<commit_message>
Fix portfolio.xlsx: inject cached formula values so previews (Gmail etc.) render correctly
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="E1" s="2">
         <f>SUM(J8:J26)</f>
-        <v/>
+        <v>1677000.4</v>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
@@ -541,7 +541,7 @@
       </c>
       <c r="G1" s="2">
         <f>SUM(L8:L26)</f>
-        <v/>
+        <v>1632729.69</v>
       </c>
     </row>
     <row r="2">
@@ -552,7 +552,7 @@
       </c>
       <c r="E2" s="2">
         <f>SUM(M8:M26)</f>
-        <v/>
+        <v>-44270.71</v>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" s="3">
         <f>IF(E1=0,"",G1/E1-1)</f>
-        <v/>
+        <v>-0.026398747430233183</v>
       </c>
     </row>
     <row r="3">
@@ -580,7 +580,7 @@
       </c>
       <c r="E3">
         <f>COUNTIF(M8:M26,"&gt;0")</f>
-        <v/>
+        <v>3</v>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
@@ -589,7 +589,7 @@
       </c>
       <c r="G3">
         <f>COUNTIF(M8:M26,"&lt;0")</f>
-        <v/>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -600,7 +600,7 @@
       </c>
       <c r="E4" s="3">
         <f>IF((E3+G3)=0,"",E3/(E3+G3))</f>
-        <v/>
+        <v>0.17647058823529413</v>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
@@ -609,7 +609,7 @@
       </c>
       <c r="G4" s="3">
         <f>AVERAGE(N8:N26)</f>
-        <v/>
+        <v>-0.026417719954767188</v>
       </c>
     </row>
     <row r="5">
@@ -618,18 +618,18 @@
           <t>Best Stock</t>
         </is>
       </c>
-      <c r="E5">
+      <c r="E5" t="str">
         <f>INDEX(B8:B26,MATCH(MAX(N8:N26),N8:N26,0))</f>
-        <v/>
+        <v>Black Box Limited</v>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
           <t>Worst Stock</t>
         </is>
       </c>
-      <c r="G5">
+      <c r="G5" t="str">
         <f>INDEX(B8:B26,MATCH(MIN(N8:N26),N8:N26,0))</f>
-        <v/>
+        <v>Lloyds Enterprises Limited</v>
       </c>
     </row>
     <row r="6">
@@ -640,7 +640,7 @@
       </c>
       <c r="E6" s="3">
         <f>AVERAGEIF(D8:D26,"4★*",N8:N26)</f>
-        <v/>
+        <v>-0.031129725497468865</v>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
@@ -649,7 +649,7 @@
       </c>
       <c r="G6" s="3">
         <f>AVERAGEIF(D8:D26,"5★*",N8:N26)</f>
-        <v/>
+        <v>-0.021116713719227798</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
@@ -774,34 +774,34 @@
       </c>
       <c r="I8" s="6">
         <f>IF(H8="","",ROUNDDOWN($B$1/H8,0))</f>
-        <v/>
+        <v>332</v>
       </c>
       <c r="J8" s="9">
         <f>IF(H8="","",H8*I8)</f>
-        <v/>
+        <v>99851.29</v>
       </c>
       <c r="K8" s="9" t="n">
         <v>299.45</v>
       </c>
       <c r="L8" s="9">
         <f>IF(OR(I8="",K8=""),"",K8*I8)</f>
-        <v/>
+        <v>99417.4</v>
       </c>
       <c r="M8" s="9">
         <f>IF(L8="","",L8-J8)</f>
-        <v/>
+        <v>-433.89</v>
       </c>
       <c r="N8" s="10">
         <f>IF(OR(H8="",K8=""),"",K8/H8-1)</f>
-        <v/>
+        <v>-0.004345396448882322</v>
       </c>
       <c r="O8" s="6">
         <f>IF(G8="","",$B$3-G8)</f>
-        <v/>
-      </c>
-      <c r="P8" s="6">
+        <v>4</v>
+      </c>
+      <c r="P8" s="6" t="str">
         <f>IF(H8="","Pending buy",IF(N8&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>In loss</v>
       </c>
       <c r="Q8" s="6" t="n">
         <v>2</v>
@@ -842,34 +842,34 @@
       </c>
       <c r="I9" s="6">
         <f>IF(H9="","",ROUNDDOWN($B$1/H9,0))</f>
-        <v/>
+        <v>53</v>
       </c>
       <c r="J9" s="9">
         <f>IF(H9="","",H9*I9)</f>
-        <v/>
+        <v>98177.53</v>
       </c>
       <c r="K9" s="9" t="n">
         <v>1764.4</v>
       </c>
       <c r="L9" s="9">
         <f>IF(OR(I9="",K9=""),"",K9*I9)</f>
-        <v/>
+        <v>93513.2</v>
       </c>
       <c r="M9" s="9">
         <f>IF(L9="","",L9-J9)</f>
-        <v/>
+        <v>-4664.33</v>
       </c>
       <c r="N9" s="10">
         <f>IF(OR(H9="",K9=""),"",K9/H9-1)</f>
-        <v/>
+        <v>-0.04750917045851566</v>
       </c>
       <c r="O9" s="6">
         <f>IF(G9="","",$B$3-G9)</f>
-        <v/>
-      </c>
-      <c r="P9" s="6">
+        <v>3</v>
+      </c>
+      <c r="P9" s="6" t="str">
         <f>IF(H9="","Pending buy",IF(N9&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>In loss</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>1</v>
@@ -910,34 +910,34 @@
       </c>
       <c r="I10" s="6">
         <f>IF(H10="","",ROUNDDOWN($B$1/H10,0))</f>
-        <v/>
+        <v>63</v>
       </c>
       <c r="J10" s="9">
         <f>IF(H10="","",H10*I10)</f>
-        <v/>
+        <v>99607.14</v>
       </c>
       <c r="K10" s="9" t="n">
         <v>1563.7</v>
       </c>
       <c r="L10" s="9">
         <f>IF(OR(I10="",K10=""),"",K10*I10)</f>
-        <v/>
+        <v>98513.1</v>
       </c>
       <c r="M10" s="9">
         <f>IF(L10="","",L10-J10)</f>
-        <v/>
+        <v>-1094.04</v>
       </c>
       <c r="N10" s="10">
         <f>IF(OR(H10="",K10=""),"",K10/H10-1)</f>
-        <v/>
+        <v>-0.010983559178772029</v>
       </c>
       <c r="O10" s="6">
         <f>IF(G10="","",$B$3-G10)</f>
-        <v/>
-      </c>
-      <c r="P10" s="6">
+        <v>3</v>
+      </c>
+      <c r="P10" s="6" t="str">
         <f>IF(H10="","Pending buy",IF(N10&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>In loss</v>
       </c>
       <c r="Q10" s="6" t="n">
         <v>1</v>
@@ -978,34 +978,34 @@
       </c>
       <c r="I11" s="6">
         <f>IF(H11="","",ROUNDDOWN($B$1/H11,0))</f>
-        <v/>
+        <v>1251</v>
       </c>
       <c r="J11" s="9">
         <f>IF(H11="","",H11*I11)</f>
-        <v/>
+        <v>99927.23</v>
       </c>
       <c r="K11" s="9" t="n">
         <v>73.73</v>
       </c>
       <c r="L11" s="9">
         <f>IF(OR(I11="",K11=""),"",K11*I11)</f>
-        <v/>
+        <v>92236.23</v>
       </c>
       <c r="M11" s="9">
         <f>IF(L11="","",L11-J11)</f>
-        <v/>
+        <v>-7691.0</v>
       </c>
       <c r="N11" s="10">
         <f>IF(OR(H11="",K11=""),"",K11/H11-1)</f>
-        <v/>
+        <v>-0.07696601169269857</v>
       </c>
       <c r="O11" s="6">
         <f>IF(G11="","",$B$3-G11)</f>
-        <v/>
-      </c>
-      <c r="P11" s="6">
+        <v>3</v>
+      </c>
+      <c r="P11" s="6" t="str">
         <f>IF(H11="","Pending buy",IF(N11&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>In loss</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>1</v>
@@ -1046,34 +1046,34 @@
       </c>
       <c r="I12" s="6">
         <f>IF(H12="","",ROUNDDOWN($B$1/H12,0))</f>
-        <v/>
+        <v>306</v>
       </c>
       <c r="J12" s="9">
         <f>IF(H12="","",H12*I12)</f>
-        <v/>
+        <v>99687.42</v>
       </c>
       <c r="K12" s="9" t="n">
         <v>323.45</v>
       </c>
       <c r="L12" s="9">
         <f>IF(OR(I12="",K12=""),"",K12*I12)</f>
-        <v/>
+        <v>98975.7</v>
       </c>
       <c r="M12" s="9">
         <f>IF(L12="","",L12-J12)</f>
-        <v/>
+        <v>-711.72</v>
       </c>
       <c r="N12" s="10">
         <f>IF(OR(H12="",K12=""),"",K12/H12-1)</f>
-        <v/>
+        <v>-0.007139518673332956</v>
       </c>
       <c r="O12" s="6">
         <f>IF(G12="","",$B$3-G12)</f>
-        <v/>
-      </c>
-      <c r="P12" s="6">
+        <v>3</v>
+      </c>
+      <c r="P12" s="6" t="str">
         <f>IF(H12="","Pending buy",IF(N12&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>In loss</v>
       </c>
       <c r="Q12" s="6" t="n">
         <v>1</v>
@@ -1114,34 +1114,34 @@
       </c>
       <c r="I13" s="6">
         <f>IF(H13="","",ROUNDDOWN($B$1/H13,0))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="J13" s="9">
         <f>IF(H13="","",H13*I13)</f>
-        <v/>
+        <v>86537.12</v>
       </c>
       <c r="K13" s="9" t="n">
         <v>20890</v>
       </c>
       <c r="L13" s="9">
         <f>IF(OR(I13="",K13=""),"",K13*I13)</f>
-        <v/>
+        <v>83560.0</v>
       </c>
       <c r="M13" s="9">
         <f>IF(L13="","",L13-J13)</f>
-        <v/>
+        <v>-2977.12</v>
       </c>
       <c r="N13" s="10">
         <f>IF(OR(H13="",K13=""),"",K13/H13-1)</f>
-        <v/>
+        <v>-0.03440276580494794</v>
       </c>
       <c r="O13" s="6">
         <f>IF(G13="","",$B$3-G13)</f>
-        <v/>
-      </c>
-      <c r="P13" s="6">
+        <v>3</v>
+      </c>
+      <c r="P13" s="6" t="str">
         <f>IF(H13="","Pending buy",IF(N13&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>In loss</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>1</v>
@@ -1182,34 +1182,34 @@
       </c>
       <c r="I14" s="6">
         <f>IF(H14="","",ROUNDDOWN($B$1/H14,0))</f>
-        <v/>
+        <v>22</v>
       </c>
       <c r="J14" s="9">
         <f>IF(H14="","",H14*I14)</f>
-        <v/>
+        <v>97667.46</v>
       </c>
       <c r="K14" s="9" t="n">
         <v>4550</v>
       </c>
       <c r="L14" s="9">
         <f>IF(OR(I14="",K14=""),"",K14*I14)</f>
-        <v/>
+        <v>100100.0</v>
       </c>
       <c r="M14" s="9">
         <f>IF(L14="","",L14-J14)</f>
-        <v/>
+        <v>2432.54</v>
       </c>
       <c r="N14" s="10">
         <f>IF(OR(H14="",K14=""),"",K14/H14-1)</f>
-        <v/>
+        <v>0.02490630672581884</v>
       </c>
       <c r="O14" s="6">
         <f>IF(G14="","",$B$3-G14)</f>
-        <v/>
-      </c>
-      <c r="P14" s="6">
+        <v>3</v>
+      </c>
+      <c r="P14" s="6" t="str">
         <f>IF(H14="","Pending buy",IF(N14&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>In profit</v>
       </c>
       <c r="Q14" s="6" t="n">
         <v>1</v>
@@ -1250,34 +1250,34 @@
       </c>
       <c r="I15" s="6">
         <f>IF(H15="","",ROUNDDOWN($B$1/H15,0))</f>
-        <v/>
+        <v>663</v>
       </c>
       <c r="J15" s="9">
         <f>IF(H15="","",H15*I15)</f>
-        <v/>
+        <v>99993.07</v>
       </c>
       <c r="K15" s="9" t="n">
         <v>142.67</v>
       </c>
       <c r="L15" s="9">
         <f>IF(OR(I15="",K15=""),"",K15*I15)</f>
-        <v/>
+        <v>94590.21</v>
       </c>
       <c r="M15" s="9">
         <f>IF(L15="","",L15-J15)</f>
-        <v/>
+        <v>-5402.86</v>
       </c>
       <c r="N15" s="10">
         <f>IF(OR(H15="",K15=""),"",K15/H15-1)</f>
-        <v/>
+        <v>-0.05403229987384306</v>
       </c>
       <c r="O15" s="6">
         <f>IF(G15="","",$B$3-G15)</f>
-        <v/>
-      </c>
-      <c r="P15" s="6">
+        <v>2</v>
+      </c>
+      <c r="P15" s="6" t="str">
         <f>IF(H15="","Pending buy",IF(N15&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>In loss</v>
       </c>
       <c r="Q15" s="6" t="n">
         <v>1</v>
@@ -1318,34 +1318,34 @@
       </c>
       <c r="I16" s="6">
         <f>IF(H16="","",ROUNDDOWN($B$1/H16,0))</f>
-        <v/>
+        <v>141</v>
       </c>
       <c r="J16" s="9">
         <f>IF(H16="","",H16*I16)</f>
-        <v/>
+        <v>99596.83</v>
       </c>
       <c r="K16" s="9" t="n">
         <v>656.65</v>
       </c>
       <c r="L16" s="9">
         <f>IF(OR(I16="",K16=""),"",K16*I16)</f>
-        <v/>
+        <v>92587.65</v>
       </c>
       <c r="M16" s="9">
         <f>IF(L16="","",L16-J16)</f>
-        <v/>
+        <v>-7009.18</v>
       </c>
       <c r="N16" s="10">
         <f>IF(OR(H16="",K16=""),"",K16/H16-1)</f>
-        <v/>
+        <v>-0.07037557586969878</v>
       </c>
       <c r="O16" s="6">
         <f>IF(G16="","",$B$3-G16)</f>
-        <v/>
-      </c>
-      <c r="P16" s="6">
+        <v>2</v>
+      </c>
+      <c r="P16" s="6" t="str">
         <f>IF(H16="","Pending buy",IF(N16&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>In loss</v>
       </c>
       <c r="Q16" s="6" t="n">
         <v>1</v>
@@ -1386,34 +1386,34 @@
       </c>
       <c r="I17" s="6">
         <f>IF(H17="","",ROUNDDOWN($B$1/H17,0))</f>
-        <v/>
+        <v>477</v>
       </c>
       <c r="J17" s="9">
         <f>IF(H17="","",H17*I17)</f>
-        <v/>
+        <v>99896.43</v>
       </c>
       <c r="K17" s="9" t="n">
         <v>200.45</v>
       </c>
       <c r="L17" s="9">
         <f>IF(OR(I17="",K17=""),"",K17*I17)</f>
-        <v/>
+        <v>95614.65</v>
       </c>
       <c r="M17" s="9">
         <f>IF(L17="","",L17-J17)</f>
-        <v/>
+        <v>-4281.78</v>
       </c>
       <c r="N17" s="10">
         <f>IF(OR(H17="",K17=""),"",K17/H17-1)</f>
-        <v/>
+        <v>-0.04286219243012823</v>
       </c>
       <c r="O17" s="6">
         <f>IF(G17="","",$B$3-G17)</f>
-        <v/>
-      </c>
-      <c r="P17" s="6">
+        <v>2</v>
+      </c>
+      <c r="P17" s="6" t="str">
         <f>IF(H17="","Pending buy",IF(N17&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>In loss</v>
       </c>
       <c r="Q17" s="6" t="n">
         <v>1</v>
@@ -1454,34 +1454,34 @@
       </c>
       <c r="I18" s="6">
         <f>IF(H18="","",ROUNDDOWN($B$1/H18,0))</f>
-        <v/>
+        <v>115</v>
       </c>
       <c r="J18" s="9">
         <f>IF(H18="","",H18*I18)</f>
-        <v/>
+        <v>99714.35</v>
       </c>
       <c r="K18" s="9" t="n">
         <v>892.1</v>
       </c>
       <c r="L18" s="9">
         <f>IF(OR(I18="",K18=""),"",K18*I18)</f>
-        <v/>
+        <v>102591.5</v>
       </c>
       <c r="M18" s="9">
         <f>IF(L18="","",L18-J18)</f>
-        <v/>
+        <v>2877.15</v>
       </c>
       <c r="N18" s="10">
         <f>IF(OR(H18="",K18=""),"",K18/H18-1)</f>
-        <v/>
+        <v>0.028853920452130977</v>
       </c>
       <c r="O18" s="6">
         <f>IF(G18="","",$B$3-G18)</f>
-        <v/>
-      </c>
-      <c r="P18" s="6">
+        <v>2</v>
+      </c>
+      <c r="P18" s="6" t="str">
         <f>IF(H18="","Pending buy",IF(N18&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>In profit</v>
       </c>
       <c r="Q18" s="6" t="n">
         <v>1</v>
@@ -1522,34 +1522,34 @@
       </c>
       <c r="I19" s="6">
         <f>IF(H19="","",ROUNDDOWN($B$1/H19,0))</f>
-        <v/>
+        <v>145</v>
       </c>
       <c r="J19" s="9">
         <f>IF(H19="","",H19*I19)</f>
-        <v/>
+        <v>99486.88</v>
       </c>
       <c r="K19" s="9" t="n">
         <v>654.85</v>
       </c>
       <c r="L19" s="9">
         <f>IF(OR(I19="",K19=""),"",K19*I19)</f>
-        <v/>
+        <v>94953.25</v>
       </c>
       <c r="M19" s="9">
         <f>IF(L19="","",L19-J19)</f>
-        <v/>
+        <v>-4533.63</v>
       </c>
       <c r="N19" s="10">
         <f>IF(OR(H19="",K19=""),"",K19/H19-1)</f>
-        <v/>
+        <v>-0.04557014086451927</v>
       </c>
       <c r="O19" s="6">
         <f>IF(G19="","",$B$3-G19)</f>
-        <v/>
-      </c>
-      <c r="P19" s="6">
+        <v>2</v>
+      </c>
+      <c r="P19" s="6" t="str">
         <f>IF(H19="","Pending buy",IF(N19&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>In loss</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>1</v>
@@ -1590,34 +1590,34 @@
       </c>
       <c r="I20" s="6">
         <f>IF(H20="","",ROUNDDOWN($B$1/H20,0))</f>
-        <v/>
+        <v>71</v>
       </c>
       <c r="J20" s="9">
         <f>IF(H20="","",H20*I20)</f>
-        <v/>
+        <v>99449.47</v>
       </c>
       <c r="K20" s="9" t="n">
         <v>1320</v>
       </c>
       <c r="L20" s="9">
         <f>IF(OR(I20="",K20=""),"",K20*I20)</f>
-        <v/>
+        <v>93720.0</v>
       </c>
       <c r="M20" s="9">
         <f>IF(L20="","",L20-J20)</f>
-        <v/>
+        <v>-5729.47</v>
       </c>
       <c r="N20" s="10">
         <f>IF(OR(H20="",K20=""),"",K20/H20-1)</f>
-        <v/>
+        <v>-0.057611835939567424</v>
       </c>
       <c r="O20" s="6">
         <f>IF(G20="","",$B$3-G20)</f>
-        <v/>
-      </c>
-      <c r="P20" s="6">
+        <v>2</v>
+      </c>
+      <c r="P20" s="6" t="str">
         <f>IF(H20="","Pending buy",IF(N20&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>In loss</v>
       </c>
       <c r="Q20" s="6" t="n">
         <v>1</v>
@@ -1658,34 +1658,34 @@
       </c>
       <c r="I21" s="6">
         <f>IF(H21="","",ROUNDDOWN($B$1/H21,0))</f>
-        <v/>
+        <v>144</v>
       </c>
       <c r="J21" s="9">
         <f>IF(H21="","",H21*I21)</f>
-        <v/>
+        <v>99837.05</v>
       </c>
       <c r="K21" s="9" t="n">
         <v>697.1</v>
       </c>
       <c r="L21" s="9">
         <f>IF(OR(I21="",K21=""),"",K21*I21)</f>
-        <v/>
+        <v>100382.4</v>
       </c>
       <c r="M21" s="9">
         <f>IF(L21="","",L21-J21)</f>
-        <v/>
+        <v>545.35</v>
       </c>
       <c r="N21" s="10">
         <f>IF(OR(H21="",K21=""),"",K21/H21-1)</f>
-        <v/>
+        <v>0.005462389702842074</v>
       </c>
       <c r="O21" s="6">
         <f>IF(G21="","",$B$3-G21)</f>
-        <v/>
-      </c>
-      <c r="P21" s="6">
+        <v>2</v>
+      </c>
+      <c r="P21" s="6" t="str">
         <f>IF(H21="","Pending buy",IF(N21&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>In profit</v>
       </c>
       <c r="Q21" s="6" t="n">
         <v>1</v>
@@ -1726,34 +1726,34 @@
       </c>
       <c r="I22" s="6">
         <f>IF(H22="","",ROUNDDOWN($B$1/H22,0))</f>
-        <v/>
+        <v>68</v>
       </c>
       <c r="J22" s="9">
         <f>IF(H22="","",H22*I22)</f>
-        <v/>
+        <v>98557.54</v>
       </c>
       <c r="K22" s="9" t="n">
         <v>1434.4</v>
       </c>
       <c r="L22" s="9">
         <f>IF(OR(I22="",K22=""),"",K22*I22)</f>
-        <v/>
+        <v>97539.2</v>
       </c>
       <c r="M22" s="9">
         <f>IF(L22="","",L22-J22)</f>
-        <v/>
+        <v>-1018.34</v>
       </c>
       <c r="N22" s="10">
         <f>IF(OR(H22="",K22=""),"",K22/H22-1)</f>
-        <v/>
+        <v>-0.01033240634859689</v>
       </c>
       <c r="O22" s="6">
         <f>IF(G22="","",$B$3-G22)</f>
-        <v/>
-      </c>
-      <c r="P22" s="6">
+        <v>2</v>
+      </c>
+      <c r="P22" s="6" t="str">
         <f>IF(H22="","Pending buy",IF(N22&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>In loss</v>
       </c>
       <c r="Q22" s="6" t="n">
         <v>2</v>
@@ -1794,34 +1794,34 @@
       </c>
       <c r="I23" s="6">
         <f>IF(H23="","",ROUNDDOWN($B$1/H23,0))</f>
-        <v/>
+        <v>64</v>
       </c>
       <c r="J23" s="9">
         <f>IF(H23="","",H23*I23)</f>
-        <v/>
+        <v>99078.19</v>
       </c>
       <c r="K23" s="9" t="n">
         <v>1479.6</v>
       </c>
       <c r="L23" s="9">
         <f>IF(OR(I23="",K23=""),"",K23*I23)</f>
-        <v/>
+        <v>94694.4</v>
       </c>
       <c r="M23" s="9">
         <f>IF(L23="","",L23-J23)</f>
-        <v/>
+        <v>-4383.79</v>
       </c>
       <c r="N23" s="10">
         <f>IF(OR(H23="",K23=""),"",K23/H23-1)</f>
-        <v/>
+        <v>-0.04424573855151881</v>
       </c>
       <c r="O23" s="6">
         <f>IF(G23="","",$B$3-G23)</f>
-        <v/>
-      </c>
-      <c r="P23" s="6">
+        <v>2</v>
+      </c>
+      <c r="P23" s="6" t="str">
         <f>IF(H23="","Pending buy",IF(N23&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>In loss</v>
       </c>
       <c r="Q23" s="6" t="n">
         <v>1</v>
@@ -1862,34 +1862,34 @@
       </c>
       <c r="I24" s="6">
         <f>IF(H24="","",ROUNDDOWN($B$1/H24,0))</f>
-        <v/>
+        <v>439</v>
       </c>
       <c r="J24" s="9">
         <f>IF(H24="","",H24*I24)</f>
-        <v/>
+        <v>99935.4</v>
       </c>
       <c r="K24" s="9" t="n">
         <v>227.2</v>
       </c>
       <c r="L24" s="9">
         <f>IF(OR(I24="",K24=""),"",K24*I24)</f>
-        <v/>
+        <v>99740.8</v>
       </c>
       <c r="M24" s="9">
         <f>IF(L24="","",L24-J24)</f>
-        <v/>
+        <v>-194.6</v>
       </c>
       <c r="N24" s="10">
         <f>IF(OR(H24="",K24=""),"",K24/H24-1)</f>
-        <v/>
+        <v>-0.0019472439768121186</v>
       </c>
       <c r="O24" s="6">
         <f>IF(G24="","",$B$3-G24)</f>
-        <v/>
-      </c>
-      <c r="P24" s="6">
+        <v>1</v>
+      </c>
+      <c r="P24" s="6" t="str">
         <f>IF(H24="","Pending buy",IF(N24&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>In loss</v>
       </c>
       <c r="Q24" s="6" t="n">
         <v>1</v>
@@ -1924,36 +1924,36 @@
       </c>
       <c r="G25" s="6" t="inlineStr"/>
       <c r="H25" s="9" t="inlineStr"/>
-      <c r="I25" s="6">
+      <c r="I25" s="6" t="str">
         <f>IF(H25="","",ROUNDDOWN($B$1/H25,0))</f>
         <v/>
       </c>
-      <c r="J25" s="9">
+      <c r="J25" s="9" t="str">
         <f>IF(H25="","",H25*I25)</f>
         <v/>
       </c>
       <c r="K25" s="9" t="n">
         <v>214.94</v>
       </c>
-      <c r="L25" s="9">
+      <c r="L25" s="9" t="str">
         <f>IF(OR(I25="",K25=""),"",K25*I25)</f>
         <v/>
       </c>
-      <c r="M25" s="9">
+      <c r="M25" s="9" t="str">
         <f>IF(L25="","",L25-J25)</f>
         <v/>
       </c>
-      <c r="N25" s="10">
+      <c r="N25" s="10" t="str">
         <f>IF(OR(H25="",K25=""),"",K25/H25-1)</f>
         <v/>
       </c>
-      <c r="O25" s="6">
+      <c r="O25" s="6" t="str">
         <f>IF(G25="","",$B$3-G25)</f>
         <v/>
       </c>
-      <c r="P25" s="6">
+      <c r="P25" s="6" t="str">
         <f>IF(H25="","Pending buy",IF(N25&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>Pending buy</v>
       </c>
       <c r="Q25" s="6" t="n">
         <v>1</v>
@@ -1988,36 +1988,36 @@
       </c>
       <c r="G26" s="6" t="inlineStr"/>
       <c r="H26" s="9" t="inlineStr"/>
-      <c r="I26" s="6">
+      <c r="I26" s="6" t="str">
         <f>IF(H26="","",ROUNDDOWN($B$1/H26,0))</f>
         <v/>
       </c>
-      <c r="J26" s="9">
+      <c r="J26" s="9" t="str">
         <f>IF(H26="","",H26*I26)</f>
         <v/>
       </c>
       <c r="K26" s="9" t="n">
         <v>788.4</v>
       </c>
-      <c r="L26" s="9">
+      <c r="L26" s="9" t="str">
         <f>IF(OR(I26="",K26=""),"",K26*I26)</f>
         <v/>
       </c>
-      <c r="M26" s="9">
+      <c r="M26" s="9" t="str">
         <f>IF(L26="","",L26-J26)</f>
         <v/>
       </c>
-      <c r="N26" s="10">
+      <c r="N26" s="10" t="str">
         <f>IF(OR(H26="",K26=""),"",K26/H26-1)</f>
         <v/>
       </c>
-      <c r="O26" s="6">
+      <c r="O26" s="6" t="str">
         <f>IF(G26="","",$B$3-G26)</f>
         <v/>
       </c>
-      <c r="P26" s="6">
+      <c r="P26" s="6" t="str">
         <f>IF(H26="","Pending buy",IF(N26&gt;=0,"In profit","In loss"))</f>
-        <v/>
+        <v>Pending buy</v>
       </c>
       <c r="Q26" s="6" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Momentum Portfolio: weekday silent update 2026-10-12
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q26"/>
+  <dimension ref="A1:Q30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -531,8 +531,8 @@
         </is>
       </c>
       <c r="E1" s="2">
-        <f>SUM(J8:J26)</f>
-        <v>1677000.4</v>
+        <f>SUM(J8:J30)</f>
+        <v>1876571.21</v>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
@@ -540,8 +540,8 @@
         </is>
       </c>
       <c r="G1" s="2">
-        <f>SUM(L8:L26)</f>
-        <v>1632729.69</v>
+        <f>SUM(L8:L30)</f>
+        <v>1851612.03</v>
       </c>
     </row>
     <row r="2">
@@ -551,8 +551,8 @@
         </is>
       </c>
       <c r="E2" s="2">
-        <f>SUM(M8:M26)</f>
-        <v>-44270.71</v>
+        <f>SUM(M8:M30)</f>
+        <v>-24959.18</v>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" s="3">
         <f>IF(E1=0,"",G1/E1-1)</f>
-        <v>-0.026398747430233183</v>
+        <v>-0.013300417200794556</v>
       </c>
     </row>
     <row r="3">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -579,8 +579,8 @@
         </is>
       </c>
       <c r="E3">
-        <f>COUNTIF(M8:M26,"&gt;0")</f>
-        <v>3</v>
+        <f>COUNTIF(M8:M30,"&gt;0")</f>
+        <v>7</v>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
@@ -588,8 +588,8 @@
         </is>
       </c>
       <c r="G3">
-        <f>COUNTIF(M8:M26,"&lt;0")</f>
-        <v>14</v>
+        <f>COUNTIF(M8:M30,"&lt;0")</f>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -600,7 +600,7 @@
       </c>
       <c r="E4" s="3">
         <f>IF((E3+G3)=0,"",E3/(E3+G3))</f>
-        <v>0.17647058823529413</v>
+        <v>0.3684210526315789</v>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
@@ -608,8 +608,8 @@
         </is>
       </c>
       <c r="G4" s="3">
-        <f>AVERAGE(N8:N26)</f>
-        <v>-0.026417719954767188</v>
+        <f>AVERAGE(N8:N30)</f>
+        <v>-0.013460471821825047</v>
       </c>
     </row>
     <row r="5">
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="E5" t="str">
-        <f>INDEX(B8:B26,MATCH(MAX(N8:N26),N8:N26,0))</f>
+        <f>INDEX(B8:B30,MATCH(MAX(N8:N30),N8:N30,0))</f>
         <v>Black Box Limited</v>
       </c>
       <c r="F5" s="1" t="inlineStr">
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="G5" t="str">
-        <f>INDEX(B8:B26,MATCH(MIN(N8:N26),N8:N26,0))</f>
+        <f>INDEX(B8:B30,MATCH(MIN(N8:N30),N8:N30,0))</f>
         <v>Lloyds Enterprises Limited</v>
       </c>
     </row>
@@ -639,8 +639,8 @@
         </is>
       </c>
       <c r="E6" s="3">
-        <f>AVERAGEIF(D8:D26,"4★*",N8:N26)</f>
-        <v>-0.031129725497468865</v>
+        <f>AVERAGEIF(D8:D30,"4★*",N8:N30)</f>
+        <v>-0.01311486671352505</v>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
@@ -648,8 +648,8 @@
         </is>
       </c>
       <c r="G6" s="3">
-        <f>AVERAGEIF(D8:D26,"5★*",N8:N26)</f>
-        <v>-0.021116713719227798</v>
+        <f>AVERAGEIF(D8:D30,"5★*",N8:N30)</f>
+        <v>-0.013935678845737542</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
@@ -781,27 +781,27 @@
         <v>99851.29</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>299.45</v>
+        <v>312.2</v>
       </c>
       <c r="L8" s="9">
         <f>IF(OR(I8="",K8=""),"",K8*I8)</f>
-        <v>99417.4</v>
+        <v>103650.4</v>
       </c>
       <c r="M8" s="9">
         <f>IF(L8="","",L8-J8)</f>
-        <v>-433.89</v>
+        <v>3799.11</v>
       </c>
       <c r="N8" s="10">
         <f>IF(OR(H8="",K8=""),"",K8/H8-1)</f>
-        <v>-0.004345396448882322</v>
+        <v>0.038047644777622125</v>
       </c>
       <c r="O8" s="6">
         <f>IF(G8="","",$B$3-G8)</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="P8" s="6" t="str">
         <f>IF(H8="","Pending buy",IF(N8&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q8" s="6" t="n">
         <v>2</v>
@@ -849,23 +849,23 @@
         <v>99687.42</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>323.45</v>
+        <v>323</v>
       </c>
       <c r="L9" s="9">
         <f>IF(OR(I9="",K9=""),"",K9*I9)</f>
-        <v>98975.7</v>
+        <v>98838.0</v>
       </c>
       <c r="M9" s="9">
         <f>IF(L9="","",L9-J9)</f>
-        <v>-711.72</v>
+        <v>-849.42</v>
       </c>
       <c r="N9" s="10">
         <f>IF(OR(H9="",K9=""),"",K9/H9-1)</f>
-        <v>-0.007139518673332956</v>
+        <v>-0.008520836393527742</v>
       </c>
       <c r="O9" s="6">
         <f>IF(G9="","",$B$3-G9)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P9" s="6" t="str">
         <f>IF(H9="","Pending buy",IF(N9&gt;=0,"In profit","In loss"))</f>
@@ -917,23 +917,23 @@
         <v>99607.14</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>1563.7</v>
+        <v>1563.1</v>
       </c>
       <c r="L10" s="9">
         <f>IF(OR(I10="",K10=""),"",K10*I10)</f>
-        <v>98513.1</v>
+        <v>98475.3</v>
       </c>
       <c r="M10" s="9">
         <f>IF(L10="","",L10-J10)</f>
-        <v>-1094.04</v>
+        <v>-1131.84</v>
       </c>
       <c r="N10" s="10">
         <f>IF(OR(H10="",K10=""),"",K10/H10-1)</f>
-        <v>-0.010983559178772029</v>
+        <v>-0.011363050043063705</v>
       </c>
       <c r="O10" s="6">
         <f>IF(G10="","",$B$3-G10)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P10" s="6" t="str">
         <f>IF(H10="","Pending buy",IF(N10&gt;=0,"In profit","In loss"))</f>
@@ -985,23 +985,23 @@
         <v>99927.23</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>73.73</v>
+        <v>71.56</v>
       </c>
       <c r="L11" s="9">
         <f>IF(OR(I11="",K11=""),"",K11*I11)</f>
-        <v>92236.23</v>
+        <v>89521.56</v>
       </c>
       <c r="M11" s="9">
         <f>IF(L11="","",L11-J11)</f>
-        <v>-7691.0</v>
+        <v>-10405.67</v>
       </c>
       <c r="N11" s="10">
         <f>IF(OR(H11="",K11=""),"",K11/H11-1)</f>
-        <v>-0.07696601169269857</v>
+        <v>-0.10413248062836711</v>
       </c>
       <c r="O11" s="6">
         <f>IF(G11="","",$B$3-G11)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P11" s="6" t="str">
         <f>IF(H11="","Pending buy",IF(N11&gt;=0,"In profit","In loss"))</f>
@@ -1053,23 +1053,23 @@
         <v>86537.12</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>20890</v>
+        <v>20565</v>
       </c>
       <c r="L12" s="9">
         <f>IF(OR(I12="",K12=""),"",K12*I12)</f>
-        <v>83560.0</v>
+        <v>82260.0</v>
       </c>
       <c r="M12" s="9">
         <f>IF(L12="","",L12-J12)</f>
-        <v>-2977.12</v>
+        <v>-4277.12</v>
       </c>
       <c r="N12" s="10">
         <f>IF(OR(H12="",K12=""),"",K12/H12-1)</f>
-        <v>-0.03440276580494794</v>
+        <v>-0.04942522157868612</v>
       </c>
       <c r="O12" s="6">
         <f>IF(G12="","",$B$3-G12)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P12" s="6" t="str">
         <f>IF(H12="","Pending buy",IF(N12&gt;=0,"In profit","In loss"))</f>
@@ -1121,27 +1121,27 @@
         <v>98177.53</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>1764.4</v>
+        <v>1868.8</v>
       </c>
       <c r="L13" s="9">
         <f>IF(OR(I13="",K13=""),"",K13*I13)</f>
-        <v>93513.2</v>
+        <v>99046.4</v>
       </c>
       <c r="M13" s="9">
         <f>IF(L13="","",L13-J13)</f>
-        <v>-4664.33</v>
+        <v>868.87</v>
       </c>
       <c r="N13" s="10">
         <f>IF(OR(H13="",K13=""),"",K13/H13-1)</f>
-        <v>-0.04750917045851566</v>
+        <v>0.008849955932399567</v>
       </c>
       <c r="O13" s="6">
         <f>IF(G13="","",$B$3-G13)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P13" s="6" t="str">
         <f>IF(H13="","Pending buy",IF(N13&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>1</v>
@@ -1189,23 +1189,23 @@
         <v>97667.46</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>4550</v>
+        <v>4555</v>
       </c>
       <c r="L14" s="9">
         <f>IF(OR(I14="",K14=""),"",K14*I14)</f>
-        <v>100100.0</v>
+        <v>100210.0</v>
       </c>
       <c r="M14" s="9">
         <f>IF(L14="","",L14-J14)</f>
-        <v>2432.54</v>
+        <v>2542.54</v>
       </c>
       <c r="N14" s="10">
         <f>IF(OR(H14="",K14=""),"",K14/H14-1)</f>
-        <v>0.02490630672581884</v>
+        <v>0.026032577392550493</v>
       </c>
       <c r="O14" s="6">
         <f>IF(G14="","",$B$3-G14)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P14" s="6" t="str">
         <f>IF(H14="","Pending buy",IF(N14&gt;=0,"In profit","In loss"))</f>
@@ -1257,30 +1257,30 @@
         <v>99078.19</v>
       </c>
       <c r="K15" s="9" t="n">
-        <v>1479.6</v>
+        <v>1540.2</v>
       </c>
       <c r="L15" s="9">
         <f>IF(OR(I15="",K15=""),"",K15*I15)</f>
-        <v>94694.4</v>
+        <v>98572.8</v>
       </c>
       <c r="M15" s="9">
         <f>IF(L15="","",L15-J15)</f>
-        <v>-4383.79</v>
+        <v>-505.39</v>
       </c>
       <c r="N15" s="10">
         <f>IF(OR(H15="",K15=""),"",K15/H15-1)</f>
-        <v>-0.04424573855151881</v>
+        <v>-0.005100896537610922</v>
       </c>
       <c r="O15" s="6">
         <f>IF(G15="","",$B$3-G15)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P15" s="6" t="str">
         <f>IF(H15="","Pending buy",IF(N15&gt;=0,"In profit","In loss"))</f>
         <v>In loss</v>
       </c>
       <c r="Q15" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -1325,27 +1325,27 @@
         <v>98557.54</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>1434.4</v>
+        <v>1511</v>
       </c>
       <c r="L16" s="9">
         <f>IF(OR(I16="",K16=""),"",K16*I16)</f>
-        <v>97539.2</v>
+        <v>102748.0</v>
       </c>
       <c r="M16" s="9">
         <f>IF(L16="","",L16-J16)</f>
-        <v>-1018.34</v>
+        <v>4190.46</v>
       </c>
       <c r="N16" s="10">
         <f>IF(OR(H16="",K16=""),"",K16/H16-1)</f>
-        <v>-0.01033240634859689</v>
+        <v>0.042517940607410765</v>
       </c>
       <c r="O16" s="6">
         <f>IF(G16="","",$B$3-G16)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P16" s="6" t="str">
         <f>IF(H16="","Pending buy",IF(N16&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q16" s="6" t="n">
         <v>2</v>
@@ -1393,23 +1393,23 @@
         <v>99714.35</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>892.1</v>
+        <v>924.6</v>
       </c>
       <c r="L17" s="9">
         <f>IF(OR(I17="",K17=""),"",K17*I17)</f>
-        <v>102591.5</v>
+        <v>106329.0</v>
       </c>
       <c r="M17" s="9">
         <f>IF(L17="","",L17-J17)</f>
-        <v>2877.15</v>
+        <v>6614.65</v>
       </c>
       <c r="N17" s="10">
         <f>IF(OR(H17="",K17=""),"",K17/H17-1)</f>
-        <v>0.028853920452130977</v>
+        <v>0.06633598794982665</v>
       </c>
       <c r="O17" s="6">
         <f>IF(G17="","",$B$3-G17)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P17" s="6" t="str">
         <f>IF(H17="","Pending buy",IF(N17&gt;=0,"In profit","In loss"))</f>
@@ -1461,23 +1461,23 @@
         <v>99596.83</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>656.65</v>
+        <v>640.25</v>
       </c>
       <c r="L18" s="9">
         <f>IF(OR(I18="",K18=""),"",K18*I18)</f>
-        <v>92587.65</v>
+        <v>90275.25</v>
       </c>
       <c r="M18" s="9">
         <f>IF(L18="","",L18-J18)</f>
-        <v>-7009.18</v>
+        <v>-9321.58</v>
       </c>
       <c r="N18" s="10">
         <f>IF(OR(H18="",K18=""),"",K18/H18-1)</f>
-        <v>-0.07037557586969878</v>
+        <v>-0.09359318122374871</v>
       </c>
       <c r="O18" s="6">
         <f>IF(G18="","",$B$3-G18)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P18" s="6" t="str">
         <f>IF(H18="","Pending buy",IF(N18&gt;=0,"In profit","In loss"))</f>
@@ -1529,30 +1529,30 @@
         <v>99993.07</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>142.67</v>
+        <v>146.19</v>
       </c>
       <c r="L19" s="9">
         <f>IF(OR(I19="",K19=""),"",K19*I19)</f>
-        <v>94590.21</v>
+        <v>96923.97</v>
       </c>
       <c r="M19" s="9">
         <f>IF(L19="","",L19-J19)</f>
-        <v>-5402.86</v>
+        <v>-3069.1</v>
       </c>
       <c r="N19" s="10">
         <f>IF(OR(H19="",K19=""),"",K19/H19-1)</f>
-        <v>-0.05403229987384306</v>
+        <v>-0.03069308136648985</v>
       </c>
       <c r="O19" s="6">
         <f>IF(G19="","",$B$3-G19)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P19" s="6" t="str">
         <f>IF(H19="","Pending buy",IF(N19&gt;=0,"In profit","In loss"))</f>
         <v>In loss</v>
       </c>
       <c r="Q19" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -1597,27 +1597,27 @@
         <v>99896.43</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>200.45</v>
+        <v>220.61</v>
       </c>
       <c r="L20" s="9">
         <f>IF(OR(I20="",K20=""),"",K20*I20)</f>
-        <v>95614.65</v>
+        <v>105230.97</v>
       </c>
       <c r="M20" s="9">
         <f>IF(L20="","",L20-J20)</f>
-        <v>-4281.78</v>
+        <v>5334.54</v>
       </c>
       <c r="N20" s="10">
         <f>IF(OR(H20="",K20=""),"",K20/H20-1)</f>
-        <v>-0.04286219243012823</v>
+        <v>0.053400707049086726</v>
       </c>
       <c r="O20" s="6">
         <f>IF(G20="","",$B$3-G20)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P20" s="6" t="str">
         <f>IF(H20="","Pending buy",IF(N20&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q20" s="6" t="n">
         <v>1</v>
@@ -1665,23 +1665,23 @@
         <v>99449.47</v>
       </c>
       <c r="K21" s="9" t="n">
-        <v>1320</v>
+        <v>1318.7</v>
       </c>
       <c r="L21" s="9">
         <f>IF(OR(I21="",K21=""),"",K21*I21)</f>
-        <v>93720.0</v>
+        <v>93627.7</v>
       </c>
       <c r="M21" s="9">
         <f>IF(L21="","",L21-J21)</f>
-        <v>-5729.47</v>
+        <v>-5821.77</v>
       </c>
       <c r="N21" s="10">
         <f>IF(OR(H21="",K21=""),"",K21/H21-1)</f>
-        <v>-0.057611835939567424</v>
+        <v>-0.05853994549508146</v>
       </c>
       <c r="O21" s="6">
         <f>IF(G21="","",$B$3-G21)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P21" s="6" t="str">
         <f>IF(H21="","Pending buy",IF(N21&gt;=0,"In profit","In loss"))</f>
@@ -1733,27 +1733,27 @@
         <v>99837.05</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>697.1</v>
+        <v>685.95</v>
       </c>
       <c r="L22" s="9">
         <f>IF(OR(I22="",K22=""),"",K22*I22)</f>
-        <v>100382.4</v>
+        <v>98776.8</v>
       </c>
       <c r="M22" s="9">
         <f>IF(L22="","",L22-J22)</f>
-        <v>545.35</v>
+        <v>-1060.25</v>
       </c>
       <c r="N22" s="10">
         <f>IF(OR(H22="",K22=""),"",K22/H22-1)</f>
-        <v>0.005462389702842074</v>
+        <v>-0.010619816071346322</v>
       </c>
       <c r="O22" s="6">
         <f>IF(G22="","",$B$3-G22)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P22" s="6" t="str">
         <f>IF(H22="","Pending buy",IF(N22&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q22" s="6" t="n">
         <v>1</v>
@@ -1801,23 +1801,23 @@
         <v>99486.88</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>654.85</v>
+        <v>653.3</v>
       </c>
       <c r="L23" s="9">
         <f>IF(OR(I23="",K23=""),"",K23*I23)</f>
-        <v>94953.25</v>
+        <v>94728.5</v>
       </c>
       <c r="M23" s="9">
         <f>IF(L23="","",L23-J23)</f>
-        <v>-4533.63</v>
+        <v>-4758.38</v>
       </c>
       <c r="N23" s="10">
         <f>IF(OR(H23="",K23=""),"",K23/H23-1)</f>
-        <v>-0.04557014086451927</v>
+        <v>-0.047829232689609036</v>
       </c>
       <c r="O23" s="6">
         <f>IF(G23="","",$B$3-G23)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P23" s="6" t="str">
         <f>IF(H23="","Pending buy",IF(N23&gt;=0,"In profit","In loss"))</f>
@@ -1869,23 +1869,23 @@
         <v>99935.4</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>227.2</v>
+        <v>224.32</v>
       </c>
       <c r="L24" s="9">
         <f>IF(OR(I24="",K24=""),"",K24*I24)</f>
-        <v>99740.8</v>
+        <v>98476.48</v>
       </c>
       <c r="M24" s="9">
         <f>IF(L24="","",L24-J24)</f>
-        <v>-194.6</v>
+        <v>-1458.92</v>
       </c>
       <c r="N24" s="10">
         <f>IF(OR(H24="",K24=""),"",K24/H24-1)</f>
-        <v>-0.0019472439768121186</v>
+        <v>-0.014598616940486364</v>
       </c>
       <c r="O24" s="6">
         <f>IF(G24="","",$B$3-G24)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P24" s="6" t="str">
         <f>IF(H24="","Pending buy",IF(N24&gt;=0,"In profit","In loss"))</f>
@@ -1922,38 +1922,42 @@
       <c r="F25" s="8" t="n">
         <v>46304</v>
       </c>
-      <c r="G25" s="6" t="inlineStr"/>
-      <c r="H25" s="9" t="inlineStr"/>
-      <c r="I25" s="6" t="str">
+      <c r="G25" s="8" t="n">
+        <v>46307</v>
+      </c>
+      <c r="H25" s="9" t="n">
+        <v>803.41</v>
+      </c>
+      <c r="I25" s="6">
         <f>IF(H25="","",ROUNDDOWN($B$1/H25,0))</f>
-        <v/>
-      </c>
-      <c r="J25" s="9" t="str">
+        <v>124</v>
+      </c>
+      <c r="J25" s="9">
         <f>IF(H25="","",H25*I25)</f>
-        <v/>
+        <v>99622.64</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>788.4</v>
-      </c>
-      <c r="L25" s="9" t="str">
+        <v>806.1</v>
+      </c>
+      <c r="L25" s="9">
         <f>IF(OR(I25="",K25=""),"",K25*I25)</f>
-        <v/>
-      </c>
-      <c r="M25" s="9" t="str">
+        <v>99956.4</v>
+      </c>
+      <c r="M25" s="9">
         <f>IF(L25="","",L25-J25)</f>
-        <v/>
-      </c>
-      <c r="N25" s="10" t="str">
+        <v>333.76</v>
+      </c>
+      <c r="N25" s="10">
         <f>IF(OR(H25="",K25=""),"",K25/H25-1)</f>
-        <v/>
-      </c>
-      <c r="O25" s="6" t="str">
+        <v>0.0033502788130068684</v>
+      </c>
+      <c r="O25" s="6">
         <f>IF(G25="","",$B$3-G25)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P25" s="6" t="str">
         <f>IF(H25="","Pending buy",IF(N25&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In profit</v>
       </c>
       <c r="Q25" s="6" t="n">
         <v>1</v>
@@ -1986,45 +1990,305 @@
       <c r="F26" s="8" t="n">
         <v>46304</v>
       </c>
-      <c r="G26" s="6" t="inlineStr"/>
-      <c r="H26" s="9" t="inlineStr"/>
-      <c r="I26" s="6" t="str">
+      <c r="G26" s="8" t="n">
+        <v>46307</v>
+      </c>
+      <c r="H26" s="9" t="n">
+        <v>210.42</v>
+      </c>
+      <c r="I26" s="6">
         <f>IF(H26="","",ROUNDDOWN($B$1/H26,0))</f>
-        <v/>
-      </c>
-      <c r="J26" s="9" t="str">
+        <v>475</v>
+      </c>
+      <c r="J26" s="9">
         <f>IF(H26="","",H26*I26)</f>
-        <v/>
+        <v>99948.17</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>214.94</v>
-      </c>
-      <c r="L26" s="9" t="str">
+        <v>197.82</v>
+      </c>
+      <c r="L26" s="9">
         <f>IF(OR(I26="",K26=""),"",K26*I26)</f>
-        <v/>
-      </c>
-      <c r="M26" s="9" t="str">
+        <v>93964.5</v>
+      </c>
+      <c r="M26" s="9">
         <f>IF(L26="","",L26-J26)</f>
-        <v/>
-      </c>
-      <c r="N26" s="10" t="str">
+        <v>-5983.67</v>
+      </c>
+      <c r="N26" s="10">
         <f>IF(OR(H26="",K26=""),"",K26/H26-1)</f>
-        <v/>
-      </c>
-      <c r="O26" s="6" t="str">
+        <v>-0.059867698168561745</v>
+      </c>
+      <c r="O26" s="6">
         <f>IF(G26="","",$B$3-G26)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P26" s="6" t="str">
         <f>IF(H26="","Pending buy",IF(N26&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q26" s="6" t="n">
         <v>1</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Commercial Syn Bags Limited</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>COMSYN</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>121026</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G27" s="6" t="inlineStr"/>
+      <c r="H27" s="9" t="inlineStr"/>
+      <c r="I27" s="6" t="str">
+        <f>IF(H27="","",ROUNDDOWN($B$1/H27,0))</f>
+        <v/>
+      </c>
+      <c r="J27" s="9" t="str">
+        <f>IF(H27="","",H27*I27)</f>
+        <v/>
+      </c>
+      <c r="K27" s="9" t="n">
+        <v>262.4</v>
+      </c>
+      <c r="L27" s="9" t="str">
+        <f>IF(OR(I27="",K27=""),"",K27*I27)</f>
+        <v/>
+      </c>
+      <c r="M27" s="9" t="str">
+        <f>IF(L27="","",L27-J27)</f>
+        <v/>
+      </c>
+      <c r="N27" s="10" t="str">
+        <f>IF(OR(H27="",K27=""),"",K27/H27-1)</f>
+        <v/>
+      </c>
+      <c r="O27" s="6" t="str">
+        <f>IF(G27="","",$B$3-G27)</f>
+        <v/>
+      </c>
+      <c r="P27" s="6" t="str">
+        <f>IF(H27="","Pending buy",IF(N27&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q27" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Craftsman Automation Limited</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>CRAFTSMAN</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>121026</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G28" s="6" t="inlineStr"/>
+      <c r="H28" s="9" t="inlineStr"/>
+      <c r="I28" s="6" t="str">
+        <f>IF(H28="","",ROUNDDOWN($B$1/H28,0))</f>
+        <v/>
+      </c>
+      <c r="J28" s="9" t="str">
+        <f>IF(H28="","",H28*I28)</f>
+        <v/>
+      </c>
+      <c r="K28" s="9" t="n">
+        <v>10815</v>
+      </c>
+      <c r="L28" s="9" t="str">
+        <f>IF(OR(I28="",K28=""),"",K28*I28)</f>
+        <v/>
+      </c>
+      <c r="M28" s="9" t="str">
+        <f>IF(L28="","",L28-J28)</f>
+        <v/>
+      </c>
+      <c r="N28" s="10" t="str">
+        <f>IF(OR(H28="",K28=""),"",K28/H28-1)</f>
+        <v/>
+      </c>
+      <c r="O28" s="6" t="str">
+        <f>IF(G28="","",$B$3-G28)</f>
+        <v/>
+      </c>
+      <c r="P28" s="6" t="str">
+        <f>IF(H28="","Pending buy",IF(N28&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q28" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Happy Forgings Limited</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>HAPPYFORGE</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>121026</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G29" s="6" t="inlineStr"/>
+      <c r="H29" s="9" t="inlineStr"/>
+      <c r="I29" s="6" t="str">
+        <f>IF(H29="","",ROUNDDOWN($B$1/H29,0))</f>
+        <v/>
+      </c>
+      <c r="J29" s="9" t="str">
+        <f>IF(H29="","",H29*I29)</f>
+        <v/>
+      </c>
+      <c r="K29" s="9" t="n">
+        <v>1966.3</v>
+      </c>
+      <c r="L29" s="9" t="str">
+        <f>IF(OR(I29="",K29=""),"",K29*I29)</f>
+        <v/>
+      </c>
+      <c r="M29" s="9" t="str">
+        <f>IF(L29="","",L29-J29)</f>
+        <v/>
+      </c>
+      <c r="N29" s="10" t="str">
+        <f>IF(OR(H29="",K29=""),"",K29/H29-1)</f>
+        <v/>
+      </c>
+      <c r="O29" s="6" t="str">
+        <f>IF(G29="","",$B$3-G29)</f>
+        <v/>
+      </c>
+      <c r="P29" s="6" t="str">
+        <f>IF(H29="","Pending buy",IF(N29&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q29" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Viji Finance Limited</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>VIJIFIN</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>121026</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="n">
+        <v>46307</v>
+      </c>
+      <c r="G30" s="6" t="inlineStr"/>
+      <c r="H30" s="9" t="inlineStr"/>
+      <c r="I30" s="6" t="str">
+        <f>IF(H30="","",ROUNDDOWN($B$1/H30,0))</f>
+        <v/>
+      </c>
+      <c r="J30" s="9" t="str">
+        <f>IF(H30="","",H30*I30)</f>
+        <v/>
+      </c>
+      <c r="K30" s="9" t="n">
+        <v>14.13</v>
+      </c>
+      <c r="L30" s="9" t="str">
+        <f>IF(OR(I30="",K30=""),"",K30*I30)</f>
+        <v/>
+      </c>
+      <c r="M30" s="9" t="str">
+        <f>IF(L30="","",L30-J30)</f>
+        <v/>
+      </c>
+      <c r="N30" s="10" t="str">
+        <f>IF(OR(H30="",K30=""),"",K30/H30-1)</f>
+        <v/>
+      </c>
+      <c r="O30" s="6" t="str">
+        <f>IF(G30="","",$B$3-G30)</f>
+        <v/>
+      </c>
+      <c r="P30" s="6" t="str">
+        <f>IF(H30="","Pending buy",IF(N30&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q30" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A8:Q26">
+  <conditionalFormatting sqref="A8:Q30">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$N8&gt;0</formula>
     </cfRule>
@@ -2042,7 +2306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2490,6 +2754,126 @@
       <c r="D22" s="11" t="inlineStr">
         <is>
           <t>Ather Energy Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>JAMNAAUTO</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>Jamna Auto Industries Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>ADOR</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>Ador Welding Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>COMSYN</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>Commercial Syn Bags Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>CRAFTSMAN</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Craftsman Automation Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>HAPPYFORGE</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>Happy Forgings Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>VIJIFIN</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Viji Finance Limited</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum Portfolio: weekday silent update 2026-10-13
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q30"/>
+  <dimension ref="A1:Q34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -531,8 +531,8 @@
         </is>
       </c>
       <c r="E1" s="2">
-        <f>SUM(J8:J30)</f>
-        <v>1876571.21</v>
+        <f>SUM(J8:J34)</f>
+        <v>2270248.6</v>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
@@ -540,8 +540,8 @@
         </is>
       </c>
       <c r="G1" s="2">
-        <f>SUM(L8:L30)</f>
-        <v>1851612.03</v>
+        <f>SUM(L8:L34)</f>
+        <v>2221023.21</v>
       </c>
     </row>
     <row r="2">
@@ -551,8 +551,8 @@
         </is>
       </c>
       <c r="E2" s="2">
-        <f>SUM(M8:M30)</f>
-        <v>-24959.18</v>
+        <f>SUM(M8:M34)</f>
+        <v>-49225.39</v>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" s="3">
         <f>IF(E1=0,"",G1/E1-1)</f>
-        <v>-0.013300417200794556</v>
+        <v>-0.021682819229576933</v>
       </c>
     </row>
     <row r="3">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -579,8 +579,8 @@
         </is>
       </c>
       <c r="E3">
-        <f>COUNTIF(M8:M30,"&gt;0")</f>
-        <v>7</v>
+        <f>COUNTIF(M8:M34,"&gt;0")</f>
+        <v>6</v>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
@@ -588,8 +588,8 @@
         </is>
       </c>
       <c r="G3">
-        <f>COUNTIF(M8:M30,"&lt;0")</f>
-        <v>12</v>
+        <f>COUNTIF(M8:M34,"&lt;0")</f>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -600,7 +600,7 @@
       </c>
       <c r="E4" s="3">
         <f>IF((E3+G3)=0,"",E3/(E3+G3))</f>
-        <v>0.3684210526315789</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
@@ -608,8 +608,8 @@
         </is>
       </c>
       <c r="G4" s="3">
-        <f>AVERAGE(N8:N30)</f>
-        <v>-0.013460471821825047</v>
+        <f>AVERAGE(N8:N34)</f>
+        <v>-0.021765836560498318</v>
       </c>
     </row>
     <row r="5">
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="E5" t="str">
-        <f>INDEX(B8:B30,MATCH(MAX(N8:N30),N8:N30,0))</f>
+        <f>INDEX(B8:B34,MATCH(MAX(N8:N34),N8:N34,0))</f>
         <v>Black Box Limited</v>
       </c>
       <c r="F5" s="1" t="inlineStr">
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="G5" t="str">
-        <f>INDEX(B8:B30,MATCH(MIN(N8:N30),N8:N30,0))</f>
+        <f>INDEX(B8:B34,MATCH(MIN(N8:N34),N8:N34,0))</f>
         <v>Lloyds Enterprises Limited</v>
       </c>
     </row>
@@ -639,8 +639,8 @@
         </is>
       </c>
       <c r="E6" s="3">
-        <f>AVERAGEIF(D8:D30,"4★*",N8:N30)</f>
-        <v>-0.01311486671352505</v>
+        <f>AVERAGEIF(D8:D34,"4★*",N8:N34)</f>
+        <v>-0.029901266488797994</v>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
@@ -648,8 +648,8 @@
         </is>
       </c>
       <c r="G6" s="3">
-        <f>AVERAGEIF(D8:D30,"5★*",N8:N30)</f>
-        <v>-0.013935678845737542</v>
+        <f>AVERAGEIF(D8:D34,"5★*",N8:N34)</f>
+        <v>-0.014308359126223616</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
@@ -781,27 +781,27 @@
         <v>99851.29</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>312.2</v>
+        <v>299.7</v>
       </c>
       <c r="L8" s="9">
         <f>IF(OR(I8="",K8=""),"",K8*I8)</f>
-        <v>103650.4</v>
+        <v>99500.4</v>
       </c>
       <c r="M8" s="9">
         <f>IF(L8="","",L8-J8)</f>
-        <v>3799.11</v>
+        <v>-350.89</v>
       </c>
       <c r="N8" s="10">
         <f>IF(OR(H8="",K8=""),"",K8/H8-1)</f>
-        <v>0.038047644777622125</v>
+        <v>-0.00351416034640184</v>
       </c>
       <c r="O8" s="6">
         <f>IF(G8="","",$B$3-G8)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P8" s="6" t="str">
         <f>IF(H8="","Pending buy",IF(N8&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q8" s="6" t="n">
         <v>2</v>
@@ -849,23 +849,23 @@
         <v>99687.42</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>323</v>
+        <v>320.45</v>
       </c>
       <c r="L9" s="9">
         <f>IF(OR(I9="",K9=""),"",K9*I9)</f>
-        <v>98838.0</v>
+        <v>98057.7</v>
       </c>
       <c r="M9" s="9">
         <f>IF(L9="","",L9-J9)</f>
-        <v>-849.42</v>
+        <v>-1629.72</v>
       </c>
       <c r="N9" s="10">
         <f>IF(OR(H9="",K9=""),"",K9/H9-1)</f>
-        <v>-0.008520836393527742</v>
+        <v>-0.016348303474631454</v>
       </c>
       <c r="O9" s="6">
         <f>IF(G9="","",$B$3-G9)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P9" s="6" t="str">
         <f>IF(H9="","Pending buy",IF(N9&gt;=0,"In profit","In loss"))</f>
@@ -917,23 +917,23 @@
         <v>99607.14</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>1563.1</v>
+        <v>1546.1</v>
       </c>
       <c r="L10" s="9">
         <f>IF(OR(I10="",K10=""),"",K10*I10)</f>
-        <v>98475.3</v>
+        <v>97404.3</v>
       </c>
       <c r="M10" s="9">
         <f>IF(L10="","",L10-J10)</f>
-        <v>-1131.84</v>
+        <v>-2202.84</v>
       </c>
       <c r="N10" s="10">
         <f>IF(OR(H10="",K10=""),"",K10/H10-1)</f>
-        <v>-0.011363050043063705</v>
+        <v>-0.022115291197991715</v>
       </c>
       <c r="O10" s="6">
         <f>IF(G10="","",$B$3-G10)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P10" s="6" t="str">
         <f>IF(H10="","Pending buy",IF(N10&gt;=0,"In profit","In loss"))</f>
@@ -985,23 +985,23 @@
         <v>99927.23</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>71.56</v>
+        <v>70.97</v>
       </c>
       <c r="L11" s="9">
         <f>IF(OR(I11="",K11=""),"",K11*I11)</f>
-        <v>89521.56</v>
+        <v>88783.47</v>
       </c>
       <c r="M11" s="9">
         <f>IF(L11="","",L11-J11)</f>
-        <v>-10405.67</v>
+        <v>-11143.76</v>
       </c>
       <c r="N11" s="10">
         <f>IF(OR(H11="",K11=""),"",K11/H11-1)</f>
-        <v>-0.10413248062836711</v>
+        <v>-0.11151875559244295</v>
       </c>
       <c r="O11" s="6">
         <f>IF(G11="","",$B$3-G11)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P11" s="6" t="str">
         <f>IF(H11="","Pending buy",IF(N11&gt;=0,"In profit","In loss"))</f>
@@ -1053,23 +1053,23 @@
         <v>86537.12</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>20565</v>
+        <v>20360</v>
       </c>
       <c r="L12" s="9">
         <f>IF(OR(I12="",K12=""),"",K12*I12)</f>
-        <v>82260.0</v>
+        <v>81440.0</v>
       </c>
       <c r="M12" s="9">
         <f>IF(L12="","",L12-J12)</f>
-        <v>-4277.12</v>
+        <v>-5097.12</v>
       </c>
       <c r="N12" s="10">
         <f>IF(OR(H12="",K12=""),"",K12/H12-1)</f>
-        <v>-0.04942522157868612</v>
+        <v>-0.058900924451351866</v>
       </c>
       <c r="O12" s="6">
         <f>IF(G12="","",$B$3-G12)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P12" s="6" t="str">
         <f>IF(H12="","Pending buy",IF(N12&gt;=0,"In profit","In loss"))</f>
@@ -1121,27 +1121,27 @@
         <v>98177.53</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>1868.8</v>
+        <v>1807.7</v>
       </c>
       <c r="L13" s="9">
         <f>IF(OR(I13="",K13=""),"",K13*I13)</f>
-        <v>99046.4</v>
+        <v>95808.1</v>
       </c>
       <c r="M13" s="9">
         <f>IF(L13="","",L13-J13)</f>
-        <v>868.87</v>
+        <v>-2369.43</v>
       </c>
       <c r="N13" s="10">
         <f>IF(OR(H13="",K13=""),"",K13/H13-1)</f>
-        <v>0.008849955932399567</v>
+        <v>-0.024134168804045952</v>
       </c>
       <c r="O13" s="6">
         <f>IF(G13="","",$B$3-G13)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P13" s="6" t="str">
         <f>IF(H13="","Pending buy",IF(N13&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>1</v>
@@ -1189,23 +1189,23 @@
         <v>97667.46</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>4555</v>
+        <v>4540</v>
       </c>
       <c r="L14" s="9">
         <f>IF(OR(I14="",K14=""),"",K14*I14)</f>
-        <v>100210.0</v>
+        <v>99880.0</v>
       </c>
       <c r="M14" s="9">
         <f>IF(L14="","",L14-J14)</f>
-        <v>2542.54</v>
+        <v>2212.54</v>
       </c>
       <c r="N14" s="10">
         <f>IF(OR(H14="",K14=""),"",K14/H14-1)</f>
-        <v>0.026032577392550493</v>
+        <v>0.02265376539235553</v>
       </c>
       <c r="O14" s="6">
         <f>IF(G14="","",$B$3-G14)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P14" s="6" t="str">
         <f>IF(H14="","Pending buy",IF(N14&gt;=0,"In profit","In loss"))</f>
@@ -1257,23 +1257,23 @@
         <v>99078.19</v>
       </c>
       <c r="K15" s="9" t="n">
-        <v>1540.2</v>
+        <v>1529</v>
       </c>
       <c r="L15" s="9">
         <f>IF(OR(I15="",K15=""),"",K15*I15)</f>
-        <v>98572.8</v>
+        <v>97856.0</v>
       </c>
       <c r="M15" s="9">
         <f>IF(L15="","",L15-J15)</f>
-        <v>-505.39</v>
+        <v>-1222.19</v>
       </c>
       <c r="N15" s="10">
         <f>IF(OR(H15="",K15=""),"",K15/H15-1)</f>
-        <v>-0.005100896537610922</v>
+        <v>-0.012335586810808485</v>
       </c>
       <c r="O15" s="6">
         <f>IF(G15="","",$B$3-G15)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P15" s="6" t="str">
         <f>IF(H15="","Pending buy",IF(N15&gt;=0,"In profit","In loss"))</f>
@@ -1325,23 +1325,23 @@
         <v>98557.54</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>1511</v>
+        <v>1494.9</v>
       </c>
       <c r="L16" s="9">
         <f>IF(OR(I16="",K16=""),"",K16*I16)</f>
-        <v>102748.0</v>
+        <v>101653.2</v>
       </c>
       <c r="M16" s="9">
         <f>IF(L16="","",L16-J16)</f>
-        <v>4190.46</v>
+        <v>3095.66</v>
       </c>
       <c r="N16" s="10">
         <f>IF(OR(H16="",K16=""),"",K16/H16-1)</f>
-        <v>0.042517940607410765</v>
+        <v>0.03140970841430746</v>
       </c>
       <c r="O16" s="6">
         <f>IF(G16="","",$B$3-G16)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P16" s="6" t="str">
         <f>IF(H16="","Pending buy",IF(N16&gt;=0,"In profit","In loss"))</f>
@@ -1393,23 +1393,23 @@
         <v>99714.35</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>924.6</v>
+        <v>921.85</v>
       </c>
       <c r="L17" s="9">
         <f>IF(OR(I17="",K17=""),"",K17*I17)</f>
-        <v>106329.0</v>
+        <v>106012.75</v>
       </c>
       <c r="M17" s="9">
         <f>IF(L17="","",L17-J17)</f>
-        <v>6614.65</v>
+        <v>6298.4</v>
       </c>
       <c r="N17" s="10">
         <f>IF(OR(H17="",K17=""),"",K17/H17-1)</f>
-        <v>0.06633598794982665</v>
+        <v>0.06316442839232939</v>
       </c>
       <c r="O17" s="6">
         <f>IF(G17="","",$B$3-G17)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P17" s="6" t="str">
         <f>IF(H17="","Pending buy",IF(N17&gt;=0,"In profit","In loss"))</f>
@@ -1461,23 +1461,23 @@
         <v>99596.83</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>640.25</v>
+        <v>637.6</v>
       </c>
       <c r="L18" s="9">
         <f>IF(OR(I18="",K18=""),"",K18*I18)</f>
-        <v>90275.25</v>
+        <v>89901.6</v>
       </c>
       <c r="M18" s="9">
         <f>IF(L18="","",L18-J18)</f>
-        <v>-9321.58</v>
+        <v>-9695.23</v>
       </c>
       <c r="N18" s="10">
         <f>IF(OR(H18="",K18=""),"",K18/H18-1)</f>
-        <v>-0.09359318122374871</v>
+        <v>-0.0973448064791288</v>
       </c>
       <c r="O18" s="6">
         <f>IF(G18="","",$B$3-G18)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P18" s="6" t="str">
         <f>IF(H18="","Pending buy",IF(N18&gt;=0,"In profit","In loss"))</f>
@@ -1529,23 +1529,23 @@
         <v>99993.07</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>146.19</v>
+        <v>145.73</v>
       </c>
       <c r="L19" s="9">
         <f>IF(OR(I19="",K19=""),"",K19*I19)</f>
-        <v>96923.97</v>
+        <v>96618.99</v>
       </c>
       <c r="M19" s="9">
         <f>IF(L19="","",L19-J19)</f>
-        <v>-3069.1</v>
+        <v>-3374.08</v>
       </c>
       <c r="N19" s="10">
         <f>IF(OR(H19="",K19=""),"",K19/H19-1)</f>
-        <v>-0.03069308136648985</v>
+        <v>-0.033743092875973546</v>
       </c>
       <c r="O19" s="6">
         <f>IF(G19="","",$B$3-G19)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P19" s="6" t="str">
         <f>IF(H19="","Pending buy",IF(N19&gt;=0,"In profit","In loss"))</f>
@@ -1597,23 +1597,23 @@
         <v>99896.43</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>220.61</v>
+        <v>212.78</v>
       </c>
       <c r="L20" s="9">
         <f>IF(OR(I20="",K20=""),"",K20*I20)</f>
-        <v>105230.97</v>
+        <v>101496.06</v>
       </c>
       <c r="M20" s="9">
         <f>IF(L20="","",L20-J20)</f>
-        <v>5334.54</v>
+        <v>1599.63</v>
       </c>
       <c r="N20" s="10">
         <f>IF(OR(H20="",K20=""),"",K20/H20-1)</f>
-        <v>0.053400707049086726</v>
+        <v>0.0160128844834988</v>
       </c>
       <c r="O20" s="6">
         <f>IF(G20="","",$B$3-G20)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P20" s="6" t="str">
         <f>IF(H20="","Pending buy",IF(N20&gt;=0,"In profit","In loss"))</f>
@@ -1665,23 +1665,23 @@
         <v>99449.47</v>
       </c>
       <c r="K21" s="9" t="n">
-        <v>1318.7</v>
+        <v>1321</v>
       </c>
       <c r="L21" s="9">
         <f>IF(OR(I21="",K21=""),"",K21*I21)</f>
-        <v>93627.7</v>
+        <v>93791.0</v>
       </c>
       <c r="M21" s="9">
         <f>IF(L21="","",L21-J21)</f>
-        <v>-5821.77</v>
+        <v>-5658.47</v>
       </c>
       <c r="N21" s="10">
         <f>IF(OR(H21="",K21=""),"",K21/H21-1)</f>
-        <v>-0.05853994549508146</v>
+        <v>-0.056897905512248936</v>
       </c>
       <c r="O21" s="6">
         <f>IF(G21="","",$B$3-G21)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P21" s="6" t="str">
         <f>IF(H21="","Pending buy",IF(N21&gt;=0,"In profit","In loss"))</f>
@@ -1733,23 +1733,23 @@
         <v>99837.05</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>685.95</v>
+        <v>677.5</v>
       </c>
       <c r="L22" s="9">
         <f>IF(OR(I22="",K22=""),"",K22*I22)</f>
-        <v>98776.8</v>
+        <v>97560.0</v>
       </c>
       <c r="M22" s="9">
         <f>IF(L22="","",L22-J22)</f>
-        <v>-1060.25</v>
+        <v>-2277.05</v>
       </c>
       <c r="N22" s="10">
         <f>IF(OR(H22="",K22=""),"",K22/H22-1)</f>
-        <v>-0.010619816071346322</v>
+        <v>-0.022807676052681858</v>
       </c>
       <c r="O22" s="6">
         <f>IF(G22="","",$B$3-G22)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P22" s="6" t="str">
         <f>IF(H22="","Pending buy",IF(N22&gt;=0,"In profit","In loss"))</f>
@@ -1801,23 +1801,23 @@
         <v>99486.88</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>653.3</v>
+        <v>645.25</v>
       </c>
       <c r="L23" s="9">
         <f>IF(OR(I23="",K23=""),"",K23*I23)</f>
-        <v>94728.5</v>
+        <v>93561.25</v>
       </c>
       <c r="M23" s="9">
         <f>IF(L23="","",L23-J23)</f>
-        <v>-4758.38</v>
+        <v>-5925.63</v>
       </c>
       <c r="N23" s="10">
         <f>IF(OR(H23="",K23=""),"",K23/H23-1)</f>
-        <v>-0.047829232689609036</v>
+        <v>-0.059561935394107146</v>
       </c>
       <c r="O23" s="6">
         <f>IF(G23="","",$B$3-G23)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P23" s="6" t="str">
         <f>IF(H23="","Pending buy",IF(N23&gt;=0,"In profit","In loss"))</f>
@@ -1869,23 +1869,23 @@
         <v>99935.4</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>224.32</v>
+        <v>223.85</v>
       </c>
       <c r="L24" s="9">
         <f>IF(OR(I24="",K24=""),"",K24*I24)</f>
-        <v>98476.48</v>
+        <v>98270.15</v>
       </c>
       <c r="M24" s="9">
         <f>IF(L24="","",L24-J24)</f>
-        <v>-1458.92</v>
+        <v>-1665.25</v>
       </c>
       <c r="N24" s="10">
         <f>IF(OR(H24="",K24=""),"",K24/H24-1)</f>
-        <v>-0.014598616940486364</v>
+        <v>-0.016663250722752543</v>
       </c>
       <c r="O24" s="6">
         <f>IF(G24="","",$B$3-G24)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P24" s="6" t="str">
         <f>IF(H24="","Pending buy",IF(N24&gt;=0,"In profit","In loss"))</f>
@@ -1937,27 +1937,27 @@
         <v>99622.64</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>806.1</v>
+        <v>783.95</v>
       </c>
       <c r="L25" s="9">
         <f>IF(OR(I25="",K25=""),"",K25*I25)</f>
-        <v>99956.4</v>
+        <v>97209.8</v>
       </c>
       <c r="M25" s="9">
         <f>IF(L25="","",L25-J25)</f>
-        <v>333.76</v>
+        <v>-2412.84</v>
       </c>
       <c r="N25" s="10">
         <f>IF(OR(H25="",K25=""),"",K25/H25-1)</f>
-        <v>0.0033502788130068684</v>
+        <v>-0.024219760482003805</v>
       </c>
       <c r="O25" s="6">
         <f>IF(G25="","",$B$3-G25)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P25" s="6" t="str">
         <f>IF(H25="","Pending buy",IF(N25&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q25" s="6" t="n">
         <v>1</v>
@@ -2005,23 +2005,23 @@
         <v>99948.17</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>197.82</v>
+        <v>194.67</v>
       </c>
       <c r="L26" s="9">
         <f>IF(OR(I26="",K26=""),"",K26*I26)</f>
-        <v>93964.5</v>
+        <v>92468.25</v>
       </c>
       <c r="M26" s="9">
         <f>IF(L26="","",L26-J26)</f>
-        <v>-5983.67</v>
+        <v>-7479.92</v>
       </c>
       <c r="N26" s="10">
         <f>IF(OR(H26="",K26=""),"",K26/H26-1)</f>
-        <v>-0.059867698168561745</v>
+        <v>-0.07483795775186497</v>
       </c>
       <c r="O26" s="6">
         <f>IF(G26="","",$B$3-G26)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P26" s="6" t="str">
         <f>IF(H26="","Pending buy",IF(N26&gt;=0,"In profit","In loss"))</f>
@@ -2058,38 +2058,42 @@
       <c r="F27" s="8" t="n">
         <v>46307</v>
       </c>
-      <c r="G27" s="6" t="inlineStr"/>
-      <c r="H27" s="9" t="inlineStr"/>
-      <c r="I27" s="6" t="str">
+      <c r="G27" s="8" t="n">
+        <v>46308</v>
+      </c>
+      <c r="H27" s="9" t="n">
+        <v>261.11</v>
+      </c>
+      <c r="I27" s="6">
         <f>IF(H27="","",ROUNDDOWN($B$1/H27,0))</f>
-        <v/>
-      </c>
-      <c r="J27" s="9" t="str">
+        <v>382</v>
+      </c>
+      <c r="J27" s="9">
         <f>IF(H27="","",H27*I27)</f>
-        <v/>
+        <v>99745.27</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>262.4</v>
-      </c>
-      <c r="L27" s="9" t="str">
+        <v>258.95</v>
+      </c>
+      <c r="L27" s="9">
         <f>IF(OR(I27="",K27=""),"",K27*I27)</f>
-        <v/>
-      </c>
-      <c r="M27" s="9" t="str">
+        <v>98918.9</v>
+      </c>
+      <c r="M27" s="9">
         <f>IF(L27="","",L27-J27)</f>
-        <v/>
-      </c>
-      <c r="N27" s="10" t="str">
+        <v>-826.37</v>
+      </c>
+      <c r="N27" s="10">
         <f>IF(OR(H27="",K27=""),"",K27/H27-1)</f>
-        <v/>
-      </c>
-      <c r="O27" s="6" t="str">
+        <v>-0.0082848333106611</v>
+      </c>
+      <c r="O27" s="6">
         <f>IF(G27="","",$B$3-G27)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P27" s="6" t="str">
         <f>IF(H27="","Pending buy",IF(N27&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q27" s="6" t="n">
         <v>1</v>
@@ -2122,38 +2126,42 @@
       <c r="F28" s="8" t="n">
         <v>46307</v>
       </c>
-      <c r="G28" s="6" t="inlineStr"/>
-      <c r="H28" s="9" t="inlineStr"/>
-      <c r="I28" s="6" t="str">
+      <c r="G28" s="8" t="n">
+        <v>46308</v>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>10592.76</v>
+      </c>
+      <c r="I28" s="6">
         <f>IF(H28="","",ROUNDDOWN($B$1/H28,0))</f>
-        <v/>
-      </c>
-      <c r="J28" s="9" t="str">
+        <v>9</v>
+      </c>
+      <c r="J28" s="9">
         <f>IF(H28="","",H28*I28)</f>
-        <v/>
+        <v>95334.84</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>10815</v>
-      </c>
-      <c r="L28" s="9" t="str">
+        <v>10674</v>
+      </c>
+      <c r="L28" s="9">
         <f>IF(OR(I28="",K28=""),"",K28*I28)</f>
-        <v/>
-      </c>
-      <c r="M28" s="9" t="str">
+        <v>96066.0</v>
+      </c>
+      <c r="M28" s="9">
         <f>IF(L28="","",L28-J28)</f>
-        <v/>
-      </c>
-      <c r="N28" s="10" t="str">
+        <v>731.16</v>
+      </c>
+      <c r="N28" s="10">
         <f>IF(OR(H28="",K28=""),"",K28/H28-1)</f>
-        <v/>
-      </c>
-      <c r="O28" s="6" t="str">
+        <v>0.007669363976900323</v>
+      </c>
+      <c r="O28" s="6">
         <f>IF(G28="","",$B$3-G28)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P28" s="6" t="str">
         <f>IF(H28="","Pending buy",IF(N28&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In profit</v>
       </c>
       <c r="Q28" s="6" t="n">
         <v>1</v>
@@ -2186,38 +2194,42 @@
       <c r="F29" s="8" t="n">
         <v>46307</v>
       </c>
-      <c r="G29" s="6" t="inlineStr"/>
-      <c r="H29" s="9" t="inlineStr"/>
-      <c r="I29" s="6" t="str">
+      <c r="G29" s="8" t="n">
+        <v>46308</v>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>1933.31</v>
+      </c>
+      <c r="I29" s="6">
         <f>IF(H29="","",ROUNDDOWN($B$1/H29,0))</f>
-        <v/>
-      </c>
-      <c r="J29" s="9" t="str">
+        <v>51</v>
+      </c>
+      <c r="J29" s="9">
         <f>IF(H29="","",H29*I29)</f>
-        <v/>
+        <v>98598.59</v>
       </c>
       <c r="K29" s="9" t="n">
-        <v>1966.3</v>
-      </c>
-      <c r="L29" s="9" t="str">
+        <v>1936.6</v>
+      </c>
+      <c r="L29" s="9">
         <f>IF(OR(I29="",K29=""),"",K29*I29)</f>
-        <v/>
-      </c>
-      <c r="M29" s="9" t="str">
+        <v>98766.6</v>
+      </c>
+      <c r="M29" s="9">
         <f>IF(L29="","",L29-J29)</f>
-        <v/>
-      </c>
-      <c r="N29" s="10" t="str">
+        <v>168.01</v>
+      </c>
+      <c r="N29" s="10">
         <f>IF(OR(H29="",K29=""),"",K29/H29-1)</f>
-        <v/>
-      </c>
-      <c r="O29" s="6" t="str">
+        <v>0.0017040177082441321</v>
+      </c>
+      <c r="O29" s="6">
         <f>IF(G29="","",$B$3-G29)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P29" s="6" t="str">
         <f>IF(H29="","Pending buy",IF(N29&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In profit</v>
       </c>
       <c r="Q29" s="6" t="n">
         <v>1</v>
@@ -2250,45 +2262,305 @@
       <c r="F30" s="8" t="n">
         <v>46307</v>
       </c>
-      <c r="G30" s="6" t="inlineStr"/>
-      <c r="H30" s="9" t="inlineStr"/>
-      <c r="I30" s="6" t="str">
+      <c r="G30" s="8" t="n">
+        <v>46308</v>
+      </c>
+      <c r="H30" s="9" t="n">
+        <v>14.83</v>
+      </c>
+      <c r="I30" s="6">
         <f>IF(H30="","",ROUNDDOWN($B$1/H30,0))</f>
-        <v/>
-      </c>
-      <c r="J30" s="9" t="str">
+        <v>6743</v>
+      </c>
+      <c r="J30" s="9">
         <f>IF(H30="","",H30*I30)</f>
-        <v/>
+        <v>99998.69</v>
       </c>
       <c r="K30" s="9" t="n">
-        <v>14.13</v>
-      </c>
-      <c r="L30" s="9" t="str">
+        <v>14.83</v>
+      </c>
+      <c r="L30" s="9">
         <f>IF(OR(I30="",K30=""),"",K30*I30)</f>
-        <v/>
-      </c>
-      <c r="M30" s="9" t="str">
+        <v>99998.69</v>
+      </c>
+      <c r="M30" s="9">
         <f>IF(L30="","",L30-J30)</f>
-        <v/>
-      </c>
-      <c r="N30" s="10" t="str">
+        <v>0.0</v>
+      </c>
+      <c r="N30" s="10">
         <f>IF(OR(H30="",K30=""),"",K30/H30-1)</f>
-        <v/>
-      </c>
-      <c r="O30" s="6" t="str">
+        <v>0.0</v>
+      </c>
+      <c r="O30" s="6">
         <f>IF(G30="","",$B$3-G30)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P30" s="6" t="str">
         <f>IF(H30="","Pending buy",IF(N30&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In profit</v>
       </c>
       <c r="Q30" s="6" t="n">
         <v>1</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Gujarat Ambuja Exports Limited</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>GAEL</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>131026</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="n">
+        <v>46308</v>
+      </c>
+      <c r="G31" s="6" t="inlineStr"/>
+      <c r="H31" s="9" t="inlineStr"/>
+      <c r="I31" s="6" t="str">
+        <f>IF(H31="","",ROUNDDOWN($B$1/H31,0))</f>
+        <v/>
+      </c>
+      <c r="J31" s="9" t="str">
+        <f>IF(H31="","",H31*I31)</f>
+        <v/>
+      </c>
+      <c r="K31" s="9" t="n">
+        <v>173.26</v>
+      </c>
+      <c r="L31" s="9" t="str">
+        <f>IF(OR(I31="",K31=""),"",K31*I31)</f>
+        <v/>
+      </c>
+      <c r="M31" s="9" t="str">
+        <f>IF(L31="","",L31-J31)</f>
+        <v/>
+      </c>
+      <c r="N31" s="10" t="str">
+        <f>IF(OR(H31="",K31=""),"",K31/H31-1)</f>
+        <v/>
+      </c>
+      <c r="O31" s="6" t="str">
+        <f>IF(G31="","",$B$3-G31)</f>
+        <v/>
+      </c>
+      <c r="P31" s="6" t="str">
+        <f>IF(H31="","Pending buy",IF(N31&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q31" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Kanoria Chemicals &amp; Industries Limited</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>KANORICHEM</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>131026</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="n">
+        <v>46308</v>
+      </c>
+      <c r="G32" s="6" t="inlineStr"/>
+      <c r="H32" s="9" t="inlineStr"/>
+      <c r="I32" s="6" t="str">
+        <f>IF(H32="","",ROUNDDOWN($B$1/H32,0))</f>
+        <v/>
+      </c>
+      <c r="J32" s="9" t="str">
+        <f>IF(H32="","",H32*I32)</f>
+        <v/>
+      </c>
+      <c r="K32" s="9" t="n">
+        <v>172.59</v>
+      </c>
+      <c r="L32" s="9" t="str">
+        <f>IF(OR(I32="",K32=""),"",K32*I32)</f>
+        <v/>
+      </c>
+      <c r="M32" s="9" t="str">
+        <f>IF(L32="","",L32-J32)</f>
+        <v/>
+      </c>
+      <c r="N32" s="10" t="str">
+        <f>IF(OR(H32="",K32=""),"",K32/H32-1)</f>
+        <v/>
+      </c>
+      <c r="O32" s="6" t="str">
+        <f>IF(G32="","",$B$3-G32)</f>
+        <v/>
+      </c>
+      <c r="P32" s="6" t="str">
+        <f>IF(H32="","Pending buy",IF(N32&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q32" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Kapston Services Limited</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>KAPSTON</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>131026</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="n">
+        <v>46308</v>
+      </c>
+      <c r="G33" s="6" t="inlineStr"/>
+      <c r="H33" s="9" t="inlineStr"/>
+      <c r="I33" s="6" t="str">
+        <f>IF(H33="","",ROUNDDOWN($B$1/H33,0))</f>
+        <v/>
+      </c>
+      <c r="J33" s="9" t="str">
+        <f>IF(H33="","",H33*I33)</f>
+        <v/>
+      </c>
+      <c r="K33" s="9" t="n">
+        <v>529.3</v>
+      </c>
+      <c r="L33" s="9" t="str">
+        <f>IF(OR(I33="",K33=""),"",K33*I33)</f>
+        <v/>
+      </c>
+      <c r="M33" s="9" t="str">
+        <f>IF(L33="","",L33-J33)</f>
+        <v/>
+      </c>
+      <c r="N33" s="10" t="str">
+        <f>IF(OR(H33="",K33=""),"",K33/H33-1)</f>
+        <v/>
+      </c>
+      <c r="O33" s="6" t="str">
+        <f>IF(G33="","",$B$3-G33)</f>
+        <v/>
+      </c>
+      <c r="P33" s="6" t="str">
+        <f>IF(H33="","Pending buy",IF(N33&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q33" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Netweb Technologies India Limited</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>NETWEB</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>131026</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="n">
+        <v>46308</v>
+      </c>
+      <c r="G34" s="6" t="inlineStr"/>
+      <c r="H34" s="9" t="inlineStr"/>
+      <c r="I34" s="6" t="str">
+        <f>IF(H34="","",ROUNDDOWN($B$1/H34,0))</f>
+        <v/>
+      </c>
+      <c r="J34" s="9" t="str">
+        <f>IF(H34="","",H34*I34)</f>
+        <v/>
+      </c>
+      <c r="K34" s="9" t="n">
+        <v>5054.6</v>
+      </c>
+      <c r="L34" s="9" t="str">
+        <f>IF(OR(I34="",K34=""),"",K34*I34)</f>
+        <v/>
+      </c>
+      <c r="M34" s="9" t="str">
+        <f>IF(L34="","",L34-J34)</f>
+        <v/>
+      </c>
+      <c r="N34" s="10" t="str">
+        <f>IF(OR(H34="",K34=""),"",K34/H34-1)</f>
+        <v/>
+      </c>
+      <c r="O34" s="6" t="str">
+        <f>IF(G34="","",$B$3-G34)</f>
+        <v/>
+      </c>
+      <c r="P34" s="6" t="str">
+        <f>IF(H34="","Pending buy",IF(N34&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q34" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A8:Q30">
+  <conditionalFormatting sqref="A8:Q34">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$N8&gt;0</formula>
     </cfRule>
@@ -2306,7 +2578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2874,6 +3146,86 @@
       <c r="D28" s="11" t="inlineStr">
         <is>
           <t>Viji Finance Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>GAEL</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>Gujarat Ambuja Exports Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>NETWEB</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>Netweb Technologies India Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>KANORICHEM</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>Kanoria Chemicals &amp; Industries Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>KAPSTON</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>Kapston Services Limited</t>
         </is>
       </c>
     </row>
@@ -2888,7 +3240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3000,6 +3352,31 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>HEALTHADD</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>DSP Nifty Healthcare ETF</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>Not in NSE official equity list; In NSE official ETF list; Name/symbol contains: ETF</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Momentum Portfolio: weekday silent update 2026-10-14
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q34"/>
+  <dimension ref="A1:Q38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -531,8 +531,8 @@
         </is>
       </c>
       <c r="E1" s="2">
-        <f>SUM(J8:J34)</f>
-        <v>2270248.6</v>
+        <f>SUM(J8:J38)</f>
+        <v>2665788.8</v>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
@@ -540,8 +540,8 @@
         </is>
       </c>
       <c r="G1" s="2">
-        <f>SUM(L8:L34)</f>
-        <v>2221023.21</v>
+        <f>SUM(L8:L38)</f>
+        <v>2623522.7</v>
       </c>
     </row>
     <row r="2">
@@ -551,8 +551,8 @@
         </is>
       </c>
       <c r="E2" s="2">
-        <f>SUM(M8:M34)</f>
-        <v>-49225.39</v>
+        <f>SUM(M8:M38)</f>
+        <v>-42266.1</v>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" s="3">
         <f>IF(E1=0,"",G1/E1-1)</f>
-        <v>-0.021682819229576933</v>
+        <v>-0.015855006968293783</v>
       </c>
     </row>
     <row r="3">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -579,8 +579,8 @@
         </is>
       </c>
       <c r="E3">
-        <f>COUNTIF(M8:M34,"&gt;0")</f>
-        <v>6</v>
+        <f>COUNTIF(M8:M38,"&gt;0")</f>
+        <v>12</v>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
@@ -588,8 +588,8 @@
         </is>
       </c>
       <c r="G3">
-        <f>COUNTIF(M8:M34,"&lt;0")</f>
-        <v>16</v>
+        <f>COUNTIF(M8:M38,"&lt;0")</f>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -600,7 +600,7 @@
       </c>
       <c r="E4" s="3">
         <f>IF((E3+G3)=0,"",E3/(E3+G3))</f>
-        <v>0.2727272727272727</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
@@ -608,8 +608,8 @@
         </is>
       </c>
       <c r="G4" s="3">
-        <f>AVERAGE(N8:N34)</f>
-        <v>-0.021765836560498318</v>
+        <f>AVERAGE(N8:N38)</f>
+        <v>-0.01597260461428871</v>
       </c>
     </row>
     <row r="5">
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="E5" t="str">
-        <f>INDEX(B8:B34,MATCH(MAX(N8:N34),N8:N34,0))</f>
+        <f>INDEX(B8:B38,MATCH(MAX(N8:N38),N8:N38,0))</f>
         <v>Black Box Limited</v>
       </c>
       <c r="F5" s="1" t="inlineStr">
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="G5" t="str">
-        <f>INDEX(B8:B34,MATCH(MIN(N8:N34),N8:N34,0))</f>
+        <f>INDEX(B8:B38,MATCH(MIN(N8:N38),N8:N38,0))</f>
         <v>Lloyds Enterprises Limited</v>
       </c>
     </row>
@@ -639,8 +639,8 @@
         </is>
       </c>
       <c r="E6" s="3">
-        <f>AVERAGEIF(D8:D34,"4★*",N8:N34)</f>
-        <v>-0.029901266488797994</v>
+        <f>AVERAGEIF(D8:D38,"4★*",N8:N38)</f>
+        <v>-0.023707883039176352</v>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
@@ -648,8 +648,8 @@
         </is>
       </c>
       <c r="G6" s="3">
-        <f>AVERAGEIF(D8:D34,"5★*",N8:N34)</f>
-        <v>-0.014308359126223616</v>
+        <f>AVERAGEIF(D8:D38,"5★*",N8:N38)</f>
+        <v>-0.008789846076893046</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
@@ -781,27 +781,27 @@
         <v>99851.29</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>299.7</v>
+        <v>302.6</v>
       </c>
       <c r="L8" s="9">
         <f>IF(OR(I8="",K8=""),"",K8*I8)</f>
-        <v>99500.4</v>
+        <v>100463.2</v>
       </c>
       <c r="M8" s="9">
         <f>IF(L8="","",L8-J8)</f>
-        <v>-350.89</v>
+        <v>611.91</v>
       </c>
       <c r="N8" s="10">
         <f>IF(OR(H8="",K8=""),"",K8/H8-1)</f>
-        <v>-0.00351416034640184</v>
+        <v>0.006128178442371901</v>
       </c>
       <c r="O8" s="6">
         <f>IF(G8="","",$B$3-G8)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P8" s="6" t="str">
         <f>IF(H8="","Pending buy",IF(N8&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q8" s="6" t="n">
         <v>2</v>
@@ -849,23 +849,23 @@
         <v>99687.42</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>320.45</v>
+        <v>316</v>
       </c>
       <c r="L9" s="9">
         <f>IF(OR(I9="",K9=""),"",K9*I9)</f>
-        <v>98057.7</v>
+        <v>96696.0</v>
       </c>
       <c r="M9" s="9">
         <f>IF(L9="","",L9-J9)</f>
-        <v>-1629.72</v>
+        <v>-2991.42</v>
       </c>
       <c r="N9" s="10">
         <f>IF(OR(H9="",K9=""),"",K9/H9-1)</f>
-        <v>-0.016348303474631454</v>
+        <v>-0.030008000929890866</v>
       </c>
       <c r="O9" s="6">
         <f>IF(G9="","",$B$3-G9)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P9" s="6" t="str">
         <f>IF(H9="","Pending buy",IF(N9&gt;=0,"In profit","In loss"))</f>
@@ -917,23 +917,23 @@
         <v>99607.14</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>1546.1</v>
+        <v>1548.4</v>
       </c>
       <c r="L10" s="9">
         <f>IF(OR(I10="",K10=""),"",K10*I10)</f>
-        <v>97404.3</v>
+        <v>97549.2</v>
       </c>
       <c r="M10" s="9">
         <f>IF(L10="","",L10-J10)</f>
-        <v>-2202.84</v>
+        <v>-2057.94</v>
       </c>
       <c r="N10" s="10">
         <f>IF(OR(H10="",K10=""),"",K10/H10-1)</f>
-        <v>-0.022115291197991715</v>
+        <v>-0.02066057621820716</v>
       </c>
       <c r="O10" s="6">
         <f>IF(G10="","",$B$3-G10)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P10" s="6" t="str">
         <f>IF(H10="","Pending buy",IF(N10&gt;=0,"In profit","In loss"))</f>
@@ -985,23 +985,23 @@
         <v>99927.23</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>70.97</v>
+        <v>71.83</v>
       </c>
       <c r="L11" s="9">
         <f>IF(OR(I11="",K11=""),"",K11*I11)</f>
-        <v>88783.47</v>
+        <v>89859.33</v>
       </c>
       <c r="M11" s="9">
         <f>IF(L11="","",L11-J11)</f>
-        <v>-11143.76</v>
+        <v>-10067.9</v>
       </c>
       <c r="N11" s="10">
         <f>IF(OR(H11="",K11=""),"",K11/H11-1)</f>
-        <v>-0.11151875559244295</v>
+        <v>-0.1007523208990444</v>
       </c>
       <c r="O11" s="6">
         <f>IF(G11="","",$B$3-G11)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P11" s="6" t="str">
         <f>IF(H11="","Pending buy",IF(N11&gt;=0,"In profit","In loss"))</f>
@@ -1053,23 +1053,23 @@
         <v>86537.12</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>20360</v>
+        <v>20200</v>
       </c>
       <c r="L12" s="9">
         <f>IF(OR(I12="",K12=""),"",K12*I12)</f>
-        <v>81440.0</v>
+        <v>80800.0</v>
       </c>
       <c r="M12" s="9">
         <f>IF(L12="","",L12-J12)</f>
-        <v>-5097.12</v>
+        <v>-5737.12</v>
       </c>
       <c r="N12" s="10">
         <f>IF(OR(H12="",K12=""),"",K12/H12-1)</f>
-        <v>-0.058900924451351866</v>
+        <v>-0.06629659498611529</v>
       </c>
       <c r="O12" s="6">
         <f>IF(G12="","",$B$3-G12)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P12" s="6" t="str">
         <f>IF(H12="","Pending buy",IF(N12&gt;=0,"In profit","In loss"))</f>
@@ -1121,23 +1121,23 @@
         <v>98177.53</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>1807.7</v>
+        <v>1746.9</v>
       </c>
       <c r="L13" s="9">
         <f>IF(OR(I13="",K13=""),"",K13*I13)</f>
-        <v>95808.1</v>
+        <v>92585.7</v>
       </c>
       <c r="M13" s="9">
         <f>IF(L13="","",L13-J13)</f>
-        <v>-2369.43</v>
+        <v>-5591.83</v>
       </c>
       <c r="N13" s="10">
         <f>IF(OR(H13="",K13=""),"",K13/H13-1)</f>
-        <v>-0.024134168804045952</v>
+        <v>-0.05695634202787403</v>
       </c>
       <c r="O13" s="6">
         <f>IF(G13="","",$B$3-G13)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P13" s="6" t="str">
         <f>IF(H13="","Pending buy",IF(N13&gt;=0,"In profit","In loss"))</f>
@@ -1189,23 +1189,23 @@
         <v>97667.46</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>4540</v>
+        <v>4554.1</v>
       </c>
       <c r="L14" s="9">
         <f>IF(OR(I14="",K14=""),"",K14*I14)</f>
-        <v>99880.0</v>
+        <v>100190.2</v>
       </c>
       <c r="M14" s="9">
         <f>IF(L14="","",L14-J14)</f>
-        <v>2212.54</v>
+        <v>2522.74</v>
       </c>
       <c r="N14" s="10">
         <f>IF(OR(H14="",K14=""),"",K14/H14-1)</f>
-        <v>0.02265376539235553</v>
+        <v>0.02582984867253879</v>
       </c>
       <c r="O14" s="6">
         <f>IF(G14="","",$B$3-G14)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P14" s="6" t="str">
         <f>IF(H14="","Pending buy",IF(N14&gt;=0,"In profit","In loss"))</f>
@@ -1257,27 +1257,27 @@
         <v>99078.19</v>
       </c>
       <c r="K15" s="9" t="n">
-        <v>1529</v>
+        <v>1557.2</v>
       </c>
       <c r="L15" s="9">
         <f>IF(OR(I15="",K15=""),"",K15*I15)</f>
-        <v>97856.0</v>
+        <v>99660.8</v>
       </c>
       <c r="M15" s="9">
         <f>IF(L15="","",L15-J15)</f>
-        <v>-1222.19</v>
+        <v>582.61</v>
       </c>
       <c r="N15" s="10">
         <f>IF(OR(H15="",K15=""),"",K15/H15-1)</f>
-        <v>-0.012335586810808485</v>
+        <v>0.005880329769920811</v>
       </c>
       <c r="O15" s="6">
         <f>IF(G15="","",$B$3-G15)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P15" s="6" t="str">
         <f>IF(H15="","Pending buy",IF(N15&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q15" s="6" t="n">
         <v>2</v>
@@ -1325,23 +1325,23 @@
         <v>98557.54</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>1494.9</v>
+        <v>1467</v>
       </c>
       <c r="L16" s="9">
         <f>IF(OR(I16="",K16=""),"",K16*I16)</f>
-        <v>101653.2</v>
+        <v>99756.0</v>
       </c>
       <c r="M16" s="9">
         <f>IF(L16="","",L16-J16)</f>
-        <v>3095.66</v>
+        <v>1198.46</v>
       </c>
       <c r="N16" s="10">
         <f>IF(OR(H16="",K16=""),"",K16/H16-1)</f>
-        <v>0.03140970841430746</v>
+        <v>0.01216003896166229</v>
       </c>
       <c r="O16" s="6">
         <f>IF(G16="","",$B$3-G16)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P16" s="6" t="str">
         <f>IF(H16="","Pending buy",IF(N16&gt;=0,"In profit","In loss"))</f>
@@ -1393,23 +1393,23 @@
         <v>99714.35</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>921.85</v>
+        <v>935.8</v>
       </c>
       <c r="L17" s="9">
         <f>IF(OR(I17="",K17=""),"",K17*I17)</f>
-        <v>106012.75</v>
+        <v>107617.0</v>
       </c>
       <c r="M17" s="9">
         <f>IF(L17="","",L17-J17)</f>
-        <v>6298.4</v>
+        <v>7902.65</v>
       </c>
       <c r="N17" s="10">
         <f>IF(OR(H17="",K17=""),"",K17/H17-1)</f>
-        <v>0.06316442839232939</v>
+        <v>0.07925288505672468</v>
       </c>
       <c r="O17" s="6">
         <f>IF(G17="","",$B$3-G17)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P17" s="6" t="str">
         <f>IF(H17="","Pending buy",IF(N17&gt;=0,"In profit","In loss"))</f>
@@ -1461,23 +1461,23 @@
         <v>99596.83</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>637.6</v>
+        <v>647.65</v>
       </c>
       <c r="L18" s="9">
         <f>IF(OR(I18="",K18=""),"",K18*I18)</f>
-        <v>89901.6</v>
+        <v>91318.65</v>
       </c>
       <c r="M18" s="9">
         <f>IF(L18="","",L18-J18)</f>
-        <v>-9695.23</v>
+        <v>-8278.18</v>
       </c>
       <c r="N18" s="10">
         <f>IF(OR(H18="",K18=""),"",K18/H18-1)</f>
-        <v>-0.0973448064791288</v>
+        <v>-0.0831169446615555</v>
       </c>
       <c r="O18" s="6">
         <f>IF(G18="","",$B$3-G18)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P18" s="6" t="str">
         <f>IF(H18="","Pending buy",IF(N18&gt;=0,"In profit","In loss"))</f>
@@ -1529,23 +1529,23 @@
         <v>99993.07</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>145.73</v>
+        <v>149.57</v>
       </c>
       <c r="L19" s="9">
         <f>IF(OR(I19="",K19=""),"",K19*I19)</f>
-        <v>96618.99</v>
+        <v>99164.91</v>
       </c>
       <c r="M19" s="9">
         <f>IF(L19="","",L19-J19)</f>
-        <v>-3374.08</v>
+        <v>-828.16</v>
       </c>
       <c r="N19" s="10">
         <f>IF(OR(H19="",K19=""),"",K19/H19-1)</f>
-        <v>-0.033743092875973546</v>
+        <v>-0.008282127231588277</v>
       </c>
       <c r="O19" s="6">
         <f>IF(G19="","",$B$3-G19)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P19" s="6" t="str">
         <f>IF(H19="","Pending buy",IF(N19&gt;=0,"In profit","In loss"))</f>
@@ -1597,27 +1597,27 @@
         <v>99896.43</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>212.78</v>
+        <v>203.32</v>
       </c>
       <c r="L20" s="9">
         <f>IF(OR(I20="",K20=""),"",K20*I20)</f>
-        <v>101496.06</v>
+        <v>96983.64</v>
       </c>
       <c r="M20" s="9">
         <f>IF(L20="","",L20-J20)</f>
-        <v>1599.63</v>
+        <v>-2912.79</v>
       </c>
       <c r="N20" s="10">
         <f>IF(OR(H20="",K20=""),"",K20/H20-1)</f>
-        <v>0.0160128844834988</v>
+        <v>-0.02915809910148992</v>
       </c>
       <c r="O20" s="6">
         <f>IF(G20="","",$B$3-G20)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P20" s="6" t="str">
         <f>IF(H20="","Pending buy",IF(N20&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q20" s="6" t="n">
         <v>1</v>
@@ -1665,23 +1665,23 @@
         <v>99449.47</v>
       </c>
       <c r="K21" s="9" t="n">
-        <v>1321</v>
+        <v>1281.5</v>
       </c>
       <c r="L21" s="9">
         <f>IF(OR(I21="",K21=""),"",K21*I21)</f>
-        <v>93791.0</v>
+        <v>90986.5</v>
       </c>
       <c r="M21" s="9">
         <f>IF(L21="","",L21-J21)</f>
-        <v>-5658.47</v>
+        <v>-8462.97</v>
       </c>
       <c r="N21" s="10">
         <f>IF(OR(H21="",K21=""),"",K21/H21-1)</f>
-        <v>-0.056897905512248936</v>
+        <v>-0.08509815739133009</v>
       </c>
       <c r="O21" s="6">
         <f>IF(G21="","",$B$3-G21)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P21" s="6" t="str">
         <f>IF(H21="","Pending buy",IF(N21&gt;=0,"In profit","In loss"))</f>
@@ -1733,23 +1733,23 @@
         <v>99837.05</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>677.5</v>
+        <v>684.4</v>
       </c>
       <c r="L22" s="9">
         <f>IF(OR(I22="",K22=""),"",K22*I22)</f>
-        <v>97560.0</v>
+        <v>98553.6</v>
       </c>
       <c r="M22" s="9">
         <f>IF(L22="","",L22-J22)</f>
-        <v>-2277.05</v>
+        <v>-1283.45</v>
       </c>
       <c r="N22" s="10">
         <f>IF(OR(H22="",K22=""),"",K22/H22-1)</f>
-        <v>-0.022807676052681858</v>
+        <v>-0.012855459026502647</v>
       </c>
       <c r="O22" s="6">
         <f>IF(G22="","",$B$3-G22)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P22" s="6" t="str">
         <f>IF(H22="","Pending buy",IF(N22&gt;=0,"In profit","In loss"))</f>
@@ -1801,23 +1801,23 @@
         <v>99486.88</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>645.25</v>
+        <v>647.7</v>
       </c>
       <c r="L23" s="9">
         <f>IF(OR(I23="",K23=""),"",K23*I23)</f>
-        <v>93561.25</v>
+        <v>93916.5</v>
       </c>
       <c r="M23" s="9">
         <f>IF(L23="","",L23-J23)</f>
-        <v>-5925.63</v>
+        <v>-5570.38</v>
       </c>
       <c r="N23" s="10">
         <f>IF(OR(H23="",K23=""),"",K23/H23-1)</f>
-        <v>-0.059561935394107146</v>
+        <v>-0.05599111283186853</v>
       </c>
       <c r="O23" s="6">
         <f>IF(G23="","",$B$3-G23)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P23" s="6" t="str">
         <f>IF(H23="","Pending buy",IF(N23&gt;=0,"In profit","In loss"))</f>
@@ -1869,23 +1869,23 @@
         <v>99935.4</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>223.85</v>
+        <v>223.71</v>
       </c>
       <c r="L24" s="9">
         <f>IF(OR(I24="",K24=""),"",K24*I24)</f>
-        <v>98270.15</v>
+        <v>98208.69</v>
       </c>
       <c r="M24" s="9">
         <f>IF(L24="","",L24-J24)</f>
-        <v>-1665.25</v>
+        <v>-1726.71</v>
       </c>
       <c r="N24" s="10">
         <f>IF(OR(H24="",K24=""),"",K24/H24-1)</f>
-        <v>-0.016663250722752543</v>
+        <v>-0.017278248019597764</v>
       </c>
       <c r="O24" s="6">
         <f>IF(G24="","",$B$3-G24)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P24" s="6" t="str">
         <f>IF(H24="","Pending buy",IF(N24&gt;=0,"In profit","In loss"))</f>
@@ -1937,27 +1937,27 @@
         <v>99622.64</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>783.95</v>
+        <v>803.9</v>
       </c>
       <c r="L25" s="9">
         <f>IF(OR(I25="",K25=""),"",K25*I25)</f>
-        <v>97209.8</v>
+        <v>99683.6</v>
       </c>
       <c r="M25" s="9">
         <f>IF(L25="","",L25-J25)</f>
-        <v>-2412.84</v>
+        <v>60.96</v>
       </c>
       <c r="N25" s="10">
         <f>IF(OR(H25="",K25=""),"",K25/H25-1)</f>
-        <v>-0.024219760482003805</v>
+        <v>0.0006119453390103224</v>
       </c>
       <c r="O25" s="6">
         <f>IF(G25="","",$B$3-G25)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P25" s="6" t="str">
         <f>IF(H25="","Pending buy",IF(N25&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q25" s="6" t="n">
         <v>1</v>
@@ -2005,23 +2005,23 @@
         <v>99948.17</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>194.67</v>
+        <v>191.41</v>
       </c>
       <c r="L26" s="9">
         <f>IF(OR(I26="",K26=""),"",K26*I26)</f>
-        <v>92468.25</v>
+        <v>90919.75</v>
       </c>
       <c r="M26" s="9">
         <f>IF(L26="","",L26-J26)</f>
-        <v>-7479.92</v>
+        <v>-9028.42</v>
       </c>
       <c r="N26" s="10">
         <f>IF(OR(H26="",K26=""),"",K26/H26-1)</f>
-        <v>-0.07483795775186497</v>
+        <v>-0.09033098830474373</v>
       </c>
       <c r="O26" s="6">
         <f>IF(G26="","",$B$3-G26)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P26" s="6" t="str">
         <f>IF(H26="","Pending buy",IF(N26&gt;=0,"In profit","In loss"))</f>
@@ -2073,23 +2073,23 @@
         <v>99745.27</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>258.95</v>
+        <v>255.05</v>
       </c>
       <c r="L27" s="9">
         <f>IF(OR(I27="",K27=""),"",K27*I27)</f>
-        <v>98918.9</v>
+        <v>97429.1</v>
       </c>
       <c r="M27" s="9">
         <f>IF(L27="","",L27-J27)</f>
-        <v>-826.37</v>
+        <v>-2316.17</v>
       </c>
       <c r="N27" s="10">
         <f>IF(OR(H27="",K27=""),"",K27/H27-1)</f>
-        <v>-0.0082848333106611</v>
+        <v>-0.023220879458907495</v>
       </c>
       <c r="O27" s="6">
         <f>IF(G27="","",$B$3-G27)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P27" s="6" t="str">
         <f>IF(H27="","Pending buy",IF(N27&gt;=0,"In profit","In loss"))</f>
@@ -2141,23 +2141,23 @@
         <v>95334.84</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>10674</v>
+        <v>10997</v>
       </c>
       <c r="L28" s="9">
         <f>IF(OR(I28="",K28=""),"",K28*I28)</f>
-        <v>96066.0</v>
+        <v>98973.0</v>
       </c>
       <c r="M28" s="9">
         <f>IF(L28="","",L28-J28)</f>
-        <v>731.16</v>
+        <v>3638.16</v>
       </c>
       <c r="N28" s="10">
         <f>IF(OR(H28="",K28=""),"",K28/H28-1)</f>
-        <v>0.007669363976900323</v>
+        <v>0.038161888294357516</v>
       </c>
       <c r="O28" s="6">
         <f>IF(G28="","",$B$3-G28)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P28" s="6" t="str">
         <f>IF(H28="","Pending buy",IF(N28&gt;=0,"In profit","In loss"))</f>
@@ -2209,27 +2209,27 @@
         <v>98598.59</v>
       </c>
       <c r="K29" s="9" t="n">
-        <v>1936.6</v>
+        <v>1917.7</v>
       </c>
       <c r="L29" s="9">
         <f>IF(OR(I29="",K29=""),"",K29*I29)</f>
-        <v>98766.6</v>
+        <v>97802.7</v>
       </c>
       <c r="M29" s="9">
         <f>IF(L29="","",L29-J29)</f>
-        <v>168.01</v>
+        <v>-795.89</v>
       </c>
       <c r="N29" s="10">
         <f>IF(OR(H29="",K29=""),"",K29/H29-1)</f>
-        <v>0.0017040177082441321</v>
+        <v>-0.008071984530052645</v>
       </c>
       <c r="O29" s="6">
         <f>IF(G29="","",$B$3-G29)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P29" s="6" t="str">
         <f>IF(H29="","Pending buy",IF(N29&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q29" s="6" t="n">
         <v>1</v>
@@ -2277,23 +2277,23 @@
         <v>99998.69</v>
       </c>
       <c r="K30" s="9" t="n">
-        <v>14.83</v>
+        <v>15.57</v>
       </c>
       <c r="L30" s="9">
         <f>IF(OR(I30="",K30=""),"",K30*I30)</f>
-        <v>99998.69</v>
+        <v>104988.51</v>
       </c>
       <c r="M30" s="9">
         <f>IF(L30="","",L30-J30)</f>
-        <v>0.0</v>
+        <v>4989.82</v>
       </c>
       <c r="N30" s="10">
         <f>IF(OR(H30="",K30=""),"",K30/H30-1)</f>
-        <v>0.0</v>
+        <v>0.049898853674983146</v>
       </c>
       <c r="O30" s="6">
         <f>IF(G30="","",$B$3-G30)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P30" s="6" t="str">
         <f>IF(H30="","Pending buy",IF(N30&gt;=0,"In profit","In loss"))</f>
@@ -2330,38 +2330,42 @@
       <c r="F31" s="8" t="n">
         <v>46308</v>
       </c>
-      <c r="G31" s="6" t="inlineStr"/>
-      <c r="H31" s="9" t="inlineStr"/>
-      <c r="I31" s="6" t="str">
+      <c r="G31" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H31" s="9" t="n">
+        <v>177.26</v>
+      </c>
+      <c r="I31" s="6">
         <f>IF(H31="","",ROUNDDOWN($B$1/H31,0))</f>
-        <v/>
-      </c>
-      <c r="J31" s="9" t="str">
+        <v>564</v>
+      </c>
+      <c r="J31" s="9">
         <f>IF(H31="","",H31*I31)</f>
-        <v/>
+        <v>99977.34</v>
       </c>
       <c r="K31" s="9" t="n">
-        <v>173.26</v>
-      </c>
-      <c r="L31" s="9" t="str">
+        <v>178.98</v>
+      </c>
+      <c r="L31" s="9">
         <f>IF(OR(I31="",K31=""),"",K31*I31)</f>
-        <v/>
-      </c>
-      <c r="M31" s="9" t="str">
+        <v>100944.72</v>
+      </c>
+      <c r="M31" s="9">
         <f>IF(L31="","",L31-J31)</f>
-        <v/>
-      </c>
-      <c r="N31" s="10" t="str">
+        <v>967.38</v>
+      </c>
+      <c r="N31" s="10">
         <f>IF(OR(H31="",K31=""),"",K31/H31-1)</f>
-        <v/>
-      </c>
-      <c r="O31" s="6" t="str">
+        <v>0.009676011000583129</v>
+      </c>
+      <c r="O31" s="6">
         <f>IF(G31="","",$B$3-G31)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P31" s="6" t="str">
         <f>IF(H31="","Pending buy",IF(N31&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In profit</v>
       </c>
       <c r="Q31" s="6" t="n">
         <v>1</v>
@@ -2394,38 +2398,42 @@
       <c r="F32" s="8" t="n">
         <v>46308</v>
       </c>
-      <c r="G32" s="6" t="inlineStr"/>
-      <c r="H32" s="9" t="inlineStr"/>
-      <c r="I32" s="6" t="str">
+      <c r="G32" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H32" s="9" t="n">
+        <v>176.86</v>
+      </c>
+      <c r="I32" s="6">
         <f>IF(H32="","",ROUNDDOWN($B$1/H32,0))</f>
-        <v/>
-      </c>
-      <c r="J32" s="9" t="str">
+        <v>565</v>
+      </c>
+      <c r="J32" s="9">
         <f>IF(H32="","",H32*I32)</f>
-        <v/>
+        <v>99923.82</v>
       </c>
       <c r="K32" s="9" t="n">
-        <v>172.59</v>
-      </c>
-      <c r="L32" s="9" t="str">
+        <v>181.21</v>
+      </c>
+      <c r="L32" s="9">
         <f>IF(OR(I32="",K32=""),"",K32*I32)</f>
-        <v/>
-      </c>
-      <c r="M32" s="9" t="str">
+        <v>102383.65</v>
+      </c>
+      <c r="M32" s="9">
         <f>IF(L32="","",L32-J32)</f>
-        <v/>
-      </c>
-      <c r="N32" s="10" t="str">
+        <v>2459.83</v>
+      </c>
+      <c r="N32" s="10">
         <f>IF(OR(H32="",K32=""),"",K32/H32-1)</f>
-        <v/>
-      </c>
-      <c r="O32" s="6" t="str">
+        <v>0.02461705665499614</v>
+      </c>
+      <c r="O32" s="6">
         <f>IF(G32="","",$B$3-G32)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P32" s="6" t="str">
         <f>IF(H32="","Pending buy",IF(N32&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In profit</v>
       </c>
       <c r="Q32" s="6" t="n">
         <v>1</v>
@@ -2458,38 +2466,42 @@
       <c r="F33" s="8" t="n">
         <v>46308</v>
       </c>
-      <c r="G33" s="6" t="inlineStr"/>
-      <c r="H33" s="9" t="inlineStr"/>
-      <c r="I33" s="6" t="str">
+      <c r="G33" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H33" s="9" t="n">
+        <v>527.03</v>
+      </c>
+      <c r="I33" s="6">
         <f>IF(H33="","",ROUNDDOWN($B$1/H33,0))</f>
-        <v/>
-      </c>
-      <c r="J33" s="9" t="str">
+        <v>189</v>
+      </c>
+      <c r="J33" s="9">
         <f>IF(H33="","",H33*I33)</f>
-        <v/>
+        <v>99608.58</v>
       </c>
       <c r="K33" s="9" t="n">
-        <v>529.3</v>
-      </c>
-      <c r="L33" s="9" t="str">
+        <v>528.05</v>
+      </c>
+      <c r="L33" s="9">
         <f>IF(OR(I33="",K33=""),"",K33*I33)</f>
-        <v/>
-      </c>
-      <c r="M33" s="9" t="str">
+        <v>99801.45</v>
+      </c>
+      <c r="M33" s="9">
         <f>IF(L33="","",L33-J33)</f>
-        <v/>
-      </c>
-      <c r="N33" s="10" t="str">
+        <v>192.87</v>
+      </c>
+      <c r="N33" s="10">
         <f>IF(OR(H33="",K33=""),"",K33/H33-1)</f>
-        <v/>
-      </c>
-      <c r="O33" s="6" t="str">
+        <v>0.0019363280497062263</v>
+      </c>
+      <c r="O33" s="6">
         <f>IF(G33="","",$B$3-G33)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P33" s="6" t="str">
         <f>IF(H33="","Pending buy",IF(N33&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In profit</v>
       </c>
       <c r="Q33" s="6" t="n">
         <v>1</v>
@@ -2522,45 +2534,305 @@
       <c r="F34" s="8" t="n">
         <v>46308</v>
       </c>
-      <c r="G34" s="6" t="inlineStr"/>
-      <c r="H34" s="9" t="inlineStr"/>
-      <c r="I34" s="6" t="str">
+      <c r="G34" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="H34" s="9" t="n">
+        <v>5054.23</v>
+      </c>
+      <c r="I34" s="6">
         <f>IF(H34="","",ROUNDDOWN($B$1/H34,0))</f>
-        <v/>
-      </c>
-      <c r="J34" s="9" t="str">
+        <v>19</v>
+      </c>
+      <c r="J34" s="9">
         <f>IF(H34="","",H34*I34)</f>
-        <v/>
+        <v>96030.46</v>
       </c>
       <c r="K34" s="9" t="n">
-        <v>5054.6</v>
-      </c>
-      <c r="L34" s="9" t="str">
+        <v>5067.7</v>
+      </c>
+      <c r="L34" s="9">
         <f>IF(OR(I34="",K34=""),"",K34*I34)</f>
-        <v/>
-      </c>
-      <c r="M34" s="9" t="str">
+        <v>96286.3</v>
+      </c>
+      <c r="M34" s="9">
         <f>IF(L34="","",L34-J34)</f>
-        <v/>
-      </c>
-      <c r="N34" s="10" t="str">
+        <v>255.84</v>
+      </c>
+      <c r="N34" s="10">
         <f>IF(OR(H34="",K34=""),"",K34/H34-1)</f>
-        <v/>
-      </c>
-      <c r="O34" s="6" t="str">
+        <v>0.0026641471161181762</v>
+      </c>
+      <c r="O34" s="6">
         <f>IF(G34="","",$B$3-G34)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P34" s="6" t="str">
         <f>IF(H34="","Pending buy",IF(N34&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In profit</v>
       </c>
       <c r="Q34" s="6" t="n">
         <v>1</v>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>CCL Products (India) Limited</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>CCL</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>141026</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G35" s="6" t="inlineStr"/>
+      <c r="H35" s="9" t="inlineStr"/>
+      <c r="I35" s="6" t="str">
+        <f>IF(H35="","",ROUNDDOWN($B$1/H35,0))</f>
+        <v/>
+      </c>
+      <c r="J35" s="9" t="str">
+        <f>IF(H35="","",H35*I35)</f>
+        <v/>
+      </c>
+      <c r="K35" s="9" t="n">
+        <v>1100.6</v>
+      </c>
+      <c r="L35" s="9" t="str">
+        <f>IF(OR(I35="",K35=""),"",K35*I35)</f>
+        <v/>
+      </c>
+      <c r="M35" s="9" t="str">
+        <f>IF(L35="","",L35-J35)</f>
+        <v/>
+      </c>
+      <c r="N35" s="10" t="str">
+        <f>IF(OR(H35="",K35=""),"",K35/H35-1)</f>
+        <v/>
+      </c>
+      <c r="O35" s="6" t="str">
+        <f>IF(G35="","",$B$3-G35)</f>
+        <v/>
+      </c>
+      <c r="P35" s="6" t="str">
+        <f>IF(H35="","Pending buy",IF(N35&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q35" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Jayaswal Neco Industries Limited</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>JAYNECOIND</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>141026</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G36" s="6" t="inlineStr"/>
+      <c r="H36" s="9" t="inlineStr"/>
+      <c r="I36" s="6" t="str">
+        <f>IF(H36="","",ROUNDDOWN($B$1/H36,0))</f>
+        <v/>
+      </c>
+      <c r="J36" s="9" t="str">
+        <f>IF(H36="","",H36*I36)</f>
+        <v/>
+      </c>
+      <c r="K36" s="9" t="n">
+        <v>98.97</v>
+      </c>
+      <c r="L36" s="9" t="str">
+        <f>IF(OR(I36="",K36=""),"",K36*I36)</f>
+        <v/>
+      </c>
+      <c r="M36" s="9" t="str">
+        <f>IF(L36="","",L36-J36)</f>
+        <v/>
+      </c>
+      <c r="N36" s="10" t="str">
+        <f>IF(OR(H36="",K36=""),"",K36/H36-1)</f>
+        <v/>
+      </c>
+      <c r="O36" s="6" t="str">
+        <f>IF(G36="","",$B$3-G36)</f>
+        <v/>
+      </c>
+      <c r="P36" s="6" t="str">
+        <f>IF(H36="","Pending buy",IF(N36&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q36" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Sakar Healthcare Limited</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>SAKAR</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>141026</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G37" s="6" t="inlineStr"/>
+      <c r="H37" s="9" t="inlineStr"/>
+      <c r="I37" s="6" t="str">
+        <f>IF(H37="","",ROUNDDOWN($B$1/H37,0))</f>
+        <v/>
+      </c>
+      <c r="J37" s="9" t="str">
+        <f>IF(H37="","",H37*I37)</f>
+        <v/>
+      </c>
+      <c r="K37" s="9" t="n">
+        <v>1020.8</v>
+      </c>
+      <c r="L37" s="9" t="str">
+        <f>IF(OR(I37="",K37=""),"",K37*I37)</f>
+        <v/>
+      </c>
+      <c r="M37" s="9" t="str">
+        <f>IF(L37="","",L37-J37)</f>
+        <v/>
+      </c>
+      <c r="N37" s="10" t="str">
+        <f>IF(OR(H37="",K37=""),"",K37/H37-1)</f>
+        <v/>
+      </c>
+      <c r="O37" s="6" t="str">
+        <f>IF(G37="","",$B$3-G37)</f>
+        <v/>
+      </c>
+      <c r="P37" s="6" t="str">
+        <f>IF(H37="","Pending buy",IF(N37&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q37" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Tamilnadu PetroProducts Limited</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>TNPETRO</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>141026</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="G38" s="6" t="inlineStr"/>
+      <c r="H38" s="9" t="inlineStr"/>
+      <c r="I38" s="6" t="str">
+        <f>IF(H38="","",ROUNDDOWN($B$1/H38,0))</f>
+        <v/>
+      </c>
+      <c r="J38" s="9" t="str">
+        <f>IF(H38="","",H38*I38)</f>
+        <v/>
+      </c>
+      <c r="K38" s="9" t="n">
+        <v>120.68</v>
+      </c>
+      <c r="L38" s="9" t="str">
+        <f>IF(OR(I38="",K38=""),"",K38*I38)</f>
+        <v/>
+      </c>
+      <c r="M38" s="9" t="str">
+        <f>IF(L38="","",L38-J38)</f>
+        <v/>
+      </c>
+      <c r="N38" s="10" t="str">
+        <f>IF(OR(H38="",K38=""),"",K38/H38-1)</f>
+        <v/>
+      </c>
+      <c r="O38" s="6" t="str">
+        <f>IF(G38="","",$B$3-G38)</f>
+        <v/>
+      </c>
+      <c r="P38" s="6" t="str">
+        <f>IF(H38="","Pending buy",IF(N38&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q38" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A8:Q34">
+  <conditionalFormatting sqref="A8:Q38">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$N8&gt;0</formula>
     </cfRule>
@@ -2578,7 +2850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3226,6 +3498,86 @@
       <c r="D32" s="11" t="inlineStr">
         <is>
           <t>Kapston Services Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>CCL</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
+        <is>
+          <t>CCL Products (India) Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>JAYNECOIND</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>Jayaswal Neco Industries Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>SAKAR</t>
+        </is>
+      </c>
+      <c r="D35" s="11" t="inlineStr">
+        <is>
+          <t>Sakar Healthcare Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>TNPETRO</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t>Tamilnadu PetroProducts Limited</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum Portfolio: weekday silent update 2026-10-15
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="E1" s="2">
         <f>SUM(J8:J38)</f>
-        <v>2665788.8</v>
+        <v>3064170.25</v>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
@@ -541,7 +541,7 @@
       </c>
       <c r="G1" s="2">
         <f>SUM(L8:L38)</f>
-        <v>2623522.7</v>
+        <v>2985740.8</v>
       </c>
     </row>
     <row r="2">
@@ -552,7 +552,7 @@
       </c>
       <c r="E2" s="2">
         <f>SUM(M8:M38)</f>
-        <v>-42266.1</v>
+        <v>-78429.45</v>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" s="3">
         <f>IF(E1=0,"",G1/E1-1)</f>
-        <v>-0.015855006968293783</v>
+        <v>-0.0255956567687452</v>
       </c>
     </row>
     <row r="3">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -580,7 +580,7 @@
       </c>
       <c r="E3">
         <f>COUNTIF(M8:M38,"&gt;0")</f>
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
@@ -589,7 +589,7 @@
       </c>
       <c r="G3">
         <f>COUNTIF(M8:M38,"&lt;0")</f>
-        <v>15</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -600,7 +600,7 @@
       </c>
       <c r="E4" s="3">
         <f>IF((E3+G3)=0,"",E3/(E3+G3))</f>
-        <v>0.4444444444444444</v>
+        <v>0.22580645161290322</v>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
@@ -609,7 +609,7 @@
       </c>
       <c r="G4" s="3">
         <f>AVERAGE(N8:N38)</f>
-        <v>-0.01597260461428871</v>
+        <v>-0.025787073050585047</v>
       </c>
     </row>
     <row r="5">
@@ -620,7 +620,7 @@
       </c>
       <c r="E5" t="str">
         <f>INDEX(B8:B38,MATCH(MAX(N8:N38),N8:N38,0))</f>
-        <v>Black Box Limited</v>
+        <v>Viji Finance Limited</v>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
@@ -640,7 +640,7 @@
       </c>
       <c r="E6" s="3">
         <f>AVERAGEIF(D8:D38,"4★*",N8:N38)</f>
-        <v>-0.023707883039176352</v>
+        <v>-0.04123686906021496</v>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
@@ -649,7 +649,7 @@
       </c>
       <c r="G6" s="3">
         <f>AVERAGEIF(D8:D38,"5★*",N8:N38)</f>
-        <v>-0.008789846076893046</v>
+        <v>-0.011302889291557004</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
@@ -781,27 +781,27 @@
         <v>99851.29</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>302.6</v>
+        <v>296.4</v>
       </c>
       <c r="L8" s="9">
         <f>IF(OR(I8="",K8=""),"",K8*I8)</f>
-        <v>100463.2</v>
+        <v>98404.8</v>
       </c>
       <c r="M8" s="9">
         <f>IF(L8="","",L8-J8)</f>
-        <v>611.91</v>
+        <v>-1446.49</v>
       </c>
       <c r="N8" s="10">
         <f>IF(OR(H8="",K8=""),"",K8/H8-1)</f>
-        <v>0.006128178442371901</v>
+        <v>-0.014486476899144174</v>
       </c>
       <c r="O8" s="6">
         <f>IF(G8="","",$B$3-G8)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P8" s="6" t="str">
         <f>IF(H8="","Pending buy",IF(N8&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q8" s="6" t="n">
         <v>2</v>
@@ -849,23 +849,23 @@
         <v>99687.42</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="L9" s="9">
         <f>IF(OR(I9="",K9=""),"",K9*I9)</f>
-        <v>96696.0</v>
+        <v>98838.0</v>
       </c>
       <c r="M9" s="9">
         <f>IF(L9="","",L9-J9)</f>
-        <v>-2991.42</v>
+        <v>-849.42</v>
       </c>
       <c r="N9" s="10">
         <f>IF(OR(H9="",K9=""),"",K9/H9-1)</f>
-        <v>-0.030008000929890866</v>
+        <v>-0.008520836393527742</v>
       </c>
       <c r="O9" s="6">
         <f>IF(G9="","",$B$3-G9)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P9" s="6" t="str">
         <f>IF(H9="","Pending buy",IF(N9&gt;=0,"In profit","In loss"))</f>
@@ -917,23 +917,23 @@
         <v>99607.14</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>1548.4</v>
+        <v>1559</v>
       </c>
       <c r="L10" s="9">
         <f>IF(OR(I10="",K10=""),"",K10*I10)</f>
-        <v>97549.2</v>
+        <v>98217.0</v>
       </c>
       <c r="M10" s="9">
         <f>IF(L10="","",L10-J10)</f>
-        <v>-2057.94</v>
+        <v>-1390.14</v>
       </c>
       <c r="N10" s="10">
         <f>IF(OR(H10="",K10=""),"",K10/H10-1)</f>
-        <v>-0.02066057621820716</v>
+        <v>-0.013956237615722733</v>
       </c>
       <c r="O10" s="6">
         <f>IF(G10="","",$B$3-G10)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P10" s="6" t="str">
         <f>IF(H10="","Pending buy",IF(N10&gt;=0,"In profit","In loss"))</f>
@@ -985,23 +985,23 @@
         <v>99927.23</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>71.83</v>
+        <v>70.31</v>
       </c>
       <c r="L11" s="9">
         <f>IF(OR(I11="",K11=""),"",K11*I11)</f>
-        <v>89859.33</v>
+        <v>87957.81</v>
       </c>
       <c r="M11" s="9">
         <f>IF(L11="","",L11-J11)</f>
-        <v>-10067.9</v>
+        <v>-11969.42</v>
       </c>
       <c r="N11" s="10">
         <f>IF(OR(H11="",K11=""),"",K11/H11-1)</f>
-        <v>-0.1007523208990444</v>
+        <v>-0.11978136826412089</v>
       </c>
       <c r="O11" s="6">
         <f>IF(G11="","",$B$3-G11)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P11" s="6" t="str">
         <f>IF(H11="","Pending buy",IF(N11&gt;=0,"In profit","In loss"))</f>
@@ -1053,23 +1053,23 @@
         <v>86537.12</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>20200</v>
+        <v>19955</v>
       </c>
       <c r="L12" s="9">
         <f>IF(OR(I12="",K12=""),"",K12*I12)</f>
-        <v>80800.0</v>
+        <v>79820.0</v>
       </c>
       <c r="M12" s="9">
         <f>IF(L12="","",L12-J12)</f>
-        <v>-5737.12</v>
+        <v>-6717.12</v>
       </c>
       <c r="N12" s="10">
         <f>IF(OR(H12="",K12=""),"",K12/H12-1)</f>
-        <v>-0.06629659498611529</v>
+        <v>-0.0776212154924718</v>
       </c>
       <c r="O12" s="6">
         <f>IF(G12="","",$B$3-G12)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P12" s="6" t="str">
         <f>IF(H12="","Pending buy",IF(N12&gt;=0,"In profit","In loss"))</f>
@@ -1121,23 +1121,23 @@
         <v>98177.53</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>1746.9</v>
+        <v>1717.2</v>
       </c>
       <c r="L13" s="9">
         <f>IF(OR(I13="",K13=""),"",K13*I13)</f>
-        <v>92585.7</v>
+        <v>91011.6</v>
       </c>
       <c r="M13" s="9">
         <f>IF(L13="","",L13-J13)</f>
-        <v>-5591.83</v>
+        <v>-7165.93</v>
       </c>
       <c r="N13" s="10">
         <f>IF(OR(H13="",K13=""),"",K13/H13-1)</f>
-        <v>-0.05695634202787403</v>
+        <v>-0.07298954177701378</v>
       </c>
       <c r="O13" s="6">
         <f>IF(G13="","",$B$3-G13)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P13" s="6" t="str">
         <f>IF(H13="","Pending buy",IF(N13&gt;=0,"In profit","In loss"))</f>
@@ -1189,23 +1189,23 @@
         <v>97667.46</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>4554.1</v>
+        <v>4449</v>
       </c>
       <c r="L14" s="9">
         <f>IF(OR(I14="",K14=""),"",K14*I14)</f>
-        <v>100190.2</v>
+        <v>97878.0</v>
       </c>
       <c r="M14" s="9">
         <f>IF(L14="","",L14-J14)</f>
-        <v>2522.74</v>
+        <v>210.54</v>
       </c>
       <c r="N14" s="10">
         <f>IF(OR(H14="",K14=""),"",K14/H14-1)</f>
-        <v>0.02582984867253879</v>
+        <v>0.002155639257839015</v>
       </c>
       <c r="O14" s="6">
         <f>IF(G14="","",$B$3-G14)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P14" s="6" t="str">
         <f>IF(H14="","Pending buy",IF(N14&gt;=0,"In profit","In loss"))</f>
@@ -1257,27 +1257,27 @@
         <v>99078.19</v>
       </c>
       <c r="K15" s="9" t="n">
-        <v>1557.2</v>
+        <v>1520.9</v>
       </c>
       <c r="L15" s="9">
         <f>IF(OR(I15="",K15=""),"",K15*I15)</f>
-        <v>99660.8</v>
+        <v>97337.6</v>
       </c>
       <c r="M15" s="9">
         <f>IF(L15="","",L15-J15)</f>
-        <v>582.61</v>
+        <v>-1740.59</v>
       </c>
       <c r="N15" s="10">
         <f>IF(OR(H15="",K15=""),"",K15/H15-1)</f>
-        <v>0.005880329769920811</v>
+        <v>-0.017567818169103022</v>
       </c>
       <c r="O15" s="6">
         <f>IF(G15="","",$B$3-G15)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P15" s="6" t="str">
         <f>IF(H15="","Pending buy",IF(N15&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q15" s="6" t="n">
         <v>2</v>
@@ -1325,23 +1325,23 @@
         <v>98557.54</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>1467</v>
+        <v>1470</v>
       </c>
       <c r="L16" s="9">
         <f>IF(OR(I16="",K16=""),"",K16*I16)</f>
-        <v>99756.0</v>
+        <v>99960.0</v>
       </c>
       <c r="M16" s="9">
         <f>IF(L16="","",L16-J16)</f>
-        <v>1198.46</v>
+        <v>1402.46</v>
       </c>
       <c r="N16" s="10">
         <f>IF(OR(H16="",K16=""),"",K16/H16-1)</f>
-        <v>0.01216003896166229</v>
+        <v>0.014229895892054145</v>
       </c>
       <c r="O16" s="6">
         <f>IF(G16="","",$B$3-G16)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P16" s="6" t="str">
         <f>IF(H16="","Pending buy",IF(N16&gt;=0,"In profit","In loss"))</f>
@@ -1393,23 +1393,23 @@
         <v>99714.35</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>935.8</v>
+        <v>880.2</v>
       </c>
       <c r="L17" s="9">
         <f>IF(OR(I17="",K17=""),"",K17*I17)</f>
-        <v>107617.0</v>
+        <v>101223.0</v>
       </c>
       <c r="M17" s="9">
         <f>IF(L17="","",L17-J17)</f>
-        <v>7902.65</v>
+        <v>1508.65</v>
       </c>
       <c r="N17" s="10">
         <f>IF(OR(H17="",K17=""),"",K17/H17-1)</f>
-        <v>0.07925288505672468</v>
+        <v>0.015129717276051835</v>
       </c>
       <c r="O17" s="6">
         <f>IF(G17="","",$B$3-G17)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P17" s="6" t="str">
         <f>IF(H17="","Pending buy",IF(N17&gt;=0,"In profit","In loss"))</f>
@@ -1461,23 +1461,23 @@
         <v>99596.83</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>647.65</v>
+        <v>625.6</v>
       </c>
       <c r="L18" s="9">
         <f>IF(OR(I18="",K18=""),"",K18*I18)</f>
-        <v>91318.65</v>
+        <v>88209.6</v>
       </c>
       <c r="M18" s="9">
         <f>IF(L18="","",L18-J18)</f>
-        <v>-8278.18</v>
+        <v>-11387.23</v>
       </c>
       <c r="N18" s="10">
         <f>IF(OR(H18="",K18=""),"",K18/H18-1)</f>
-        <v>-0.0831169446615555</v>
+        <v>-0.11433329820160443</v>
       </c>
       <c r="O18" s="6">
         <f>IF(G18="","",$B$3-G18)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P18" s="6" t="str">
         <f>IF(H18="","Pending buy",IF(N18&gt;=0,"In profit","In loss"))</f>
@@ -1529,23 +1529,23 @@
         <v>99993.07</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>149.57</v>
+        <v>142.54</v>
       </c>
       <c r="L19" s="9">
         <f>IF(OR(I19="",K19=""),"",K19*I19)</f>
-        <v>99164.91</v>
+        <v>94504.02</v>
       </c>
       <c r="M19" s="9">
         <f>IF(L19="","",L19-J19)</f>
-        <v>-828.16</v>
+        <v>-5489.05</v>
       </c>
       <c r="N19" s="10">
         <f>IF(OR(H19="",K19=""),"",K19/H19-1)</f>
-        <v>-0.008282127231588277</v>
+        <v>-0.054894259648262334</v>
       </c>
       <c r="O19" s="6">
         <f>IF(G19="","",$B$3-G19)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P19" s="6" t="str">
         <f>IF(H19="","Pending buy",IF(N19&gt;=0,"In profit","In loss"))</f>
@@ -1597,23 +1597,23 @@
         <v>99896.43</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>203.32</v>
+        <v>202.72</v>
       </c>
       <c r="L20" s="9">
         <f>IF(OR(I20="",K20=""),"",K20*I20)</f>
-        <v>96983.64</v>
+        <v>96697.44</v>
       </c>
       <c r="M20" s="9">
         <f>IF(L20="","",L20-J20)</f>
-        <v>-2912.79</v>
+        <v>-3198.99</v>
       </c>
       <c r="N20" s="10">
         <f>IF(OR(H20="",K20=""),"",K20/H20-1)</f>
-        <v>-0.02915809910148992</v>
+        <v>-0.0320230663478952</v>
       </c>
       <c r="O20" s="6">
         <f>IF(G20="","",$B$3-G20)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P20" s="6" t="str">
         <f>IF(H20="","Pending buy",IF(N20&gt;=0,"In profit","In loss"))</f>
@@ -1665,23 +1665,23 @@
         <v>99449.47</v>
       </c>
       <c r="K21" s="9" t="n">
-        <v>1281.5</v>
+        <v>1258.8</v>
       </c>
       <c r="L21" s="9">
         <f>IF(OR(I21="",K21=""),"",K21*I21)</f>
-        <v>90986.5</v>
+        <v>89374.8</v>
       </c>
       <c r="M21" s="9">
         <f>IF(L21="","",L21-J21)</f>
-        <v>-8462.97</v>
+        <v>-10074.67</v>
       </c>
       <c r="N21" s="10">
         <f>IF(OR(H21="",K21=""),"",K21/H21-1)</f>
-        <v>-0.08509815739133009</v>
+        <v>-0.10130437809146031</v>
       </c>
       <c r="O21" s="6">
         <f>IF(G21="","",$B$3-G21)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P21" s="6" t="str">
         <f>IF(H21="","Pending buy",IF(N21&gt;=0,"In profit","In loss"))</f>
@@ -1733,23 +1733,23 @@
         <v>99837.05</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>684.4</v>
+        <v>663.25</v>
       </c>
       <c r="L22" s="9">
         <f>IF(OR(I22="",K22=""),"",K22*I22)</f>
-        <v>98553.6</v>
+        <v>95508.0</v>
       </c>
       <c r="M22" s="9">
         <f>IF(L22="","",L22-J22)</f>
-        <v>-1283.45</v>
+        <v>-4329.05</v>
       </c>
       <c r="N22" s="10">
         <f>IF(OR(H22="",K22=""),"",K22/H22-1)</f>
-        <v>-0.012855459026502647</v>
+        <v>-0.04336116773718268</v>
       </c>
       <c r="O22" s="6">
         <f>IF(G22="","",$B$3-G22)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P22" s="6" t="str">
         <f>IF(H22="","Pending buy",IF(N22&gt;=0,"In profit","In loss"))</f>
@@ -1801,23 +1801,23 @@
         <v>99486.88</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>647.7</v>
+        <v>640.5</v>
       </c>
       <c r="L23" s="9">
         <f>IF(OR(I23="",K23=""),"",K23*I23)</f>
-        <v>93916.5</v>
+        <v>92872.5</v>
       </c>
       <c r="M23" s="9">
         <f>IF(L23="","",L23-J23)</f>
-        <v>-5570.38</v>
+        <v>-6614.38</v>
       </c>
       <c r="N23" s="10">
         <f>IF(OR(H23="",K23=""),"",K23/H23-1)</f>
-        <v>-0.05599111283186853</v>
+        <v>-0.06648495872905946</v>
       </c>
       <c r="O23" s="6">
         <f>IF(G23="","",$B$3-G23)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P23" s="6" t="str">
         <f>IF(H23="","Pending buy",IF(N23&gt;=0,"In profit","In loss"))</f>
@@ -1869,23 +1869,23 @@
         <v>99935.4</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>223.71</v>
+        <v>221.03</v>
       </c>
       <c r="L24" s="9">
         <f>IF(OR(I24="",K24=""),"",K24*I24)</f>
-        <v>98208.69</v>
+        <v>97032.17</v>
       </c>
       <c r="M24" s="9">
         <f>IF(L24="","",L24-J24)</f>
-        <v>-1726.71</v>
+        <v>-2903.23</v>
       </c>
       <c r="N24" s="10">
         <f>IF(OR(H24="",K24=""),"",K24/H24-1)</f>
-        <v>-0.017278248019597764</v>
+        <v>-0.02905105341635017</v>
       </c>
       <c r="O24" s="6">
         <f>IF(G24="","",$B$3-G24)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P24" s="6" t="str">
         <f>IF(H24="","Pending buy",IF(N24&gt;=0,"In profit","In loss"))</f>
@@ -1937,27 +1937,27 @@
         <v>99622.64</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>803.9</v>
+        <v>790.65</v>
       </c>
       <c r="L25" s="9">
         <f>IF(OR(I25="",K25=""),"",K25*I25)</f>
-        <v>99683.6</v>
+        <v>98040.6</v>
       </c>
       <c r="M25" s="9">
         <f>IF(L25="","",L25-J25)</f>
-        <v>60.96</v>
+        <v>-1582.04</v>
       </c>
       <c r="N25" s="10">
         <f>IF(OR(H25="",K25=""),"",K25/H25-1)</f>
-        <v>0.0006119453390103224</v>
+        <v>-0.01588029035665084</v>
       </c>
       <c r="O25" s="6">
         <f>IF(G25="","",$B$3-G25)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P25" s="6" t="str">
         <f>IF(H25="","Pending buy",IF(N25&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q25" s="6" t="n">
         <v>1</v>
@@ -2005,23 +2005,23 @@
         <v>99948.17</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>191.41</v>
+        <v>196.99</v>
       </c>
       <c r="L26" s="9">
         <f>IF(OR(I26="",K26=""),"",K26*I26)</f>
-        <v>90919.75</v>
+        <v>93570.25</v>
       </c>
       <c r="M26" s="9">
         <f>IF(L26="","",L26-J26)</f>
-        <v>-9028.42</v>
+        <v>-6377.92</v>
       </c>
       <c r="N26" s="10">
         <f>IF(OR(H26="",K26=""),"",K26/H26-1)</f>
-        <v>-0.09033098830474373</v>
+        <v>-0.06381224275717812</v>
       </c>
       <c r="O26" s="6">
         <f>IF(G26="","",$B$3-G26)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P26" s="6" t="str">
         <f>IF(H26="","Pending buy",IF(N26&gt;=0,"In profit","In loss"))</f>
@@ -2073,23 +2073,23 @@
         <v>99745.27</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>255.05</v>
+        <v>251.05</v>
       </c>
       <c r="L27" s="9">
         <f>IF(OR(I27="",K27=""),"",K27*I27)</f>
-        <v>97429.1</v>
+        <v>95901.1</v>
       </c>
       <c r="M27" s="9">
         <f>IF(L27="","",L27-J27)</f>
-        <v>-2316.17</v>
+        <v>-3844.17</v>
       </c>
       <c r="N27" s="10">
         <f>IF(OR(H27="",K27=""),"",K27/H27-1)</f>
-        <v>-0.023220879458907495</v>
+        <v>-0.038539901149416744</v>
       </c>
       <c r="O27" s="6">
         <f>IF(G27="","",$B$3-G27)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P27" s="6" t="str">
         <f>IF(H27="","Pending buy",IF(N27&gt;=0,"In profit","In loss"))</f>
@@ -2141,23 +2141,23 @@
         <v>95334.84</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>10997</v>
+        <v>10941</v>
       </c>
       <c r="L28" s="9">
         <f>IF(OR(I28="",K28=""),"",K28*I28)</f>
-        <v>98973.0</v>
+        <v>98469.0</v>
       </c>
       <c r="M28" s="9">
         <f>IF(L28="","",L28-J28)</f>
-        <v>3638.16</v>
+        <v>3134.16</v>
       </c>
       <c r="N28" s="10">
         <f>IF(OR(H28="",K28=""),"",K28/H28-1)</f>
-        <v>0.038161888294357516</v>
+        <v>0.03287525869133079</v>
       </c>
       <c r="O28" s="6">
         <f>IF(G28="","",$B$3-G28)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P28" s="6" t="str">
         <f>IF(H28="","Pending buy",IF(N28&gt;=0,"In profit","In loss"))</f>
@@ -2209,23 +2209,23 @@
         <v>98598.59</v>
       </c>
       <c r="K29" s="9" t="n">
-        <v>1917.7</v>
+        <v>1873.2</v>
       </c>
       <c r="L29" s="9">
         <f>IF(OR(I29="",K29=""),"",K29*I29)</f>
-        <v>97802.7</v>
+        <v>95533.2</v>
       </c>
       <c r="M29" s="9">
         <f>IF(L29="","",L29-J29)</f>
-        <v>-795.89</v>
+        <v>-3065.39</v>
       </c>
       <c r="N29" s="10">
         <f>IF(OR(H29="",K29=""),"",K29/H29-1)</f>
-        <v>-0.008071984530052645</v>
+        <v>-0.031089555937682922</v>
       </c>
       <c r="O29" s="6">
         <f>IF(G29="","",$B$3-G29)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P29" s="6" t="str">
         <f>IF(H29="","Pending buy",IF(N29&gt;=0,"In profit","In loss"))</f>
@@ -2277,23 +2277,23 @@
         <v>99998.69</v>
       </c>
       <c r="K30" s="9" t="n">
-        <v>15.57</v>
+        <v>16.34</v>
       </c>
       <c r="L30" s="9">
         <f>IF(OR(I30="",K30=""),"",K30*I30)</f>
-        <v>104988.51</v>
+        <v>110180.62</v>
       </c>
       <c r="M30" s="9">
         <f>IF(L30="","",L30-J30)</f>
-        <v>4989.82</v>
+        <v>10181.93</v>
       </c>
       <c r="N30" s="10">
         <f>IF(OR(H30="",K30=""),"",K30/H30-1)</f>
-        <v>0.049898853674983146</v>
+        <v>0.10182063385030338</v>
       </c>
       <c r="O30" s="6">
         <f>IF(G30="","",$B$3-G30)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P30" s="6" t="str">
         <f>IF(H30="","Pending buy",IF(N30&gt;=0,"In profit","In loss"))</f>
@@ -2345,27 +2345,27 @@
         <v>99977.34</v>
       </c>
       <c r="K31" s="9" t="n">
-        <v>178.98</v>
+        <v>173.7</v>
       </c>
       <c r="L31" s="9">
         <f>IF(OR(I31="",K31=""),"",K31*I31)</f>
-        <v>100944.72</v>
+        <v>97966.8</v>
       </c>
       <c r="M31" s="9">
         <f>IF(L31="","",L31-J31)</f>
-        <v>967.38</v>
+        <v>-2010.54</v>
       </c>
       <c r="N31" s="10">
         <f>IF(OR(H31="",K31=""),"",K31/H31-1)</f>
-        <v>0.009676011000583129</v>
+        <v>-0.020109939038991498</v>
       </c>
       <c r="O31" s="6">
         <f>IF(G31="","",$B$3-G31)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P31" s="6" t="str">
         <f>IF(H31="","Pending buy",IF(N31&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q31" s="6" t="n">
         <v>1</v>
@@ -2413,23 +2413,23 @@
         <v>99923.82</v>
       </c>
       <c r="K32" s="9" t="n">
-        <v>181.21</v>
+        <v>190.04</v>
       </c>
       <c r="L32" s="9">
         <f>IF(OR(I32="",K32=""),"",K32*I32)</f>
-        <v>102383.65</v>
+        <v>107372.6</v>
       </c>
       <c r="M32" s="9">
         <f>IF(L32="","",L32-J32)</f>
-        <v>2459.83</v>
+        <v>7448.78</v>
       </c>
       <c r="N32" s="10">
         <f>IF(OR(H32="",K32=""),"",K32/H32-1)</f>
-        <v>0.02461705665499614</v>
+        <v>0.07454459161589022</v>
       </c>
       <c r="O32" s="6">
         <f>IF(G32="","",$B$3-G32)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P32" s="6" t="str">
         <f>IF(H32="","Pending buy",IF(N32&gt;=0,"In profit","In loss"))</f>
@@ -2481,23 +2481,23 @@
         <v>99608.58</v>
       </c>
       <c r="K33" s="9" t="n">
-        <v>528.05</v>
+        <v>529.6</v>
       </c>
       <c r="L33" s="9">
         <f>IF(OR(I33="",K33=""),"",K33*I33)</f>
-        <v>99801.45</v>
+        <v>100094.4</v>
       </c>
       <c r="M33" s="9">
         <f>IF(L33="","",L33-J33)</f>
-        <v>192.87</v>
+        <v>485.82</v>
       </c>
       <c r="N33" s="10">
         <f>IF(OR(H33="",K33=""),"",K33/H33-1)</f>
-        <v>0.0019363280497062263</v>
+        <v>0.004877339901760092</v>
       </c>
       <c r="O33" s="6">
         <f>IF(G33="","",$B$3-G33)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P33" s="6" t="str">
         <f>IF(H33="","Pending buy",IF(N33&gt;=0,"In profit","In loss"))</f>
@@ -2549,27 +2549,27 @@
         <v>96030.46</v>
       </c>
       <c r="K34" s="9" t="n">
-        <v>5067.7</v>
+        <v>4712.1</v>
       </c>
       <c r="L34" s="9">
         <f>IF(OR(I34="",K34=""),"",K34*I34)</f>
-        <v>96286.3</v>
+        <v>89529.9</v>
       </c>
       <c r="M34" s="9">
         <f>IF(L34="","",L34-J34)</f>
-        <v>255.84</v>
+        <v>-6500.56</v>
       </c>
       <c r="N34" s="10">
         <f>IF(OR(H34="",K34=""),"",K34/H34-1)</f>
-        <v>0.0026641471161181762</v>
+        <v>-0.06769269537939093</v>
       </c>
       <c r="O34" s="6">
         <f>IF(G34="","",$B$3-G34)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P34" s="6" t="str">
         <f>IF(H34="","Pending buy",IF(N34&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q34" s="6" t="n">
         <v>1</v>
@@ -2602,38 +2602,42 @@
       <c r="F35" s="8" t="n">
         <v>46309</v>
       </c>
-      <c r="G35" s="6" t="inlineStr"/>
-      <c r="H35" s="9" t="inlineStr"/>
-      <c r="I35" s="6" t="str">
+      <c r="G35" s="8" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H35" s="9" t="n">
+        <v>1088.82</v>
+      </c>
+      <c r="I35" s="6">
         <f>IF(H35="","",ROUNDDOWN($B$1/H35,0))</f>
-        <v/>
-      </c>
-      <c r="J35" s="9" t="str">
+        <v>91</v>
+      </c>
+      <c r="J35" s="9">
         <f>IF(H35="","",H35*I35)</f>
-        <v/>
+        <v>99082.89</v>
       </c>
       <c r="K35" s="9" t="n">
-        <v>1100.6</v>
-      </c>
-      <c r="L35" s="9" t="str">
+        <v>1085.4</v>
+      </c>
+      <c r="L35" s="9">
         <f>IF(OR(I35="",K35=""),"",K35*I35)</f>
-        <v/>
-      </c>
-      <c r="M35" s="9" t="str">
+        <v>98771.4</v>
+      </c>
+      <c r="M35" s="9">
         <f>IF(L35="","",L35-J35)</f>
-        <v/>
-      </c>
-      <c r="N35" s="10" t="str">
+        <v>-311.49</v>
+      </c>
+      <c r="N35" s="10">
         <f>IF(OR(H35="",K35=""),"",K35/H35-1)</f>
-        <v/>
-      </c>
-      <c r="O35" s="6" t="str">
+        <v>-0.003143761658230937</v>
+      </c>
+      <c r="O35" s="6">
         <f>IF(G35="","",$B$3-G35)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P35" s="6" t="str">
         <f>IF(H35="","Pending buy",IF(N35&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q35" s="6" t="n">
         <v>1</v>
@@ -2666,38 +2670,42 @@
       <c r="F36" s="8" t="n">
         <v>46309</v>
       </c>
-      <c r="G36" s="6" t="inlineStr"/>
-      <c r="H36" s="9" t="inlineStr"/>
-      <c r="I36" s="6" t="str">
+      <c r="G36" s="8" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H36" s="9" t="n">
+        <v>97.47</v>
+      </c>
+      <c r="I36" s="6">
         <f>IF(H36="","",ROUNDDOWN($B$1/H36,0))</f>
-        <v/>
-      </c>
-      <c r="J36" s="9" t="str">
+        <v>1025</v>
+      </c>
+      <c r="J36" s="9">
         <f>IF(H36="","",H36*I36)</f>
-        <v/>
+        <v>99910.57</v>
       </c>
       <c r="K36" s="9" t="n">
-        <v>98.97</v>
-      </c>
-      <c r="L36" s="9" t="str">
+        <v>96.34999999999999</v>
+      </c>
+      <c r="L36" s="9">
         <f>IF(OR(I36="",K36=""),"",K36*I36)</f>
-        <v/>
-      </c>
-      <c r="M36" s="9" t="str">
+        <v>98758.75</v>
+      </c>
+      <c r="M36" s="9">
         <f>IF(L36="","",L36-J36)</f>
-        <v/>
-      </c>
-      <c r="N36" s="10" t="str">
+        <v>-1151.82</v>
+      </c>
+      <c r="N36" s="10">
         <f>IF(OR(H36="",K36=""),"",K36/H36-1)</f>
-        <v/>
-      </c>
-      <c r="O36" s="6" t="str">
+        <v>-0.011528521818720217</v>
+      </c>
+      <c r="O36" s="6">
         <f>IF(G36="","",$B$3-G36)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P36" s="6" t="str">
         <f>IF(H36="","Pending buy",IF(N36&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q36" s="6" t="n">
         <v>1</v>
@@ -2730,38 +2738,42 @@
       <c r="F37" s="8" t="n">
         <v>46309</v>
       </c>
-      <c r="G37" s="6" t="inlineStr"/>
-      <c r="H37" s="9" t="inlineStr"/>
-      <c r="I37" s="6" t="str">
+      <c r="G37" s="8" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H37" s="9" t="n">
+        <v>994.37</v>
+      </c>
+      <c r="I37" s="6">
         <f>IF(H37="","",ROUNDDOWN($B$1/H37,0))</f>
-        <v/>
-      </c>
-      <c r="J37" s="9" t="str">
+        <v>100</v>
+      </c>
+      <c r="J37" s="9">
         <f>IF(H37="","",H37*I37)</f>
-        <v/>
+        <v>99436.51</v>
       </c>
       <c r="K37" s="9" t="n">
-        <v>1020.8</v>
-      </c>
-      <c r="L37" s="9" t="str">
+        <v>989.5</v>
+      </c>
+      <c r="L37" s="9">
         <f>IF(OR(I37="",K37=""),"",K37*I37)</f>
-        <v/>
-      </c>
-      <c r="M37" s="9" t="str">
+        <v>98950.0</v>
+      </c>
+      <c r="M37" s="9">
         <f>IF(L37="","",L37-J37)</f>
-        <v/>
-      </c>
-      <c r="N37" s="10" t="str">
+        <v>-486.51</v>
+      </c>
+      <c r="N37" s="10">
         <f>IF(OR(H37="",K37=""),"",K37/H37-1)</f>
-        <v/>
-      </c>
-      <c r="O37" s="6" t="str">
+        <v>-0.004892698726163824</v>
+      </c>
+      <c r="O37" s="6">
         <f>IF(G37="","",$B$3-G37)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P37" s="6" t="str">
         <f>IF(H37="","Pending buy",IF(N37&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q37" s="6" t="n">
         <v>1</v>
@@ -2794,38 +2806,42 @@
       <c r="F38" s="8" t="n">
         <v>46309</v>
       </c>
-      <c r="G38" s="6" t="inlineStr"/>
-      <c r="H38" s="9" t="inlineStr"/>
-      <c r="I38" s="6" t="str">
+      <c r="G38" s="8" t="n">
+        <v>46310</v>
+      </c>
+      <c r="H38" s="9" t="n">
+        <v>122.04</v>
+      </c>
+      <c r="I38" s="6">
         <f>IF(H38="","",ROUNDDOWN($B$1/H38,0))</f>
-        <v/>
-      </c>
-      <c r="J38" s="9" t="str">
+        <v>819</v>
+      </c>
+      <c r="J38" s="9">
         <f>IF(H38="","",H38*I38)</f>
-        <v/>
+        <v>99951.48</v>
       </c>
       <c r="K38" s="9" t="n">
-        <v>120.68</v>
-      </c>
-      <c r="L38" s="9" t="str">
+        <v>119.36</v>
+      </c>
+      <c r="L38" s="9">
         <f>IF(OR(I38="",K38=""),"",K38*I38)</f>
-        <v/>
-      </c>
-      <c r="M38" s="9" t="str">
+        <v>97755.84</v>
+      </c>
+      <c r="M38" s="9">
         <f>IF(L38="","",L38-J38)</f>
-        <v/>
-      </c>
-      <c r="N38" s="10" t="str">
+        <v>-2195.64</v>
+      </c>
+      <c r="N38" s="10">
         <f>IF(OR(H38="",K38=""),"",K38/H38-1)</f>
-        <v/>
-      </c>
-      <c r="O38" s="6" t="str">
+        <v>-0.021967057448021188</v>
+      </c>
+      <c r="O38" s="6">
         <f>IF(G38="","",$B$3-G38)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P38" s="6" t="str">
         <f>IF(H38="","Pending buy",IF(N38&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q38" s="6" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Momentum Portfolio: Friday report 2026-10-16
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q38"/>
+  <dimension ref="A1:Q40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="E1" s="2">
-        <f>SUM(J8:J38)</f>
+        <f>SUM(J8:J40)</f>
         <v>3064170.25</v>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -540,8 +540,8 @@
         </is>
       </c>
       <c r="G1" s="2">
-        <f>SUM(L8:L38)</f>
-        <v>2985740.8</v>
+        <f>SUM(L8:L40)</f>
+        <v>2986700.38</v>
       </c>
     </row>
     <row r="2">
@@ -551,8 +551,8 @@
         </is>
       </c>
       <c r="E2" s="2">
-        <f>SUM(M8:M38)</f>
-        <v>-78429.45</v>
+        <f>SUM(M8:M40)</f>
+        <v>-77469.87</v>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" s="3">
         <f>IF(E1=0,"",G1/E1-1)</f>
-        <v>-0.0255956567687452</v>
+        <v>-0.02528249531826765</v>
       </c>
     </row>
     <row r="3">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -579,8 +579,8 @@
         </is>
       </c>
       <c r="E3">
-        <f>COUNTIF(M8:M38,"&gt;0")</f>
-        <v>7</v>
+        <f>COUNTIF(M8:M40,"&gt;0")</f>
+        <v>9</v>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
@@ -588,8 +588,8 @@
         </is>
       </c>
       <c r="G3">
-        <f>COUNTIF(M8:M38,"&lt;0")</f>
-        <v>24</v>
+        <f>COUNTIF(M8:M40,"&lt;0")</f>
+        <v>22</v>
       </c>
     </row>
     <row r="4">
@@ -600,7 +600,7 @@
       </c>
       <c r="E4" s="3">
         <f>IF((E3+G3)=0,"",E3/(E3+G3))</f>
-        <v>0.22580645161290322</v>
+        <v>0.2903225806451613</v>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
@@ -608,8 +608,8 @@
         </is>
       </c>
       <c r="G4" s="3">
-        <f>AVERAGE(N8:N38)</f>
-        <v>-0.025787073050585047</v>
+        <f>AVERAGE(N8:N40)</f>
+        <v>-0.025541884760128506</v>
       </c>
     </row>
     <row r="5">
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="E5" t="str">
-        <f>INDEX(B8:B38,MATCH(MAX(N8:N38),N8:N38,0))</f>
+        <f>INDEX(B8:B40,MATCH(MAX(N8:N40),N8:N40,0))</f>
         <v>Viji Finance Limited</v>
       </c>
       <c r="F5" s="1" t="inlineStr">
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="G5" t="str">
-        <f>INDEX(B8:B38,MATCH(MIN(N8:N38),N8:N38,0))</f>
+        <f>INDEX(B8:B40,MATCH(MIN(N8:N40),N8:N40,0))</f>
         <v>Lloyds Enterprises Limited</v>
       </c>
     </row>
@@ -639,8 +639,8 @@
         </is>
       </c>
       <c r="E6" s="3">
-        <f>AVERAGEIF(D8:D38,"4★*",N8:N38)</f>
-        <v>-0.04123686906021496</v>
+        <f>AVERAGEIF(D8:D40,"4★*",N8:N40)</f>
+        <v>-0.04560827146453346</v>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
@@ -648,8 +648,8 @@
         </is>
       </c>
       <c r="G6" s="3">
-        <f>AVERAGEIF(D8:D38,"5★*",N8:N38)</f>
-        <v>-0.011302889291557004</v>
+        <f>AVERAGEIF(D8:D40,"5★*",N8:N40)</f>
+        <v>-0.006729647224748864</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
@@ -781,23 +781,23 @@
         <v>99851.29</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>296.4</v>
+        <v>287.65</v>
       </c>
       <c r="L8" s="9">
         <f>IF(OR(I8="",K8=""),"",K8*I8)</f>
-        <v>98404.8</v>
+        <v>95499.8</v>
       </c>
       <c r="M8" s="9">
         <f>IF(L8="","",L8-J8)</f>
-        <v>-1446.49</v>
+        <v>-4351.49</v>
       </c>
       <c r="N8" s="10">
         <f>IF(OR(H8="",K8=""),"",K8/H8-1)</f>
-        <v>-0.014486476899144174</v>
+        <v>-0.043579740485960916</v>
       </c>
       <c r="O8" s="6">
         <f>IF(G8="","",$B$3-G8)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P8" s="6" t="str">
         <f>IF(H8="","Pending buy",IF(N8&gt;=0,"In profit","In loss"))</f>
@@ -849,23 +849,23 @@
         <v>99687.42</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>323</v>
+        <v>325.3</v>
       </c>
       <c r="L9" s="9">
         <f>IF(OR(I9="",K9=""),"",K9*I9)</f>
-        <v>98838.0</v>
+        <v>99541.8</v>
       </c>
       <c r="M9" s="9">
         <f>IF(L9="","",L9-J9)</f>
-        <v>-849.42</v>
+        <v>-145.62</v>
       </c>
       <c r="N9" s="10">
         <f>IF(OR(H9="",K9=""),"",K9/H9-1)</f>
-        <v>-0.008520836393527742</v>
+        <v>-0.0014607680458654793</v>
       </c>
       <c r="O9" s="6">
         <f>IF(G9="","",$B$3-G9)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P9" s="6" t="str">
         <f>IF(H9="","Pending buy",IF(N9&gt;=0,"In profit","In loss"))</f>
@@ -917,23 +917,23 @@
         <v>99607.14</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>1559</v>
+        <v>1532.4</v>
       </c>
       <c r="L10" s="9">
         <f>IF(OR(I10="",K10=""),"",K10*I10)</f>
-        <v>98217.0</v>
+        <v>96541.2</v>
       </c>
       <c r="M10" s="9">
         <f>IF(L10="","",L10-J10)</f>
-        <v>-1390.14</v>
+        <v>-3065.94</v>
       </c>
       <c r="N10" s="10">
         <f>IF(OR(H10="",K10=""),"",K10/H10-1)</f>
-        <v>-0.013956237615722733</v>
+        <v>-0.030780332599315896</v>
       </c>
       <c r="O10" s="6">
         <f>IF(G10="","",$B$3-G10)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P10" s="6" t="str">
         <f>IF(H10="","Pending buy",IF(N10&gt;=0,"In profit","In loss"))</f>
@@ -985,23 +985,23 @@
         <v>99927.23</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>70.31</v>
+        <v>70.42</v>
       </c>
       <c r="L11" s="9">
         <f>IF(OR(I11="",K11=""),"",K11*I11)</f>
-        <v>87957.81</v>
+        <v>88095.42</v>
       </c>
       <c r="M11" s="9">
         <f>IF(L11="","",L11-J11)</f>
-        <v>-11969.42</v>
+        <v>-11831.81</v>
       </c>
       <c r="N11" s="10">
         <f>IF(OR(H11="",K11=""),"",K11/H11-1)</f>
-        <v>-0.11978136826412089</v>
+        <v>-0.11840426615217459</v>
       </c>
       <c r="O11" s="6">
         <f>IF(G11="","",$B$3-G11)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P11" s="6" t="str">
         <f>IF(H11="","Pending buy",IF(N11&gt;=0,"In profit","In loss"))</f>
@@ -1053,23 +1053,23 @@
         <v>86537.12</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>19955</v>
+        <v>19675</v>
       </c>
       <c r="L12" s="9">
         <f>IF(OR(I12="",K12=""),"",K12*I12)</f>
-        <v>79820.0</v>
+        <v>78700.0</v>
       </c>
       <c r="M12" s="9">
         <f>IF(L12="","",L12-J12)</f>
-        <v>-6717.12</v>
+        <v>-7837.12</v>
       </c>
       <c r="N12" s="10">
         <f>IF(OR(H12="",K12=""),"",K12/H12-1)</f>
-        <v>-0.0776212154924718</v>
+        <v>-0.09056363892830777</v>
       </c>
       <c r="O12" s="6">
         <f>IF(G12="","",$B$3-G12)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P12" s="6" t="str">
         <f>IF(H12="","Pending buy",IF(N12&gt;=0,"In profit","In loss"))</f>
@@ -1121,23 +1121,23 @@
         <v>98177.53</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>1717.2</v>
+        <v>1706.1</v>
       </c>
       <c r="L13" s="9">
         <f>IF(OR(I13="",K13=""),"",K13*I13)</f>
-        <v>91011.6</v>
+        <v>90423.3</v>
       </c>
       <c r="M13" s="9">
         <f>IF(L13="","",L13-J13)</f>
-        <v>-7165.93</v>
+        <v>-7754.23</v>
       </c>
       <c r="N13" s="10">
         <f>IF(OR(H13="",K13=""),"",K13/H13-1)</f>
-        <v>-0.07298954177701378</v>
+        <v>-0.07898174774386402</v>
       </c>
       <c r="O13" s="6">
         <f>IF(G13="","",$B$3-G13)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P13" s="6" t="str">
         <f>IF(H13="","Pending buy",IF(N13&gt;=0,"In profit","In loss"))</f>
@@ -1189,23 +1189,23 @@
         <v>97667.46</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>4449</v>
+        <v>4473.4</v>
       </c>
       <c r="L14" s="9">
         <f>IF(OR(I14="",K14=""),"",K14*I14)</f>
-        <v>97878.0</v>
+        <v>98414.8</v>
       </c>
       <c r="M14" s="9">
         <f>IF(L14="","",L14-J14)</f>
-        <v>210.54</v>
+        <v>747.34</v>
       </c>
       <c r="N14" s="10">
         <f>IF(OR(H14="",K14=""),"",K14/H14-1)</f>
-        <v>0.002155639257839015</v>
+        <v>0.007651840111489561</v>
       </c>
       <c r="O14" s="6">
         <f>IF(G14="","",$B$3-G14)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P14" s="6" t="str">
         <f>IF(H14="","Pending buy",IF(N14&gt;=0,"In profit","In loss"))</f>
@@ -1257,23 +1257,23 @@
         <v>99078.19</v>
       </c>
       <c r="K15" s="9" t="n">
-        <v>1520.9</v>
+        <v>1500.8</v>
       </c>
       <c r="L15" s="9">
         <f>IF(OR(I15="",K15=""),"",K15*I15)</f>
-        <v>97337.6</v>
+        <v>96051.2</v>
       </c>
       <c r="M15" s="9">
         <f>IF(L15="","",L15-J15)</f>
-        <v>-1740.59</v>
+        <v>-3026.99</v>
       </c>
       <c r="N15" s="10">
         <f>IF(OR(H15="",K15=""),"",K15/H15-1)</f>
-        <v>-0.017567818169103022</v>
+        <v>-0.030551503391537893</v>
       </c>
       <c r="O15" s="6">
         <f>IF(G15="","",$B$3-G15)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P15" s="6" t="str">
         <f>IF(H15="","Pending buy",IF(N15&gt;=0,"In profit","In loss"))</f>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="O16" s="6">
         <f>IF(G16="","",$B$3-G16)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P16" s="6" t="str">
         <f>IF(H16="","Pending buy",IF(N16&gt;=0,"In profit","In loss"))</f>
@@ -1393,23 +1393,23 @@
         <v>99714.35</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>880.2</v>
+        <v>907.25</v>
       </c>
       <c r="L17" s="9">
         <f>IF(OR(I17="",K17=""),"",K17*I17)</f>
-        <v>101223.0</v>
+        <v>104333.75</v>
       </c>
       <c r="M17" s="9">
         <f>IF(L17="","",L17-J17)</f>
-        <v>1508.65</v>
+        <v>4619.4</v>
       </c>
       <c r="N17" s="10">
         <f>IF(OR(H17="",K17=""),"",K17/H17-1)</f>
-        <v>0.015129717276051835</v>
+        <v>0.04632633037797995</v>
       </c>
       <c r="O17" s="6">
         <f>IF(G17="","",$B$3-G17)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P17" s="6" t="str">
         <f>IF(H17="","Pending buy",IF(N17&gt;=0,"In profit","In loss"))</f>
@@ -1461,23 +1461,23 @@
         <v>99596.83</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>625.6</v>
+        <v>638.8</v>
       </c>
       <c r="L18" s="9">
         <f>IF(OR(I18="",K18=""),"",K18*I18)</f>
-        <v>88209.6</v>
+        <v>90070.8</v>
       </c>
       <c r="M18" s="9">
         <f>IF(L18="","",L18-J18)</f>
-        <v>-11387.23</v>
+        <v>-9526.03</v>
       </c>
       <c r="N18" s="10">
         <f>IF(OR(H18="",K18=""),"",K18/H18-1)</f>
-        <v>-0.11433329820160443</v>
+        <v>-0.0956459573068813</v>
       </c>
       <c r="O18" s="6">
         <f>IF(G18="","",$B$3-G18)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P18" s="6" t="str">
         <f>IF(H18="","Pending buy",IF(N18&gt;=0,"In profit","In loss"))</f>
@@ -1529,23 +1529,23 @@
         <v>99993.07</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>142.54</v>
+        <v>140.85</v>
       </c>
       <c r="L19" s="9">
         <f>IF(OR(I19="",K19=""),"",K19*I19)</f>
-        <v>94504.02</v>
+        <v>93383.55</v>
       </c>
       <c r="M19" s="9">
         <f>IF(L19="","",L19-J19)</f>
-        <v>-5489.05</v>
+        <v>-6609.52</v>
       </c>
       <c r="N19" s="10">
         <f>IF(OR(H19="",K19=""),"",K19/H19-1)</f>
-        <v>-0.054894259648262334</v>
+        <v>-0.06609973671571312</v>
       </c>
       <c r="O19" s="6">
         <f>IF(G19="","",$B$3-G19)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P19" s="6" t="str">
         <f>IF(H19="","Pending buy",IF(N19&gt;=0,"In profit","In loss"))</f>
@@ -1597,23 +1597,23 @@
         <v>99896.43</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>202.72</v>
+        <v>206.31</v>
       </c>
       <c r="L20" s="9">
         <f>IF(OR(I20="",K20=""),"",K20*I20)</f>
-        <v>96697.44</v>
+        <v>98409.87</v>
       </c>
       <c r="M20" s="9">
         <f>IF(L20="","",L20-J20)</f>
-        <v>-3198.99</v>
+        <v>-1486.56</v>
       </c>
       <c r="N20" s="10">
         <f>IF(OR(H20="",K20=""),"",K20/H20-1)</f>
-        <v>-0.0320230663478952</v>
+        <v>-0.014881012323570642</v>
       </c>
       <c r="O20" s="6">
         <f>IF(G20="","",$B$3-G20)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P20" s="6" t="str">
         <f>IF(H20="","Pending buy",IF(N20&gt;=0,"In profit","In loss"))</f>
@@ -1665,23 +1665,23 @@
         <v>99449.47</v>
       </c>
       <c r="K21" s="9" t="n">
-        <v>1258.8</v>
+        <v>1318.4</v>
       </c>
       <c r="L21" s="9">
         <f>IF(OR(I21="",K21=""),"",K21*I21)</f>
-        <v>89374.8</v>
+        <v>93606.4</v>
       </c>
       <c r="M21" s="9">
         <f>IF(L21="","",L21-J21)</f>
-        <v>-10074.67</v>
+        <v>-5843.07</v>
       </c>
       <c r="N21" s="10">
         <f>IF(OR(H21="",K21=""),"",K21/H21-1)</f>
-        <v>-0.10130437809146031</v>
+        <v>-0.058754124623277004</v>
       </c>
       <c r="O21" s="6">
         <f>IF(G21="","",$B$3-G21)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P21" s="6" t="str">
         <f>IF(H21="","Pending buy",IF(N21&gt;=0,"In profit","In loss"))</f>
@@ -1733,23 +1733,23 @@
         <v>99837.05</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>663.25</v>
+        <v>675.9</v>
       </c>
       <c r="L22" s="9">
         <f>IF(OR(I22="",K22=""),"",K22*I22)</f>
-        <v>95508.0</v>
+        <v>97329.6</v>
       </c>
       <c r="M22" s="9">
         <f>IF(L22="","",L22-J22)</f>
-        <v>-4329.05</v>
+        <v>-2507.45</v>
       </c>
       <c r="N22" s="10">
         <f>IF(OR(H22="",K22=""),"",K22/H22-1)</f>
-        <v>-0.04336116773718268</v>
+        <v>-0.025115436522520573</v>
       </c>
       <c r="O22" s="6">
         <f>IF(G22="","",$B$3-G22)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P22" s="6" t="str">
         <f>IF(H22="","Pending buy",IF(N22&gt;=0,"In profit","In loss"))</f>
@@ -1801,23 +1801,23 @@
         <v>99486.88</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>640.5</v>
+        <v>641.35</v>
       </c>
       <c r="L23" s="9">
         <f>IF(OR(I23="",K23=""),"",K23*I23)</f>
-        <v>92872.5</v>
+        <v>92995.75</v>
       </c>
       <c r="M23" s="9">
         <f>IF(L23="","",L23-J23)</f>
-        <v>-6614.38</v>
+        <v>-6491.13</v>
       </c>
       <c r="N23" s="10">
         <f>IF(OR(H23="",K23=""),"",K23/H23-1)</f>
-        <v>-0.06648495872905946</v>
+        <v>-0.06524610192175218</v>
       </c>
       <c r="O23" s="6">
         <f>IF(G23="","",$B$3-G23)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P23" s="6" t="str">
         <f>IF(H23="","Pending buy",IF(N23&gt;=0,"In profit","In loss"))</f>
@@ -1869,23 +1869,23 @@
         <v>99935.4</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>221.03</v>
+        <v>216.88</v>
       </c>
       <c r="L24" s="9">
         <f>IF(OR(I24="",K24=""),"",K24*I24)</f>
-        <v>97032.17</v>
+        <v>95210.32</v>
       </c>
       <c r="M24" s="9">
         <f>IF(L24="","",L24-J24)</f>
-        <v>-2903.23</v>
+        <v>-4725.08</v>
       </c>
       <c r="N24" s="10">
         <f>IF(OR(H24="",K24=""),"",K24/H24-1)</f>
-        <v>-0.02905105341635017</v>
+        <v>-0.04728133042997806</v>
       </c>
       <c r="O24" s="6">
         <f>IF(G24="","",$B$3-G24)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P24" s="6" t="str">
         <f>IF(H24="","Pending buy",IF(N24&gt;=0,"In profit","In loss"))</f>
@@ -1937,23 +1937,23 @@
         <v>99622.64</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>790.65</v>
+        <v>794.2</v>
       </c>
       <c r="L25" s="9">
         <f>IF(OR(I25="",K25=""),"",K25*I25)</f>
-        <v>98040.6</v>
+        <v>98480.8</v>
       </c>
       <c r="M25" s="9">
         <f>IF(L25="","",L25-J25)</f>
-        <v>-1582.04</v>
+        <v>-1141.84</v>
       </c>
       <c r="N25" s="10">
         <f>IF(OR(H25="",K25=""),"",K25/H25-1)</f>
-        <v>-0.01588029035665084</v>
+        <v>-0.011461615887247145</v>
       </c>
       <c r="O25" s="6">
         <f>IF(G25="","",$B$3-G25)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P25" s="6" t="str">
         <f>IF(H25="","Pending buy",IF(N25&gt;=0,"In profit","In loss"))</f>
@@ -2005,23 +2005,23 @@
         <v>99948.17</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>196.99</v>
+        <v>189.33</v>
       </c>
       <c r="L26" s="9">
         <f>IF(OR(I26="",K26=""),"",K26*I26)</f>
-        <v>93570.25</v>
+        <v>89931.75</v>
       </c>
       <c r="M26" s="9">
         <f>IF(L26="","",L26-J26)</f>
-        <v>-6377.92</v>
+        <v>-10016.42</v>
       </c>
       <c r="N26" s="10">
         <f>IF(OR(H26="",K26=""),"",K26/H26-1)</f>
-        <v>-0.06381224275717812</v>
+        <v>-0.10021611209308345</v>
       </c>
       <c r="O26" s="6">
         <f>IF(G26="","",$B$3-G26)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P26" s="6" t="str">
         <f>IF(H26="","Pending buy",IF(N26&gt;=0,"In profit","In loss"))</f>
@@ -2073,23 +2073,23 @@
         <v>99745.27</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>251.05</v>
+        <v>251.4</v>
       </c>
       <c r="L27" s="9">
         <f>IF(OR(I27="",K27=""),"",K27*I27)</f>
-        <v>95901.1</v>
+        <v>96034.8</v>
       </c>
       <c r="M27" s="9">
         <f>IF(L27="","",L27-J27)</f>
-        <v>-3844.17</v>
+        <v>-3710.47</v>
       </c>
       <c r="N27" s="10">
         <f>IF(OR(H27="",K27=""),"",K27/H27-1)</f>
-        <v>-0.038539901149416744</v>
+        <v>-0.0371994867514972</v>
       </c>
       <c r="O27" s="6">
         <f>IF(G27="","",$B$3-G27)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P27" s="6" t="str">
         <f>IF(H27="","Pending buy",IF(N27&gt;=0,"In profit","In loss"))</f>
@@ -2141,23 +2141,23 @@
         <v>95334.84</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>10941</v>
+        <v>10960</v>
       </c>
       <c r="L28" s="9">
         <f>IF(OR(I28="",K28=""),"",K28*I28)</f>
-        <v>98469.0</v>
+        <v>98640.0</v>
       </c>
       <c r="M28" s="9">
         <f>IF(L28="","",L28-J28)</f>
-        <v>3134.16</v>
+        <v>3305.16</v>
       </c>
       <c r="N28" s="10">
         <f>IF(OR(H28="",K28=""),"",K28/H28-1)</f>
-        <v>0.03287525869133079</v>
+        <v>0.03466893659235781</v>
       </c>
       <c r="O28" s="6">
         <f>IF(G28="","",$B$3-G28)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P28" s="6" t="str">
         <f>IF(H28="","Pending buy",IF(N28&gt;=0,"In profit","In loss"))</f>
@@ -2209,23 +2209,23 @@
         <v>98598.59</v>
       </c>
       <c r="K29" s="9" t="n">
-        <v>1873.2</v>
+        <v>1866</v>
       </c>
       <c r="L29" s="9">
         <f>IF(OR(I29="",K29=""),"",K29*I29)</f>
-        <v>95533.2</v>
+        <v>95166.0</v>
       </c>
       <c r="M29" s="9">
         <f>IF(L29="","",L29-J29)</f>
-        <v>-3065.39</v>
+        <v>-3432.59</v>
       </c>
       <c r="N29" s="10">
         <f>IF(OR(H29="",K29=""),"",K29/H29-1)</f>
-        <v>-0.031089555937682922</v>
+        <v>-0.03481374726655795</v>
       </c>
       <c r="O29" s="6">
         <f>IF(G29="","",$B$3-G29)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P29" s="6" t="str">
         <f>IF(H29="","Pending buy",IF(N29&gt;=0,"In profit","In loss"))</f>
@@ -2277,23 +2277,23 @@
         <v>99998.69</v>
       </c>
       <c r="K30" s="9" t="n">
-        <v>16.34</v>
+        <v>16.66</v>
       </c>
       <c r="L30" s="9">
         <f>IF(OR(I30="",K30=""),"",K30*I30)</f>
-        <v>110180.62</v>
+        <v>112338.38</v>
       </c>
       <c r="M30" s="9">
         <f>IF(L30="","",L30-J30)</f>
-        <v>10181.93</v>
+        <v>12339.69</v>
       </c>
       <c r="N30" s="10">
         <f>IF(OR(H30="",K30=""),"",K30/H30-1)</f>
-        <v>0.10182063385030338</v>
+        <v>0.12339851652056644</v>
       </c>
       <c r="O30" s="6">
         <f>IF(G30="","",$B$3-G30)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P30" s="6" t="str">
         <f>IF(H30="","Pending buy",IF(N30&gt;=0,"In profit","In loss"))</f>
@@ -2345,23 +2345,23 @@
         <v>99977.34</v>
       </c>
       <c r="K31" s="9" t="n">
-        <v>173.7</v>
+        <v>174.14</v>
       </c>
       <c r="L31" s="9">
         <f>IF(OR(I31="",K31=""),"",K31*I31)</f>
-        <v>97966.8</v>
+        <v>98214.96</v>
       </c>
       <c r="M31" s="9">
         <f>IF(L31="","",L31-J31)</f>
-        <v>-2010.54</v>
+        <v>-1762.38</v>
       </c>
       <c r="N31" s="10">
         <f>IF(OR(H31="",K31=""),"",K31/H31-1)</f>
-        <v>-0.020109939038991498</v>
+        <v>-0.017627776535693696</v>
       </c>
       <c r="O31" s="6">
         <f>IF(G31="","",$B$3-G31)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P31" s="6" t="str">
         <f>IF(H31="","Pending buy",IF(N31&gt;=0,"In profit","In loss"))</f>
@@ -2413,23 +2413,23 @@
         <v>99923.82</v>
       </c>
       <c r="K32" s="9" t="n">
-        <v>190.04</v>
+        <v>187.7</v>
       </c>
       <c r="L32" s="9">
         <f>IF(OR(I32="",K32=""),"",K32*I32)</f>
-        <v>107372.6</v>
+        <v>106050.5</v>
       </c>
       <c r="M32" s="9">
         <f>IF(L32="","",L32-J32)</f>
-        <v>7448.78</v>
+        <v>6126.68</v>
       </c>
       <c r="N32" s="10">
         <f>IF(OR(H32="",K32=""),"",K32/H32-1)</f>
-        <v>0.07454459161589022</v>
+        <v>0.061313512135879655</v>
       </c>
       <c r="O32" s="6">
         <f>IF(G32="","",$B$3-G32)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P32" s="6" t="str">
         <f>IF(H32="","Pending buy",IF(N32&gt;=0,"In profit","In loss"))</f>
@@ -2481,23 +2481,23 @@
         <v>99608.58</v>
       </c>
       <c r="K33" s="9" t="n">
-        <v>529.6</v>
+        <v>539.3</v>
       </c>
       <c r="L33" s="9">
         <f>IF(OR(I33="",K33=""),"",K33*I33)</f>
-        <v>100094.4</v>
+        <v>101927.7</v>
       </c>
       <c r="M33" s="9">
         <f>IF(L33="","",L33-J33)</f>
-        <v>485.82</v>
+        <v>2319.12</v>
       </c>
       <c r="N33" s="10">
         <f>IF(OR(H33="",K33=""),"",K33/H33-1)</f>
-        <v>0.004877339901760092</v>
+        <v>0.023282381814613284</v>
       </c>
       <c r="O33" s="6">
         <f>IF(G33="","",$B$3-G33)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P33" s="6" t="str">
         <f>IF(H33="","Pending buy",IF(N33&gt;=0,"In profit","In loss"))</f>
@@ -2549,23 +2549,23 @@
         <v>96030.46</v>
       </c>
       <c r="K34" s="9" t="n">
-        <v>4712.1</v>
+        <v>4731.7</v>
       </c>
       <c r="L34" s="9">
         <f>IF(OR(I34="",K34=""),"",K34*I34)</f>
-        <v>89529.9</v>
+        <v>89902.3</v>
       </c>
       <c r="M34" s="9">
         <f>IF(L34="","",L34-J34)</f>
-        <v>-6500.56</v>
+        <v>-6128.16</v>
       </c>
       <c r="N34" s="10">
         <f>IF(OR(H34="",K34=""),"",K34/H34-1)</f>
-        <v>-0.06769269537939093</v>
+        <v>-0.06381475917885115</v>
       </c>
       <c r="O34" s="6">
         <f>IF(G34="","",$B$3-G34)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P34" s="6" t="str">
         <f>IF(H34="","Pending buy",IF(N34&gt;=0,"In profit","In loss"))</f>
@@ -2617,23 +2617,23 @@
         <v>99082.89</v>
       </c>
       <c r="K35" s="9" t="n">
-        <v>1085.4</v>
+        <v>1008.3</v>
       </c>
       <c r="L35" s="9">
         <f>IF(OR(I35="",K35=""),"",K35*I35)</f>
-        <v>98771.4</v>
+        <v>91755.3</v>
       </c>
       <c r="M35" s="9">
         <f>IF(L35="","",L35-J35)</f>
-        <v>-311.49</v>
+        <v>-7327.59</v>
       </c>
       <c r="N35" s="10">
         <f>IF(OR(H35="",K35=""),"",K35/H35-1)</f>
-        <v>-0.003143761658230937</v>
+        <v>-0.07395416885940154</v>
       </c>
       <c r="O35" s="6">
         <f>IF(G35="","",$B$3-G35)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P35" s="6" t="str">
         <f>IF(H35="","Pending buy",IF(N35&gt;=0,"In profit","In loss"))</f>
@@ -2685,27 +2685,27 @@
         <v>99910.57</v>
       </c>
       <c r="K36" s="9" t="n">
-        <v>96.34999999999999</v>
+        <v>100.62</v>
       </c>
       <c r="L36" s="9">
         <f>IF(OR(I36="",K36=""),"",K36*I36)</f>
-        <v>98758.75</v>
+        <v>103135.5</v>
       </c>
       <c r="M36" s="9">
         <f>IF(L36="","",L36-J36)</f>
-        <v>-1151.82</v>
+        <v>3224.93</v>
       </c>
       <c r="N36" s="10">
         <f>IF(OR(H36="",K36=""),"",K36/H36-1)</f>
-        <v>-0.011528521818720217</v>
+        <v>0.03227815396575373</v>
       </c>
       <c r="O36" s="6">
         <f>IF(G36="","",$B$3-G36)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P36" s="6" t="str">
         <f>IF(H36="","Pending buy",IF(N36&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q36" s="6" t="n">
         <v>1</v>
@@ -2753,23 +2753,23 @@
         <v>99436.51</v>
       </c>
       <c r="K37" s="9" t="n">
-        <v>989.5</v>
+        <v>961.7</v>
       </c>
       <c r="L37" s="9">
         <f>IF(OR(I37="",K37=""),"",K37*I37)</f>
-        <v>98950.0</v>
+        <v>96170.0</v>
       </c>
       <c r="M37" s="9">
         <f>IF(L37="","",L37-J37)</f>
-        <v>-486.51</v>
+        <v>-3266.51</v>
       </c>
       <c r="N37" s="10">
         <f>IF(OR(H37="",K37=""),"",K37/H37-1)</f>
-        <v>-0.004892698726163824</v>
+        <v>-0.032850235841285214</v>
       </c>
       <c r="O37" s="6">
         <f>IF(G37="","",$B$3-G37)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P37" s="6" t="str">
         <f>IF(H37="","Pending buy",IF(N37&gt;=0,"In profit","In loss"))</f>
@@ -2821,34 +2821,162 @@
         <v>99951.48</v>
       </c>
       <c r="K38" s="9" t="n">
-        <v>119.36</v>
+        <v>122.57</v>
       </c>
       <c r="L38" s="9">
         <f>IF(OR(I38="",K38=""),"",K38*I38)</f>
-        <v>97755.84</v>
+        <v>100384.83</v>
       </c>
       <c r="M38" s="9">
         <f>IF(L38="","",L38-J38)</f>
-        <v>-2195.64</v>
+        <v>433.35</v>
       </c>
       <c r="N38" s="10">
         <f>IF(OR(H38="",K38=""),"",K38/H38-1)</f>
-        <v>-0.021967057448021188</v>
+        <v>0.00433560462965854</v>
       </c>
       <c r="O38" s="6">
         <f>IF(G38="","",$B$3-G38)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P38" s="6" t="str">
         <f>IF(H38="","Pending buy",IF(N38&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q38" s="6" t="n">
         <v>1</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Authum Investment &amp; Infrastructure Limited</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>AIIL</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>161026</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G39" s="6" t="inlineStr"/>
+      <c r="H39" s="9" t="inlineStr"/>
+      <c r="I39" s="6" t="str">
+        <f>IF(H39="","",ROUNDDOWN($B$1/H39,0))</f>
+        <v/>
+      </c>
+      <c r="J39" s="9" t="str">
+        <f>IF(H39="","",H39*I39)</f>
+        <v/>
+      </c>
+      <c r="K39" s="9" t="n">
+        <v>571.9</v>
+      </c>
+      <c r="L39" s="9" t="str">
+        <f>IF(OR(I39="",K39=""),"",K39*I39)</f>
+        <v/>
+      </c>
+      <c r="M39" s="9" t="str">
+        <f>IF(L39="","",L39-J39)</f>
+        <v/>
+      </c>
+      <c r="N39" s="10" t="str">
+        <f>IF(OR(H39="",K39=""),"",K39/H39-1)</f>
+        <v/>
+      </c>
+      <c r="O39" s="6" t="str">
+        <f>IF(G39="","",$B$3-G39)</f>
+        <v/>
+      </c>
+      <c r="P39" s="6" t="str">
+        <f>IF(H39="","Pending buy",IF(N39&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q39" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Kesoram Industries Limited</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>KESORAMIND</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>161026</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G40" s="6" t="inlineStr"/>
+      <c r="H40" s="9" t="inlineStr"/>
+      <c r="I40" s="6" t="str">
+        <f>IF(H40="","",ROUNDDOWN($B$1/H40,0))</f>
+        <v/>
+      </c>
+      <c r="J40" s="9" t="str">
+        <f>IF(H40="","",H40*I40)</f>
+        <v/>
+      </c>
+      <c r="K40" s="9" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="L40" s="9" t="str">
+        <f>IF(OR(I40="",K40=""),"",K40*I40)</f>
+        <v/>
+      </c>
+      <c r="M40" s="9" t="str">
+        <f>IF(L40="","",L40-J40)</f>
+        <v/>
+      </c>
+      <c r="N40" s="10" t="str">
+        <f>IF(OR(H40="",K40=""),"",K40/H40-1)</f>
+        <v/>
+      </c>
+      <c r="O40" s="6" t="str">
+        <f>IF(G40="","",$B$3-G40)</f>
+        <v/>
+      </c>
+      <c r="P40" s="6" t="str">
+        <f>IF(H40="","Pending buy",IF(N40&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q40" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A8:Q38">
+  <conditionalFormatting sqref="A8:Q40">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$N8&gt;0</formula>
     </cfRule>
@@ -2866,7 +2994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3594,6 +3722,46 @@
       <c r="D36" s="11" t="inlineStr">
         <is>
           <t>Tamilnadu PetroProducts Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>AIIL</t>
+        </is>
+      </c>
+      <c r="D37" s="11" t="inlineStr">
+        <is>
+          <t>Authum Investment &amp; Infrastructure Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>KESORAMIND</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="inlineStr">
+        <is>
+          <t>Kesoram Industries Limited</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum Portfolio: weekday silent update 2026-10-19
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:Q42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -531,8 +531,8 @@
         </is>
       </c>
       <c r="E1" s="2">
-        <f>SUM(J8:J40)</f>
-        <v>3064170.25</v>
+        <f>SUM(J8:J42)</f>
+        <v>3263835.67</v>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
@@ -540,8 +540,8 @@
         </is>
       </c>
       <c r="G1" s="2">
-        <f>SUM(L8:L40)</f>
-        <v>2986700.38</v>
+        <f>SUM(L8:L42)</f>
+        <v>3131700.46</v>
       </c>
     </row>
     <row r="2">
@@ -551,8 +551,8 @@
         </is>
       </c>
       <c r="E2" s="2">
-        <f>SUM(M8:M40)</f>
-        <v>-77469.87</v>
+        <f>SUM(M8:M42)</f>
+        <v>-132135.21</v>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" s="3">
         <f>IF(E1=0,"",G1/E1-1)</f>
-        <v>-0.02528249531826765</v>
+        <v>-0.040484639350730545</v>
       </c>
     </row>
     <row r="3">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -579,8 +579,8 @@
         </is>
       </c>
       <c r="E3">
-        <f>COUNTIF(M8:M40,"&gt;0")</f>
-        <v>9</v>
+        <f>COUNTIF(M8:M42,"&gt;0")</f>
+        <v>8</v>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
@@ -588,8 +588,8 @@
         </is>
       </c>
       <c r="G3">
-        <f>COUNTIF(M8:M40,"&lt;0")</f>
-        <v>22</v>
+        <f>COUNTIF(M8:M42,"&lt;0")</f>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -600,7 +600,7 @@
       </c>
       <c r="E4" s="3">
         <f>IF((E3+G3)=0,"",E3/(E3+G3))</f>
-        <v>0.2903225806451613</v>
+        <v>0.24242424242424243</v>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
@@ -608,8 +608,8 @@
         </is>
       </c>
       <c r="G4" s="3">
-        <f>AVERAGE(N8:N40)</f>
-        <v>-0.025541884760128506</v>
+        <f>AVERAGE(N8:N42)</f>
+        <v>-0.0406912464443625</v>
       </c>
     </row>
     <row r="5">
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="E5" t="str">
-        <f>INDEX(B8:B40,MATCH(MAX(N8:N40),N8:N40,0))</f>
+        <f>INDEX(B8:B42,MATCH(MAX(N8:N42),N8:N42,0))</f>
         <v>Viji Finance Limited</v>
       </c>
       <c r="F5" s="1" t="inlineStr">
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="G5" t="str">
-        <f>INDEX(B8:B40,MATCH(MIN(N8:N40),N8:N40,0))</f>
+        <f>INDEX(B8:B42,MATCH(MIN(N8:N42),N8:N42,0))</f>
         <v>Lloyds Enterprises Limited</v>
       </c>
     </row>
@@ -639,8 +639,8 @@
         </is>
       </c>
       <c r="E6" s="3">
-        <f>AVERAGEIF(D8:D40,"4★*",N8:N40)</f>
-        <v>-0.04560827146453346</v>
+        <f>AVERAGEIF(D8:D42,"4★*",N8:N42)</f>
+        <v>-0.05945869664085087</v>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
@@ -648,8 +648,8 @@
         </is>
       </c>
       <c r="G6" s="3">
-        <f>AVERAGEIF(D8:D40,"5★*",N8:N40)</f>
-        <v>-0.006729647224748864</v>
+        <f>AVERAGEIF(D8:D42,"5★*",N8:N42)</f>
+        <v>-0.0207508306105936</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
@@ -781,23 +781,23 @@
         <v>99851.29</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>287.65</v>
+        <v>285.6</v>
       </c>
       <c r="L8" s="9">
         <f>IF(OR(I8="",K8=""),"",K8*I8)</f>
-        <v>95499.8</v>
+        <v>94819.2</v>
       </c>
       <c r="M8" s="9">
         <f>IF(L8="","",L8-J8)</f>
-        <v>-4351.49</v>
+        <v>-5032.09</v>
       </c>
       <c r="N8" s="10">
         <f>IF(OR(H8="",K8=""),"",K8/H8-1)</f>
-        <v>-0.043579740485960916</v>
+        <v>-0.05039587652630073</v>
       </c>
       <c r="O8" s="6">
         <f>IF(G8="","",$B$3-G8)</f>
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="P8" s="6" t="str">
         <f>IF(H8="","Pending buy",IF(N8&gt;=0,"In profit","In loss"))</f>
@@ -849,23 +849,23 @@
         <v>99687.42</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>325.3</v>
+        <v>320.2</v>
       </c>
       <c r="L9" s="9">
         <f>IF(OR(I9="",K9=""),"",K9*I9)</f>
-        <v>99541.8</v>
+        <v>97981.2</v>
       </c>
       <c r="M9" s="9">
         <f>IF(L9="","",L9-J9)</f>
-        <v>-145.62</v>
+        <v>-1706.22</v>
       </c>
       <c r="N9" s="10">
         <f>IF(OR(H9="",K9=""),"",K9/H9-1)</f>
-        <v>-0.0014607680458654793</v>
+        <v>-0.017115702208073014</v>
       </c>
       <c r="O9" s="6">
         <f>IF(G9="","",$B$3-G9)</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="P9" s="6" t="str">
         <f>IF(H9="","Pending buy",IF(N9&gt;=0,"In profit","In loss"))</f>
@@ -917,23 +917,23 @@
         <v>99607.14</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>1532.4</v>
+        <v>1538.3</v>
       </c>
       <c r="L10" s="9">
         <f>IF(OR(I10="",K10=""),"",K10*I10)</f>
-        <v>96541.2</v>
+        <v>96912.9</v>
       </c>
       <c r="M10" s="9">
         <f>IF(L10="","",L10-J10)</f>
-        <v>-3065.94</v>
+        <v>-2694.24</v>
       </c>
       <c r="N10" s="10">
         <f>IF(OR(H10="",K10=""),"",K10/H10-1)</f>
-        <v>-0.030780332599315896</v>
+        <v>-0.027048672433782173</v>
       </c>
       <c r="O10" s="6">
         <f>IF(G10="","",$B$3-G10)</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="P10" s="6" t="str">
         <f>IF(H10="","Pending buy",IF(N10&gt;=0,"In profit","In loss"))</f>
@@ -985,23 +985,23 @@
         <v>99927.23</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>70.42</v>
+        <v>68.72</v>
       </c>
       <c r="L11" s="9">
         <f>IF(OR(I11="",K11=""),"",K11*I11)</f>
-        <v>88095.42</v>
+        <v>85968.72</v>
       </c>
       <c r="M11" s="9">
         <f>IF(L11="","",L11-J11)</f>
-        <v>-11831.81</v>
+        <v>-13958.51</v>
       </c>
       <c r="N11" s="10">
         <f>IF(OR(H11="",K11=""),"",K11/H11-1)</f>
-        <v>-0.11840426615217459</v>
+        <v>-0.1396867533367998</v>
       </c>
       <c r="O11" s="6">
         <f>IF(G11="","",$B$3-G11)</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="P11" s="6" t="str">
         <f>IF(H11="","Pending buy",IF(N11&gt;=0,"In profit","In loss"))</f>
@@ -1053,23 +1053,23 @@
         <v>86537.12</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>19675</v>
+        <v>19220</v>
       </c>
       <c r="L12" s="9">
         <f>IF(OR(I12="",K12=""),"",K12*I12)</f>
-        <v>78700.0</v>
+        <v>76880.0</v>
       </c>
       <c r="M12" s="9">
         <f>IF(L12="","",L12-J12)</f>
-        <v>-7837.12</v>
+        <v>-9657.12</v>
       </c>
       <c r="N12" s="10">
         <f>IF(OR(H12="",K12=""),"",K12/H12-1)</f>
-        <v>-0.09056363892830777</v>
+        <v>-0.11159507701154137</v>
       </c>
       <c r="O12" s="6">
         <f>IF(G12="","",$B$3-G12)</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="P12" s="6" t="str">
         <f>IF(H12="","Pending buy",IF(N12&gt;=0,"In profit","In loss"))</f>
@@ -1121,23 +1121,23 @@
         <v>98177.53</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>1706.1</v>
+        <v>1683.8</v>
       </c>
       <c r="L13" s="9">
         <f>IF(OR(I13="",K13=""),"",K13*I13)</f>
-        <v>90423.3</v>
+        <v>89241.4</v>
       </c>
       <c r="M13" s="9">
         <f>IF(L13="","",L13-J13)</f>
-        <v>-7754.23</v>
+        <v>-8936.13</v>
       </c>
       <c r="N13" s="10">
         <f>IF(OR(H13="",K13=""),"",K13/H13-1)</f>
-        <v>-0.07898174774386402</v>
+        <v>-0.09102014351510357</v>
       </c>
       <c r="O13" s="6">
         <f>IF(G13="","",$B$3-G13)</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="P13" s="6" t="str">
         <f>IF(H13="","Pending buy",IF(N13&gt;=0,"In profit","In loss"))</f>
@@ -1189,27 +1189,27 @@
         <v>97667.46</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>4473.4</v>
+        <v>4435.5</v>
       </c>
       <c r="L14" s="9">
         <f>IF(OR(I14="",K14=""),"",K14*I14)</f>
-        <v>98414.8</v>
+        <v>97581.0</v>
       </c>
       <c r="M14" s="9">
         <f>IF(L14="","",L14-J14)</f>
-        <v>747.34</v>
+        <v>-86.46</v>
       </c>
       <c r="N14" s="10">
         <f>IF(OR(H14="",K14=""),"",K14/H14-1)</f>
-        <v>0.007651840111489561</v>
+        <v>-0.0008852915423364083</v>
       </c>
       <c r="O14" s="6">
         <f>IF(G14="","",$B$3-G14)</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="P14" s="6" t="str">
         <f>IF(H14="","Pending buy",IF(N14&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q14" s="6" t="n">
         <v>1</v>
@@ -1257,23 +1257,23 @@
         <v>99078.19</v>
       </c>
       <c r="K15" s="9" t="n">
-        <v>1500.8</v>
+        <v>1478.1</v>
       </c>
       <c r="L15" s="9">
         <f>IF(OR(I15="",K15=""),"",K15*I15)</f>
-        <v>96051.2</v>
+        <v>94598.4</v>
       </c>
       <c r="M15" s="9">
         <f>IF(L15="","",L15-J15)</f>
-        <v>-3026.99</v>
+        <v>-4479.79</v>
       </c>
       <c r="N15" s="10">
         <f>IF(OR(H15="",K15=""),"",K15/H15-1)</f>
-        <v>-0.030551503391537893</v>
+        <v>-0.04521467028453641</v>
       </c>
       <c r="O15" s="6">
         <f>IF(G15="","",$B$3-G15)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P15" s="6" t="str">
         <f>IF(H15="","Pending buy",IF(N15&gt;=0,"In profit","In loss"))</f>
@@ -1325,23 +1325,23 @@
         <v>98557.54</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>1470</v>
+        <v>1459</v>
       </c>
       <c r="L16" s="9">
         <f>IF(OR(I16="",K16=""),"",K16*I16)</f>
-        <v>99960.0</v>
+        <v>99212.0</v>
       </c>
       <c r="M16" s="9">
         <f>IF(L16="","",L16-J16)</f>
-        <v>1402.46</v>
+        <v>654.46</v>
       </c>
       <c r="N16" s="10">
         <f>IF(OR(H16="",K16=""),"",K16/H16-1)</f>
-        <v>0.014229895892054145</v>
+        <v>0.006640420480616971</v>
       </c>
       <c r="O16" s="6">
         <f>IF(G16="","",$B$3-G16)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P16" s="6" t="str">
         <f>IF(H16="","Pending buy",IF(N16&gt;=0,"In profit","In loss"))</f>
@@ -1393,23 +1393,23 @@
         <v>99714.35</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>907.25</v>
+        <v>894.45</v>
       </c>
       <c r="L17" s="9">
         <f>IF(OR(I17="",K17=""),"",K17*I17)</f>
-        <v>104333.75</v>
+        <v>102861.75</v>
       </c>
       <c r="M17" s="9">
         <f>IF(L17="","",L17-J17)</f>
-        <v>4619.4</v>
+        <v>3147.4</v>
       </c>
       <c r="N17" s="10">
         <f>IF(OR(H17="",K17=""),"",K17/H17-1)</f>
-        <v>0.04632633037797995</v>
+        <v>0.03156416225581071</v>
       </c>
       <c r="O17" s="6">
         <f>IF(G17="","",$B$3-G17)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P17" s="6" t="str">
         <f>IF(H17="","Pending buy",IF(N17&gt;=0,"In profit","In loss"))</f>
@@ -1461,23 +1461,23 @@
         <v>99596.83</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>638.8</v>
+        <v>622.15</v>
       </c>
       <c r="L18" s="9">
         <f>IF(OR(I18="",K18=""),"",K18*I18)</f>
-        <v>90070.8</v>
+        <v>87723.15</v>
       </c>
       <c r="M18" s="9">
         <f>IF(L18="","",L18-J18)</f>
-        <v>-9526.03</v>
+        <v>-11873.68</v>
       </c>
       <c r="N18" s="10">
         <f>IF(OR(H18="",K18=""),"",K18/H18-1)</f>
-        <v>-0.0956459573068813</v>
+        <v>-0.11921748957181622</v>
       </c>
       <c r="O18" s="6">
         <f>IF(G18="","",$B$3-G18)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P18" s="6" t="str">
         <f>IF(H18="","Pending buy",IF(N18&gt;=0,"In profit","In loss"))</f>
@@ -1529,23 +1529,23 @@
         <v>99993.07</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>140.85</v>
+        <v>139.02</v>
       </c>
       <c r="L19" s="9">
         <f>IF(OR(I19="",K19=""),"",K19*I19)</f>
-        <v>93383.55</v>
+        <v>92170.26</v>
       </c>
       <c r="M19" s="9">
         <f>IF(L19="","",L19-J19)</f>
-        <v>-6609.52</v>
+        <v>-7822.81</v>
       </c>
       <c r="N19" s="10">
         <f>IF(OR(H19="",K19=""),"",K19/H19-1)</f>
-        <v>-0.06609973671571312</v>
+        <v>-0.07823347815561532</v>
       </c>
       <c r="O19" s="6">
         <f>IF(G19="","",$B$3-G19)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P19" s="6" t="str">
         <f>IF(H19="","Pending buy",IF(N19&gt;=0,"In profit","In loss"))</f>
@@ -1597,23 +1597,23 @@
         <v>99896.43</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>206.31</v>
+        <v>202.32</v>
       </c>
       <c r="L20" s="9">
         <f>IF(OR(I20="",K20=""),"",K20*I20)</f>
-        <v>98409.87</v>
+        <v>96506.64</v>
       </c>
       <c r="M20" s="9">
         <f>IF(L20="","",L20-J20)</f>
-        <v>-1486.56</v>
+        <v>-3389.79</v>
       </c>
       <c r="N20" s="10">
         <f>IF(OR(H20="",K20=""),"",K20/H20-1)</f>
-        <v>-0.014881012323570642</v>
+        <v>-0.03393304451216528</v>
       </c>
       <c r="O20" s="6">
         <f>IF(G20="","",$B$3-G20)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P20" s="6" t="str">
         <f>IF(H20="","Pending buy",IF(N20&gt;=0,"In profit","In loss"))</f>
@@ -1665,23 +1665,23 @@
         <v>99449.47</v>
       </c>
       <c r="K21" s="9" t="n">
-        <v>1318.4</v>
+        <v>1253.6</v>
       </c>
       <c r="L21" s="9">
         <f>IF(OR(I21="",K21=""),"",K21*I21)</f>
-        <v>93606.4</v>
+        <v>89005.6</v>
       </c>
       <c r="M21" s="9">
         <f>IF(L21="","",L21-J21)</f>
-        <v>-5843.07</v>
+        <v>-10443.87</v>
       </c>
       <c r="N21" s="10">
         <f>IF(OR(H21="",K21=""),"",K21/H21-1)</f>
-        <v>-0.058754124623277004</v>
+        <v>-0.10501681631351656</v>
       </c>
       <c r="O21" s="6">
         <f>IF(G21="","",$B$3-G21)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P21" s="6" t="str">
         <f>IF(H21="","Pending buy",IF(N21&gt;=0,"In profit","In loss"))</f>
@@ -1733,23 +1733,23 @@
         <v>99837.05</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>675.9</v>
+        <v>668.4</v>
       </c>
       <c r="L22" s="9">
         <f>IF(OR(I22="",K22=""),"",K22*I22)</f>
-        <v>97329.6</v>
+        <v>96249.6</v>
       </c>
       <c r="M22" s="9">
         <f>IF(L22="","",L22-J22)</f>
-        <v>-2507.45</v>
+        <v>-3587.45</v>
       </c>
       <c r="N22" s="10">
         <f>IF(OR(H22="",K22=""),"",K22/H22-1)</f>
-        <v>-0.025115436522520573</v>
+        <v>-0.03593306372488947</v>
       </c>
       <c r="O22" s="6">
         <f>IF(G22="","",$B$3-G22)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P22" s="6" t="str">
         <f>IF(H22="","Pending buy",IF(N22&gt;=0,"In profit","In loss"))</f>
@@ -1801,23 +1801,23 @@
         <v>99486.88</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>641.35</v>
+        <v>615.6</v>
       </c>
       <c r="L23" s="9">
         <f>IF(OR(I23="",K23=""),"",K23*I23)</f>
-        <v>92995.75</v>
+        <v>89262.0</v>
       </c>
       <c r="M23" s="9">
         <f>IF(L23="","",L23-J23)</f>
-        <v>-6491.13</v>
+        <v>-10224.88</v>
       </c>
       <c r="N23" s="10">
         <f>IF(OR(H23="",K23=""),"",K23/H23-1)</f>
-        <v>-0.06524610192175218</v>
+        <v>-0.10277617579017795</v>
       </c>
       <c r="O23" s="6">
         <f>IF(G23="","",$B$3-G23)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P23" s="6" t="str">
         <f>IF(H23="","Pending buy",IF(N23&gt;=0,"In profit","In loss"))</f>
@@ -1869,23 +1869,23 @@
         <v>99935.4</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>216.88</v>
+        <v>215.77</v>
       </c>
       <c r="L24" s="9">
         <f>IF(OR(I24="",K24=""),"",K24*I24)</f>
-        <v>95210.32</v>
+        <v>94723.03</v>
       </c>
       <c r="M24" s="9">
         <f>IF(L24="","",L24-J24)</f>
-        <v>-4725.08</v>
+        <v>-5212.37</v>
       </c>
       <c r="N24" s="10">
         <f>IF(OR(H24="",K24=""),"",K24/H24-1)</f>
-        <v>-0.04728133042997806</v>
+        <v>-0.05215738042639406</v>
       </c>
       <c r="O24" s="6">
         <f>IF(G24="","",$B$3-G24)</f>
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="P24" s="6" t="str">
         <f>IF(H24="","Pending buy",IF(N24&gt;=0,"In profit","In loss"))</f>
@@ -1937,23 +1937,23 @@
         <v>99622.64</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>794.2</v>
+        <v>751.75</v>
       </c>
       <c r="L25" s="9">
         <f>IF(OR(I25="",K25=""),"",K25*I25)</f>
-        <v>98480.8</v>
+        <v>93217.0</v>
       </c>
       <c r="M25" s="9">
         <f>IF(L25="","",L25-J25)</f>
-        <v>-1141.84</v>
+        <v>-6405.64</v>
       </c>
       <c r="N25" s="10">
         <f>IF(OR(H25="",K25=""),"",K25/H25-1)</f>
-        <v>-0.011461615887247145</v>
+        <v>-0.06429900496504426</v>
       </c>
       <c r="O25" s="6">
         <f>IF(G25="","",$B$3-G25)</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="P25" s="6" t="str">
         <f>IF(H25="","Pending buy",IF(N25&gt;=0,"In profit","In loss"))</f>
@@ -2005,23 +2005,23 @@
         <v>99948.17</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>189.33</v>
+        <v>183</v>
       </c>
       <c r="L26" s="9">
         <f>IF(OR(I26="",K26=""),"",K26*I26)</f>
-        <v>89931.75</v>
+        <v>86925.0</v>
       </c>
       <c r="M26" s="9">
         <f>IF(L26="","",L26-J26)</f>
-        <v>-10016.42</v>
+        <v>-13023.17</v>
       </c>
       <c r="N26" s="10">
         <f>IF(OR(H26="",K26=""),"",K26/H26-1)</f>
-        <v>-0.10021611209308345</v>
+        <v>-0.1302992051604832</v>
       </c>
       <c r="O26" s="6">
         <f>IF(G26="","",$B$3-G26)</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="P26" s="6" t="str">
         <f>IF(H26="","Pending buy",IF(N26&gt;=0,"In profit","In loss"))</f>
@@ -2073,23 +2073,23 @@
         <v>99745.27</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>251.4</v>
+        <v>240.6</v>
       </c>
       <c r="L27" s="9">
         <f>IF(OR(I27="",K27=""),"",K27*I27)</f>
-        <v>96034.8</v>
+        <v>91909.2</v>
       </c>
       <c r="M27" s="9">
         <f>IF(L27="","",L27-J27)</f>
-        <v>-3710.47</v>
+        <v>-7836.07</v>
       </c>
       <c r="N27" s="10">
         <f>IF(OR(H27="",K27=""),"",K27/H27-1)</f>
-        <v>-0.0371994867514972</v>
+        <v>-0.07856084531587204</v>
       </c>
       <c r="O27" s="6">
         <f>IF(G27="","",$B$3-G27)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P27" s="6" t="str">
         <f>IF(H27="","Pending buy",IF(N27&gt;=0,"In profit","In loss"))</f>
@@ -2141,23 +2141,23 @@
         <v>95334.84</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>10960</v>
+        <v>11158</v>
       </c>
       <c r="L28" s="9">
         <f>IF(OR(I28="",K28=""),"",K28*I28)</f>
-        <v>98640.0</v>
+        <v>100422.0</v>
       </c>
       <c r="M28" s="9">
         <f>IF(L28="","",L28-J28)</f>
-        <v>3305.16</v>
+        <v>5087.16</v>
       </c>
       <c r="N28" s="10">
         <f>IF(OR(H28="",K28=""),"",K28/H28-1)</f>
-        <v>0.03466893659235781</v>
+        <v>0.05336094840305905</v>
       </c>
       <c r="O28" s="6">
         <f>IF(G28="","",$B$3-G28)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P28" s="6" t="str">
         <f>IF(H28="","Pending buy",IF(N28&gt;=0,"In profit","In loss"))</f>
@@ -2209,23 +2209,23 @@
         <v>98598.59</v>
       </c>
       <c r="K29" s="9" t="n">
-        <v>1866</v>
+        <v>1866.8</v>
       </c>
       <c r="L29" s="9">
         <f>IF(OR(I29="",K29=""),"",K29*I29)</f>
-        <v>95166.0</v>
+        <v>95206.8</v>
       </c>
       <c r="M29" s="9">
         <f>IF(L29="","",L29-J29)</f>
-        <v>-3432.59</v>
+        <v>-3391.79</v>
       </c>
       <c r="N29" s="10">
         <f>IF(OR(H29="",K29=""),"",K29/H29-1)</f>
-        <v>-0.03481374726655795</v>
+        <v>-0.03439994823001635</v>
       </c>
       <c r="O29" s="6">
         <f>IF(G29="","",$B$3-G29)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P29" s="6" t="str">
         <f>IF(H29="","Pending buy",IF(N29&gt;=0,"In profit","In loss"))</f>
@@ -2277,23 +2277,23 @@
         <v>99998.69</v>
       </c>
       <c r="K30" s="9" t="n">
-        <v>16.66</v>
+        <v>16.99</v>
       </c>
       <c r="L30" s="9">
         <f>IF(OR(I30="",K30=""),"",K30*I30)</f>
-        <v>112338.38</v>
+        <v>114563.57</v>
       </c>
       <c r="M30" s="9">
         <f>IF(L30="","",L30-J30)</f>
-        <v>12339.69</v>
+        <v>14564.88</v>
       </c>
       <c r="N30" s="10">
         <f>IF(OR(H30="",K30=""),"",K30/H30-1)</f>
-        <v>0.12339851652056644</v>
+        <v>0.14565070802427504</v>
       </c>
       <c r="O30" s="6">
         <f>IF(G30="","",$B$3-G30)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="P30" s="6" t="str">
         <f>IF(H30="","Pending buy",IF(N30&gt;=0,"In profit","In loss"))</f>
@@ -2345,23 +2345,23 @@
         <v>99977.34</v>
       </c>
       <c r="K31" s="9" t="n">
-        <v>174.14</v>
+        <v>165.45</v>
       </c>
       <c r="L31" s="9">
         <f>IF(OR(I31="",K31=""),"",K31*I31)</f>
-        <v>98214.96</v>
+        <v>93313.8</v>
       </c>
       <c r="M31" s="9">
         <f>IF(L31="","",L31-J31)</f>
-        <v>-1762.38</v>
+        <v>-6663.54</v>
       </c>
       <c r="N31" s="10">
         <f>IF(OR(H31="",K31=""),"",K31/H31-1)</f>
-        <v>-0.017627776535693696</v>
+        <v>-0.06665048597582701</v>
       </c>
       <c r="O31" s="6">
         <f>IF(G31="","",$B$3-G31)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P31" s="6" t="str">
         <f>IF(H31="","Pending buy",IF(N31&gt;=0,"In profit","In loss"))</f>
@@ -2413,23 +2413,23 @@
         <v>99923.82</v>
       </c>
       <c r="K32" s="9" t="n">
-        <v>187.7</v>
+        <v>178.32</v>
       </c>
       <c r="L32" s="9">
         <f>IF(OR(I32="",K32=""),"",K32*I32)</f>
-        <v>106050.5</v>
+        <v>100750.8</v>
       </c>
       <c r="M32" s="9">
         <f>IF(L32="","",L32-J32)</f>
-        <v>6126.68</v>
+        <v>826.98</v>
       </c>
       <c r="N32" s="10">
         <f>IF(OR(H32="",K32=""),"",K32/H32-1)</f>
-        <v>0.061313512135879655</v>
+        <v>0.008276108066436194</v>
       </c>
       <c r="O32" s="6">
         <f>IF(G32="","",$B$3-G32)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P32" s="6" t="str">
         <f>IF(H32="","Pending buy",IF(N32&gt;=0,"In profit","In loss"))</f>
@@ -2481,23 +2481,23 @@
         <v>99608.58</v>
       </c>
       <c r="K33" s="9" t="n">
-        <v>539.3</v>
+        <v>542.5</v>
       </c>
       <c r="L33" s="9">
         <f>IF(OR(I33="",K33=""),"",K33*I33)</f>
-        <v>101927.7</v>
+        <v>102532.5</v>
       </c>
       <c r="M33" s="9">
         <f>IF(L33="","",L33-J33)</f>
-        <v>2319.12</v>
+        <v>2923.92</v>
       </c>
       <c r="N33" s="10">
         <f>IF(OR(H33="",K33=""),"",K33/H33-1)</f>
-        <v>0.023282381814613284</v>
+        <v>0.029354148218853515</v>
       </c>
       <c r="O33" s="6">
         <f>IF(G33="","",$B$3-G33)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P33" s="6" t="str">
         <f>IF(H33="","Pending buy",IF(N33&gt;=0,"In profit","In loss"))</f>
@@ -2549,23 +2549,23 @@
         <v>96030.46</v>
       </c>
       <c r="K34" s="9" t="n">
-        <v>4731.7</v>
+        <v>4699.9</v>
       </c>
       <c r="L34" s="9">
         <f>IF(OR(I34="",K34=""),"",K34*I34)</f>
-        <v>89902.3</v>
+        <v>89298.1</v>
       </c>
       <c r="M34" s="9">
         <f>IF(L34="","",L34-J34)</f>
-        <v>-6128.16</v>
+        <v>-6732.36</v>
       </c>
       <c r="N34" s="10">
         <f>IF(OR(H34="",K34=""),"",K34/H34-1)</f>
-        <v>-0.06381475917885115</v>
+        <v>-0.07010651281033942</v>
       </c>
       <c r="O34" s="6">
         <f>IF(G34="","",$B$3-G34)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P34" s="6" t="str">
         <f>IF(H34="","Pending buy",IF(N34&gt;=0,"In profit","In loss"))</f>
@@ -2617,23 +2617,23 @@
         <v>99082.89</v>
       </c>
       <c r="K35" s="9" t="n">
-        <v>1008.3</v>
+        <v>986.8</v>
       </c>
       <c r="L35" s="9">
         <f>IF(OR(I35="",K35=""),"",K35*I35)</f>
-        <v>91755.3</v>
+        <v>89798.8</v>
       </c>
       <c r="M35" s="9">
         <f>IF(L35="","",L35-J35)</f>
-        <v>-7327.59</v>
+        <v>-9284.09</v>
       </c>
       <c r="N35" s="10">
         <f>IF(OR(H35="",K35=""),"",K35/H35-1)</f>
-        <v>-0.07395416885940154</v>
+        <v>-0.09370026165869028</v>
       </c>
       <c r="O35" s="6">
         <f>IF(G35="","",$B$3-G35)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P35" s="6" t="str">
         <f>IF(H35="","Pending buy",IF(N35&gt;=0,"In profit","In loss"))</f>
@@ -2685,23 +2685,23 @@
         <v>99910.57</v>
       </c>
       <c r="K36" s="9" t="n">
-        <v>100.62</v>
+        <v>97.98</v>
       </c>
       <c r="L36" s="9">
         <f>IF(OR(I36="",K36=""),"",K36*I36)</f>
-        <v>103135.5</v>
+        <v>100429.5</v>
       </c>
       <c r="M36" s="9">
         <f>IF(L36="","",L36-J36)</f>
-        <v>3224.93</v>
+        <v>518.93</v>
       </c>
       <c r="N36" s="10">
         <f>IF(OR(H36="",K36=""),"",K36/H36-1)</f>
-        <v>0.03227815396575373</v>
+        <v>0.005193932871840223</v>
       </c>
       <c r="O36" s="6">
         <f>IF(G36="","",$B$3-G36)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P36" s="6" t="str">
         <f>IF(H36="","Pending buy",IF(N36&gt;=0,"In profit","In loss"))</f>
@@ -2753,23 +2753,23 @@
         <v>99436.51</v>
       </c>
       <c r="K37" s="9" t="n">
-        <v>961.7</v>
+        <v>923.2</v>
       </c>
       <c r="L37" s="9">
         <f>IF(OR(I37="",K37=""),"",K37*I37)</f>
-        <v>96170.0</v>
+        <v>92320.0</v>
       </c>
       <c r="M37" s="9">
         <f>IF(L37="","",L37-J37)</f>
-        <v>-3266.51</v>
+        <v>-7116.51</v>
       </c>
       <c r="N37" s="10">
         <f>IF(OR(H37="",K37=""),"",K37/H37-1)</f>
-        <v>-0.032850235841285214</v>
+        <v>-0.07156840774532025</v>
       </c>
       <c r="O37" s="6">
         <f>IF(G37="","",$B$3-G37)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P37" s="6" t="str">
         <f>IF(H37="","Pending buy",IF(N37&gt;=0,"In profit","In loss"))</f>
@@ -2821,23 +2821,23 @@
         <v>99951.48</v>
       </c>
       <c r="K38" s="9" t="n">
-        <v>122.57</v>
+        <v>125.43</v>
       </c>
       <c r="L38" s="9">
         <f>IF(OR(I38="",K38=""),"",K38*I38)</f>
-        <v>100384.83</v>
+        <v>102727.17</v>
       </c>
       <c r="M38" s="9">
         <f>IF(L38="","",L38-J38)</f>
-        <v>433.35</v>
+        <v>2775.69</v>
       </c>
       <c r="N38" s="10">
         <f>IF(OR(H38="",K38=""),"",K38/H38-1)</f>
-        <v>0.00433560462965854</v>
+        <v>0.02777037520354142</v>
       </c>
       <c r="O38" s="6">
         <f>IF(G38="","",$B$3-G38)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P38" s="6" t="str">
         <f>IF(H38="","Pending buy",IF(N38&gt;=0,"In profit","In loss"))</f>
@@ -2874,38 +2874,42 @@
       <c r="F39" s="8" t="n">
         <v>46311</v>
       </c>
-      <c r="G39" s="6" t="inlineStr"/>
-      <c r="H39" s="9" t="inlineStr"/>
-      <c r="I39" s="6" t="str">
+      <c r="G39" s="8" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H39" s="9" t="n">
+        <v>556.8</v>
+      </c>
+      <c r="I39" s="6">
         <f>IF(H39="","",ROUNDDOWN($B$1/H39,0))</f>
-        <v/>
-      </c>
-      <c r="J39" s="9" t="str">
+        <v>179</v>
+      </c>
+      <c r="J39" s="9">
         <f>IF(H39="","",H39*I39)</f>
-        <v/>
+        <v>99666.78</v>
       </c>
       <c r="K39" s="9" t="n">
-        <v>571.9</v>
-      </c>
-      <c r="L39" s="9" t="str">
+        <v>548.95</v>
+      </c>
+      <c r="L39" s="9">
         <f>IF(OR(I39="",K39=""),"",K39*I39)</f>
-        <v/>
-      </c>
-      <c r="M39" s="9" t="str">
+        <v>98262.05</v>
+      </c>
+      <c r="M39" s="9">
         <f>IF(L39="","",L39-J39)</f>
-        <v/>
-      </c>
-      <c r="N39" s="10" t="str">
+        <v>-1404.73</v>
+      </c>
+      <c r="N39" s="10">
         <f>IF(OR(H39="",K39=""),"",K39/H39-1)</f>
-        <v/>
-      </c>
-      <c r="O39" s="6" t="str">
+        <v>-0.014094226607630378</v>
+      </c>
+      <c r="O39" s="6">
         <f>IF(G39="","",$B$3-G39)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P39" s="6" t="str">
         <f>IF(H39="","Pending buy",IF(N39&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q39" s="6" t="n">
         <v>1</v>
@@ -2938,45 +2942,177 @@
       <c r="F40" s="8" t="n">
         <v>46311</v>
       </c>
-      <c r="G40" s="6" t="inlineStr"/>
-      <c r="H40" s="9" t="inlineStr"/>
-      <c r="I40" s="6" t="str">
+      <c r="G40" s="8" t="n">
+        <v>46314</v>
+      </c>
+      <c r="H40" s="9" t="n">
+        <v>12.96</v>
+      </c>
+      <c r="I40" s="6">
         <f>IF(H40="","",ROUNDDOWN($B$1/H40,0))</f>
-        <v/>
-      </c>
-      <c r="J40" s="9" t="str">
+        <v>7718</v>
+      </c>
+      <c r="J40" s="9">
         <f>IF(H40="","",H40*I40)</f>
-        <v/>
+        <v>99998.64</v>
       </c>
       <c r="K40" s="9" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="L40" s="9" t="str">
+        <v>12.74</v>
+      </c>
+      <c r="L40" s="9">
         <f>IF(OR(I40="",K40=""),"",K40*I40)</f>
-        <v/>
-      </c>
-      <c r="M40" s="9" t="str">
+        <v>98327.32</v>
+      </c>
+      <c r="M40" s="9">
         <f>IF(L40="","",L40-J40)</f>
-        <v/>
-      </c>
-      <c r="N40" s="10" t="str">
+        <v>-1671.32</v>
+      </c>
+      <c r="N40" s="10">
         <f>IF(OR(H40="",K40=""),"",K40/H40-1)</f>
-        <v/>
-      </c>
-      <c r="O40" s="6" t="str">
+        <v>-0.016713402366124064</v>
+      </c>
+      <c r="O40" s="6">
         <f>IF(G40="","",$B$3-G40)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P40" s="6" t="str">
         <f>IF(H40="","Pending buy",IF(N40&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q40" s="6" t="n">
         <v>1</v>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>AvenuesAI Limited</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>CCAVENUE</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>191026</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G41" s="6" t="inlineStr"/>
+      <c r="H41" s="9" t="inlineStr"/>
+      <c r="I41" s="6" t="str">
+        <f>IF(H41="","",ROUNDDOWN($B$1/H41,0))</f>
+        <v/>
+      </c>
+      <c r="J41" s="9" t="str">
+        <f>IF(H41="","",H41*I41)</f>
+        <v/>
+      </c>
+      <c r="K41" s="9" t="n">
+        <v>130.05</v>
+      </c>
+      <c r="L41" s="9" t="str">
+        <f>IF(OR(I41="",K41=""),"",K41*I41)</f>
+        <v/>
+      </c>
+      <c r="M41" s="9" t="str">
+        <f>IF(L41="","",L41-J41)</f>
+        <v/>
+      </c>
+      <c r="N41" s="10" t="str">
+        <f>IF(OR(H41="",K41=""),"",K41/H41-1)</f>
+        <v/>
+      </c>
+      <c r="O41" s="6" t="str">
+        <f>IF(G41="","",$B$3-G41)</f>
+        <v/>
+      </c>
+      <c r="P41" s="6" t="str">
+        <f>IF(H41="","Pending buy",IF(N41&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q41" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Pashupati Cotspin Limited</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>PASHUPATI</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>191026</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G42" s="6" t="inlineStr"/>
+      <c r="H42" s="9" t="inlineStr"/>
+      <c r="I42" s="6" t="str">
+        <f>IF(H42="","",ROUNDDOWN($B$1/H42,0))</f>
+        <v/>
+      </c>
+      <c r="J42" s="9" t="str">
+        <f>IF(H42="","",H42*I42)</f>
+        <v/>
+      </c>
+      <c r="K42" s="9" t="n">
+        <v>89.52</v>
+      </c>
+      <c r="L42" s="9" t="str">
+        <f>IF(OR(I42="",K42=""),"",K42*I42)</f>
+        <v/>
+      </c>
+      <c r="M42" s="9" t="str">
+        <f>IF(L42="","",L42-J42)</f>
+        <v/>
+      </c>
+      <c r="N42" s="10" t="str">
+        <f>IF(OR(H42="",K42=""),"",K42/H42-1)</f>
+        <v/>
+      </c>
+      <c r="O42" s="6" t="str">
+        <f>IF(G42="","",$B$3-G42)</f>
+        <v/>
+      </c>
+      <c r="P42" s="6" t="str">
+        <f>IF(H42="","Pending buy",IF(N42&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q42" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A8:Q40">
+  <conditionalFormatting sqref="A8:Q42">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$N8&gt;0</formula>
     </cfRule>
@@ -2994,7 +3130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3762,6 +3898,46 @@
       <c r="D38" s="11" t="inlineStr">
         <is>
           <t>Kesoram Industries Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>PASHUPATI</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
+        <is>
+          <t>Pashupati Cotspin Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>CCAVENUE</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="inlineStr">
+        <is>
+          <t>AvenuesAI Limited</t>
         </is>
       </c>
     </row>
@@ -3776,7 +3952,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3913,6 +4089,31 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>EBBETF0433</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Bharat Bond ETF - April 2033</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
+          <t>Not in NSE official equity list; In NSE official ETF list; Name/symbol contains: ETF</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Momentum Portfolio: weekday silent update 2026-10-20
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -3044,7 +3044,7 @@
         <v>Pending buy</v>
       </c>
       <c r="Q41" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42">
@@ -3108,7 +3108,7 @@
         <v>Pending buy</v>
       </c>
       <c r="Q42" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -3130,7 +3130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3936,6 +3936,46 @@
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
+        <is>
+          <t>AvenuesAI Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>PASHUPATI</t>
+        </is>
+      </c>
+      <c r="D41" s="11" t="inlineStr">
+        <is>
+          <t>Pashupati Cotspin Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>CCAVENUE</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="inlineStr">
         <is>
           <t>AvenuesAI Limited</t>
         </is>

</xml_diff>

<commit_message>
Momentum Portfolio: weekday silent update 2026-10-21
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="E1" s="2">
         <f>SUM(J8:J42)</f>
-        <v>3263835.67</v>
+        <v>3463650.69</v>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
@@ -541,7 +541,7 @@
       </c>
       <c r="G1" s="2">
         <f>SUM(L8:L42)</f>
-        <v>3131700.46</v>
+        <v>3242257.44</v>
       </c>
     </row>
     <row r="2">
@@ -552,7 +552,7 @@
       </c>
       <c r="E2" s="2">
         <f>SUM(M8:M42)</f>
-        <v>-132135.21</v>
+        <v>-221393.25</v>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" s="3">
         <f>IF(E1=0,"",G1/E1-1)</f>
-        <v>-0.040484639350730545</v>
+        <v>-0.06391904664035275</v>
       </c>
     </row>
     <row r="3">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>46314</v>
+        <v>46316</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -580,7 +580,7 @@
       </c>
       <c r="E3">
         <f>COUNTIF(M8:M42,"&gt;0")</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
@@ -589,7 +589,7 @@
       </c>
       <c r="G3">
         <f>COUNTIF(M8:M42,"&lt;0")</f>
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4">
@@ -600,7 +600,7 @@
       </c>
       <c r="E4" s="3">
         <f>IF((E3+G3)=0,"",E3/(E3+G3))</f>
-        <v>0.24242424242424243</v>
+        <v>0.2</v>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
@@ -609,7 +609,7 @@
       </c>
       <c r="G4" s="3">
         <f>AVERAGE(N8:N42)</f>
-        <v>-0.0406912464443625</v>
+        <v>-0.06402909789029841</v>
       </c>
     </row>
     <row r="5">
@@ -629,7 +629,7 @@
       </c>
       <c r="G5" t="str">
         <f>INDEX(B8:B42,MATCH(MIN(N8:N42),N8:N42,0))</f>
-        <v>Lloyds Enterprises Limited</v>
+        <v>Ujaas Energy Limited</v>
       </c>
     </row>
     <row r="6">
@@ -640,7 +640,7 @@
       </c>
       <c r="E6" s="3">
         <f>AVERAGEIF(D8:D42,"4★*",N8:N42)</f>
-        <v>-0.05945869664085087</v>
+        <v>-0.08477898089107445</v>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
@@ -649,7 +649,7 @@
       </c>
       <c r="G6" s="3">
         <f>AVERAGEIF(D8:D42,"5★*",N8:N42)</f>
-        <v>-0.0207508306105936</v>
+        <v>-0.042058633536535536</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
@@ -781,23 +781,23 @@
         <v>99851.29</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>285.6</v>
+        <v>274.3</v>
       </c>
       <c r="L8" s="9">
         <f>IF(OR(I8="",K8=""),"",K8*I8)</f>
-        <v>94819.2</v>
+        <v>91067.6</v>
       </c>
       <c r="M8" s="9">
         <f>IF(L8="","",L8-J8)</f>
-        <v>-5032.09</v>
+        <v>-8783.69</v>
       </c>
       <c r="N8" s="10">
         <f>IF(OR(H8="",K8=""),"",K8/H8-1)</f>
-        <v>-0.05039587652630073</v>
+        <v>-0.08796774835841836</v>
       </c>
       <c r="O8" s="6">
         <f>IF(G8="","",$B$3-G8)</f>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="P8" s="6" t="str">
         <f>IF(H8="","Pending buy",IF(N8&gt;=0,"In profit","In loss"))</f>
@@ -849,23 +849,23 @@
         <v>99687.42</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>320.2</v>
+        <v>312.35</v>
       </c>
       <c r="L9" s="9">
         <f>IF(OR(I9="",K9=""),"",K9*I9)</f>
-        <v>97981.2</v>
+        <v>95579.1</v>
       </c>
       <c r="M9" s="9">
         <f>IF(L9="","",L9-J9)</f>
-        <v>-1706.22</v>
+        <v>-4108.32</v>
       </c>
       <c r="N9" s="10">
         <f>IF(OR(H9="",K9=""),"",K9/H9-1)</f>
-        <v>-0.017115702208073014</v>
+        <v>-0.041212022438137375</v>
       </c>
       <c r="O9" s="6">
         <f>IF(G9="","",$B$3-G9)</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="P9" s="6" t="str">
         <f>IF(H9="","Pending buy",IF(N9&gt;=0,"In profit","In loss"))</f>
@@ -917,30 +917,30 @@
         <v>99607.14</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>1538.3</v>
+        <v>1583.8</v>
       </c>
       <c r="L10" s="9">
         <f>IF(OR(I10="",K10=""),"",K10*I10)</f>
-        <v>96912.9</v>
+        <v>99779.4</v>
       </c>
       <c r="M10" s="9">
         <f>IF(L10="","",L10-J10)</f>
-        <v>-2694.24</v>
+        <v>172.26</v>
       </c>
       <c r="N10" s="10">
         <f>IF(OR(H10="",K10=""),"",K10/H10-1)</f>
-        <v>-0.027048672433782173</v>
+        <v>0.0017293847749957347</v>
       </c>
       <c r="O10" s="6">
         <f>IF(G10="","",$B$3-G10)</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="P10" s="6" t="str">
         <f>IF(H10="","Pending buy",IF(N10&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -985,23 +985,23 @@
         <v>99927.23</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>68.72</v>
+        <v>66.02</v>
       </c>
       <c r="L11" s="9">
         <f>IF(OR(I11="",K11=""),"",K11*I11)</f>
-        <v>85968.72</v>
+        <v>82591.02</v>
       </c>
       <c r="M11" s="9">
         <f>IF(L11="","",L11-J11)</f>
-        <v>-13958.51</v>
+        <v>-17336.21</v>
       </c>
       <c r="N11" s="10">
         <f>IF(OR(H11="",K11=""),"",K11/H11-1)</f>
-        <v>-0.1396867533367998</v>
+        <v>-0.173488350630028</v>
       </c>
       <c r="O11" s="6">
         <f>IF(G11="","",$B$3-G11)</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="P11" s="6" t="str">
         <f>IF(H11="","Pending buy",IF(N11&gt;=0,"In profit","In loss"))</f>
@@ -1053,23 +1053,23 @@
         <v>86537.12</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>19220</v>
+        <v>18975</v>
       </c>
       <c r="L12" s="9">
         <f>IF(OR(I12="",K12=""),"",K12*I12)</f>
-        <v>76880.0</v>
+        <v>75900.0</v>
       </c>
       <c r="M12" s="9">
         <f>IF(L12="","",L12-J12)</f>
-        <v>-9657.12</v>
+        <v>-10637.12</v>
       </c>
       <c r="N12" s="10">
         <f>IF(OR(H12="",K12=""),"",K12/H12-1)</f>
-        <v>-0.11159507701154137</v>
+        <v>-0.12291969751789789</v>
       </c>
       <c r="O12" s="6">
         <f>IF(G12="","",$B$3-G12)</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="P12" s="6" t="str">
         <f>IF(H12="","Pending buy",IF(N12&gt;=0,"In profit","In loss"))</f>
@@ -1121,23 +1121,23 @@
         <v>98177.53</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>1683.8</v>
+        <v>1695.8</v>
       </c>
       <c r="L13" s="9">
         <f>IF(OR(I13="",K13=""),"",K13*I13)</f>
-        <v>89241.4</v>
+        <v>89877.4</v>
       </c>
       <c r="M13" s="9">
         <f>IF(L13="","",L13-J13)</f>
-        <v>-8936.13</v>
+        <v>-8300.13</v>
       </c>
       <c r="N13" s="10">
         <f>IF(OR(H13="",K13=""),"",K13/H13-1)</f>
-        <v>-0.09102014351510357</v>
+        <v>-0.08454208301040067</v>
       </c>
       <c r="O13" s="6">
         <f>IF(G13="","",$B$3-G13)</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="P13" s="6" t="str">
         <f>IF(H13="","Pending buy",IF(N13&gt;=0,"In profit","In loss"))</f>
@@ -1189,23 +1189,23 @@
         <v>97667.46</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>4435.5</v>
+        <v>4356.1</v>
       </c>
       <c r="L14" s="9">
         <f>IF(OR(I14="",K14=""),"",K14*I14)</f>
-        <v>97581.0</v>
+        <v>95834.2</v>
       </c>
       <c r="M14" s="9">
         <f>IF(L14="","",L14-J14)</f>
-        <v>-86.46</v>
+        <v>-1833.26</v>
       </c>
       <c r="N14" s="10">
         <f>IF(OR(H14="",K14=""),"",K14/H14-1)</f>
-        <v>-0.0008852915423364083</v>
+        <v>-0.018770469730035266</v>
       </c>
       <c r="O14" s="6">
         <f>IF(G14="","",$B$3-G14)</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="P14" s="6" t="str">
         <f>IF(H14="","Pending buy",IF(N14&gt;=0,"In profit","In loss"))</f>
@@ -1257,23 +1257,23 @@
         <v>99078.19</v>
       </c>
       <c r="K15" s="9" t="n">
-        <v>1478.1</v>
+        <v>1441</v>
       </c>
       <c r="L15" s="9">
         <f>IF(OR(I15="",K15=""),"",K15*I15)</f>
-        <v>94598.4</v>
+        <v>92224.0</v>
       </c>
       <c r="M15" s="9">
         <f>IF(L15="","",L15-J15)</f>
-        <v>-4479.79</v>
+        <v>-6854.19</v>
       </c>
       <c r="N15" s="10">
         <f>IF(OR(H15="",K15=""),"",K15/H15-1)</f>
-        <v>-0.04521467028453641</v>
+        <v>-0.06917958181450301</v>
       </c>
       <c r="O15" s="6">
         <f>IF(G15="","",$B$3-G15)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P15" s="6" t="str">
         <f>IF(H15="","Pending buy",IF(N15&gt;=0,"In profit","In loss"))</f>
@@ -1325,27 +1325,27 @@
         <v>98557.54</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>1459</v>
+        <v>1447.2</v>
       </c>
       <c r="L16" s="9">
         <f>IF(OR(I16="",K16=""),"",K16*I16)</f>
-        <v>99212.0</v>
+        <v>98409.6</v>
       </c>
       <c r="M16" s="9">
         <f>IF(L16="","",L16-J16)</f>
-        <v>654.46</v>
+        <v>-147.94</v>
       </c>
       <c r="N16" s="10">
         <f>IF(OR(H16="",K16=""),"",K16/H16-1)</f>
-        <v>0.006640420480616971</v>
+        <v>-0.0015010167789245576</v>
       </c>
       <c r="O16" s="6">
         <f>IF(G16="","",$B$3-G16)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P16" s="6" t="str">
         <f>IF(H16="","Pending buy",IF(N16&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q16" s="6" t="n">
         <v>2</v>
@@ -1393,23 +1393,23 @@
         <v>99714.35</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>894.45</v>
+        <v>896.8</v>
       </c>
       <c r="L17" s="9">
         <f>IF(OR(I17="",K17=""),"",K17*I17)</f>
-        <v>102861.75</v>
+        <v>103132.0</v>
       </c>
       <c r="M17" s="9">
         <f>IF(L17="","",L17-J17)</f>
-        <v>3147.4</v>
+        <v>3417.65</v>
       </c>
       <c r="N17" s="10">
         <f>IF(OR(H17="",K17=""),"",K17/H17-1)</f>
-        <v>0.03156416225581071</v>
+        <v>0.034274404059490005</v>
       </c>
       <c r="O17" s="6">
         <f>IF(G17="","",$B$3-G17)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P17" s="6" t="str">
         <f>IF(H17="","Pending buy",IF(N17&gt;=0,"In profit","In loss"))</f>
@@ -1461,23 +1461,23 @@
         <v>99596.83</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>622.15</v>
+        <v>598.75</v>
       </c>
       <c r="L18" s="9">
         <f>IF(OR(I18="",K18=""),"",K18*I18)</f>
-        <v>87723.15</v>
+        <v>84423.75</v>
       </c>
       <c r="M18" s="9">
         <f>IF(L18="","",L18-J18)</f>
-        <v>-11873.68</v>
+        <v>-15173.08</v>
       </c>
       <c r="N18" s="10">
         <f>IF(OR(H18="",K18=""),"",K18/H18-1)</f>
-        <v>-0.11921748957181622</v>
+        <v>-0.15234504843064356</v>
       </c>
       <c r="O18" s="6">
         <f>IF(G18="","",$B$3-G18)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P18" s="6" t="str">
         <f>IF(H18="","Pending buy",IF(N18&gt;=0,"In profit","In loss"))</f>
@@ -1529,23 +1529,23 @@
         <v>99993.07</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>139.02</v>
+        <v>133.92</v>
       </c>
       <c r="L19" s="9">
         <f>IF(OR(I19="",K19=""),"",K19*I19)</f>
-        <v>92170.26</v>
+        <v>88788.96</v>
       </c>
       <c r="M19" s="9">
         <f>IF(L19="","",L19-J19)</f>
-        <v>-7822.81</v>
+        <v>-11204.11</v>
       </c>
       <c r="N19" s="10">
         <f>IF(OR(H19="",K19=""),"",K19/H19-1)</f>
-        <v>-0.07823347815561532</v>
+        <v>-0.11204882315206466</v>
       </c>
       <c r="O19" s="6">
         <f>IF(G19="","",$B$3-G19)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P19" s="6" t="str">
         <f>IF(H19="","Pending buy",IF(N19&gt;=0,"In profit","In loss"))</f>
@@ -1597,23 +1597,23 @@
         <v>99896.43</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>202.32</v>
+        <v>193.59</v>
       </c>
       <c r="L20" s="9">
         <f>IF(OR(I20="",K20=""),"",K20*I20)</f>
-        <v>96506.64</v>
+        <v>92342.43</v>
       </c>
       <c r="M20" s="9">
         <f>IF(L20="","",L20-J20)</f>
-        <v>-3389.79</v>
+        <v>-7554.0</v>
       </c>
       <c r="N20" s="10">
         <f>IF(OR(H20="",K20=""),"",K20/H20-1)</f>
-        <v>-0.03393304451216528</v>
+        <v>-0.07561831794736096</v>
       </c>
       <c r="O20" s="6">
         <f>IF(G20="","",$B$3-G20)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P20" s="6" t="str">
         <f>IF(H20="","Pending buy",IF(N20&gt;=0,"In profit","In loss"))</f>
@@ -1665,23 +1665,23 @@
         <v>99449.47</v>
       </c>
       <c r="K21" s="9" t="n">
-        <v>1253.6</v>
+        <v>1224.1</v>
       </c>
       <c r="L21" s="9">
         <f>IF(OR(I21="",K21=""),"",K21*I21)</f>
-        <v>89005.6</v>
+        <v>86911.1</v>
       </c>
       <c r="M21" s="9">
         <f>IF(L21="","",L21-J21)</f>
-        <v>-10443.87</v>
+        <v>-12538.37</v>
       </c>
       <c r="N21" s="10">
         <f>IF(OR(H21="",K21=""),"",K21/H21-1)</f>
-        <v>-0.10501681631351656</v>
+        <v>-0.1260777639194126</v>
       </c>
       <c r="O21" s="6">
         <f>IF(G21="","",$B$3-G21)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P21" s="6" t="str">
         <f>IF(H21="","Pending buy",IF(N21&gt;=0,"In profit","In loss"))</f>
@@ -1733,23 +1733,23 @@
         <v>99837.05</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>668.4</v>
+        <v>635</v>
       </c>
       <c r="L22" s="9">
         <f>IF(OR(I22="",K22=""),"",K22*I22)</f>
-        <v>96249.6</v>
+        <v>91440.0</v>
       </c>
       <c r="M22" s="9">
         <f>IF(L22="","",L22-J22)</f>
-        <v>-3587.45</v>
+        <v>-8397.05</v>
       </c>
       <c r="N22" s="10">
         <f>IF(OR(H22="",K22=""),"",K22/H22-1)</f>
-        <v>-0.03593306372488947</v>
+        <v>-0.08410756353277193</v>
       </c>
       <c r="O22" s="6">
         <f>IF(G22="","",$B$3-G22)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P22" s="6" t="str">
         <f>IF(H22="","Pending buy",IF(N22&gt;=0,"In profit","In loss"))</f>
@@ -1801,23 +1801,23 @@
         <v>99486.88</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>615.6</v>
+        <v>591.6</v>
       </c>
       <c r="L23" s="9">
         <f>IF(OR(I23="",K23=""),"",K23*I23)</f>
-        <v>89262.0</v>
+        <v>85782.0</v>
       </c>
       <c r="M23" s="9">
         <f>IF(L23="","",L23-J23)</f>
-        <v>-10224.88</v>
+        <v>-13704.88</v>
       </c>
       <c r="N23" s="10">
         <f>IF(OR(H23="",K23=""),"",K23/H23-1)</f>
-        <v>-0.10277617579017795</v>
+        <v>-0.13775566211414758</v>
       </c>
       <c r="O23" s="6">
         <f>IF(G23="","",$B$3-G23)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="P23" s="6" t="str">
         <f>IF(H23="","Pending buy",IF(N23&gt;=0,"In profit","In loss"))</f>
@@ -1869,23 +1869,23 @@
         <v>99935.4</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>215.77</v>
+        <v>211.53</v>
       </c>
       <c r="L24" s="9">
         <f>IF(OR(I24="",K24=""),"",K24*I24)</f>
-        <v>94723.03</v>
+        <v>92861.67</v>
       </c>
       <c r="M24" s="9">
         <f>IF(L24="","",L24-J24)</f>
-        <v>-5212.37</v>
+        <v>-7073.73</v>
       </c>
       <c r="N24" s="10">
         <f>IF(OR(H24="",K24=""),"",K24/H24-1)</f>
-        <v>-0.05215738042639406</v>
+        <v>-0.07078301284513666</v>
       </c>
       <c r="O24" s="6">
         <f>IF(G24="","",$B$3-G24)</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="P24" s="6" t="str">
         <f>IF(H24="","Pending buy",IF(N24&gt;=0,"In profit","In loss"))</f>
@@ -1937,23 +1937,23 @@
         <v>99622.64</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>751.75</v>
+        <v>717.55</v>
       </c>
       <c r="L25" s="9">
         <f>IF(OR(I25="",K25=""),"",K25*I25)</f>
-        <v>93217.0</v>
+        <v>88976.2</v>
       </c>
       <c r="M25" s="9">
         <f>IF(L25="","",L25-J25)</f>
-        <v>-6405.64</v>
+        <v>-10646.44</v>
       </c>
       <c r="N25" s="10">
         <f>IF(OR(H25="",K25=""),"",K25/H25-1)</f>
-        <v>-0.06429900496504426</v>
+        <v>-0.10686764351535416</v>
       </c>
       <c r="O25" s="6">
         <f>IF(G25="","",$B$3-G25)</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P25" s="6" t="str">
         <f>IF(H25="","Pending buy",IF(N25&gt;=0,"In profit","In loss"))</f>
@@ -2005,23 +2005,23 @@
         <v>99948.17</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>183</v>
+        <v>171.42</v>
       </c>
       <c r="L26" s="9">
         <f>IF(OR(I26="",K26=""),"",K26*I26)</f>
-        <v>86925.0</v>
+        <v>81424.5</v>
       </c>
       <c r="M26" s="9">
         <f>IF(L26="","",L26-J26)</f>
-        <v>-13023.17</v>
+        <v>-18523.67</v>
       </c>
       <c r="N26" s="10">
         <f>IF(OR(H26="",K26=""),"",K26/H26-1)</f>
-        <v>-0.1302992051604832</v>
+        <v>-0.18533273086672153</v>
       </c>
       <c r="O26" s="6">
         <f>IF(G26="","",$B$3-G26)</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="P26" s="6" t="str">
         <f>IF(H26="","Pending buy",IF(N26&gt;=0,"In profit","In loss"))</f>
@@ -2073,23 +2073,23 @@
         <v>99745.27</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>240.6</v>
+        <v>236.75</v>
       </c>
       <c r="L27" s="9">
         <f>IF(OR(I27="",K27=""),"",K27*I27)</f>
-        <v>91909.2</v>
+        <v>90438.5</v>
       </c>
       <c r="M27" s="9">
         <f>IF(L27="","",L27-J27)</f>
-        <v>-7836.07</v>
+        <v>-9306.77</v>
       </c>
       <c r="N27" s="10">
         <f>IF(OR(H27="",K27=""),"",K27/H27-1)</f>
-        <v>-0.07856084531587204</v>
+        <v>-0.09330540369298712</v>
       </c>
       <c r="O27" s="6">
         <f>IF(G27="","",$B$3-G27)</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P27" s="6" t="str">
         <f>IF(H27="","Pending buy",IF(N27&gt;=0,"In profit","In loss"))</f>
@@ -2141,23 +2141,23 @@
         <v>95334.84</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>11158</v>
+        <v>10989</v>
       </c>
       <c r="L28" s="9">
         <f>IF(OR(I28="",K28=""),"",K28*I28)</f>
-        <v>100422.0</v>
+        <v>98901.0</v>
       </c>
       <c r="M28" s="9">
         <f>IF(L28="","",L28-J28)</f>
-        <v>5087.16</v>
+        <v>3566.16</v>
       </c>
       <c r="N28" s="10">
         <f>IF(OR(H28="",K28=""),"",K28/H28-1)</f>
-        <v>0.05336094840305905</v>
+        <v>0.03740665549392519</v>
       </c>
       <c r="O28" s="6">
         <f>IF(G28="","",$B$3-G28)</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P28" s="6" t="str">
         <f>IF(H28="","Pending buy",IF(N28&gt;=0,"In profit","In loss"))</f>
@@ -2209,23 +2209,23 @@
         <v>98598.59</v>
       </c>
       <c r="K29" s="9" t="n">
-        <v>1866.8</v>
+        <v>1825.7</v>
       </c>
       <c r="L29" s="9">
         <f>IF(OR(I29="",K29=""),"",K29*I29)</f>
-        <v>95206.8</v>
+        <v>93110.7</v>
       </c>
       <c r="M29" s="9">
         <f>IF(L29="","",L29-J29)</f>
-        <v>-3391.79</v>
+        <v>-5487.89</v>
       </c>
       <c r="N29" s="10">
         <f>IF(OR(H29="",K29=""),"",K29/H29-1)</f>
-        <v>-0.03439994823001635</v>
+        <v>-0.05565887373234457</v>
       </c>
       <c r="O29" s="6">
         <f>IF(G29="","",$B$3-G29)</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P29" s="6" t="str">
         <f>IF(H29="","Pending buy",IF(N29&gt;=0,"In profit","In loss"))</f>
@@ -2277,23 +2277,23 @@
         <v>99998.69</v>
       </c>
       <c r="K30" s="9" t="n">
-        <v>16.99</v>
+        <v>16.66</v>
       </c>
       <c r="L30" s="9">
         <f>IF(OR(I30="",K30=""),"",K30*I30)</f>
-        <v>114563.57</v>
+        <v>112338.38</v>
       </c>
       <c r="M30" s="9">
         <f>IF(L30="","",L30-J30)</f>
-        <v>14564.88</v>
+        <v>12339.69</v>
       </c>
       <c r="N30" s="10">
         <f>IF(OR(H30="",K30=""),"",K30/H30-1)</f>
-        <v>0.14565070802427504</v>
+        <v>0.12339851652056644</v>
       </c>
       <c r="O30" s="6">
         <f>IF(G30="","",$B$3-G30)</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P30" s="6" t="str">
         <f>IF(H30="","Pending buy",IF(N30&gt;=0,"In profit","In loss"))</f>
@@ -2345,23 +2345,23 @@
         <v>99977.34</v>
       </c>
       <c r="K31" s="9" t="n">
-        <v>165.45</v>
+        <v>161.24</v>
       </c>
       <c r="L31" s="9">
         <f>IF(OR(I31="",K31=""),"",K31*I31)</f>
-        <v>93313.8</v>
+        <v>90939.36</v>
       </c>
       <c r="M31" s="9">
         <f>IF(L31="","",L31-J31)</f>
-        <v>-6663.54</v>
+        <v>-9037.98</v>
       </c>
       <c r="N31" s="10">
         <f>IF(OR(H31="",K31=""),"",K31/H31-1)</f>
-        <v>-0.06665048597582701</v>
+        <v>-0.0904002681096544</v>
       </c>
       <c r="O31" s="6">
         <f>IF(G31="","",$B$3-G31)</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P31" s="6" t="str">
         <f>IF(H31="","Pending buy",IF(N31&gt;=0,"In profit","In loss"))</f>
@@ -2413,27 +2413,27 @@
         <v>99923.82</v>
       </c>
       <c r="K32" s="9" t="n">
-        <v>178.32</v>
+        <v>169.68</v>
       </c>
       <c r="L32" s="9">
         <f>IF(OR(I32="",K32=""),"",K32*I32)</f>
-        <v>100750.8</v>
+        <v>95869.2</v>
       </c>
       <c r="M32" s="9">
         <f>IF(L32="","",L32-J32)</f>
-        <v>826.98</v>
+        <v>-4054.62</v>
       </c>
       <c r="N32" s="10">
         <f>IF(OR(H32="",K32=""),"",K32/H32-1)</f>
-        <v>0.008276108066436194</v>
+        <v>-0.04057710847514073</v>
       </c>
       <c r="O32" s="6">
         <f>IF(G32="","",$B$3-G32)</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P32" s="6" t="str">
         <f>IF(H32="","Pending buy",IF(N32&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q32" s="6" t="n">
         <v>1</v>
@@ -2481,23 +2481,23 @@
         <v>99608.58</v>
       </c>
       <c r="K33" s="9" t="n">
-        <v>542.5</v>
+        <v>530.15</v>
       </c>
       <c r="L33" s="9">
         <f>IF(OR(I33="",K33=""),"",K33*I33)</f>
-        <v>102532.5</v>
+        <v>100198.35</v>
       </c>
       <c r="M33" s="9">
         <f>IF(L33="","",L33-J33)</f>
-        <v>2923.92</v>
+        <v>589.77</v>
       </c>
       <c r="N33" s="10">
         <f>IF(OR(H33="",K33=""),"",K33/H33-1)</f>
-        <v>0.029354148218853515</v>
+        <v>0.005920924752488954</v>
       </c>
       <c r="O33" s="6">
         <f>IF(G33="","",$B$3-G33)</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P33" s="6" t="str">
         <f>IF(H33="","Pending buy",IF(N33&gt;=0,"In profit","In loss"))</f>
@@ -2549,23 +2549,23 @@
         <v>96030.46</v>
       </c>
       <c r="K34" s="9" t="n">
-        <v>4699.9</v>
+        <v>4594.1</v>
       </c>
       <c r="L34" s="9">
         <f>IF(OR(I34="",K34=""),"",K34*I34)</f>
-        <v>89298.1</v>
+        <v>87287.9</v>
       </c>
       <c r="M34" s="9">
         <f>IF(L34="","",L34-J34)</f>
-        <v>-6732.36</v>
+        <v>-8742.56</v>
       </c>
       <c r="N34" s="10">
         <f>IF(OR(H34="",K34=""),"",K34/H34-1)</f>
-        <v>-0.07010651281033942</v>
+        <v>-0.09103945413774328</v>
       </c>
       <c r="O34" s="6">
         <f>IF(G34="","",$B$3-G34)</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="P34" s="6" t="str">
         <f>IF(H34="","Pending buy",IF(N34&gt;=0,"In profit","In loss"))</f>
@@ -2617,23 +2617,23 @@
         <v>99082.89</v>
       </c>
       <c r="K35" s="9" t="n">
-        <v>986.8</v>
+        <v>951.8</v>
       </c>
       <c r="L35" s="9">
         <f>IF(OR(I35="",K35=""),"",K35*I35)</f>
-        <v>89798.8</v>
+        <v>86613.8</v>
       </c>
       <c r="M35" s="9">
         <f>IF(L35="","",L35-J35)</f>
-        <v>-9284.09</v>
+        <v>-12469.09</v>
       </c>
       <c r="N35" s="10">
         <f>IF(OR(H35="",K35=""),"",K35/H35-1)</f>
-        <v>-0.09370026165869028</v>
+        <v>-0.12584506389009065</v>
       </c>
       <c r="O35" s="6">
         <f>IF(G35="","",$B$3-G35)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P35" s="6" t="str">
         <f>IF(H35="","Pending buy",IF(N35&gt;=0,"In profit","In loss"))</f>
@@ -2685,27 +2685,27 @@
         <v>99910.57</v>
       </c>
       <c r="K36" s="9" t="n">
-        <v>97.98</v>
+        <v>93.06</v>
       </c>
       <c r="L36" s="9">
         <f>IF(OR(I36="",K36=""),"",K36*I36)</f>
-        <v>100429.5</v>
+        <v>95386.5</v>
       </c>
       <c r="M36" s="9">
         <f>IF(L36="","",L36-J36)</f>
-        <v>518.93</v>
+        <v>-4524.07</v>
       </c>
       <c r="N36" s="10">
         <f>IF(OR(H36="",K36=""),"",K36/H36-1)</f>
-        <v>0.005193932871840223</v>
+        <v>-0.045281206439544364</v>
       </c>
       <c r="O36" s="6">
         <f>IF(G36="","",$B$3-G36)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P36" s="6" t="str">
         <f>IF(H36="","Pending buy",IF(N36&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q36" s="6" t="n">
         <v>1</v>
@@ -2753,23 +2753,23 @@
         <v>99436.51</v>
       </c>
       <c r="K37" s="9" t="n">
-        <v>923.2</v>
+        <v>904.8</v>
       </c>
       <c r="L37" s="9">
         <f>IF(OR(I37="",K37=""),"",K37*I37)</f>
-        <v>92320.0</v>
+        <v>90480.0</v>
       </c>
       <c r="M37" s="9">
         <f>IF(L37="","",L37-J37)</f>
-        <v>-7116.51</v>
+        <v>-8956.51</v>
       </c>
       <c r="N37" s="10">
         <f>IF(OR(H37="",K37=""),"",K37/H37-1)</f>
-        <v>-0.07156840774532025</v>
+        <v>-0.09007267691504095</v>
       </c>
       <c r="O37" s="6">
         <f>IF(G37="","",$B$3-G37)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P37" s="6" t="str">
         <f>IF(H37="","Pending buy",IF(N37&gt;=0,"In profit","In loss"))</f>
@@ -2821,23 +2821,23 @@
         <v>99951.48</v>
       </c>
       <c r="K38" s="9" t="n">
-        <v>125.43</v>
+        <v>123.9</v>
       </c>
       <c r="L38" s="9">
         <f>IF(OR(I38="",K38=""),"",K38*I38)</f>
-        <v>102727.17</v>
+        <v>101474.1</v>
       </c>
       <c r="M38" s="9">
         <f>IF(L38="","",L38-J38)</f>
-        <v>2775.69</v>
+        <v>1522.62</v>
       </c>
       <c r="N38" s="10">
         <f>IF(OR(H38="",K38=""),"",K38/H38-1)</f>
-        <v>0.02777037520354142</v>
+        <v>0.015233592344086722</v>
       </c>
       <c r="O38" s="6">
         <f>IF(G38="","",$B$3-G38)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="P38" s="6" t="str">
         <f>IF(H38="","Pending buy",IF(N38&gt;=0,"In profit","In loss"))</f>
@@ -2889,23 +2889,23 @@
         <v>99666.78</v>
       </c>
       <c r="K39" s="9" t="n">
-        <v>548.95</v>
+        <v>521.75</v>
       </c>
       <c r="L39" s="9">
         <f>IF(OR(I39="",K39=""),"",K39*I39)</f>
-        <v>98262.05</v>
+        <v>93393.25</v>
       </c>
       <c r="M39" s="9">
         <f>IF(L39="","",L39-J39)</f>
-        <v>-1404.73</v>
+        <v>-6273.53</v>
       </c>
       <c r="N39" s="10">
         <f>IF(OR(H39="",K39=""),"",K39/H39-1)</f>
-        <v>-0.014094226607630378</v>
+        <v>-0.06294500907647538</v>
       </c>
       <c r="O39" s="6">
         <f>IF(G39="","",$B$3-G39)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P39" s="6" t="str">
         <f>IF(H39="","Pending buy",IF(N39&gt;=0,"In profit","In loss"))</f>
@@ -2957,23 +2957,23 @@
         <v>99998.64</v>
       </c>
       <c r="K40" s="9" t="n">
-        <v>12.74</v>
+        <v>11.67</v>
       </c>
       <c r="L40" s="9">
         <f>IF(OR(I40="",K40=""),"",K40*I40)</f>
-        <v>98327.32</v>
+        <v>90069.06</v>
       </c>
       <c r="M40" s="9">
         <f>IF(L40="","",L40-J40)</f>
-        <v>-1671.32</v>
+        <v>-9929.58</v>
       </c>
       <c r="N40" s="10">
         <f>IF(OR(H40="",K40=""),"",K40/H40-1)</f>
-        <v>-0.016713402366124064</v>
+        <v>-0.09929712759911047</v>
       </c>
       <c r="O40" s="6">
         <f>IF(G40="","",$B$3-G40)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P40" s="6" t="str">
         <f>IF(H40="","Pending buy",IF(N40&gt;=0,"In profit","In loss"))</f>
@@ -3010,38 +3010,42 @@
       <c r="F41" s="8" t="n">
         <v>46314</v>
       </c>
-      <c r="G41" s="6" t="inlineStr"/>
-      <c r="H41" s="9" t="inlineStr"/>
-      <c r="I41" s="6" t="str">
+      <c r="G41" s="8" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H41" s="9" t="n">
+        <v>125.65</v>
+      </c>
+      <c r="I41" s="6">
         <f>IF(H41="","",ROUNDDOWN($B$1/H41,0))</f>
-        <v/>
-      </c>
-      <c r="J41" s="9" t="str">
+        <v>795</v>
+      </c>
+      <c r="J41" s="9">
         <f>IF(H41="","",H41*I41)</f>
-        <v/>
+        <v>99889.82</v>
       </c>
       <c r="K41" s="9" t="n">
-        <v>130.05</v>
-      </c>
-      <c r="L41" s="9" t="str">
+        <v>123.66</v>
+      </c>
+      <c r="L41" s="9">
         <f>IF(OR(I41="",K41=""),"",K41*I41)</f>
-        <v/>
-      </c>
-      <c r="M41" s="9" t="str">
+        <v>98309.7</v>
+      </c>
+      <c r="M41" s="9">
         <f>IF(L41="","",L41-J41)</f>
-        <v/>
-      </c>
-      <c r="N41" s="10" t="str">
+        <v>-1580.12</v>
+      </c>
+      <c r="N41" s="10">
         <f>IF(OR(H41="",K41=""),"",K41/H41-1)</f>
-        <v/>
-      </c>
-      <c r="O41" s="6" t="str">
+        <v>-0.01581861857082778</v>
+      </c>
+      <c r="O41" s="6">
         <f>IF(G41="","",$B$3-G41)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P41" s="6" t="str">
         <f>IF(H41="","Pending buy",IF(N41&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q41" s="6" t="n">
         <v>2</v>
@@ -3074,38 +3078,42 @@
       <c r="F42" s="8" t="n">
         <v>46314</v>
       </c>
-      <c r="G42" s="6" t="inlineStr"/>
-      <c r="H42" s="9" t="inlineStr"/>
-      <c r="I42" s="6" t="str">
+      <c r="G42" s="8" t="n">
+        <v>46316</v>
+      </c>
+      <c r="H42" s="9" t="n">
+        <v>94</v>
+      </c>
+      <c r="I42" s="6">
         <f>IF(H42="","",ROUNDDOWN($B$1/H42,0))</f>
-        <v/>
-      </c>
-      <c r="J42" s="9" t="str">
+        <v>1063</v>
+      </c>
+      <c r="J42" s="9">
         <f>IF(H42="","",H42*I42)</f>
-        <v/>
+        <v>99925.2</v>
       </c>
       <c r="K42" s="9" t="n">
-        <v>89.52</v>
-      </c>
-      <c r="L42" s="9" t="str">
+        <v>94.17</v>
+      </c>
+      <c r="L42" s="9">
         <f>IF(OR(I42="",K42=""),"",K42*I42)</f>
-        <v/>
-      </c>
-      <c r="M42" s="9" t="str">
+        <v>100102.71</v>
+      </c>
+      <c r="M42" s="9">
         <f>IF(L42="","",L42-J42)</f>
-        <v/>
-      </c>
-      <c r="N42" s="10" t="str">
+        <v>177.51</v>
+      </c>
+      <c r="N42" s="10">
         <f>IF(OR(H42="",K42=""),"",K42/H42-1)</f>
-        <v/>
-      </c>
-      <c r="O42" s="6" t="str">
+        <v>0.0017764431349212018</v>
+      </c>
+      <c r="O42" s="6">
         <f>IF(G42="","",$B$3-G42)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P42" s="6" t="str">
         <f>IF(H42="","Pending buy",IF(N42&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In profit</v>
       </c>
       <c r="Q42" s="6" t="n">
         <v>2</v>
@@ -3130,7 +3138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3978,6 +3986,26 @@
       <c r="D42" s="11" t="inlineStr">
         <is>
           <t>AvenuesAI Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>HALEOSLABS</t>
+        </is>
+      </c>
+      <c r="D43" s="11" t="inlineStr">
+        <is>
+          <t>HALEOS LABS LIMITED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum Portfolio: weekday silent update 2026-10-22
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q42"/>
+  <dimension ref="A1:Q48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="E1" s="2">
-        <f>SUM(J8:J42)</f>
+        <f>SUM(J8:J48)</f>
         <v>3463650.69</v>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -540,8 +540,8 @@
         </is>
       </c>
       <c r="G1" s="2">
-        <f>SUM(L8:L42)</f>
-        <v>3242257.44</v>
+        <f>SUM(L8:L48)</f>
+        <v>3201499.22</v>
       </c>
     </row>
     <row r="2">
@@ -551,8 +551,8 @@
         </is>
       </c>
       <c r="E2" s="2">
-        <f>SUM(M8:M42)</f>
-        <v>-221393.25</v>
+        <f>SUM(M8:M48)</f>
+        <v>-262151.47</v>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" s="3">
         <f>IF(E1=0,"",G1/E1-1)</f>
-        <v>-0.06391904664035275</v>
+        <v>-0.07568646305958748</v>
       </c>
     </row>
     <row r="3">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -579,8 +579,8 @@
         </is>
       </c>
       <c r="E3">
-        <f>COUNTIF(M8:M42,"&gt;0")</f>
-        <v>7</v>
+        <f>COUNTIF(M8:M48,"&gt;0")</f>
+        <v>5</v>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
@@ -588,8 +588,8 @@
         </is>
       </c>
       <c r="G3">
-        <f>COUNTIF(M8:M42,"&lt;0")</f>
-        <v>28</v>
+        <f>COUNTIF(M8:M48,"&lt;0")</f>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
@@ -600,7 +600,7 @@
       </c>
       <c r="E4" s="3">
         <f>IF((E3+G3)=0,"",E3/(E3+G3))</f>
-        <v>0.2</v>
+        <v>0.14285714285714285</v>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
@@ -608,8 +608,8 @@
         </is>
       </c>
       <c r="G4" s="3">
-        <f>AVERAGE(N8:N42)</f>
-        <v>-0.06402909789029841</v>
+        <f>AVERAGE(N8:N48)</f>
+        <v>-0.07574536961562824</v>
       </c>
     </row>
     <row r="5">
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="E5" t="str">
-        <f>INDEX(B8:B42,MATCH(MAX(N8:N42),N8:N42,0))</f>
+        <f>INDEX(B8:B48,MATCH(MAX(N8:N48),N8:N48,0))</f>
         <v>Viji Finance Limited</v>
       </c>
       <c r="F5" s="1" t="inlineStr">
@@ -628,8 +628,8 @@
         </is>
       </c>
       <c r="G5" t="str">
-        <f>INDEX(B8:B42,MATCH(MIN(N8:N42),N8:N42,0))</f>
-        <v>Ujaas Energy Limited</v>
+        <f>INDEX(B8:B48,MATCH(MIN(N8:N48),N8:N48,0))</f>
+        <v>Lloyds Enterprises Limited</v>
       </c>
     </row>
     <row r="6">
@@ -639,8 +639,8 @@
         </is>
       </c>
       <c r="E6" s="3">
-        <f>AVERAGEIF(D8:D42,"4★*",N8:N42)</f>
-        <v>-0.08477898089107445</v>
+        <f>AVERAGEIF(D8:D48,"4★*",N8:N48)</f>
+        <v>-0.08912510970554093</v>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
@@ -648,8 +648,8 @@
         </is>
       </c>
       <c r="G6" s="3">
-        <f>AVERAGEIF(D8:D42,"5★*",N8:N42)</f>
-        <v>-0.042058633536535536</v>
+        <f>AVERAGEIF(D8:D48,"5★*",N8:N48)</f>
+        <v>-0.06157858599101481</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
@@ -781,23 +781,23 @@
         <v>99851.29</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>274.3</v>
+        <v>271.3</v>
       </c>
       <c r="L8" s="9">
         <f>IF(OR(I8="",K8=""),"",K8*I8)</f>
-        <v>91067.6</v>
+        <v>90071.6</v>
       </c>
       <c r="M8" s="9">
         <f>IF(L8="","",L8-J8)</f>
-        <v>-8783.69</v>
+        <v>-9779.69</v>
       </c>
       <c r="N8" s="10">
         <f>IF(OR(H8="",K8=""),"",K8/H8-1)</f>
-        <v>-0.08796774835841836</v>
+        <v>-0.09794258158818414</v>
       </c>
       <c r="O8" s="6">
         <f>IF(G8="","",$B$3-G8)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P8" s="6" t="str">
         <f>IF(H8="","Pending buy",IF(N8&gt;=0,"In profit","In loss"))</f>
@@ -849,23 +849,23 @@
         <v>99687.42</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>312.35</v>
+        <v>304.45</v>
       </c>
       <c r="L9" s="9">
         <f>IF(OR(I9="",K9=""),"",K9*I9)</f>
-        <v>95579.1</v>
+        <v>93161.7</v>
       </c>
       <c r="M9" s="9">
         <f>IF(L9="","",L9-J9)</f>
-        <v>-4108.32</v>
+        <v>-6525.72</v>
       </c>
       <c r="N9" s="10">
         <f>IF(OR(H9="",K9=""),"",K9/H9-1)</f>
-        <v>-0.041212022438137375</v>
+        <v>-0.06546182241489018</v>
       </c>
       <c r="O9" s="6">
         <f>IF(G9="","",$B$3-G9)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P9" s="6" t="str">
         <f>IF(H9="","Pending buy",IF(N9&gt;=0,"In profit","In loss"))</f>
@@ -917,23 +917,23 @@
         <v>99607.14</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>1583.8</v>
+        <v>1611.3</v>
       </c>
       <c r="L10" s="9">
         <f>IF(OR(I10="",K10=""),"",K10*I10)</f>
-        <v>99779.4</v>
+        <v>101511.9</v>
       </c>
       <c r="M10" s="9">
         <f>IF(L10="","",L10-J10)</f>
-        <v>172.26</v>
+        <v>1904.76</v>
       </c>
       <c r="N10" s="10">
         <f>IF(OR(H10="",K10=""),"",K10/H10-1)</f>
-        <v>0.0017293847749957347</v>
+        <v>0.019122716055026245</v>
       </c>
       <c r="O10" s="6">
         <f>IF(G10="","",$B$3-G10)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P10" s="6" t="str">
         <f>IF(H10="","Pending buy",IF(N10&gt;=0,"In profit","In loss"))</f>
@@ -985,23 +985,23 @@
         <v>99927.23</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>66.02</v>
+        <v>63.74</v>
       </c>
       <c r="L11" s="9">
         <f>IF(OR(I11="",K11=""),"",K11*I11)</f>
-        <v>82591.02</v>
+        <v>79738.74</v>
       </c>
       <c r="M11" s="9">
         <f>IF(L11="","",L11-J11)</f>
-        <v>-17336.21</v>
+        <v>-20188.49</v>
       </c>
       <c r="N11" s="10">
         <f>IF(OR(H11="",K11=""),"",K11/H11-1)</f>
-        <v>-0.173488350630028</v>
+        <v>-0.20203192167764283</v>
       </c>
       <c r="O11" s="6">
         <f>IF(G11="","",$B$3-G11)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P11" s="6" t="str">
         <f>IF(H11="","Pending buy",IF(N11&gt;=0,"In profit","In loss"))</f>
@@ -1053,23 +1053,23 @@
         <v>86537.12</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>18975</v>
+        <v>18935</v>
       </c>
       <c r="L12" s="9">
         <f>IF(OR(I12="",K12=""),"",K12*I12)</f>
-        <v>75900.0</v>
+        <v>75740.0</v>
       </c>
       <c r="M12" s="9">
         <f>IF(L12="","",L12-J12)</f>
-        <v>-10637.12</v>
+        <v>-10797.12</v>
       </c>
       <c r="N12" s="10">
         <f>IF(OR(H12="",K12=""),"",K12/H12-1)</f>
-        <v>-0.12291969751789789</v>
+        <v>-0.12476861515158877</v>
       </c>
       <c r="O12" s="6">
         <f>IF(G12="","",$B$3-G12)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P12" s="6" t="str">
         <f>IF(H12="","Pending buy",IF(N12&gt;=0,"In profit","In loss"))</f>
@@ -1121,23 +1121,23 @@
         <v>98177.53</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>1695.8</v>
+        <v>1669.5</v>
       </c>
       <c r="L13" s="9">
         <f>IF(OR(I13="",K13=""),"",K13*I13)</f>
-        <v>89877.4</v>
+        <v>88483.5</v>
       </c>
       <c r="M13" s="9">
         <f>IF(L13="","",L13-J13)</f>
-        <v>-8300.13</v>
+        <v>-9694.03</v>
       </c>
       <c r="N13" s="10">
         <f>IF(OR(H13="",K13=""),"",K13/H13-1)</f>
-        <v>-0.08454208301040067</v>
+        <v>-0.09873983228320782</v>
       </c>
       <c r="O13" s="6">
         <f>IF(G13="","",$B$3-G13)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P13" s="6" t="str">
         <f>IF(H13="","Pending buy",IF(N13&gt;=0,"In profit","In loss"))</f>
@@ -1189,23 +1189,23 @@
         <v>97667.46</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>4356.1</v>
+        <v>4201.3</v>
       </c>
       <c r="L14" s="9">
         <f>IF(OR(I14="",K14=""),"",K14*I14)</f>
-        <v>95834.2</v>
+        <v>92428.6</v>
       </c>
       <c r="M14" s="9">
         <f>IF(L14="","",L14-J14)</f>
-        <v>-1833.26</v>
+        <v>-5238.86</v>
       </c>
       <c r="N14" s="10">
         <f>IF(OR(H14="",K14=""),"",K14/H14-1)</f>
-        <v>-0.018770469730035266</v>
+        <v>-0.053639809572047725</v>
       </c>
       <c r="O14" s="6">
         <f>IF(G14="","",$B$3-G14)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P14" s="6" t="str">
         <f>IF(H14="","Pending buy",IF(N14&gt;=0,"In profit","In loss"))</f>
@@ -1257,23 +1257,23 @@
         <v>99078.19</v>
       </c>
       <c r="K15" s="9" t="n">
-        <v>1441</v>
+        <v>1345</v>
       </c>
       <c r="L15" s="9">
         <f>IF(OR(I15="",K15=""),"",K15*I15)</f>
-        <v>92224.0</v>
+        <v>86080.0</v>
       </c>
       <c r="M15" s="9">
         <f>IF(L15="","",L15-J15)</f>
-        <v>-6854.19</v>
+        <v>-12998.19</v>
       </c>
       <c r="N15" s="10">
         <f>IF(OR(H15="",K15=""),"",K15/H15-1)</f>
-        <v>-0.06917958181450301</v>
+        <v>-0.13119121272762424</v>
       </c>
       <c r="O15" s="6">
         <f>IF(G15="","",$B$3-G15)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P15" s="6" t="str">
         <f>IF(H15="","Pending buy",IF(N15&gt;=0,"In profit","In loss"))</f>
@@ -1325,23 +1325,23 @@
         <v>98557.54</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>1447.2</v>
+        <v>1425.3</v>
       </c>
       <c r="L16" s="9">
         <f>IF(OR(I16="",K16=""),"",K16*I16)</f>
-        <v>98409.6</v>
+        <v>96920.4</v>
       </c>
       <c r="M16" s="9">
         <f>IF(L16="","",L16-J16)</f>
-        <v>-147.94</v>
+        <v>-1637.14</v>
       </c>
       <c r="N16" s="10">
         <f>IF(OR(H16="",K16=""),"",K16/H16-1)</f>
-        <v>-0.0015010167789245576</v>
+        <v>-0.016610972370785904</v>
       </c>
       <c r="O16" s="6">
         <f>IF(G16="","",$B$3-G16)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P16" s="6" t="str">
         <f>IF(H16="","Pending buy",IF(N16&gt;=0,"In profit","In loss"))</f>
@@ -1393,23 +1393,23 @@
         <v>99714.35</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>896.8</v>
+        <v>885</v>
       </c>
       <c r="L17" s="9">
         <f>IF(OR(I17="",K17=""),"",K17*I17)</f>
-        <v>103132.0</v>
+        <v>101775.0</v>
       </c>
       <c r="M17" s="9">
         <f>IF(L17="","",L17-J17)</f>
-        <v>3417.65</v>
+        <v>2060.65</v>
       </c>
       <c r="N17" s="10">
         <f>IF(OR(H17="",K17=""),"",K17/H17-1)</f>
-        <v>0.034274404059490005</v>
+        <v>0.020665530321865244</v>
       </c>
       <c r="O17" s="6">
         <f>IF(G17="","",$B$3-G17)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P17" s="6" t="str">
         <f>IF(H17="","Pending buy",IF(N17&gt;=0,"In profit","In loss"))</f>
@@ -1461,23 +1461,23 @@
         <v>99596.83</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>598.75</v>
+        <v>608.9</v>
       </c>
       <c r="L18" s="9">
         <f>IF(OR(I18="",K18=""),"",K18*I18)</f>
-        <v>84423.75</v>
+        <v>85854.9</v>
       </c>
       <c r="M18" s="9">
         <f>IF(L18="","",L18-J18)</f>
-        <v>-15173.08</v>
+        <v>-13741.93</v>
       </c>
       <c r="N18" s="10">
         <f>IF(OR(H18="",K18=""),"",K18/H18-1)</f>
-        <v>-0.15234504843064356</v>
+        <v>-0.13797561584871632</v>
       </c>
       <c r="O18" s="6">
         <f>IF(G18="","",$B$3-G18)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P18" s="6" t="str">
         <f>IF(H18="","Pending buy",IF(N18&gt;=0,"In profit","In loss"))</f>
@@ -1529,23 +1529,23 @@
         <v>99993.07</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>133.92</v>
+        <v>128.14</v>
       </c>
       <c r="L19" s="9">
         <f>IF(OR(I19="",K19=""),"",K19*I19)</f>
-        <v>88788.96</v>
+        <v>84956.82</v>
       </c>
       <c r="M19" s="9">
         <f>IF(L19="","",L19-J19)</f>
-        <v>-11204.11</v>
+        <v>-15036.25</v>
       </c>
       <c r="N19" s="10">
         <f>IF(OR(H19="",K19=""),"",K19/H19-1)</f>
-        <v>-0.11204882315206466</v>
+        <v>-0.150372880814707</v>
       </c>
       <c r="O19" s="6">
         <f>IF(G19="","",$B$3-G19)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P19" s="6" t="str">
         <f>IF(H19="","Pending buy",IF(N19&gt;=0,"In profit","In loss"))</f>
@@ -1597,23 +1597,23 @@
         <v>99896.43</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>193.59</v>
+        <v>193.7</v>
       </c>
       <c r="L20" s="9">
         <f>IF(OR(I20="",K20=""),"",K20*I20)</f>
-        <v>92342.43</v>
+        <v>92394.9</v>
       </c>
       <c r="M20" s="9">
         <f>IF(L20="","",L20-J20)</f>
-        <v>-7554.0</v>
+        <v>-7501.53</v>
       </c>
       <c r="N20" s="10">
         <f>IF(OR(H20="",K20=""),"",K20/H20-1)</f>
-        <v>-0.07561831794736096</v>
+        <v>-0.07509307395218678</v>
       </c>
       <c r="O20" s="6">
         <f>IF(G20="","",$B$3-G20)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P20" s="6" t="str">
         <f>IF(H20="","Pending buy",IF(N20&gt;=0,"In profit","In loss"))</f>
@@ -1665,23 +1665,23 @@
         <v>99449.47</v>
       </c>
       <c r="K21" s="9" t="n">
-        <v>1224.1</v>
+        <v>1202.6</v>
       </c>
       <c r="L21" s="9">
         <f>IF(OR(I21="",K21=""),"",K21*I21)</f>
-        <v>86911.1</v>
+        <v>85384.6</v>
       </c>
       <c r="M21" s="9">
         <f>IF(L21="","",L21-J21)</f>
-        <v>-12538.37</v>
+        <v>-14064.87</v>
       </c>
       <c r="N21" s="10">
         <f>IF(OR(H21="",K21=""),"",K21/H21-1)</f>
-        <v>-0.1260777639194126</v>
+        <v>-0.14142726810676054</v>
       </c>
       <c r="O21" s="6">
         <f>IF(G21="","",$B$3-G21)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P21" s="6" t="str">
         <f>IF(H21="","Pending buy",IF(N21&gt;=0,"In profit","In loss"))</f>
@@ -1733,23 +1733,23 @@
         <v>99837.05</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>635</v>
+        <v>603.25</v>
       </c>
       <c r="L22" s="9">
         <f>IF(OR(I22="",K22=""),"",K22*I22)</f>
-        <v>91440.0</v>
+        <v>86868.0</v>
       </c>
       <c r="M22" s="9">
         <f>IF(L22="","",L22-J22)</f>
-        <v>-8397.05</v>
+        <v>-12969.05</v>
       </c>
       <c r="N22" s="10">
         <f>IF(OR(H22="",K22=""),"",K22/H22-1)</f>
-        <v>-0.08410756353277193</v>
+        <v>-0.1299021853561334</v>
       </c>
       <c r="O22" s="6">
         <f>IF(G22="","",$B$3-G22)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P22" s="6" t="str">
         <f>IF(H22="","Pending buy",IF(N22&gt;=0,"In profit","In loss"))</f>
@@ -1801,23 +1801,23 @@
         <v>99486.88</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>591.6</v>
+        <v>589.1</v>
       </c>
       <c r="L23" s="9">
         <f>IF(OR(I23="",K23=""),"",K23*I23)</f>
-        <v>85782.0</v>
+        <v>85419.5</v>
       </c>
       <c r="M23" s="9">
         <f>IF(L23="","",L23-J23)</f>
-        <v>-13704.88</v>
+        <v>-14067.38</v>
       </c>
       <c r="N23" s="10">
         <f>IF(OR(H23="",K23=""),"",K23/H23-1)</f>
-        <v>-0.13775566211414758</v>
+        <v>-0.14139935860622777</v>
       </c>
       <c r="O23" s="6">
         <f>IF(G23="","",$B$3-G23)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P23" s="6" t="str">
         <f>IF(H23="","Pending buy",IF(N23&gt;=0,"In profit","In loss"))</f>
@@ -1869,23 +1869,23 @@
         <v>99935.4</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>211.53</v>
+        <v>209.91</v>
       </c>
       <c r="L24" s="9">
         <f>IF(OR(I24="",K24=""),"",K24*I24)</f>
-        <v>92861.67</v>
+        <v>92150.49</v>
       </c>
       <c r="M24" s="9">
         <f>IF(L24="","",L24-J24)</f>
-        <v>-7073.73</v>
+        <v>-7784.91</v>
       </c>
       <c r="N24" s="10">
         <f>IF(OR(H24="",K24=""),"",K24/H24-1)</f>
-        <v>-0.07078301284513666</v>
+        <v>-0.07789941013720347</v>
       </c>
       <c r="O24" s="6">
         <f>IF(G24="","",$B$3-G24)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P24" s="6" t="str">
         <f>IF(H24="","Pending buy",IF(N24&gt;=0,"In profit","In loss"))</f>
@@ -1937,23 +1937,23 @@
         <v>99622.64</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>717.55</v>
+        <v>727.7</v>
       </c>
       <c r="L25" s="9">
         <f>IF(OR(I25="",K25=""),"",K25*I25)</f>
-        <v>88976.2</v>
+        <v>90234.8</v>
       </c>
       <c r="M25" s="9">
         <f>IF(L25="","",L25-J25)</f>
-        <v>-10646.44</v>
+        <v>-9387.84</v>
       </c>
       <c r="N25" s="10">
         <f>IF(OR(H25="",K25=""),"",K25/H25-1)</f>
-        <v>-0.10686764351535416</v>
+        <v>-0.09423396862396094</v>
       </c>
       <c r="O25" s="6">
         <f>IF(G25="","",$B$3-G25)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P25" s="6" t="str">
         <f>IF(H25="","Pending buy",IF(N25&gt;=0,"In profit","In loss"))</f>
@@ -2005,23 +2005,23 @@
         <v>99948.17</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>171.42</v>
+        <v>176.37</v>
       </c>
       <c r="L26" s="9">
         <f>IF(OR(I26="",K26=""),"",K26*I26)</f>
-        <v>81424.5</v>
+        <v>83775.75</v>
       </c>
       <c r="M26" s="9">
         <f>IF(L26="","",L26-J26)</f>
-        <v>-18523.67</v>
+        <v>-16172.42</v>
       </c>
       <c r="N26" s="10">
         <f>IF(OR(H26="",K26=""),"",K26/H26-1)</f>
-        <v>-0.18533273086672153</v>
+        <v>-0.1618080372358165</v>
       </c>
       <c r="O26" s="6">
         <f>IF(G26="","",$B$3-G26)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P26" s="6" t="str">
         <f>IF(H26="","Pending buy",IF(N26&gt;=0,"In profit","In loss"))</f>
@@ -2073,23 +2073,23 @@
         <v>99745.27</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>236.75</v>
+        <v>231.15</v>
       </c>
       <c r="L27" s="9">
         <f>IF(OR(I27="",K27=""),"",K27*I27)</f>
-        <v>90438.5</v>
+        <v>88299.3</v>
       </c>
       <c r="M27" s="9">
         <f>IF(L27="","",L27-J27)</f>
-        <v>-9306.77</v>
+        <v>-11445.97</v>
       </c>
       <c r="N27" s="10">
         <f>IF(OR(H27="",K27=""),"",K27/H27-1)</f>
-        <v>-0.09330540369298712</v>
+        <v>-0.11475203405969991</v>
       </c>
       <c r="O27" s="6">
         <f>IF(G27="","",$B$3-G27)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P27" s="6" t="str">
         <f>IF(H27="","Pending buy",IF(N27&gt;=0,"In profit","In loss"))</f>
@@ -2141,23 +2141,23 @@
         <v>95334.84</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>10989</v>
+        <v>10998</v>
       </c>
       <c r="L28" s="9">
         <f>IF(OR(I28="",K28=""),"",K28*I28)</f>
-        <v>98901.0</v>
+        <v>98982.0</v>
       </c>
       <c r="M28" s="9">
         <f>IF(L28="","",L28-J28)</f>
-        <v>3566.16</v>
+        <v>3647.16</v>
       </c>
       <c r="N28" s="10">
         <f>IF(OR(H28="",K28=""),"",K28/H28-1)</f>
-        <v>0.03740665549392519</v>
+        <v>0.03825629239441164</v>
       </c>
       <c r="O28" s="6">
         <f>IF(G28="","",$B$3-G28)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P28" s="6" t="str">
         <f>IF(H28="","Pending buy",IF(N28&gt;=0,"In profit","In loss"))</f>
@@ -2209,23 +2209,23 @@
         <v>98598.59</v>
       </c>
       <c r="K29" s="9" t="n">
-        <v>1825.7</v>
+        <v>1818</v>
       </c>
       <c r="L29" s="9">
         <f>IF(OR(I29="",K29=""),"",K29*I29)</f>
-        <v>93110.7</v>
+        <v>92718.0</v>
       </c>
       <c r="M29" s="9">
         <f>IF(L29="","",L29-J29)</f>
-        <v>-5487.89</v>
+        <v>-5880.59</v>
       </c>
       <c r="N29" s="10">
         <f>IF(OR(H29="",K29=""),"",K29/H29-1)</f>
-        <v>-0.05565887373234457</v>
+        <v>-0.05964168945905812</v>
       </c>
       <c r="O29" s="6">
         <f>IF(G29="","",$B$3-G29)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P29" s="6" t="str">
         <f>IF(H29="","Pending buy",IF(N29&gt;=0,"In profit","In loss"))</f>
@@ -2277,23 +2277,23 @@
         <v>99998.69</v>
       </c>
       <c r="K30" s="9" t="n">
-        <v>16.66</v>
+        <v>16.33</v>
       </c>
       <c r="L30" s="9">
         <f>IF(OR(I30="",K30=""),"",K30*I30)</f>
-        <v>112338.38</v>
+        <v>110113.19</v>
       </c>
       <c r="M30" s="9">
         <f>IF(L30="","",L30-J30)</f>
-        <v>12339.69</v>
+        <v>10114.5</v>
       </c>
       <c r="N30" s="10">
         <f>IF(OR(H30="",K30=""),"",K30/H30-1)</f>
-        <v>0.12339851652056644</v>
+        <v>0.10114632501685761</v>
       </c>
       <c r="O30" s="6">
         <f>IF(G30="","",$B$3-G30)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P30" s="6" t="str">
         <f>IF(H30="","Pending buy",IF(N30&gt;=0,"In profit","In loss"))</f>
@@ -2345,23 +2345,23 @@
         <v>99977.34</v>
       </c>
       <c r="K31" s="9" t="n">
-        <v>161.24</v>
+        <v>158.57</v>
       </c>
       <c r="L31" s="9">
         <f>IF(OR(I31="",K31=""),"",K31*I31)</f>
-        <v>90939.36</v>
+        <v>89433.48</v>
       </c>
       <c r="M31" s="9">
         <f>IF(L31="","",L31-J31)</f>
-        <v>-9037.98</v>
+        <v>-10543.86</v>
       </c>
       <c r="N31" s="10">
         <f>IF(OR(H31="",K31=""),"",K31/H31-1)</f>
-        <v>-0.0904002681096544</v>
+        <v>-0.10546248148193949</v>
       </c>
       <c r="O31" s="6">
         <f>IF(G31="","",$B$3-G31)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P31" s="6" t="str">
         <f>IF(H31="","Pending buy",IF(N31&gt;=0,"In profit","In loss"))</f>
@@ -2413,23 +2413,23 @@
         <v>99923.82</v>
       </c>
       <c r="K32" s="9" t="n">
-        <v>169.68</v>
+        <v>168.78</v>
       </c>
       <c r="L32" s="9">
         <f>IF(OR(I32="",K32=""),"",K32*I32)</f>
-        <v>95869.2</v>
+        <v>95360.7</v>
       </c>
       <c r="M32" s="9">
         <f>IF(L32="","",L32-J32)</f>
-        <v>-4054.62</v>
+        <v>-4563.12</v>
       </c>
       <c r="N32" s="10">
         <f>IF(OR(H32="",K32=""),"",K32/H32-1)</f>
-        <v>-0.04057710847514073</v>
+        <v>-0.04566598519822174</v>
       </c>
       <c r="O32" s="6">
         <f>IF(G32="","",$B$3-G32)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P32" s="6" t="str">
         <f>IF(H32="","Pending buy",IF(N32&gt;=0,"In profit","In loss"))</f>
@@ -2481,27 +2481,27 @@
         <v>99608.58</v>
       </c>
       <c r="K33" s="9" t="n">
-        <v>530.15</v>
+        <v>515.15</v>
       </c>
       <c r="L33" s="9">
         <f>IF(OR(I33="",K33=""),"",K33*I33)</f>
-        <v>100198.35</v>
+        <v>97363.35</v>
       </c>
       <c r="M33" s="9">
         <f>IF(L33="","",L33-J33)</f>
-        <v>589.77</v>
+        <v>-2245.23</v>
       </c>
       <c r="N33" s="10">
         <f>IF(OR(H33="",K33=""),"",K33/H33-1)</f>
-        <v>0.005920924752488954</v>
+        <v>-0.02254048026738731</v>
       </c>
       <c r="O33" s="6">
         <f>IF(G33="","",$B$3-G33)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P33" s="6" t="str">
         <f>IF(H33="","Pending buy",IF(N33&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q33" s="6" t="n">
         <v>1</v>
@@ -2549,23 +2549,23 @@
         <v>96030.46</v>
       </c>
       <c r="K34" s="9" t="n">
-        <v>4594.1</v>
+        <v>4592.9</v>
       </c>
       <c r="L34" s="9">
         <f>IF(OR(I34="",K34=""),"",K34*I34)</f>
-        <v>87287.9</v>
+        <v>87265.1</v>
       </c>
       <c r="M34" s="9">
         <f>IF(L34="","",L34-J34)</f>
-        <v>-8742.56</v>
+        <v>-8765.36</v>
       </c>
       <c r="N34" s="10">
         <f>IF(OR(H34="",K34=""),"",K34/H34-1)</f>
-        <v>-0.09103945413774328</v>
+        <v>-0.09127687880308255</v>
       </c>
       <c r="O34" s="6">
         <f>IF(G34="","",$B$3-G34)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P34" s="6" t="str">
         <f>IF(H34="","Pending buy",IF(N34&gt;=0,"In profit","In loss"))</f>
@@ -2617,23 +2617,23 @@
         <v>99082.89</v>
       </c>
       <c r="K35" s="9" t="n">
-        <v>951.8</v>
+        <v>927.8</v>
       </c>
       <c r="L35" s="9">
         <f>IF(OR(I35="",K35=""),"",K35*I35)</f>
-        <v>86613.8</v>
+        <v>84429.8</v>
       </c>
       <c r="M35" s="9">
         <f>IF(L35="","",L35-J35)</f>
-        <v>-12469.09</v>
+        <v>-14653.09</v>
       </c>
       <c r="N35" s="10">
         <f>IF(OR(H35="",K35=""),"",K35/H35-1)</f>
-        <v>-0.12584506389009065</v>
+        <v>-0.1478872139916223</v>
       </c>
       <c r="O35" s="6">
         <f>IF(G35="","",$B$3-G35)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P35" s="6" t="str">
         <f>IF(H35="","Pending buy",IF(N35&gt;=0,"In profit","In loss"))</f>
@@ -2685,23 +2685,23 @@
         <v>99910.57</v>
       </c>
       <c r="K36" s="9" t="n">
-        <v>93.06</v>
+        <v>91.04000000000001</v>
       </c>
       <c r="L36" s="9">
         <f>IF(OR(I36="",K36=""),"",K36*I36)</f>
-        <v>95386.5</v>
+        <v>93316.0</v>
       </c>
       <c r="M36" s="9">
         <f>IF(L36="","",L36-J36)</f>
-        <v>-4524.07</v>
+        <v>-6594.57</v>
       </c>
       <c r="N36" s="10">
         <f>IF(OR(H36="",K36=""),"",K36/H36-1)</f>
-        <v>-0.045281206439544364</v>
+        <v>-0.06600473924625094</v>
       </c>
       <c r="O36" s="6">
         <f>IF(G36="","",$B$3-G36)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P36" s="6" t="str">
         <f>IF(H36="","Pending buy",IF(N36&gt;=0,"In profit","In loss"))</f>
@@ -2753,23 +2753,23 @@
         <v>99436.51</v>
       </c>
       <c r="K37" s="9" t="n">
-        <v>904.8</v>
+        <v>951.8</v>
       </c>
       <c r="L37" s="9">
         <f>IF(OR(I37="",K37=""),"",K37*I37)</f>
-        <v>90480.0</v>
+        <v>95180.0</v>
       </c>
       <c r="M37" s="9">
         <f>IF(L37="","",L37-J37)</f>
-        <v>-8956.51</v>
+        <v>-4256.51</v>
       </c>
       <c r="N37" s="10">
         <f>IF(OR(H37="",K37=""),"",K37/H37-1)</f>
-        <v>-0.09007267691504095</v>
+        <v>-0.04280633718803717</v>
       </c>
       <c r="O37" s="6">
         <f>IF(G37="","",$B$3-G37)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P37" s="6" t="str">
         <f>IF(H37="","Pending buy",IF(N37&gt;=0,"In profit","In loss"))</f>
@@ -2821,27 +2821,27 @@
         <v>99951.48</v>
       </c>
       <c r="K38" s="9" t="n">
-        <v>123.9</v>
+        <v>118.73</v>
       </c>
       <c r="L38" s="9">
         <f>IF(OR(I38="",K38=""),"",K38*I38)</f>
-        <v>101474.1</v>
+        <v>97239.87</v>
       </c>
       <c r="M38" s="9">
         <f>IF(L38="","",L38-J38)</f>
-        <v>1522.62</v>
+        <v>-2711.61</v>
       </c>
       <c r="N38" s="10">
         <f>IF(OR(H38="",K38=""),"",K38/H38-1)</f>
-        <v>0.015233592344086722</v>
+        <v>-0.02712926215485545</v>
       </c>
       <c r="O38" s="6">
         <f>IF(G38="","",$B$3-G38)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P38" s="6" t="str">
         <f>IF(H38="","Pending buy",IF(N38&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q38" s="6" t="n">
         <v>1</v>
@@ -2889,23 +2889,23 @@
         <v>99666.78</v>
       </c>
       <c r="K39" s="9" t="n">
-        <v>521.75</v>
+        <v>515.8</v>
       </c>
       <c r="L39" s="9">
         <f>IF(OR(I39="",K39=""),"",K39*I39)</f>
-        <v>93393.25</v>
+        <v>92328.2</v>
       </c>
       <c r="M39" s="9">
         <f>IF(L39="","",L39-J39)</f>
-        <v>-6273.53</v>
+        <v>-7338.58</v>
       </c>
       <c r="N39" s="10">
         <f>IF(OR(H39="",K39=""),"",K39/H39-1)</f>
-        <v>-0.06294500907647538</v>
+        <v>-0.0736311177415353</v>
       </c>
       <c r="O39" s="6">
         <f>IF(G39="","",$B$3-G39)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P39" s="6" t="str">
         <f>IF(H39="","Pending buy",IF(N39&gt;=0,"In profit","In loss"))</f>
@@ -2957,23 +2957,23 @@
         <v>99998.64</v>
       </c>
       <c r="K40" s="9" t="n">
-        <v>11.67</v>
+        <v>11.4</v>
       </c>
       <c r="L40" s="9">
         <f>IF(OR(I40="",K40=""),"",K40*I40)</f>
-        <v>90069.06</v>
+        <v>87985.2</v>
       </c>
       <c r="M40" s="9">
         <f>IF(L40="","",L40-J40)</f>
-        <v>-9929.58</v>
+        <v>-12013.44</v>
       </c>
       <c r="N40" s="10">
         <f>IF(OR(H40="",K40=""),"",K40/H40-1)</f>
-        <v>-0.09929712759911047</v>
+        <v>-0.12013601153640607</v>
       </c>
       <c r="O40" s="6">
         <f>IF(G40="","",$B$3-G40)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P40" s="6" t="str">
         <f>IF(H40="","Pending buy",IF(N40&gt;=0,"In profit","In loss"))</f>
@@ -3025,23 +3025,23 @@
         <v>99889.82</v>
       </c>
       <c r="K41" s="9" t="n">
-        <v>123.66</v>
+        <v>116.94</v>
       </c>
       <c r="L41" s="9">
         <f>IF(OR(I41="",K41=""),"",K41*I41)</f>
-        <v>98309.7</v>
+        <v>92967.3</v>
       </c>
       <c r="M41" s="9">
         <f>IF(L41="","",L41-J41)</f>
-        <v>-1580.12</v>
+        <v>-6922.52</v>
       </c>
       <c r="N41" s="10">
         <f>IF(OR(H41="",K41=""),"",K41/H41-1)</f>
-        <v>-0.01581861857082778</v>
+        <v>-0.06930154662520294</v>
       </c>
       <c r="O41" s="6">
         <f>IF(G41="","",$B$3-G41)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P41" s="6" t="str">
         <f>IF(H41="","Pending buy",IF(N41&gt;=0,"In profit","In loss"))</f>
@@ -3093,23 +3093,23 @@
         <v>99925.2</v>
       </c>
       <c r="K42" s="9" t="n">
-        <v>94.17</v>
+        <v>99.31</v>
       </c>
       <c r="L42" s="9">
         <f>IF(OR(I42="",K42=""),"",K42*I42)</f>
-        <v>100102.71</v>
+        <v>105566.53</v>
       </c>
       <c r="M42" s="9">
         <f>IF(L42="","",L42-J42)</f>
-        <v>177.51</v>
+        <v>5641.33</v>
       </c>
       <c r="N42" s="10">
         <f>IF(OR(H42="",K42=""),"",K42/H42-1)</f>
-        <v>0.0017764431349212018</v>
+        <v>0.056455543885834514</v>
       </c>
       <c r="O42" s="6">
         <f>IF(G42="","",$B$3-G42)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P42" s="6" t="str">
         <f>IF(H42="","Pending buy",IF(N42&gt;=0,"In profit","In loss"))</f>
@@ -3119,8 +3119,392 @@
         <v>2</v>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Bliss GVS Pharma Limited</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>BLISSGVS</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>221026</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="G43" s="6" t="inlineStr"/>
+      <c r="H43" s="9" t="inlineStr"/>
+      <c r="I43" s="6" t="str">
+        <f>IF(H43="","",ROUNDDOWN($B$1/H43,0))</f>
+        <v/>
+      </c>
+      <c r="J43" s="9" t="str">
+        <f>IF(H43="","",H43*I43)</f>
+        <v/>
+      </c>
+      <c r="K43" s="9" t="n">
+        <v>642.7</v>
+      </c>
+      <c r="L43" s="9" t="str">
+        <f>IF(OR(I43="",K43=""),"",K43*I43)</f>
+        <v/>
+      </c>
+      <c r="M43" s="9" t="str">
+        <f>IF(L43="","",L43-J43)</f>
+        <v/>
+      </c>
+      <c r="N43" s="10" t="str">
+        <f>IF(OR(H43="",K43=""),"",K43/H43-1)</f>
+        <v/>
+      </c>
+      <c r="O43" s="6" t="str">
+        <f>IF(G43="","",$B$3-G43)</f>
+        <v/>
+      </c>
+      <c r="P43" s="6" t="str">
+        <f>IF(H43="","Pending buy",IF(N43&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q43" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Ind-Swift Laboratories Limited</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>INDSWFTLAB</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>221026</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="G44" s="6" t="inlineStr"/>
+      <c r="H44" s="9" t="inlineStr"/>
+      <c r="I44" s="6" t="str">
+        <f>IF(H44="","",ROUNDDOWN($B$1/H44,0))</f>
+        <v/>
+      </c>
+      <c r="J44" s="9" t="str">
+        <f>IF(H44="","",H44*I44)</f>
+        <v/>
+      </c>
+      <c r="K44" s="9" t="n">
+        <v>345.35</v>
+      </c>
+      <c r="L44" s="9" t="str">
+        <f>IF(OR(I44="",K44=""),"",K44*I44)</f>
+        <v/>
+      </c>
+      <c r="M44" s="9" t="str">
+        <f>IF(L44="","",L44-J44)</f>
+        <v/>
+      </c>
+      <c r="N44" s="10" t="str">
+        <f>IF(OR(H44="",K44=""),"",K44/H44-1)</f>
+        <v/>
+      </c>
+      <c r="O44" s="6" t="str">
+        <f>IF(G44="","",$B$3-G44)</f>
+        <v/>
+      </c>
+      <c r="P44" s="6" t="str">
+        <f>IF(H44="","Pending buy",IF(N44&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q44" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Menon Bearings Limited</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>MENONBE</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>221026</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="G45" s="6" t="inlineStr"/>
+      <c r="H45" s="9" t="inlineStr"/>
+      <c r="I45" s="6" t="str">
+        <f>IF(H45="","",ROUNDDOWN($B$1/H45,0))</f>
+        <v/>
+      </c>
+      <c r="J45" s="9" t="str">
+        <f>IF(H45="","",H45*I45)</f>
+        <v/>
+      </c>
+      <c r="K45" s="9" t="n">
+        <v>270.15</v>
+      </c>
+      <c r="L45" s="9" t="str">
+        <f>IF(OR(I45="",K45=""),"",K45*I45)</f>
+        <v/>
+      </c>
+      <c r="M45" s="9" t="str">
+        <f>IF(L45="","",L45-J45)</f>
+        <v/>
+      </c>
+      <c r="N45" s="10" t="str">
+        <f>IF(OR(H45="",K45=""),"",K45/H45-1)</f>
+        <v/>
+      </c>
+      <c r="O45" s="6" t="str">
+        <f>IF(G45="","",$B$3-G45)</f>
+        <v/>
+      </c>
+      <c r="P45" s="6" t="str">
+        <f>IF(H45="","Pending buy",IF(N45&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q45" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Redington Limited</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>REDINGTON</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>221026</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="G46" s="6" t="inlineStr"/>
+      <c r="H46" s="9" t="inlineStr"/>
+      <c r="I46" s="6" t="str">
+        <f>IF(H46="","",ROUNDDOWN($B$1/H46,0))</f>
+        <v/>
+      </c>
+      <c r="J46" s="9" t="str">
+        <f>IF(H46="","",H46*I46)</f>
+        <v/>
+      </c>
+      <c r="K46" s="9" t="n">
+        <v>367.1</v>
+      </c>
+      <c r="L46" s="9" t="str">
+        <f>IF(OR(I46="",K46=""),"",K46*I46)</f>
+        <v/>
+      </c>
+      <c r="M46" s="9" t="str">
+        <f>IF(L46="","",L46-J46)</f>
+        <v/>
+      </c>
+      <c r="N46" s="10" t="str">
+        <f>IF(OR(H46="",K46=""),"",K46/H46-1)</f>
+        <v/>
+      </c>
+      <c r="O46" s="6" t="str">
+        <f>IF(G46="","",$B$3-G46)</f>
+        <v/>
+      </c>
+      <c r="P46" s="6" t="str">
+        <f>IF(H46="","Pending buy",IF(N46&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q46" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Sheetal Cool Products Limited</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>SCPL</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>221026</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="G47" s="6" t="inlineStr"/>
+      <c r="H47" s="9" t="inlineStr"/>
+      <c r="I47" s="6" t="str">
+        <f>IF(H47="","",ROUNDDOWN($B$1/H47,0))</f>
+        <v/>
+      </c>
+      <c r="J47" s="9" t="str">
+        <f>IF(H47="","",H47*I47)</f>
+        <v/>
+      </c>
+      <c r="K47" s="9" t="n">
+        <v>592.35</v>
+      </c>
+      <c r="L47" s="9" t="str">
+        <f>IF(OR(I47="",K47=""),"",K47*I47)</f>
+        <v/>
+      </c>
+      <c r="M47" s="9" t="str">
+        <f>IF(L47="","",L47-J47)</f>
+        <v/>
+      </c>
+      <c r="N47" s="10" t="str">
+        <f>IF(OR(H47="",K47=""),"",K47/H47-1)</f>
+        <v/>
+      </c>
+      <c r="O47" s="6" t="str">
+        <f>IF(G47="","",$B$3-G47)</f>
+        <v/>
+      </c>
+      <c r="P47" s="6" t="str">
+        <f>IF(H47="","Pending buy",IF(N47&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q47" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Union Bank of India</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>UNIONBANK</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>221026</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="G48" s="6" t="inlineStr"/>
+      <c r="H48" s="9" t="inlineStr"/>
+      <c r="I48" s="6" t="str">
+        <f>IF(H48="","",ROUNDDOWN($B$1/H48,0))</f>
+        <v/>
+      </c>
+      <c r="J48" s="9" t="str">
+        <f>IF(H48="","",H48*I48)</f>
+        <v/>
+      </c>
+      <c r="K48" s="9" t="n">
+        <v>182.85</v>
+      </c>
+      <c r="L48" s="9" t="str">
+        <f>IF(OR(I48="",K48=""),"",K48*I48)</f>
+        <v/>
+      </c>
+      <c r="M48" s="9" t="str">
+        <f>IF(L48="","",L48-J48)</f>
+        <v/>
+      </c>
+      <c r="N48" s="10" t="str">
+        <f>IF(OR(H48="",K48=""),"",K48/H48-1)</f>
+        <v/>
+      </c>
+      <c r="O48" s="6" t="str">
+        <f>IF(G48="","",$B$3-G48)</f>
+        <v/>
+      </c>
+      <c r="P48" s="6" t="str">
+        <f>IF(H48="","Pending buy",IF(N48&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q48" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A8:Q42">
+  <conditionalFormatting sqref="A8:Q48">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$N8&gt;0</formula>
     </cfRule>
@@ -3138,7 +3522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4006,6 +4390,126 @@
       <c r="D43" s="11" t="inlineStr">
         <is>
           <t>HALEOS LABS LIMITED</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>UNIONBANK</t>
+        </is>
+      </c>
+      <c r="D44" s="11" t="inlineStr">
+        <is>
+          <t>Union Bank of India</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>BLISSGVS</t>
+        </is>
+      </c>
+      <c r="D45" s="11" t="inlineStr">
+        <is>
+          <t>Bliss GVS Pharma Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>INDSWFTLAB</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="inlineStr">
+        <is>
+          <t>Ind-Swift Laboratories Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>MENONBE</t>
+        </is>
+      </c>
+      <c r="D47" s="11" t="inlineStr">
+        <is>
+          <t>Menon Bearings Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>REDINGTON</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="inlineStr">
+        <is>
+          <t>Redington Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>SCPL</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="inlineStr">
+        <is>
+          <t>Sheetal Cool Products Limited</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum Portfolio: Friday report 2026-10-23
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="E1" s="2">
         <f>SUM(J8:J48)</f>
-        <v>3463650.69</v>
+        <v>4062646.89</v>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
@@ -541,7 +541,7 @@
       </c>
       <c r="G1" s="2">
         <f>SUM(L8:L48)</f>
-        <v>3201499.22</v>
+        <v>3709129.13</v>
       </c>
     </row>
     <row r="2">
@@ -552,7 +552,7 @@
       </c>
       <c r="E2" s="2">
         <f>SUM(M8:M48)</f>
-        <v>-262151.47</v>
+        <v>-353517.76</v>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" s="3">
         <f>IF(E1=0,"",G1/E1-1)</f>
-        <v>-0.07568646305958748</v>
+        <v>-0.08701661000126948</v>
       </c>
     </row>
     <row r="3">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -580,7 +580,7 @@
       </c>
       <c r="E3">
         <f>COUNTIF(M8:M48,"&gt;0")</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
@@ -589,7 +589,7 @@
       </c>
       <c r="G3">
         <f>COUNTIF(M8:M48,"&lt;0")</f>
-        <v>30</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4">
@@ -600,7 +600,7 @@
       </c>
       <c r="E4" s="3">
         <f>IF((E3+G3)=0,"",E3/(E3+G3))</f>
-        <v>0.14285714285714285</v>
+        <v>0.04878048780487805</v>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
@@ -609,7 +609,7 @@
       </c>
       <c r="G4" s="3">
         <f>AVERAGE(N8:N48)</f>
-        <v>-0.07574536961562824</v>
+        <v>-0.08714148760251178</v>
       </c>
     </row>
     <row r="5">
@@ -620,7 +620,7 @@
       </c>
       <c r="E5" t="str">
         <f>INDEX(B8:B48,MATCH(MAX(N8:N48),N8:N48,0))</f>
-        <v>Viji Finance Limited</v>
+        <v>Pashupati Cotspin Limited</v>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
@@ -640,7 +640,7 @@
       </c>
       <c r="E6" s="3">
         <f>AVERAGEIF(D8:D48,"4★*",N8:N48)</f>
-        <v>-0.08912510970554093</v>
+        <v>-0.11065143816567073</v>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
@@ -649,7 +649,7 @@
       </c>
       <c r="G6" s="3">
         <f>AVERAGEIF(D8:D48,"5★*",N8:N48)</f>
-        <v>-0.06157858599101481</v>
+        <v>-0.0668374393888745</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
@@ -781,23 +781,23 @@
         <v>99851.29</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>271.3</v>
+        <v>267.75</v>
       </c>
       <c r="L8" s="9">
         <f>IF(OR(I8="",K8=""),"",K8*I8)</f>
-        <v>90071.6</v>
+        <v>88893.0</v>
       </c>
       <c r="M8" s="9">
         <f>IF(L8="","",L8-J8)</f>
-        <v>-9779.69</v>
+        <v>-10958.29</v>
       </c>
       <c r="N8" s="10">
         <f>IF(OR(H8="",K8=""),"",K8/H8-1)</f>
-        <v>-0.09794258158818414</v>
+        <v>-0.10974613424340696</v>
       </c>
       <c r="O8" s="6">
         <f>IF(G8="","",$B$3-G8)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="P8" s="6" t="str">
         <f>IF(H8="","Pending buy",IF(N8&gt;=0,"In profit","In loss"))</f>
@@ -849,23 +849,23 @@
         <v>99687.42</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>304.45</v>
+        <v>317.4</v>
       </c>
       <c r="L9" s="9">
         <f>IF(OR(I9="",K9=""),"",K9*I9)</f>
-        <v>93161.7</v>
+        <v>97124.4</v>
       </c>
       <c r="M9" s="9">
         <f>IF(L9="","",L9-J9)</f>
-        <v>-6525.72</v>
+        <v>-2563.02</v>
       </c>
       <c r="N9" s="10">
         <f>IF(OR(H9="",K9=""),"",K9/H9-1)</f>
-        <v>-0.06546182241489018</v>
+        <v>-0.025710568022618285</v>
       </c>
       <c r="O9" s="6">
         <f>IF(G9="","",$B$3-G9)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P9" s="6" t="str">
         <f>IF(H9="","Pending buy",IF(N9&gt;=0,"In profit","In loss"))</f>
@@ -917,27 +917,27 @@
         <v>99607.14</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>1611.3</v>
+        <v>1498.5</v>
       </c>
       <c r="L10" s="9">
         <f>IF(OR(I10="",K10=""),"",K10*I10)</f>
-        <v>101511.9</v>
+        <v>94405.5</v>
       </c>
       <c r="M10" s="9">
         <f>IF(L10="","",L10-J10)</f>
-        <v>1904.76</v>
+        <v>-5201.64</v>
       </c>
       <c r="N10" s="10">
         <f>IF(OR(H10="",K10=""),"",K10/H10-1)</f>
-        <v>0.019122716055026245</v>
+        <v>-0.05222156643178999</v>
       </c>
       <c r="O10" s="6">
         <f>IF(G10="","",$B$3-G10)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P10" s="6" t="str">
         <f>IF(H10="","Pending buy",IF(N10&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q10" s="6" t="n">
         <v>2</v>
@@ -985,23 +985,23 @@
         <v>99927.23</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>63.74</v>
+        <v>62.36</v>
       </c>
       <c r="L11" s="9">
         <f>IF(OR(I11="",K11=""),"",K11*I11)</f>
-        <v>79738.74</v>
+        <v>78012.36</v>
       </c>
       <c r="M11" s="9">
         <f>IF(L11="","",L11-J11)</f>
-        <v>-20188.49</v>
+        <v>-21914.87</v>
       </c>
       <c r="N11" s="10">
         <f>IF(OR(H11="",K11=""),"",K11/H11-1)</f>
-        <v>-0.20203192167764283</v>
+        <v>-0.21930829362751503</v>
       </c>
       <c r="O11" s="6">
         <f>IF(G11="","",$B$3-G11)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P11" s="6" t="str">
         <f>IF(H11="","Pending buy",IF(N11&gt;=0,"In profit","In loss"))</f>
@@ -1053,23 +1053,23 @@
         <v>86537.12</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>18935</v>
+        <v>18865</v>
       </c>
       <c r="L12" s="9">
         <f>IF(OR(I12="",K12=""),"",K12*I12)</f>
-        <v>75740.0</v>
+        <v>75460.0</v>
       </c>
       <c r="M12" s="9">
         <f>IF(L12="","",L12-J12)</f>
-        <v>-10797.12</v>
+        <v>-11077.12</v>
       </c>
       <c r="N12" s="10">
         <f>IF(OR(H12="",K12=""),"",K12/H12-1)</f>
-        <v>-0.12476861515158877</v>
+        <v>-0.12800422101054776</v>
       </c>
       <c r="O12" s="6">
         <f>IF(G12="","",$B$3-G12)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P12" s="6" t="str">
         <f>IF(H12="","Pending buy",IF(N12&gt;=0,"In profit","In loss"))</f>
@@ -1121,23 +1121,23 @@
         <v>98177.53</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>1669.5</v>
+        <v>1661.9</v>
       </c>
       <c r="L13" s="9">
         <f>IF(OR(I13="",K13=""),"",K13*I13)</f>
-        <v>88483.5</v>
+        <v>88080.7</v>
       </c>
       <c r="M13" s="9">
         <f>IF(L13="","",L13-J13)</f>
-        <v>-9694.03</v>
+        <v>-10096.83</v>
       </c>
       <c r="N13" s="10">
         <f>IF(OR(H13="",K13=""),"",K13/H13-1)</f>
-        <v>-0.09873983228320782</v>
+        <v>-0.10284260393618627</v>
       </c>
       <c r="O13" s="6">
         <f>IF(G13="","",$B$3-G13)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P13" s="6" t="str">
         <f>IF(H13="","Pending buy",IF(N13&gt;=0,"In profit","In loss"))</f>
@@ -1189,23 +1189,23 @@
         <v>97667.46</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>4201.3</v>
+        <v>4157.3</v>
       </c>
       <c r="L14" s="9">
         <f>IF(OR(I14="",K14=""),"",K14*I14)</f>
-        <v>92428.6</v>
+        <v>91460.6</v>
       </c>
       <c r="M14" s="9">
         <f>IF(L14="","",L14-J14)</f>
-        <v>-5238.86</v>
+        <v>-6206.86</v>
       </c>
       <c r="N14" s="10">
         <f>IF(OR(H14="",K14=""),"",K14/H14-1)</f>
-        <v>-0.053639809572047725</v>
+        <v>-0.06355099143928644</v>
       </c>
       <c r="O14" s="6">
         <f>IF(G14="","",$B$3-G14)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P14" s="6" t="str">
         <f>IF(H14="","Pending buy",IF(N14&gt;=0,"In profit","In loss"))</f>
@@ -1257,23 +1257,23 @@
         <v>99078.19</v>
       </c>
       <c r="K15" s="9" t="n">
-        <v>1345</v>
+        <v>1295.3</v>
       </c>
       <c r="L15" s="9">
         <f>IF(OR(I15="",K15=""),"",K15*I15)</f>
-        <v>86080.0</v>
+        <v>82899.2</v>
       </c>
       <c r="M15" s="9">
         <f>IF(L15="","",L15-J15)</f>
-        <v>-12998.19</v>
+        <v>-16178.99</v>
       </c>
       <c r="N15" s="10">
         <f>IF(OR(H15="",K15=""),"",K15/H15-1)</f>
-        <v>-0.13119121272762424</v>
+        <v>-0.16329515081493806</v>
       </c>
       <c r="O15" s="6">
         <f>IF(G15="","",$B$3-G15)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P15" s="6" t="str">
         <f>IF(H15="","Pending buy",IF(N15&gt;=0,"In profit","In loss"))</f>
@@ -1325,23 +1325,23 @@
         <v>98557.54</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>1425.3</v>
+        <v>1380</v>
       </c>
       <c r="L16" s="9">
         <f>IF(OR(I16="",K16=""),"",K16*I16)</f>
-        <v>96920.4</v>
+        <v>93840.0</v>
       </c>
       <c r="M16" s="9">
         <f>IF(L16="","",L16-J16)</f>
-        <v>-1637.14</v>
+        <v>-4717.54</v>
       </c>
       <c r="N16" s="10">
         <f>IF(OR(H16="",K16=""),"",K16/H16-1)</f>
-        <v>-0.016610972370785904</v>
+        <v>-0.0478658120197043</v>
       </c>
       <c r="O16" s="6">
         <f>IF(G16="","",$B$3-G16)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P16" s="6" t="str">
         <f>IF(H16="","Pending buy",IF(N16&gt;=0,"In profit","In loss"))</f>
@@ -1393,27 +1393,27 @@
         <v>99714.35</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>885</v>
+        <v>805.1</v>
       </c>
       <c r="L17" s="9">
         <f>IF(OR(I17="",K17=""),"",K17*I17)</f>
-        <v>101775.0</v>
+        <v>92586.5</v>
       </c>
       <c r="M17" s="9">
         <f>IF(L17="","",L17-J17)</f>
-        <v>2060.65</v>
+        <v>-7127.85</v>
       </c>
       <c r="N17" s="10">
         <f>IF(OR(H17="",K17=""),"",K17/H17-1)</f>
-        <v>0.020665530321865244</v>
+        <v>-0.07148269100323879</v>
       </c>
       <c r="O17" s="6">
         <f>IF(G17="","",$B$3-G17)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P17" s="6" t="str">
         <f>IF(H17="","Pending buy",IF(N17&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q17" s="6" t="n">
         <v>1</v>
@@ -1461,23 +1461,23 @@
         <v>99596.83</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>608.9</v>
+        <v>589.75</v>
       </c>
       <c r="L18" s="9">
         <f>IF(OR(I18="",K18=""),"",K18*I18)</f>
-        <v>85854.9</v>
+        <v>83154.75</v>
       </c>
       <c r="M18" s="9">
         <f>IF(L18="","",L18-J18)</f>
-        <v>-13741.93</v>
+        <v>-16442.08</v>
       </c>
       <c r="N18" s="10">
         <f>IF(OR(H18="",K18=""),"",K18/H18-1)</f>
-        <v>-0.13797561584871632</v>
+        <v>-0.16508641722250028</v>
       </c>
       <c r="O18" s="6">
         <f>IF(G18="","",$B$3-G18)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P18" s="6" t="str">
         <f>IF(H18="","Pending buy",IF(N18&gt;=0,"In profit","In loss"))</f>
@@ -1529,23 +1529,23 @@
         <v>99993.07</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>128.14</v>
+        <v>123.16</v>
       </c>
       <c r="L19" s="9">
         <f>IF(OR(I19="",K19=""),"",K19*I19)</f>
-        <v>84956.82</v>
+        <v>81655.08</v>
       </c>
       <c r="M19" s="9">
         <f>IF(L19="","",L19-J19)</f>
-        <v>-15036.25</v>
+        <v>-18337.99</v>
       </c>
       <c r="N19" s="10">
         <f>IF(OR(H19="",K19=""),"",K19/H19-1)</f>
-        <v>-0.150372880814707</v>
+        <v>-0.1833925706347691</v>
       </c>
       <c r="O19" s="6">
         <f>IF(G19="","",$B$3-G19)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P19" s="6" t="str">
         <f>IF(H19="","Pending buy",IF(N19&gt;=0,"In profit","In loss"))</f>
@@ -1597,23 +1597,23 @@
         <v>99896.43</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>193.7</v>
+        <v>185.49</v>
       </c>
       <c r="L20" s="9">
         <f>IF(OR(I20="",K20=""),"",K20*I20)</f>
-        <v>92394.9</v>
+        <v>88478.73</v>
       </c>
       <c r="M20" s="9">
         <f>IF(L20="","",L20-J20)</f>
-        <v>-7501.53</v>
+        <v>-11417.7</v>
       </c>
       <c r="N20" s="10">
         <f>IF(OR(H20="",K20=""),"",K20/H20-1)</f>
-        <v>-0.07509307395218678</v>
+        <v>-0.1142953757738312</v>
       </c>
       <c r="O20" s="6">
         <f>IF(G20="","",$B$3-G20)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P20" s="6" t="str">
         <f>IF(H20="","Pending buy",IF(N20&gt;=0,"In profit","In loss"))</f>
@@ -1665,23 +1665,23 @@
         <v>99449.47</v>
       </c>
       <c r="K21" s="9" t="n">
-        <v>1202.6</v>
+        <v>1215.3</v>
       </c>
       <c r="L21" s="9">
         <f>IF(OR(I21="",K21=""),"",K21*I21)</f>
-        <v>85384.6</v>
+        <v>86286.3</v>
       </c>
       <c r="M21" s="9">
         <f>IF(L21="","",L21-J21)</f>
-        <v>-14064.87</v>
+        <v>-13163.17</v>
       </c>
       <c r="N21" s="10">
         <f>IF(OR(H21="",K21=""),"",K21/H21-1)</f>
-        <v>-0.14142726810676054</v>
+        <v>-0.1323603516798154</v>
       </c>
       <c r="O21" s="6">
         <f>IF(G21="","",$B$3-G21)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P21" s="6" t="str">
         <f>IF(H21="","Pending buy",IF(N21&gt;=0,"In profit","In loss"))</f>
@@ -1733,23 +1733,23 @@
         <v>99837.05</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>603.25</v>
+        <v>604.25</v>
       </c>
       <c r="L22" s="9">
         <f>IF(OR(I22="",K22=""),"",K22*I22)</f>
-        <v>86868.0</v>
+        <v>87012.0</v>
       </c>
       <c r="M22" s="9">
         <f>IF(L22="","",L22-J22)</f>
-        <v>-12969.05</v>
+        <v>-12825.05</v>
       </c>
       <c r="N22" s="10">
         <f>IF(OR(H22="",K22=""),"",K22/H22-1)</f>
-        <v>-0.1299021853561334</v>
+        <v>-0.12845983506248415</v>
       </c>
       <c r="O22" s="6">
         <f>IF(G22="","",$B$3-G22)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P22" s="6" t="str">
         <f>IF(H22="","Pending buy",IF(N22&gt;=0,"In profit","In loss"))</f>
@@ -1801,23 +1801,23 @@
         <v>99486.88</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>589.1</v>
+        <v>566.25</v>
       </c>
       <c r="L23" s="9">
         <f>IF(OR(I23="",K23=""),"",K23*I23)</f>
-        <v>85419.5</v>
+        <v>82106.25</v>
       </c>
       <c r="M23" s="9">
         <f>IF(L23="","",L23-J23)</f>
-        <v>-14067.38</v>
+        <v>-17380.63</v>
       </c>
       <c r="N23" s="10">
         <f>IF(OR(H23="",K23=""),"",K23/H23-1)</f>
-        <v>-0.14139935860622777</v>
+        <v>-0.1747027445438406</v>
       </c>
       <c r="O23" s="6">
         <f>IF(G23="","",$B$3-G23)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P23" s="6" t="str">
         <f>IF(H23="","Pending buy",IF(N23&gt;=0,"In profit","In loss"))</f>
@@ -1869,23 +1869,23 @@
         <v>99935.4</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>209.91</v>
+        <v>205.51</v>
       </c>
       <c r="L24" s="9">
         <f>IF(OR(I24="",K24=""),"",K24*I24)</f>
-        <v>92150.49</v>
+        <v>90218.89</v>
       </c>
       <c r="M24" s="9">
         <f>IF(L24="","",L24-J24)</f>
-        <v>-7784.91</v>
+        <v>-9716.51</v>
       </c>
       <c r="N24" s="10">
         <f>IF(OR(H24="",K24=""),"",K24/H24-1)</f>
-        <v>-0.07789941013720347</v>
+        <v>-0.0972278966094835</v>
       </c>
       <c r="O24" s="6">
         <f>IF(G24="","",$B$3-G24)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P24" s="6" t="str">
         <f>IF(H24="","Pending buy",IF(N24&gt;=0,"In profit","In loss"))</f>
@@ -1937,23 +1937,23 @@
         <v>99622.64</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>727.7</v>
+        <v>703.6</v>
       </c>
       <c r="L25" s="9">
         <f>IF(OR(I25="",K25=""),"",K25*I25)</f>
-        <v>90234.8</v>
+        <v>87246.4</v>
       </c>
       <c r="M25" s="9">
         <f>IF(L25="","",L25-J25)</f>
-        <v>-9387.84</v>
+        <v>-12376.24</v>
       </c>
       <c r="N25" s="10">
         <f>IF(OR(H25="",K25=""),"",K25/H25-1)</f>
-        <v>-0.09423396862396094</v>
+        <v>-0.1242311671345595</v>
       </c>
       <c r="O25" s="6">
         <f>IF(G25="","",$B$3-G25)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P25" s="6" t="str">
         <f>IF(H25="","Pending buy",IF(N25&gt;=0,"In profit","In loss"))</f>
@@ -2005,23 +2005,23 @@
         <v>99948.17</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>176.37</v>
+        <v>170.77</v>
       </c>
       <c r="L26" s="9">
         <f>IF(OR(I26="",K26=""),"",K26*I26)</f>
-        <v>83775.75</v>
+        <v>81115.75</v>
       </c>
       <c r="M26" s="9">
         <f>IF(L26="","",L26-J26)</f>
-        <v>-16172.42</v>
+        <v>-18832.42</v>
       </c>
       <c r="N26" s="10">
         <f>IF(OR(H26="",K26=""),"",K26/H26-1)</f>
-        <v>-0.1618080372358165</v>
+        <v>-0.18842183205057772</v>
       </c>
       <c r="O26" s="6">
         <f>IF(G26="","",$B$3-G26)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P26" s="6" t="str">
         <f>IF(H26="","Pending buy",IF(N26&gt;=0,"In profit","In loss"))</f>
@@ -2073,23 +2073,23 @@
         <v>99745.27</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>231.15</v>
+        <v>210</v>
       </c>
       <c r="L27" s="9">
         <f>IF(OR(I27="",K27=""),"",K27*I27)</f>
-        <v>88299.3</v>
+        <v>80220.0</v>
       </c>
       <c r="M27" s="9">
         <f>IF(L27="","",L27-J27)</f>
-        <v>-11445.97</v>
+        <v>-19525.27</v>
       </c>
       <c r="N27" s="10">
         <f>IF(OR(H27="",K27=""),"",K27/H27-1)</f>
-        <v>-0.11475203405969991</v>
+        <v>-0.1957513612482673</v>
       </c>
       <c r="O27" s="6">
         <f>IF(G27="","",$B$3-G27)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P27" s="6" t="str">
         <f>IF(H27="","Pending buy",IF(N27&gt;=0,"In profit","In loss"))</f>
@@ -2141,27 +2141,27 @@
         <v>95334.84</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>10998</v>
+        <v>10488</v>
       </c>
       <c r="L28" s="9">
         <f>IF(OR(I28="",K28=""),"",K28*I28)</f>
-        <v>98982.0</v>
+        <v>94392.0</v>
       </c>
       <c r="M28" s="9">
         <f>IF(L28="","",L28-J28)</f>
-        <v>3647.16</v>
+        <v>-942.84</v>
       </c>
       <c r="N28" s="10">
         <f>IF(OR(H28="",K28=""),"",K28/H28-1)</f>
-        <v>0.03825629239441164</v>
+        <v>-0.009889798633152536</v>
       </c>
       <c r="O28" s="6">
         <f>IF(G28="","",$B$3-G28)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P28" s="6" t="str">
         <f>IF(H28="","Pending buy",IF(N28&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q28" s="6" t="n">
         <v>1</v>
@@ -2209,23 +2209,23 @@
         <v>98598.59</v>
       </c>
       <c r="K29" s="9" t="n">
-        <v>1818</v>
+        <v>1762</v>
       </c>
       <c r="L29" s="9">
         <f>IF(OR(I29="",K29=""),"",K29*I29)</f>
-        <v>92718.0</v>
+        <v>89862.0</v>
       </c>
       <c r="M29" s="9">
         <f>IF(L29="","",L29-J29)</f>
-        <v>-5880.59</v>
+        <v>-8736.59</v>
       </c>
       <c r="N29" s="10">
         <f>IF(OR(H29="",K29=""),"",K29/H29-1)</f>
-        <v>-0.05964168945905812</v>
+        <v>-0.08860762201697492</v>
       </c>
       <c r="O29" s="6">
         <f>IF(G29="","",$B$3-G29)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P29" s="6" t="str">
         <f>IF(H29="","Pending buy",IF(N29&gt;=0,"In profit","In loss"))</f>
@@ -2277,23 +2277,23 @@
         <v>99998.69</v>
       </c>
       <c r="K30" s="9" t="n">
-        <v>16.33</v>
+        <v>16.01</v>
       </c>
       <c r="L30" s="9">
         <f>IF(OR(I30="",K30=""),"",K30*I30)</f>
-        <v>110113.19</v>
+        <v>107955.43</v>
       </c>
       <c r="M30" s="9">
         <f>IF(L30="","",L30-J30)</f>
-        <v>10114.5</v>
+        <v>7956.74</v>
       </c>
       <c r="N30" s="10">
         <f>IF(OR(H30="",K30=""),"",K30/H30-1)</f>
-        <v>0.10114632501685761</v>
+        <v>0.07956844234659477</v>
       </c>
       <c r="O30" s="6">
         <f>IF(G30="","",$B$3-G30)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P30" s="6" t="str">
         <f>IF(H30="","Pending buy",IF(N30&gt;=0,"In profit","In loss"))</f>
@@ -2345,23 +2345,23 @@
         <v>99977.34</v>
       </c>
       <c r="K31" s="9" t="n">
-        <v>158.57</v>
+        <v>153.83</v>
       </c>
       <c r="L31" s="9">
         <f>IF(OR(I31="",K31=""),"",K31*I31)</f>
-        <v>89433.48</v>
+        <v>86760.12</v>
       </c>
       <c r="M31" s="9">
         <f>IF(L31="","",L31-J31)</f>
-        <v>-10543.86</v>
+        <v>-13217.22</v>
       </c>
       <c r="N31" s="10">
         <f>IF(OR(H31="",K31=""),"",K31/H31-1)</f>
-        <v>-0.10546248148193949</v>
+        <v>-0.1322021411765576</v>
       </c>
       <c r="O31" s="6">
         <f>IF(G31="","",$B$3-G31)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P31" s="6" t="str">
         <f>IF(H31="","Pending buy",IF(N31&gt;=0,"In profit","In loss"))</f>
@@ -2413,23 +2413,23 @@
         <v>99923.82</v>
       </c>
       <c r="K32" s="9" t="n">
-        <v>168.78</v>
+        <v>167.84</v>
       </c>
       <c r="L32" s="9">
         <f>IF(OR(I32="",K32=""),"",K32*I32)</f>
-        <v>95360.7</v>
+        <v>94829.6</v>
       </c>
       <c r="M32" s="9">
         <f>IF(L32="","",L32-J32)</f>
-        <v>-4563.12</v>
+        <v>-5094.22</v>
       </c>
       <c r="N32" s="10">
         <f>IF(OR(H32="",K32=""),"",K32/H32-1)</f>
-        <v>-0.04566598519822174</v>
+        <v>-0.05098103422010625</v>
       </c>
       <c r="O32" s="6">
         <f>IF(G32="","",$B$3-G32)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P32" s="6" t="str">
         <f>IF(H32="","Pending buy",IF(N32&gt;=0,"In profit","In loss"))</f>
@@ -2481,23 +2481,23 @@
         <v>99608.58</v>
       </c>
       <c r="K33" s="9" t="n">
-        <v>515.15</v>
+        <v>508.1</v>
       </c>
       <c r="L33" s="9">
         <f>IF(OR(I33="",K33=""),"",K33*I33)</f>
-        <v>97363.35</v>
+        <v>96030.9</v>
       </c>
       <c r="M33" s="9">
         <f>IF(L33="","",L33-J33)</f>
-        <v>-2245.23</v>
+        <v>-3577.68</v>
       </c>
       <c r="N33" s="10">
         <f>IF(OR(H33="",K33=""),"",K33/H33-1)</f>
-        <v>-0.02254048026738731</v>
+        <v>-0.03591734062672891</v>
       </c>
       <c r="O33" s="6">
         <f>IF(G33="","",$B$3-G33)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P33" s="6" t="str">
         <f>IF(H33="","Pending buy",IF(N33&gt;=0,"In profit","In loss"))</f>
@@ -2549,23 +2549,23 @@
         <v>96030.46</v>
       </c>
       <c r="K34" s="9" t="n">
-        <v>4592.9</v>
+        <v>4335.8</v>
       </c>
       <c r="L34" s="9">
         <f>IF(OR(I34="",K34=""),"",K34*I34)</f>
-        <v>87265.1</v>
+        <v>82380.2</v>
       </c>
       <c r="M34" s="9">
         <f>IF(L34="","",L34-J34)</f>
-        <v>-8765.36</v>
+        <v>-13650.26</v>
       </c>
       <c r="N34" s="10">
         <f>IF(OR(H34="",K34=""),"",K34/H34-1)</f>
-        <v>-0.09127687880308255</v>
+        <v>-0.14214511335200086</v>
       </c>
       <c r="O34" s="6">
         <f>IF(G34="","",$B$3-G34)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P34" s="6" t="str">
         <f>IF(H34="","Pending buy",IF(N34&gt;=0,"In profit","In loss"))</f>
@@ -2617,23 +2617,23 @@
         <v>99082.89</v>
       </c>
       <c r="K35" s="9" t="n">
-        <v>927.8</v>
+        <v>907.5</v>
       </c>
       <c r="L35" s="9">
         <f>IF(OR(I35="",K35=""),"",K35*I35)</f>
-        <v>84429.8</v>
+        <v>82582.5</v>
       </c>
       <c r="M35" s="9">
         <f>IF(L35="","",L35-J35)</f>
-        <v>-14653.09</v>
+        <v>-16500.39</v>
       </c>
       <c r="N35" s="10">
         <f>IF(OR(H35="",K35=""),"",K35/H35-1)</f>
-        <v>-0.1478872139916223</v>
+        <v>-0.16653119928583437</v>
       </c>
       <c r="O35" s="6">
         <f>IF(G35="","",$B$3-G35)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P35" s="6" t="str">
         <f>IF(H35="","Pending buy",IF(N35&gt;=0,"In profit","In loss"))</f>
@@ -2685,23 +2685,23 @@
         <v>99910.57</v>
       </c>
       <c r="K36" s="9" t="n">
-        <v>91.04000000000001</v>
+        <v>88.69</v>
       </c>
       <c r="L36" s="9">
         <f>IF(OR(I36="",K36=""),"",K36*I36)</f>
-        <v>93316.0</v>
+        <v>90907.25</v>
       </c>
       <c r="M36" s="9">
         <f>IF(L36="","",L36-J36)</f>
-        <v>-6594.57</v>
+        <v>-9003.32</v>
       </c>
       <c r="N36" s="10">
         <f>IF(OR(H36="",K36=""),"",K36/H36-1)</f>
-        <v>-0.06600473924625094</v>
+        <v>-0.0901137996896969</v>
       </c>
       <c r="O36" s="6">
         <f>IF(G36="","",$B$3-G36)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P36" s="6" t="str">
         <f>IF(H36="","Pending buy",IF(N36&gt;=0,"In profit","In loss"))</f>
@@ -2753,23 +2753,23 @@
         <v>99436.51</v>
       </c>
       <c r="K37" s="9" t="n">
-        <v>951.8</v>
+        <v>889.8</v>
       </c>
       <c r="L37" s="9">
         <f>IF(OR(I37="",K37=""),"",K37*I37)</f>
-        <v>95180.0</v>
+        <v>88980.0</v>
       </c>
       <c r="M37" s="9">
         <f>IF(L37="","",L37-J37)</f>
-        <v>-4256.51</v>
+        <v>-10456.51</v>
       </c>
       <c r="N37" s="10">
         <f>IF(OR(H37="",K37=""),"",K37/H37-1)</f>
-        <v>-0.04280633718803717</v>
+        <v>-0.10515767895557415</v>
       </c>
       <c r="O37" s="6">
         <f>IF(G37="","",$B$3-G37)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P37" s="6" t="str">
         <f>IF(H37="","Pending buy",IF(N37&gt;=0,"In profit","In loss"))</f>
@@ -2821,23 +2821,23 @@
         <v>99951.48</v>
       </c>
       <c r="K38" s="9" t="n">
-        <v>118.73</v>
+        <v>113.02</v>
       </c>
       <c r="L38" s="9">
         <f>IF(OR(I38="",K38=""),"",K38*I38)</f>
-        <v>97239.87</v>
+        <v>92563.38</v>
       </c>
       <c r="M38" s="9">
         <f>IF(L38="","",L38-J38)</f>
-        <v>-2711.61</v>
+        <v>-7388.1</v>
       </c>
       <c r="N38" s="10">
         <f>IF(OR(H38="",K38=""),"",K38/H38-1)</f>
-        <v>-0.02712926215485545</v>
+        <v>-0.07391686354536997</v>
       </c>
       <c r="O38" s="6">
         <f>IF(G38="","",$B$3-G38)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P38" s="6" t="str">
         <f>IF(H38="","Pending buy",IF(N38&gt;=0,"In profit","In loss"))</f>
@@ -2889,23 +2889,23 @@
         <v>99666.78</v>
       </c>
       <c r="K39" s="9" t="n">
-        <v>515.8</v>
+        <v>496.75</v>
       </c>
       <c r="L39" s="9">
         <f>IF(OR(I39="",K39=""),"",K39*I39)</f>
-        <v>92328.2</v>
+        <v>88918.25</v>
       </c>
       <c r="M39" s="9">
         <f>IF(L39="","",L39-J39)</f>
-        <v>-7338.58</v>
+        <v>-10748.53</v>
       </c>
       <c r="N39" s="10">
         <f>IF(OR(H39="",K39=""),"",K39/H39-1)</f>
-        <v>-0.0736311177415353</v>
+        <v>-0.10784462531622263</v>
       </c>
       <c r="O39" s="6">
         <f>IF(G39="","",$B$3-G39)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P39" s="6" t="str">
         <f>IF(H39="","Pending buy",IF(N39&gt;=0,"In profit","In loss"))</f>
@@ -2957,23 +2957,23 @@
         <v>99998.64</v>
       </c>
       <c r="K40" s="9" t="n">
-        <v>11.4</v>
+        <v>11.12</v>
       </c>
       <c r="L40" s="9">
         <f>IF(OR(I40="",K40=""),"",K40*I40)</f>
-        <v>87985.2</v>
+        <v>85824.16</v>
       </c>
       <c r="M40" s="9">
         <f>IF(L40="","",L40-J40)</f>
-        <v>-12013.44</v>
+        <v>-14174.48</v>
       </c>
       <c r="N40" s="10">
         <f>IF(OR(H40="",K40=""),"",K40/H40-1)</f>
-        <v>-0.12013601153640607</v>
+        <v>-0.14174670598989791</v>
       </c>
       <c r="O40" s="6">
         <f>IF(G40="","",$B$3-G40)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P40" s="6" t="str">
         <f>IF(H40="","Pending buy",IF(N40&gt;=0,"In profit","In loss"))</f>
@@ -3025,23 +3025,23 @@
         <v>99889.82</v>
       </c>
       <c r="K41" s="9" t="n">
-        <v>116.94</v>
+        <v>116.3</v>
       </c>
       <c r="L41" s="9">
         <f>IF(OR(I41="",K41=""),"",K41*I41)</f>
-        <v>92967.3</v>
+        <v>92458.5</v>
       </c>
       <c r="M41" s="9">
         <f>IF(L41="","",L41-J41)</f>
-        <v>-6922.52</v>
+        <v>-7431.32</v>
       </c>
       <c r="N41" s="10">
         <f>IF(OR(H41="",K41=""),"",K41/H41-1)</f>
-        <v>-0.06930154662520294</v>
+        <v>-0.07439515882085779</v>
       </c>
       <c r="O41" s="6">
         <f>IF(G41="","",$B$3-G41)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P41" s="6" t="str">
         <f>IF(H41="","Pending buy",IF(N41&gt;=0,"In profit","In loss"))</f>
@@ -3093,23 +3093,23 @@
         <v>99925.2</v>
       </c>
       <c r="K42" s="9" t="n">
-        <v>99.31</v>
+        <v>104.31</v>
       </c>
       <c r="L42" s="9">
         <f>IF(OR(I42="",K42=""),"",K42*I42)</f>
-        <v>105566.53</v>
+        <v>110881.53</v>
       </c>
       <c r="M42" s="9">
         <f>IF(L42="","",L42-J42)</f>
-        <v>5641.33</v>
+        <v>10956.33</v>
       </c>
       <c r="N42" s="10">
         <f>IF(OR(H42="",K42=""),"",K42/H42-1)</f>
-        <v>0.056455543885834514</v>
+        <v>0.10964533060851278</v>
       </c>
       <c r="O42" s="6">
         <f>IF(G42="","",$B$3-G42)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P42" s="6" t="str">
         <f>IF(H42="","Pending buy",IF(N42&gt;=0,"In profit","In loss"))</f>
@@ -3146,38 +3146,42 @@
       <c r="F43" s="8" t="n">
         <v>46317</v>
       </c>
-      <c r="G43" s="6" t="inlineStr"/>
-      <c r="H43" s="9" t="inlineStr"/>
-      <c r="I43" s="6" t="str">
+      <c r="G43" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H43" s="9" t="n">
+        <v>633.09</v>
+      </c>
+      <c r="I43" s="6">
         <f>IF(H43="","",ROUNDDOWN($B$1/H43,0))</f>
-        <v/>
-      </c>
-      <c r="J43" s="9" t="str">
+        <v>157</v>
+      </c>
+      <c r="J43" s="9">
         <f>IF(H43="","",H43*I43)</f>
-        <v/>
+        <v>99394.67</v>
       </c>
       <c r="K43" s="9" t="n">
-        <v>642.7</v>
-      </c>
-      <c r="L43" s="9" t="str">
+        <v>623.35</v>
+      </c>
+      <c r="L43" s="9">
         <f>IF(OR(I43="",K43=""),"",K43*I43)</f>
-        <v/>
-      </c>
-      <c r="M43" s="9" t="str">
+        <v>97865.95</v>
+      </c>
+      <c r="M43" s="9">
         <f>IF(L43="","",L43-J43)</f>
-        <v/>
-      </c>
-      <c r="N43" s="10" t="str">
+        <v>-1528.72</v>
+      </c>
+      <c r="N43" s="10">
         <f>IF(OR(H43="",K43=""),"",K43/H43-1)</f>
-        <v/>
-      </c>
-      <c r="O43" s="6" t="str">
+        <v>-0.01538032325423333</v>
+      </c>
+      <c r="O43" s="6">
         <f>IF(G43="","",$B$3-G43)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P43" s="6" t="str">
         <f>IF(H43="","Pending buy",IF(N43&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q43" s="6" t="n">
         <v>1</v>
@@ -3210,38 +3214,42 @@
       <c r="F44" s="8" t="n">
         <v>46317</v>
       </c>
-      <c r="G44" s="6" t="inlineStr"/>
-      <c r="H44" s="9" t="inlineStr"/>
-      <c r="I44" s="6" t="str">
+      <c r="G44" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H44" s="9" t="n">
+        <v>330.5</v>
+      </c>
+      <c r="I44" s="6">
         <f>IF(H44="","",ROUNDDOWN($B$1/H44,0))</f>
-        <v/>
-      </c>
-      <c r="J44" s="9" t="str">
+        <v>302</v>
+      </c>
+      <c r="J44" s="9">
         <f>IF(H44="","",H44*I44)</f>
-        <v/>
+        <v>99810.88</v>
       </c>
       <c r="K44" s="9" t="n">
-        <v>345.35</v>
-      </c>
-      <c r="L44" s="9" t="str">
+        <v>327.45</v>
+      </c>
+      <c r="L44" s="9">
         <f>IF(OR(I44="",K44=""),"",K44*I44)</f>
-        <v/>
-      </c>
-      <c r="M44" s="9" t="str">
+        <v>98889.9</v>
+      </c>
+      <c r="M44" s="9">
         <f>IF(L44="","",L44-J44)</f>
-        <v/>
-      </c>
-      <c r="N44" s="10" t="str">
+        <v>-920.98</v>
+      </c>
+      <c r="N44" s="10">
         <f>IF(OR(H44="",K44=""),"",K44/H44-1)</f>
-        <v/>
-      </c>
-      <c r="O44" s="6" t="str">
+        <v>-0.009227254626302028</v>
+      </c>
+      <c r="O44" s="6">
         <f>IF(G44="","",$B$3-G44)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P44" s="6" t="str">
         <f>IF(H44="","Pending buy",IF(N44&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q44" s="6" t="n">
         <v>1</v>
@@ -3274,38 +3282,42 @@
       <c r="F45" s="8" t="n">
         <v>46317</v>
       </c>
-      <c r="G45" s="6" t="inlineStr"/>
-      <c r="H45" s="9" t="inlineStr"/>
-      <c r="I45" s="6" t="str">
+      <c r="G45" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H45" s="9" t="n">
+        <v>269.53</v>
+      </c>
+      <c r="I45" s="6">
         <f>IF(H45="","",ROUNDDOWN($B$1/H45,0))</f>
-        <v/>
-      </c>
-      <c r="J45" s="9" t="str">
+        <v>371</v>
+      </c>
+      <c r="J45" s="9">
         <f>IF(H45="","",H45*I45)</f>
-        <v/>
+        <v>99997.44</v>
       </c>
       <c r="K45" s="9" t="n">
-        <v>270.15</v>
-      </c>
-      <c r="L45" s="9" t="str">
+        <v>263.95</v>
+      </c>
+      <c r="L45" s="9">
         <f>IF(OR(I45="",K45=""),"",K45*I45)</f>
-        <v/>
-      </c>
-      <c r="M45" s="9" t="str">
+        <v>97925.45</v>
+      </c>
+      <c r="M45" s="9">
         <f>IF(L45="","",L45-J45)</f>
-        <v/>
-      </c>
-      <c r="N45" s="10" t="str">
+        <v>-2071.99</v>
+      </c>
+      <c r="N45" s="10">
         <f>IF(OR(H45="",K45=""),"",K45/H45-1)</f>
-        <v/>
-      </c>
-      <c r="O45" s="6" t="str">
+        <v>-0.020720406077919362</v>
+      </c>
+      <c r="O45" s="6">
         <f>IF(G45="","",$B$3-G45)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P45" s="6" t="str">
         <f>IF(H45="","Pending buy",IF(N45&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q45" s="6" t="n">
         <v>1</v>
@@ -3338,38 +3350,42 @@
       <c r="F46" s="8" t="n">
         <v>46317</v>
       </c>
-      <c r="G46" s="6" t="inlineStr"/>
-      <c r="H46" s="9" t="inlineStr"/>
-      <c r="I46" s="6" t="str">
+      <c r="G46" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H46" s="9" t="n">
+        <v>359.25</v>
+      </c>
+      <c r="I46" s="6">
         <f>IF(H46="","",ROUNDDOWN($B$1/H46,0))</f>
-        <v/>
-      </c>
-      <c r="J46" s="9" t="str">
+        <v>278</v>
+      </c>
+      <c r="J46" s="9">
         <f>IF(H46="","",H46*I46)</f>
-        <v/>
+        <v>99870.37</v>
       </c>
       <c r="K46" s="9" t="n">
-        <v>367.1</v>
-      </c>
-      <c r="L46" s="9" t="str">
+        <v>359.1</v>
+      </c>
+      <c r="L46" s="9">
         <f>IF(OR(I46="",K46=""),"",K46*I46)</f>
-        <v/>
-      </c>
-      <c r="M46" s="9" t="str">
+        <v>99829.8</v>
+      </c>
+      <c r="M46" s="9">
         <f>IF(L46="","",L46-J46)</f>
-        <v/>
-      </c>
-      <c r="N46" s="10" t="str">
+        <v>-40.57</v>
+      </c>
+      <c r="N46" s="10">
         <f>IF(OR(H46="",K46=""),"",K46/H46-1)</f>
-        <v/>
-      </c>
-      <c r="O46" s="6" t="str">
+        <v>-0.000406178588785</v>
+      </c>
+      <c r="O46" s="6">
         <f>IF(G46="","",$B$3-G46)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P46" s="6" t="str">
         <f>IF(H46="","Pending buy",IF(N46&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q46" s="6" t="n">
         <v>1</v>
@@ -3402,38 +3418,42 @@
       <c r="F47" s="8" t="n">
         <v>46317</v>
       </c>
-      <c r="G47" s="6" t="inlineStr"/>
-      <c r="H47" s="9" t="inlineStr"/>
-      <c r="I47" s="6" t="str">
+      <c r="G47" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H47" s="9" t="n">
+        <v>577.79</v>
+      </c>
+      <c r="I47" s="6">
         <f>IF(H47="","",ROUNDDOWN($B$1/H47,0))</f>
-        <v/>
-      </c>
-      <c r="J47" s="9" t="str">
+        <v>173</v>
+      </c>
+      <c r="J47" s="9">
         <f>IF(H47="","",H47*I47)</f>
-        <v/>
+        <v>99957.4</v>
       </c>
       <c r="K47" s="9" t="n">
-        <v>592.35</v>
-      </c>
-      <c r="L47" s="9" t="str">
+        <v>574.5</v>
+      </c>
+      <c r="L47" s="9">
         <f>IF(OR(I47="",K47=""),"",K47*I47)</f>
-        <v/>
-      </c>
-      <c r="M47" s="9" t="str">
+        <v>99388.5</v>
+      </c>
+      <c r="M47" s="9">
         <f>IF(L47="","",L47-J47)</f>
-        <v/>
-      </c>
-      <c r="N47" s="10" t="str">
+        <v>-568.9</v>
+      </c>
+      <c r="N47" s="10">
         <f>IF(OR(H47="",K47=""),"",K47/H47-1)</f>
-        <v/>
-      </c>
-      <c r="O47" s="6" t="str">
+        <v>-0.005691413694327241</v>
+      </c>
+      <c r="O47" s="6">
         <f>IF(G47="","",$B$3-G47)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P47" s="6" t="str">
         <f>IF(H47="","Pending buy",IF(N47&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q47" s="6" t="n">
         <v>1</v>
@@ -3466,38 +3486,42 @@
       <c r="F48" s="8" t="n">
         <v>46317</v>
       </c>
-      <c r="G48" s="6" t="inlineStr"/>
-      <c r="H48" s="9" t="inlineStr"/>
-      <c r="I48" s="6" t="str">
+      <c r="G48" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="H48" s="9" t="n">
+        <v>179.47</v>
+      </c>
+      <c r="I48" s="6">
         <f>IF(H48="","",ROUNDDOWN($B$1/H48,0))</f>
-        <v/>
-      </c>
-      <c r="J48" s="9" t="str">
+        <v>557</v>
+      </c>
+      <c r="J48" s="9">
         <f>IF(H48="","",H48*I48)</f>
-        <v/>
+        <v>99965.44</v>
       </c>
       <c r="K48" s="9" t="n">
-        <v>182.85</v>
-      </c>
-      <c r="L48" s="9" t="str">
+        <v>178.9</v>
+      </c>
+      <c r="L48" s="9">
         <f>IF(OR(I48="",K48=""),"",K48*I48)</f>
-        <v/>
-      </c>
-      <c r="M48" s="9" t="str">
+        <v>99647.3</v>
+      </c>
+      <c r="M48" s="9">
         <f>IF(L48="","",L48-J48)</f>
-        <v/>
-      </c>
-      <c r="N48" s="10" t="str">
+        <v>-318.14</v>
+      </c>
+      <c r="N48" s="10">
         <f>IF(OR(H48="",K48=""),"",K48/H48-1)</f>
-        <v/>
-      </c>
-      <c r="O48" s="6" t="str">
+        <v>-0.003182522278188049</v>
+      </c>
+      <c r="O48" s="6">
         <f>IF(G48="","",$B$3-G48)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P48" s="6" t="str">
         <f>IF(H48="","Pending buy",IF(N48&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q48" s="6" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Momentum Portfolio: weekday silent update 2026-10-26
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q48"/>
+  <dimension ref="A1:Q53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -531,8 +531,8 @@
         </is>
       </c>
       <c r="E1" s="2">
-        <f>SUM(J8:J48)</f>
-        <v>4062646.89</v>
+        <f>SUM(J8:J53)</f>
+        <v>4162632.59</v>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
@@ -540,8 +540,8 @@
         </is>
       </c>
       <c r="G1" s="2">
-        <f>SUM(L8:L48)</f>
-        <v>3709129.13</v>
+        <f>SUM(L8:L53)</f>
+        <v>3864882.18</v>
       </c>
     </row>
     <row r="2">
@@ -551,8 +551,8 @@
         </is>
       </c>
       <c r="E2" s="2">
-        <f>SUM(M8:M48)</f>
-        <v>-353517.76</v>
+        <f>SUM(M8:M53)</f>
+        <v>-297750.41</v>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" s="3">
         <f>IF(E1=0,"",G1/E1-1)</f>
-        <v>-0.08701661000126948</v>
+        <v>-0.0715293515731591</v>
       </c>
     </row>
     <row r="3">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -579,8 +579,8 @@
         </is>
       </c>
       <c r="E3">
-        <f>COUNTIF(M8:M48,"&gt;0")</f>
-        <v>2</v>
+        <f>COUNTIF(M8:M53,"&gt;0")</f>
+        <v>9</v>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
@@ -588,8 +588,8 @@
         </is>
       </c>
       <c r="G3">
-        <f>COUNTIF(M8:M48,"&lt;0")</f>
-        <v>39</v>
+        <f>COUNTIF(M8:M53,"&lt;0")</f>
+        <v>33</v>
       </c>
     </row>
     <row r="4">
@@ -600,7 +600,7 @@
       </c>
       <c r="E4" s="3">
         <f>IF((E3+G3)=0,"",E3/(E3+G3))</f>
-        <v>0.04878048780487805</v>
+        <v>0.21428571428571427</v>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
@@ -608,8 +608,8 @@
         </is>
       </c>
       <c r="G4" s="3">
-        <f>AVERAGE(N8:N48)</f>
-        <v>-0.08714148760251178</v>
+        <f>AVERAGE(N8:N53)</f>
+        <v>-0.07167628534450934</v>
       </c>
     </row>
     <row r="5">
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="E5" t="str">
-        <f>INDEX(B8:B48,MATCH(MAX(N8:N48),N8:N48,0))</f>
+        <f>INDEX(B8:B53,MATCH(MAX(N8:N53),N8:N53,0))</f>
         <v>Pashupati Cotspin Limited</v>
       </c>
       <c r="F5" s="1" t="inlineStr">
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="G5" t="str">
-        <f>INDEX(B8:B48,MATCH(MIN(N8:N48),N8:N48,0))</f>
+        <f>INDEX(B8:B53,MATCH(MIN(N8:N53),N8:N53,0))</f>
         <v>Lloyds Enterprises Limited</v>
       </c>
     </row>
@@ -639,8 +639,8 @@
         </is>
       </c>
       <c r="E6" s="3">
-        <f>AVERAGEIF(D8:D48,"4★*",N8:N48)</f>
-        <v>-0.11065143816567073</v>
+        <f>AVERAGEIF(D8:D53,"4★*",N8:N53)</f>
+        <v>-0.10690773576489473</v>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
@@ -648,8 +648,8 @@
         </is>
       </c>
       <c r="G6" s="3">
-        <f>AVERAGEIF(D8:D48,"5★*",N8:N48)</f>
-        <v>-0.0668374393888745</v>
+        <f>AVERAGEIF(D8:D53,"5★*",N8:N53)</f>
+        <v>-0.042572043692886634</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
@@ -781,23 +781,23 @@
         <v>99851.29</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>267.75</v>
+        <v>273.8</v>
       </c>
       <c r="L8" s="9">
         <f>IF(OR(I8="",K8=""),"",K8*I8)</f>
-        <v>88893.0</v>
+        <v>90901.6</v>
       </c>
       <c r="M8" s="9">
         <f>IF(L8="","",L8-J8)</f>
-        <v>-10958.29</v>
+        <v>-8949.69</v>
       </c>
       <c r="N8" s="10">
         <f>IF(OR(H8="",K8=""),"",K8/H8-1)</f>
-        <v>-0.10974613424340696</v>
+        <v>-0.08963022056337933</v>
       </c>
       <c r="O8" s="6">
         <f>IF(G8="","",$B$3-G8)</f>
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="P8" s="6" t="str">
         <f>IF(H8="","Pending buy",IF(N8&gt;=0,"In profit","In loss"))</f>
@@ -849,23 +849,23 @@
         <v>99687.42</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>317.4</v>
+        <v>325.55</v>
       </c>
       <c r="L9" s="9">
         <f>IF(OR(I9="",K9=""),"",K9*I9)</f>
-        <v>97124.4</v>
+        <v>99618.3</v>
       </c>
       <c r="M9" s="9">
         <f>IF(L9="","",L9-J9)</f>
-        <v>-2563.02</v>
+        <v>-69.12</v>
       </c>
       <c r="N9" s="10">
         <f>IF(OR(H9="",K9=""),"",K9/H9-1)</f>
-        <v>-0.025710568022618285</v>
+        <v>-0.0006933693124239193</v>
       </c>
       <c r="O9" s="6">
         <f>IF(G9="","",$B$3-G9)</f>
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="P9" s="6" t="str">
         <f>IF(H9="","Pending buy",IF(N9&gt;=0,"In profit","In loss"))</f>
@@ -917,23 +917,23 @@
         <v>99607.14</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>1498.5</v>
+        <v>1463.7</v>
       </c>
       <c r="L10" s="9">
         <f>IF(OR(I10="",K10=""),"",K10*I10)</f>
-        <v>94405.5</v>
+        <v>92213.1</v>
       </c>
       <c r="M10" s="9">
         <f>IF(L10="","",L10-J10)</f>
-        <v>-5201.64</v>
+        <v>-7394.04</v>
       </c>
       <c r="N10" s="10">
         <f>IF(OR(H10="",K10=""),"",K10/H10-1)</f>
-        <v>-0.05222156643178999</v>
+        <v>-0.07423203656070132</v>
       </c>
       <c r="O10" s="6">
         <f>IF(G10="","",$B$3-G10)</f>
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="P10" s="6" t="str">
         <f>IF(H10="","Pending buy",IF(N10&gt;=0,"In profit","In loss"))</f>
@@ -985,23 +985,23 @@
         <v>99927.23</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>62.36</v>
+        <v>60.91</v>
       </c>
       <c r="L11" s="9">
         <f>IF(OR(I11="",K11=""),"",K11*I11)</f>
-        <v>78012.36</v>
+        <v>76198.41</v>
       </c>
       <c r="M11" s="9">
         <f>IF(L11="","",L11-J11)</f>
-        <v>-21914.87</v>
+        <v>-23728.82</v>
       </c>
       <c r="N11" s="10">
         <f>IF(OR(H11="",K11=""),"",K11/H11-1)</f>
-        <v>-0.21930829362751503</v>
+        <v>-0.23746100328498954</v>
       </c>
       <c r="O11" s="6">
         <f>IF(G11="","",$B$3-G11)</f>
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="P11" s="6" t="str">
         <f>IF(H11="","Pending buy",IF(N11&gt;=0,"In profit","In loss"))</f>
@@ -1053,23 +1053,23 @@
         <v>86537.12</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>18865</v>
+        <v>19055</v>
       </c>
       <c r="L12" s="9">
         <f>IF(OR(I12="",K12=""),"",K12*I12)</f>
-        <v>75460.0</v>
+        <v>76220.0</v>
       </c>
       <c r="M12" s="9">
         <f>IF(L12="","",L12-J12)</f>
-        <v>-11077.12</v>
+        <v>-10317.12</v>
       </c>
       <c r="N12" s="10">
         <f>IF(OR(H12="",K12=""),"",K12/H12-1)</f>
-        <v>-0.12800422101054776</v>
+        <v>-0.11922186225051612</v>
       </c>
       <c r="O12" s="6">
         <f>IF(G12="","",$B$3-G12)</f>
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="P12" s="6" t="str">
         <f>IF(H12="","Pending buy",IF(N12&gt;=0,"In profit","In loss"))</f>
@@ -1121,23 +1121,23 @@
         <v>98177.53</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>1661.9</v>
+        <v>1659</v>
       </c>
       <c r="L13" s="9">
         <f>IF(OR(I13="",K13=""),"",K13*I13)</f>
-        <v>88080.7</v>
+        <v>87927.0</v>
       </c>
       <c r="M13" s="9">
         <f>IF(L13="","",L13-J13)</f>
-        <v>-10096.83</v>
+        <v>-10250.53</v>
       </c>
       <c r="N13" s="10">
         <f>IF(OR(H13="",K13=""),"",K13/H13-1)</f>
-        <v>-0.10284260393618627</v>
+        <v>-0.10440813522482284</v>
       </c>
       <c r="O13" s="6">
         <f>IF(G13="","",$B$3-G13)</f>
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="P13" s="6" t="str">
         <f>IF(H13="","Pending buy",IF(N13&gt;=0,"In profit","In loss"))</f>
@@ -1189,23 +1189,23 @@
         <v>97667.46</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>4157.3</v>
+        <v>4200</v>
       </c>
       <c r="L14" s="9">
         <f>IF(OR(I14="",K14=""),"",K14*I14)</f>
-        <v>91460.6</v>
+        <v>92400.0</v>
       </c>
       <c r="M14" s="9">
         <f>IF(L14="","",L14-J14)</f>
-        <v>-6206.86</v>
+        <v>-5267.46</v>
       </c>
       <c r="N14" s="10">
         <f>IF(OR(H14="",K14=""),"",K14/H14-1)</f>
-        <v>-0.06355099143928644</v>
+        <v>-0.0539326399453981</v>
       </c>
       <c r="O14" s="6">
         <f>IF(G14="","",$B$3-G14)</f>
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="P14" s="6" t="str">
         <f>IF(H14="","Pending buy",IF(N14&gt;=0,"In profit","In loss"))</f>
@@ -1257,23 +1257,23 @@
         <v>99078.19</v>
       </c>
       <c r="K15" s="9" t="n">
-        <v>1295.3</v>
+        <v>1305.7</v>
       </c>
       <c r="L15" s="9">
         <f>IF(OR(I15="",K15=""),"",K15*I15)</f>
-        <v>82899.2</v>
+        <v>83564.8</v>
       </c>
       <c r="M15" s="9">
         <f>IF(L15="","",L15-J15)</f>
-        <v>-16178.99</v>
+        <v>-15513.39</v>
       </c>
       <c r="N15" s="10">
         <f>IF(OR(H15="",K15=""),"",K15/H15-1)</f>
-        <v>-0.16329515081493806</v>
+        <v>-0.15657722413268316</v>
       </c>
       <c r="O15" s="6">
         <f>IF(G15="","",$B$3-G15)</f>
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="P15" s="6" t="str">
         <f>IF(H15="","Pending buy",IF(N15&gt;=0,"In profit","In loss"))</f>
@@ -1325,30 +1325,30 @@
         <v>98557.54</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>1380</v>
+        <v>1575</v>
       </c>
       <c r="L16" s="9">
         <f>IF(OR(I16="",K16=""),"",K16*I16)</f>
-        <v>93840.0</v>
+        <v>107100.0</v>
       </c>
       <c r="M16" s="9">
         <f>IF(L16="","",L16-J16)</f>
-        <v>-4717.54</v>
+        <v>8542.46</v>
       </c>
       <c r="N16" s="10">
         <f>IF(OR(H16="",K16=""),"",K16/H16-1)</f>
-        <v>-0.0478658120197043</v>
+        <v>0.08667488845577243</v>
       </c>
       <c r="O16" s="6">
         <f>IF(G16="","",$B$3-G16)</f>
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="P16" s="6" t="str">
         <f>IF(H16="","Pending buy",IF(N16&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q16" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -1393,23 +1393,23 @@
         <v>99714.35</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>805.1</v>
+        <v>796</v>
       </c>
       <c r="L17" s="9">
         <f>IF(OR(I17="",K17=""),"",K17*I17)</f>
-        <v>92586.5</v>
+        <v>91540.0</v>
       </c>
       <c r="M17" s="9">
         <f>IF(L17="","",L17-J17)</f>
-        <v>-7127.85</v>
+        <v>-8174.35</v>
       </c>
       <c r="N17" s="10">
         <f>IF(OR(H17="",K17=""),"",K17/H17-1)</f>
-        <v>-0.07148269100323879</v>
+        <v>-0.08197766990259359</v>
       </c>
       <c r="O17" s="6">
         <f>IF(G17="","",$B$3-G17)</f>
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="P17" s="6" t="str">
         <f>IF(H17="","Pending buy",IF(N17&gt;=0,"In profit","In loss"))</f>
@@ -1461,23 +1461,23 @@
         <v>99596.83</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>589.75</v>
+        <v>575.8</v>
       </c>
       <c r="L18" s="9">
         <f>IF(OR(I18="",K18=""),"",K18*I18)</f>
-        <v>83154.75</v>
+        <v>81187.8</v>
       </c>
       <c r="M18" s="9">
         <f>IF(L18="","",L18-J18)</f>
-        <v>-16442.08</v>
+        <v>-18409.03</v>
       </c>
       <c r="N18" s="10">
         <f>IF(OR(H18="",K18=""),"",K18/H18-1)</f>
-        <v>-0.16508641722250028</v>
+        <v>-0.18483553884987824</v>
       </c>
       <c r="O18" s="6">
         <f>IF(G18="","",$B$3-G18)</f>
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="P18" s="6" t="str">
         <f>IF(H18="","Pending buy",IF(N18&gt;=0,"In profit","In loss"))</f>
@@ -1529,23 +1529,23 @@
         <v>99993.07</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>123.16</v>
+        <v>124.69</v>
       </c>
       <c r="L19" s="9">
         <f>IF(OR(I19="",K19=""),"",K19*I19)</f>
-        <v>81655.08</v>
+        <v>82669.47</v>
       </c>
       <c r="M19" s="9">
         <f>IF(L19="","",L19-J19)</f>
-        <v>-18337.99</v>
+        <v>-17323.6</v>
       </c>
       <c r="N19" s="10">
         <f>IF(OR(H19="",K19=""),"",K19/H19-1)</f>
-        <v>-0.1833925706347691</v>
+        <v>-0.17324796713583435</v>
       </c>
       <c r="O19" s="6">
         <f>IF(G19="","",$B$3-G19)</f>
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="P19" s="6" t="str">
         <f>IF(H19="","Pending buy",IF(N19&gt;=0,"In profit","In loss"))</f>
@@ -1597,23 +1597,23 @@
         <v>99896.43</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>185.49</v>
+        <v>190.71</v>
       </c>
       <c r="L20" s="9">
         <f>IF(OR(I20="",K20=""),"",K20*I20)</f>
-        <v>88478.73</v>
+        <v>90968.67</v>
       </c>
       <c r="M20" s="9">
         <f>IF(L20="","",L20-J20)</f>
-        <v>-11417.7</v>
+        <v>-8927.76</v>
       </c>
       <c r="N20" s="10">
         <f>IF(OR(H20="",K20=""),"",K20/H20-1)</f>
-        <v>-0.1142953757738312</v>
+        <v>-0.08937016073010595</v>
       </c>
       <c r="O20" s="6">
         <f>IF(G20="","",$B$3-G20)</f>
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="P20" s="6" t="str">
         <f>IF(H20="","Pending buy",IF(N20&gt;=0,"In profit","In loss"))</f>
@@ -1665,23 +1665,23 @@
         <v>99449.47</v>
       </c>
       <c r="K21" s="9" t="n">
-        <v>1215.3</v>
+        <v>1245.5</v>
       </c>
       <c r="L21" s="9">
         <f>IF(OR(I21="",K21=""),"",K21*I21)</f>
-        <v>86286.3</v>
+        <v>88430.5</v>
       </c>
       <c r="M21" s="9">
         <f>IF(L21="","",L21-J21)</f>
-        <v>-13163.17</v>
+        <v>-11018.97</v>
       </c>
       <c r="N21" s="10">
         <f>IF(OR(H21="",K21=""),"",K21/H21-1)</f>
-        <v>-0.1323603516798154</v>
+        <v>-0.11079965277479642</v>
       </c>
       <c r="O21" s="6">
         <f>IF(G21="","",$B$3-G21)</f>
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="P21" s="6" t="str">
         <f>IF(H21="","Pending buy",IF(N21&gt;=0,"In profit","In loss"))</f>
@@ -1733,23 +1733,23 @@
         <v>99837.05</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>604.25</v>
+        <v>624.8</v>
       </c>
       <c r="L22" s="9">
         <f>IF(OR(I22="",K22=""),"",K22*I22)</f>
-        <v>87012.0</v>
+        <v>89971.2</v>
       </c>
       <c r="M22" s="9">
         <f>IF(L22="","",L22-J22)</f>
-        <v>-12825.05</v>
+        <v>-9865.85</v>
       </c>
       <c r="N22" s="10">
         <f>IF(OR(H22="",K22=""),"",K22/H22-1)</f>
-        <v>-0.12845983506248415</v>
+        <v>-0.09881953652799369</v>
       </c>
       <c r="O22" s="6">
         <f>IF(G22="","",$B$3-G22)</f>
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="P22" s="6" t="str">
         <f>IF(H22="","Pending buy",IF(N22&gt;=0,"In profit","In loss"))</f>
@@ -1801,23 +1801,23 @@
         <v>99486.88</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>566.25</v>
+        <v>560.35</v>
       </c>
       <c r="L23" s="9">
         <f>IF(OR(I23="",K23=""),"",K23*I23)</f>
-        <v>82106.25</v>
+        <v>81250.75</v>
       </c>
       <c r="M23" s="9">
         <f>IF(L23="","",L23-J23)</f>
-        <v>-17380.63</v>
+        <v>-18236.13</v>
       </c>
       <c r="N23" s="10">
         <f>IF(OR(H23="",K23=""),"",K23/H23-1)</f>
-        <v>-0.1747027445438406</v>
+        <v>-0.18330186826514983</v>
       </c>
       <c r="O23" s="6">
         <f>IF(G23="","",$B$3-G23)</f>
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="P23" s="6" t="str">
         <f>IF(H23="","Pending buy",IF(N23&gt;=0,"In profit","In loss"))</f>
@@ -1869,23 +1869,23 @@
         <v>99935.4</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>205.51</v>
+        <v>210.37</v>
       </c>
       <c r="L24" s="9">
         <f>IF(OR(I24="",K24=""),"",K24*I24)</f>
-        <v>90218.89</v>
+        <v>92352.43</v>
       </c>
       <c r="M24" s="9">
         <f>IF(L24="","",L24-J24)</f>
-        <v>-9716.51</v>
+        <v>-7582.97</v>
       </c>
       <c r="N24" s="10">
         <f>IF(OR(H24="",K24=""),"",K24/H24-1)</f>
-        <v>-0.0972278966094835</v>
+        <v>-0.07587870473328329</v>
       </c>
       <c r="O24" s="6">
         <f>IF(G24="","",$B$3-G24)</f>
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="P24" s="6" t="str">
         <f>IF(H24="","Pending buy",IF(N24&gt;=0,"In profit","In loss"))</f>
@@ -1937,23 +1937,23 @@
         <v>99622.64</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>703.6</v>
+        <v>713.55</v>
       </c>
       <c r="L25" s="9">
         <f>IF(OR(I25="",K25=""),"",K25*I25)</f>
-        <v>87246.4</v>
+        <v>88480.2</v>
       </c>
       <c r="M25" s="9">
         <f>IF(L25="","",L25-J25)</f>
-        <v>-12376.24</v>
+        <v>-11142.44</v>
       </c>
       <c r="N25" s="10">
         <f>IF(OR(H25="",K25=""),"",K25/H25-1)</f>
-        <v>-0.1242311671345595</v>
+        <v>-0.11184643164989339</v>
       </c>
       <c r="O25" s="6">
         <f>IF(G25="","",$B$3-G25)</f>
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="P25" s="6" t="str">
         <f>IF(H25="","Pending buy",IF(N25&gt;=0,"In profit","In loss"))</f>
@@ -2005,23 +2005,23 @@
         <v>99948.17</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>170.77</v>
+        <v>170.94</v>
       </c>
       <c r="L26" s="9">
         <f>IF(OR(I26="",K26=""),"",K26*I26)</f>
-        <v>81115.75</v>
+        <v>81196.5</v>
       </c>
       <c r="M26" s="9">
         <f>IF(L26="","",L26-J26)</f>
-        <v>-18832.42</v>
+        <v>-18751.67</v>
       </c>
       <c r="N26" s="10">
         <f>IF(OR(H26="",K26=""),"",K26/H26-1)</f>
-        <v>-0.18842183205057772</v>
+        <v>-0.18761391327941535</v>
       </c>
       <c r="O26" s="6">
         <f>IF(G26="","",$B$3-G26)</f>
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="P26" s="6" t="str">
         <f>IF(H26="","Pending buy",IF(N26&gt;=0,"In profit","In loss"))</f>
@@ -2073,23 +2073,23 @@
         <v>99745.27</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>210</v>
+        <v>208.45</v>
       </c>
       <c r="L27" s="9">
         <f>IF(OR(I27="",K27=""),"",K27*I27)</f>
-        <v>80220.0</v>
+        <v>79627.9</v>
       </c>
       <c r="M27" s="9">
         <f>IF(L27="","",L27-J27)</f>
-        <v>-19525.27</v>
+        <v>-20117.37</v>
       </c>
       <c r="N27" s="10">
         <f>IF(OR(H27="",K27=""),"",K27/H27-1)</f>
-        <v>-0.1957513612482673</v>
+        <v>-0.20168748215333965</v>
       </c>
       <c r="O27" s="6">
         <f>IF(G27="","",$B$3-G27)</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="P27" s="6" t="str">
         <f>IF(H27="","Pending buy",IF(N27&gt;=0,"In profit","In loss"))</f>
@@ -2141,27 +2141,27 @@
         <v>95334.84</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>10488</v>
+        <v>10726</v>
       </c>
       <c r="L28" s="9">
         <f>IF(OR(I28="",K28=""),"",K28*I28)</f>
-        <v>94392.0</v>
+        <v>96534.0</v>
       </c>
       <c r="M28" s="9">
         <f>IF(L28="","",L28-J28)</f>
-        <v>-942.84</v>
+        <v>1199.16</v>
       </c>
       <c r="N28" s="10">
         <f>IF(OR(H28="",K28=""),"",K28/H28-1)</f>
-        <v>-0.009889798633152536</v>
+        <v>0.012578377179710776</v>
       </c>
       <c r="O28" s="6">
         <f>IF(G28="","",$B$3-G28)</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="P28" s="6" t="str">
         <f>IF(H28="","Pending buy",IF(N28&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q28" s="6" t="n">
         <v>1</v>
@@ -2209,23 +2209,23 @@
         <v>98598.59</v>
       </c>
       <c r="K29" s="9" t="n">
-        <v>1762</v>
+        <v>1758.4</v>
       </c>
       <c r="L29" s="9">
         <f>IF(OR(I29="",K29=""),"",K29*I29)</f>
-        <v>89862.0</v>
+        <v>89678.4</v>
       </c>
       <c r="M29" s="9">
         <f>IF(L29="","",L29-J29)</f>
-        <v>-8736.59</v>
+        <v>-8920.19</v>
       </c>
       <c r="N29" s="10">
         <f>IF(OR(H29="",K29=""),"",K29/H29-1)</f>
-        <v>-0.08860762201697492</v>
+        <v>-0.09046971768141243</v>
       </c>
       <c r="O29" s="6">
         <f>IF(G29="","",$B$3-G29)</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="P29" s="6" t="str">
         <f>IF(H29="","Pending buy",IF(N29&gt;=0,"In profit","In loss"))</f>
@@ -2277,23 +2277,23 @@
         <v>99998.69</v>
       </c>
       <c r="K30" s="9" t="n">
-        <v>16.01</v>
+        <v>15.69</v>
       </c>
       <c r="L30" s="9">
         <f>IF(OR(I30="",K30=""),"",K30*I30)</f>
-        <v>107955.43</v>
+        <v>105797.67</v>
       </c>
       <c r="M30" s="9">
         <f>IF(L30="","",L30-J30)</f>
-        <v>7956.74</v>
+        <v>5798.98</v>
       </c>
       <c r="N30" s="10">
         <f>IF(OR(H30="",K30=""),"",K30/H30-1)</f>
-        <v>0.07956844234659477</v>
+        <v>0.05799055967633171</v>
       </c>
       <c r="O30" s="6">
         <f>IF(G30="","",$B$3-G30)</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="P30" s="6" t="str">
         <f>IF(H30="","Pending buy",IF(N30&gt;=0,"In profit","In loss"))</f>
@@ -2345,23 +2345,23 @@
         <v>99977.34</v>
       </c>
       <c r="K31" s="9" t="n">
-        <v>153.83</v>
+        <v>141.07</v>
       </c>
       <c r="L31" s="9">
         <f>IF(OR(I31="",K31=""),"",K31*I31)</f>
-        <v>86760.12</v>
+        <v>79563.48</v>
       </c>
       <c r="M31" s="9">
         <f>IF(L31="","",L31-J31)</f>
-        <v>-13217.22</v>
+        <v>-20413.86</v>
       </c>
       <c r="N31" s="10">
         <f>IF(OR(H31="",K31=""),"",K31/H31-1)</f>
-        <v>-0.1322021411765576</v>
+        <v>-0.20418485377219653</v>
       </c>
       <c r="O31" s="6">
         <f>IF(G31="","",$B$3-G31)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P31" s="6" t="str">
         <f>IF(H31="","Pending buy",IF(N31&gt;=0,"In profit","In loss"))</f>
@@ -2413,23 +2413,23 @@
         <v>99923.82</v>
       </c>
       <c r="K32" s="9" t="n">
-        <v>167.84</v>
+        <v>176.23</v>
       </c>
       <c r="L32" s="9">
         <f>IF(OR(I32="",K32=""),"",K32*I32)</f>
-        <v>94829.6</v>
+        <v>99569.95</v>
       </c>
       <c r="M32" s="9">
         <f>IF(L32="","",L32-J32)</f>
-        <v>-5094.22</v>
+        <v>-353.87</v>
       </c>
       <c r="N32" s="10">
         <f>IF(OR(H32="",K32=""),"",K32/H32-1)</f>
-        <v>-0.05098103422010625</v>
+        <v>-0.003541394546051735</v>
       </c>
       <c r="O32" s="6">
         <f>IF(G32="","",$B$3-G32)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P32" s="6" t="str">
         <f>IF(H32="","Pending buy",IF(N32&gt;=0,"In profit","In loss"))</f>
@@ -2481,30 +2481,30 @@
         <v>99608.58</v>
       </c>
       <c r="K33" s="9" t="n">
-        <v>508.1</v>
+        <v>522.8</v>
       </c>
       <c r="L33" s="9">
         <f>IF(OR(I33="",K33=""),"",K33*I33)</f>
-        <v>96030.9</v>
+        <v>98809.2</v>
       </c>
       <c r="M33" s="9">
         <f>IF(L33="","",L33-J33)</f>
-        <v>-3577.68</v>
+        <v>-799.38</v>
       </c>
       <c r="N33" s="10">
         <f>IF(OR(H33="",K33=""),"",K33/H33-1)</f>
-        <v>-0.03591734062672891</v>
+        <v>-0.008025163707250482</v>
       </c>
       <c r="O33" s="6">
         <f>IF(G33="","",$B$3-G33)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P33" s="6" t="str">
         <f>IF(H33="","Pending buy",IF(N33&gt;=0,"In profit","In loss"))</f>
         <v>In loss</v>
       </c>
       <c r="Q33" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
@@ -2549,23 +2549,23 @@
         <v>96030.46</v>
       </c>
       <c r="K34" s="9" t="n">
-        <v>4335.8</v>
+        <v>4286</v>
       </c>
       <c r="L34" s="9">
         <f>IF(OR(I34="",K34=""),"",K34*I34)</f>
-        <v>82380.2</v>
+        <v>81434.0</v>
       </c>
       <c r="M34" s="9">
         <f>IF(L34="","",L34-J34)</f>
-        <v>-13650.26</v>
+        <v>-14596.46</v>
       </c>
       <c r="N34" s="10">
         <f>IF(OR(H34="",K34=""),"",K34/H34-1)</f>
-        <v>-0.14214511335200086</v>
+        <v>-0.15199823696357673</v>
       </c>
       <c r="O34" s="6">
         <f>IF(G34="","",$B$3-G34)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="P34" s="6" t="str">
         <f>IF(H34="","Pending buy",IF(N34&gt;=0,"In profit","In loss"))</f>
@@ -2617,23 +2617,23 @@
         <v>99082.89</v>
       </c>
       <c r="K35" s="9" t="n">
-        <v>907.5</v>
+        <v>903.2</v>
       </c>
       <c r="L35" s="9">
         <f>IF(OR(I35="",K35=""),"",K35*I35)</f>
-        <v>82582.5</v>
+        <v>82191.2</v>
       </c>
       <c r="M35" s="9">
         <f>IF(L35="","",L35-J35)</f>
-        <v>-16500.39</v>
+        <v>-16891.69</v>
       </c>
       <c r="N35" s="10">
         <f>IF(OR(H35="",K35=""),"",K35/H35-1)</f>
-        <v>-0.16653119928583437</v>
+        <v>-0.17048041784569212</v>
       </c>
       <c r="O35" s="6">
         <f>IF(G35="","",$B$3-G35)</f>
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="P35" s="6" t="str">
         <f>IF(H35="","Pending buy",IF(N35&gt;=0,"In profit","In loss"))</f>
@@ -2685,23 +2685,23 @@
         <v>99910.57</v>
       </c>
       <c r="K36" s="9" t="n">
-        <v>88.69</v>
+        <v>88.64</v>
       </c>
       <c r="L36" s="9">
         <f>IF(OR(I36="",K36=""),"",K36*I36)</f>
-        <v>90907.25</v>
+        <v>90856.0</v>
       </c>
       <c r="M36" s="9">
         <f>IF(L36="","",L36-J36)</f>
-        <v>-9003.32</v>
+        <v>-9054.57</v>
       </c>
       <c r="N36" s="10">
         <f>IF(OR(H36="",K36=""),"",K36/H36-1)</f>
-        <v>-0.0901137996896969</v>
+        <v>-0.09062675842253609</v>
       </c>
       <c r="O36" s="6">
         <f>IF(G36="","",$B$3-G36)</f>
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="P36" s="6" t="str">
         <f>IF(H36="","Pending buy",IF(N36&gt;=0,"In profit","In loss"))</f>
@@ -2753,23 +2753,23 @@
         <v>99436.51</v>
       </c>
       <c r="K37" s="9" t="n">
-        <v>889.8</v>
+        <v>970.8</v>
       </c>
       <c r="L37" s="9">
         <f>IF(OR(I37="",K37=""),"",K37*I37)</f>
-        <v>88980.0</v>
+        <v>97080.0</v>
       </c>
       <c r="M37" s="9">
         <f>IF(L37="","",L37-J37)</f>
-        <v>-10456.51</v>
+        <v>-2356.51</v>
       </c>
       <c r="N37" s="10">
         <f>IF(OR(H37="",K37=""),"",K37/H37-1)</f>
-        <v>-0.10515767895557415</v>
+        <v>-0.023698667936695172</v>
       </c>
       <c r="O37" s="6">
         <f>IF(G37="","",$B$3-G37)</f>
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="P37" s="6" t="str">
         <f>IF(H37="","Pending buy",IF(N37&gt;=0,"In profit","In loss"))</f>
@@ -2821,23 +2821,23 @@
         <v>99951.48</v>
       </c>
       <c r="K38" s="9" t="n">
-        <v>113.02</v>
+        <v>112.6</v>
       </c>
       <c r="L38" s="9">
         <f>IF(OR(I38="",K38=""),"",K38*I38)</f>
-        <v>92563.38</v>
+        <v>92219.4</v>
       </c>
       <c r="M38" s="9">
         <f>IF(L38="","",L38-J38)</f>
-        <v>-7388.1</v>
+        <v>-7732.08</v>
       </c>
       <c r="N38" s="10">
         <f>IF(OR(H38="",K38=""),"",K38/H38-1)</f>
-        <v>-0.07391686354536997</v>
+        <v>-0.07735833334992626</v>
       </c>
       <c r="O38" s="6">
         <f>IF(G38="","",$B$3-G38)</f>
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="P38" s="6" t="str">
         <f>IF(H38="","Pending buy",IF(N38&gt;=0,"In profit","In loss"))</f>
@@ -2889,23 +2889,23 @@
         <v>99666.78</v>
       </c>
       <c r="K39" s="9" t="n">
-        <v>496.75</v>
+        <v>486.75</v>
       </c>
       <c r="L39" s="9">
         <f>IF(OR(I39="",K39=""),"",K39*I39)</f>
-        <v>88918.25</v>
+        <v>87128.25</v>
       </c>
       <c r="M39" s="9">
         <f>IF(L39="","",L39-J39)</f>
-        <v>-10748.53</v>
+        <v>-12538.53</v>
       </c>
       <c r="N39" s="10">
         <f>IF(OR(H39="",K39=""),"",K39/H39-1)</f>
-        <v>-0.10784462531622263</v>
+        <v>-0.1258044718121215</v>
       </c>
       <c r="O39" s="6">
         <f>IF(G39="","",$B$3-G39)</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="P39" s="6" t="str">
         <f>IF(H39="","Pending buy",IF(N39&gt;=0,"In profit","In loss"))</f>
@@ -2957,23 +2957,23 @@
         <v>99998.64</v>
       </c>
       <c r="K40" s="9" t="n">
-        <v>11.12</v>
+        <v>12.23</v>
       </c>
       <c r="L40" s="9">
         <f>IF(OR(I40="",K40=""),"",K40*I40)</f>
-        <v>85824.16</v>
+        <v>94391.14</v>
       </c>
       <c r="M40" s="9">
         <f>IF(L40="","",L40-J40)</f>
-        <v>-14174.48</v>
+        <v>-5607.5</v>
       </c>
       <c r="N40" s="10">
         <f>IF(OR(H40="",K40=""),"",K40/H40-1)</f>
-        <v>-0.14174670598989791</v>
+        <v>-0.0560757386921269</v>
       </c>
       <c r="O40" s="6">
         <f>IF(G40="","",$B$3-G40)</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="P40" s="6" t="str">
         <f>IF(H40="","Pending buy",IF(N40&gt;=0,"In profit","In loss"))</f>
@@ -3025,23 +3025,23 @@
         <v>99889.82</v>
       </c>
       <c r="K41" s="9" t="n">
-        <v>116.3</v>
+        <v>119.81</v>
       </c>
       <c r="L41" s="9">
         <f>IF(OR(I41="",K41=""),"",K41*I41)</f>
-        <v>92458.5</v>
+        <v>95248.95</v>
       </c>
       <c r="M41" s="9">
         <f>IF(L41="","",L41-J41)</f>
-        <v>-7431.32</v>
+        <v>-4640.87</v>
       </c>
       <c r="N41" s="10">
         <f>IF(OR(H41="",K41=""),"",K41/H41-1)</f>
-        <v>-0.07439515882085779</v>
+        <v>-0.04645987943531349</v>
       </c>
       <c r="O41" s="6">
         <f>IF(G41="","",$B$3-G41)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P41" s="6" t="str">
         <f>IF(H41="","Pending buy",IF(N41&gt;=0,"In profit","In loss"))</f>
@@ -3093,23 +3093,23 @@
         <v>99925.2</v>
       </c>
       <c r="K42" s="9" t="n">
-        <v>104.31</v>
+        <v>109.87</v>
       </c>
       <c r="L42" s="9">
         <f>IF(OR(I42="",K42=""),"",K42*I42)</f>
-        <v>110881.53</v>
+        <v>116791.81</v>
       </c>
       <c r="M42" s="9">
         <f>IF(L42="","",L42-J42)</f>
-        <v>10956.33</v>
+        <v>16866.61</v>
       </c>
       <c r="N42" s="10">
         <f>IF(OR(H42="",K42=""),"",K42/H42-1)</f>
-        <v>0.10964533060851278</v>
+        <v>0.168792373444131</v>
       </c>
       <c r="O42" s="6">
         <f>IF(G42="","",$B$3-G42)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="P42" s="6" t="str">
         <f>IF(H42="","Pending buy",IF(N42&gt;=0,"In profit","In loss"))</f>
@@ -3161,23 +3161,23 @@
         <v>99394.67</v>
       </c>
       <c r="K43" s="9" t="n">
-        <v>623.35</v>
+        <v>620.05</v>
       </c>
       <c r="L43" s="9">
         <f>IF(OR(I43="",K43=""),"",K43*I43)</f>
-        <v>97865.95</v>
+        <v>97347.85</v>
       </c>
       <c r="M43" s="9">
         <f>IF(L43="","",L43-J43)</f>
-        <v>-1528.72</v>
+        <v>-2046.82</v>
       </c>
       <c r="N43" s="10">
         <f>IF(OR(H43="",K43=""),"",K43/H43-1)</f>
-        <v>-0.01538032325423333</v>
+        <v>-0.020592876287458872</v>
       </c>
       <c r="O43" s="6">
         <f>IF(G43="","",$B$3-G43)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P43" s="6" t="str">
         <f>IF(H43="","Pending buy",IF(N43&gt;=0,"In profit","In loss"))</f>
@@ -3229,30 +3229,30 @@
         <v>99810.88</v>
       </c>
       <c r="K44" s="9" t="n">
-        <v>327.45</v>
+        <v>337.05</v>
       </c>
       <c r="L44" s="9">
         <f>IF(OR(I44="",K44=""),"",K44*I44)</f>
-        <v>98889.9</v>
+        <v>101789.1</v>
       </c>
       <c r="M44" s="9">
         <f>IF(L44="","",L44-J44)</f>
-        <v>-920.98</v>
+        <v>1978.22</v>
       </c>
       <c r="N44" s="10">
         <f>IF(OR(H44="",K44=""),"",K44/H44-1)</f>
-        <v>-0.009227254626302028</v>
+        <v>0.019819678815712116</v>
       </c>
       <c r="O44" s="6">
         <f>IF(G44="","",$B$3-G44)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P44" s="6" t="str">
         <f>IF(H44="","Pending buy",IF(N44&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q44" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45">
@@ -3297,27 +3297,27 @@
         <v>99997.44</v>
       </c>
       <c r="K45" s="9" t="n">
-        <v>263.95</v>
+        <v>271.2</v>
       </c>
       <c r="L45" s="9">
         <f>IF(OR(I45="",K45=""),"",K45*I45)</f>
-        <v>97925.45</v>
+        <v>100615.2</v>
       </c>
       <c r="M45" s="9">
         <f>IF(L45="","",L45-J45)</f>
-        <v>-2071.99</v>
+        <v>617.76</v>
       </c>
       <c r="N45" s="10">
         <f>IF(OR(H45="",K45=""),"",K45/H45-1)</f>
-        <v>-0.020720406077919362</v>
+        <v>0.006177783184952768</v>
       </c>
       <c r="O45" s="6">
         <f>IF(G45="","",$B$3-G45)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P45" s="6" t="str">
         <f>IF(H45="","Pending buy",IF(N45&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q45" s="6" t="n">
         <v>1</v>
@@ -3365,27 +3365,27 @@
         <v>99870.37</v>
       </c>
       <c r="K46" s="9" t="n">
-        <v>359.1</v>
+        <v>366.75</v>
       </c>
       <c r="L46" s="9">
         <f>IF(OR(I46="",K46=""),"",K46*I46)</f>
-        <v>99829.8</v>
+        <v>101956.5</v>
       </c>
       <c r="M46" s="9">
         <f>IF(L46="","",L46-J46)</f>
-        <v>-40.57</v>
+        <v>2086.13</v>
       </c>
       <c r="N46" s="10">
         <f>IF(OR(H46="",K46=""),"",K46/H46-1)</f>
-        <v>-0.000406178588785</v>
+        <v>0.02088842662924839</v>
       </c>
       <c r="O46" s="6">
         <f>IF(G46="","",$B$3-G46)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P46" s="6" t="str">
         <f>IF(H46="","Pending buy",IF(N46&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q46" s="6" t="n">
         <v>1</v>
@@ -3433,23 +3433,23 @@
         <v>99957.4</v>
       </c>
       <c r="K47" s="9" t="n">
-        <v>574.5</v>
+        <v>560.85</v>
       </c>
       <c r="L47" s="9">
         <f>IF(OR(I47="",K47=""),"",K47*I47)</f>
-        <v>99388.5</v>
+        <v>97027.05</v>
       </c>
       <c r="M47" s="9">
         <f>IF(L47="","",L47-J47)</f>
-        <v>-568.9</v>
+        <v>-2930.35</v>
       </c>
       <c r="N47" s="10">
         <f>IF(OR(H47="",K47=""),"",K47/H47-1)</f>
-        <v>-0.005691413694327241</v>
+        <v>-0.029315978016472344</v>
       </c>
       <c r="O47" s="6">
         <f>IF(G47="","",$B$3-G47)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P47" s="6" t="str">
         <f>IF(H47="","Pending buy",IF(N47&gt;=0,"In profit","In loss"))</f>
@@ -3501,34 +3501,358 @@
         <v>99965.44</v>
       </c>
       <c r="K48" s="9" t="n">
-        <v>178.9</v>
+        <v>181.2</v>
       </c>
       <c r="L48" s="9">
         <f>IF(OR(I48="",K48=""),"",K48*I48)</f>
-        <v>99647.3</v>
+        <v>100928.4</v>
       </c>
       <c r="M48" s="9">
         <f>IF(L48="","",L48-J48)</f>
-        <v>-318.14</v>
+        <v>962.96</v>
       </c>
       <c r="N48" s="10">
         <f>IF(OR(H48="",K48=""),"",K48/H48-1)</f>
-        <v>-0.003182522278188049</v>
+        <v>0.009632906446016332</v>
       </c>
       <c r="O48" s="6">
         <f>IF(G48="","",$B$3-G48)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P48" s="6" t="str">
         <f>IF(H48="","Pending buy",IF(N48&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q48" s="6" t="n">
         <v>1</v>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="6" t="n">
+        <v>42</v>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Sterlite Technologies Limited</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>STLTECH</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>231026</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="G49" s="8" t="n">
+        <v>46321</v>
+      </c>
+      <c r="H49" s="9" t="n">
+        <v>833.21</v>
+      </c>
+      <c r="I49" s="6">
+        <f>IF(H49="","",ROUNDDOWN($B$1/H49,0))</f>
+        <v>120</v>
+      </c>
+      <c r="J49" s="9">
+        <f>IF(H49="","",H49*I49)</f>
+        <v>99985.7</v>
+      </c>
+      <c r="K49" s="9" t="n">
+        <v>867.55</v>
+      </c>
+      <c r="L49" s="9">
+        <f>IF(OR(I49="",K49=""),"",K49*I49)</f>
+        <v>104106.0</v>
+      </c>
+      <c r="M49" s="9">
+        <f>IF(L49="","",L49-J49)</f>
+        <v>4120.3</v>
+      </c>
+      <c r="N49" s="10">
+        <f>IF(OR(H49="",K49=""),"",K49/H49-1)</f>
+        <v>0.0412089274447609</v>
+      </c>
+      <c r="O49" s="6">
+        <f>IF(G49="","",$B$3-G49)</f>
+        <v>0</v>
+      </c>
+      <c r="P49" s="6" t="str">
+        <f>IF(H49="","Pending buy",IF(N49&gt;=0,"In profit","In loss"))</f>
+        <v>In profit</v>
+      </c>
+      <c r="Q49" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Filatex India Limited</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>FILATEX</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>261026</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="n">
+        <v>46321</v>
+      </c>
+      <c r="G50" s="6" t="inlineStr"/>
+      <c r="H50" s="9" t="inlineStr"/>
+      <c r="I50" s="6" t="str">
+        <f>IF(H50="","",ROUNDDOWN($B$1/H50,0))</f>
+        <v/>
+      </c>
+      <c r="J50" s="9" t="str">
+        <f>IF(H50="","",H50*I50)</f>
+        <v/>
+      </c>
+      <c r="K50" s="9" t="n">
+        <v>94.62</v>
+      </c>
+      <c r="L50" s="9" t="str">
+        <f>IF(OR(I50="",K50=""),"",K50*I50)</f>
+        <v/>
+      </c>
+      <c r="M50" s="9" t="str">
+        <f>IF(L50="","",L50-J50)</f>
+        <v/>
+      </c>
+      <c r="N50" s="10" t="str">
+        <f>IF(OR(H50="",K50=""),"",K50/H50-1)</f>
+        <v/>
+      </c>
+      <c r="O50" s="6" t="str">
+        <f>IF(G50="","",$B$3-G50)</f>
+        <v/>
+      </c>
+      <c r="P50" s="6" t="str">
+        <f>IF(H50="","Pending buy",IF(N50&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q50" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Gland Pharma Limited</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>GLAND</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>261026</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="n">
+        <v>46321</v>
+      </c>
+      <c r="G51" s="6" t="inlineStr"/>
+      <c r="H51" s="9" t="inlineStr"/>
+      <c r="I51" s="6" t="str">
+        <f>IF(H51="","",ROUNDDOWN($B$1/H51,0))</f>
+        <v/>
+      </c>
+      <c r="J51" s="9" t="str">
+        <f>IF(H51="","",H51*I51)</f>
+        <v/>
+      </c>
+      <c r="K51" s="9" t="n">
+        <v>2843.9</v>
+      </c>
+      <c r="L51" s="9" t="str">
+        <f>IF(OR(I51="",K51=""),"",K51*I51)</f>
+        <v/>
+      </c>
+      <c r="M51" s="9" t="str">
+        <f>IF(L51="","",L51-J51)</f>
+        <v/>
+      </c>
+      <c r="N51" s="10" t="str">
+        <f>IF(OR(H51="",K51=""),"",K51/H51-1)</f>
+        <v/>
+      </c>
+      <c r="O51" s="6" t="str">
+        <f>IF(G51="","",$B$3-G51)</f>
+        <v/>
+      </c>
+      <c r="P51" s="6" t="str">
+        <f>IF(H51="","Pending buy",IF(N51&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q51" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Shilpa Medicare Limited</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>SHILPAMED</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>261026</t>
+        </is>
+      </c>
+      <c r="F52" s="8" t="n">
+        <v>46321</v>
+      </c>
+      <c r="G52" s="6" t="inlineStr"/>
+      <c r="H52" s="9" t="inlineStr"/>
+      <c r="I52" s="6" t="str">
+        <f>IF(H52="","",ROUNDDOWN($B$1/H52,0))</f>
+        <v/>
+      </c>
+      <c r="J52" s="9" t="str">
+        <f>IF(H52="","",H52*I52)</f>
+        <v/>
+      </c>
+      <c r="K52" s="9" t="n">
+        <v>900.8</v>
+      </c>
+      <c r="L52" s="9" t="str">
+        <f>IF(OR(I52="",K52=""),"",K52*I52)</f>
+        <v/>
+      </c>
+      <c r="M52" s="9" t="str">
+        <f>IF(L52="","",L52-J52)</f>
+        <v/>
+      </c>
+      <c r="N52" s="10" t="str">
+        <f>IF(OR(H52="",K52=""),"",K52/H52-1)</f>
+        <v/>
+      </c>
+      <c r="O52" s="6" t="str">
+        <f>IF(G52="","",$B$3-G52)</f>
+        <v/>
+      </c>
+      <c r="P52" s="6" t="str">
+        <f>IF(H52="","Pending buy",IF(N52&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q52" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Sona BLW Precision Forgings Limited</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>SONACOMS</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>261026</t>
+        </is>
+      </c>
+      <c r="F53" s="8" t="n">
+        <v>46321</v>
+      </c>
+      <c r="G53" s="6" t="inlineStr"/>
+      <c r="H53" s="9" t="inlineStr"/>
+      <c r="I53" s="6" t="str">
+        <f>IF(H53="","",ROUNDDOWN($B$1/H53,0))</f>
+        <v/>
+      </c>
+      <c r="J53" s="9" t="str">
+        <f>IF(H53="","",H53*I53)</f>
+        <v/>
+      </c>
+      <c r="K53" s="9" t="n">
+        <v>781.9</v>
+      </c>
+      <c r="L53" s="9" t="str">
+        <f>IF(OR(I53="",K53=""),"",K53*I53)</f>
+        <v/>
+      </c>
+      <c r="M53" s="9" t="str">
+        <f>IF(L53="","",L53-J53)</f>
+        <v/>
+      </c>
+      <c r="N53" s="10" t="str">
+        <f>IF(OR(H53="",K53=""),"",K53/H53-1)</f>
+        <v/>
+      </c>
+      <c r="O53" s="6" t="str">
+        <f>IF(G53="","",$B$3-G53)</f>
+        <v/>
+      </c>
+      <c r="P53" s="6" t="str">
+        <f>IF(H53="","Pending buy",IF(N53&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q53" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A8:Q48">
+  <conditionalFormatting sqref="A8:Q53">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$N8&gt;0</formula>
     </cfRule>
@@ -3546,7 +3870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4534,6 +4858,166 @@
       <c r="D49" s="11" t="inlineStr">
         <is>
           <t>Sheetal Cool Products Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>STLTECH</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="inlineStr">
+        <is>
+          <t>Sterlite Technologies Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>ATHERENERG</t>
+        </is>
+      </c>
+      <c r="D51" s="11" t="inlineStr">
+        <is>
+          <t>Ather Energy Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>FILATEX</t>
+        </is>
+      </c>
+      <c r="D52" s="11" t="inlineStr">
+        <is>
+          <t>Filatex India Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>GLAND</t>
+        </is>
+      </c>
+      <c r="D53" s="11" t="inlineStr">
+        <is>
+          <t>Gland Pharma Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>INDSWFTLAB</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="inlineStr">
+        <is>
+          <t>Ind-Swift Laboratories Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>KAPSTON</t>
+        </is>
+      </c>
+      <c r="D55" s="11" t="inlineStr">
+        <is>
+          <t>Kapston Services Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>SHILPAMED</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
+        <is>
+          <t>Shilpa Medicare Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>SONACOMS</t>
+        </is>
+      </c>
+      <c r="D57" s="11" t="inlineStr">
+        <is>
+          <t>Sona BLW Precision Forgings Limited</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum Portfolio: weekday silent update 2026-10-27
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q53"/>
+  <dimension ref="A1:Q58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -531,8 +531,8 @@
         </is>
       </c>
       <c r="E1" s="2">
-        <f>SUM(J8:J53)</f>
-        <v>4162632.59</v>
+        <f>SUM(J8:J58)</f>
+        <v>4559576.06</v>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
@@ -540,8 +540,8 @@
         </is>
       </c>
       <c r="G1" s="2">
-        <f>SUM(L8:L53)</f>
-        <v>3864882.18</v>
+        <f>SUM(L8:L58)</f>
+        <v>4353060.57</v>
       </c>
     </row>
     <row r="2">
@@ -551,8 +551,8 @@
         </is>
       </c>
       <c r="E2" s="2">
-        <f>SUM(M8:M53)</f>
-        <v>-297750.41</v>
+        <f>SUM(M8:M58)</f>
+        <v>-206515.49</v>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" s="3">
         <f>IF(E1=0,"",G1/E1-1)</f>
-        <v>-0.0715293515731591</v>
+        <v>-0.04529269547923698</v>
       </c>
     </row>
     <row r="3">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -579,8 +579,8 @@
         </is>
       </c>
       <c r="E3">
-        <f>COUNTIF(M8:M53,"&gt;0")</f>
-        <v>9</v>
+        <f>COUNTIF(M8:M58,"&gt;0")</f>
+        <v>13</v>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="G3">
-        <f>COUNTIF(M8:M53,"&lt;0")</f>
+        <f>COUNTIF(M8:M58,"&lt;0")</f>
         <v>33</v>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="E4" s="3">
         <f>IF((E3+G3)=0,"",E3/(E3+G3))</f>
-        <v>0.21428571428571427</v>
+        <v>0.2826086956521739</v>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
@@ -608,8 +608,8 @@
         </is>
       </c>
       <c r="G4" s="3">
-        <f>AVERAGE(N8:N53)</f>
-        <v>-0.07167628534450934</v>
+        <f>AVERAGE(N8:N58)</f>
+        <v>-0.045462774731276995</v>
       </c>
     </row>
     <row r="5">
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="E5" t="str">
-        <f>INDEX(B8:B53,MATCH(MAX(N8:N53),N8:N53,0))</f>
+        <f>INDEX(B8:B58,MATCH(MAX(N8:N58),N8:N58,0))</f>
         <v>Pashupati Cotspin Limited</v>
       </c>
       <c r="F5" s="1" t="inlineStr">
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="G5" t="str">
-        <f>INDEX(B8:B53,MATCH(MIN(N8:N53),N8:N53,0))</f>
+        <f>INDEX(B8:B58,MATCH(MIN(N8:N58),N8:N58,0))</f>
         <v>Lloyds Enterprises Limited</v>
       </c>
     </row>
@@ -639,8 +639,8 @@
         </is>
       </c>
       <c r="E6" s="3">
-        <f>AVERAGEIF(D8:D53,"4★*",N8:N53)</f>
-        <v>-0.10690773576489473</v>
+        <f>AVERAGEIF(D8:D58,"4★*",N8:N58)</f>
+        <v>-0.08442613176186621</v>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
@@ -648,8 +648,8 @@
         </is>
       </c>
       <c r="G6" s="3">
-        <f>AVERAGEIF(D8:D53,"5★*",N8:N53)</f>
-        <v>-0.042572043692886634</v>
+        <f>AVERAGEIF(D8:D58,"5★*",N8:N58)</f>
+        <v>-0.01804411608012162</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
@@ -781,23 +781,23 @@
         <v>99851.29</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>273.8</v>
+        <v>278.7</v>
       </c>
       <c r="L8" s="9">
         <f>IF(OR(I8="",K8=""),"",K8*I8)</f>
-        <v>90901.6</v>
+        <v>92528.4</v>
       </c>
       <c r="M8" s="9">
         <f>IF(L8="","",L8-J8)</f>
-        <v>-8949.69</v>
+        <v>-7322.89</v>
       </c>
       <c r="N8" s="10">
         <f>IF(OR(H8="",K8=""),"",K8/H8-1)</f>
-        <v>-0.08963022056337933</v>
+        <v>-0.07333799295476207</v>
       </c>
       <c r="O8" s="6">
         <f>IF(G8="","",$B$3-G8)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P8" s="6" t="str">
         <f>IF(H8="","Pending buy",IF(N8&gt;=0,"In profit","In loss"))</f>
@@ -849,27 +849,27 @@
         <v>99687.42</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>325.55</v>
+        <v>331</v>
       </c>
       <c r="L9" s="9">
         <f>IF(OR(I9="",K9=""),"",K9*I9)</f>
-        <v>99618.3</v>
+        <v>101286.0</v>
       </c>
       <c r="M9" s="9">
         <f>IF(L9="","",L9-J9)</f>
-        <v>-69.12</v>
+        <v>1598.58</v>
       </c>
       <c r="N9" s="10">
         <f>IF(OR(H9="",K9=""),"",K9/H9-1)</f>
-        <v>-0.0006933693124239193</v>
+        <v>0.01603592307660162</v>
       </c>
       <c r="O9" s="6">
         <f>IF(G9="","",$B$3-G9)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P9" s="6" t="str">
         <f>IF(H9="","Pending buy",IF(N9&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>1</v>
@@ -917,23 +917,23 @@
         <v>99607.14</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>1463.7</v>
+        <v>1474</v>
       </c>
       <c r="L10" s="9">
         <f>IF(OR(I10="",K10=""),"",K10*I10)</f>
-        <v>92213.1</v>
+        <v>92862.0</v>
       </c>
       <c r="M10" s="9">
         <f>IF(L10="","",L10-J10)</f>
-        <v>-7394.04</v>
+        <v>-6745.14</v>
       </c>
       <c r="N10" s="10">
         <f>IF(OR(H10="",K10=""),"",K10/H10-1)</f>
-        <v>-0.07423203656070132</v>
+        <v>-0.06771744339036267</v>
       </c>
       <c r="O10" s="6">
         <f>IF(G10="","",$B$3-G10)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P10" s="6" t="str">
         <f>IF(H10="","Pending buy",IF(N10&gt;=0,"In profit","In loss"))</f>
@@ -985,23 +985,23 @@
         <v>99927.23</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>60.91</v>
+        <v>61.25</v>
       </c>
       <c r="L11" s="9">
         <f>IF(OR(I11="",K11=""),"",K11*I11)</f>
-        <v>76198.41</v>
+        <v>76623.75</v>
       </c>
       <c r="M11" s="9">
         <f>IF(L11="","",L11-J11)</f>
-        <v>-23728.82</v>
+        <v>-23303.48</v>
       </c>
       <c r="N11" s="10">
         <f>IF(OR(H11="",K11=""),"",K11/H11-1)</f>
-        <v>-0.23746100328498954</v>
+        <v>-0.2332045058480644</v>
       </c>
       <c r="O11" s="6">
         <f>IF(G11="","",$B$3-G11)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P11" s="6" t="str">
         <f>IF(H11="","Pending buy",IF(N11&gt;=0,"In profit","In loss"))</f>
@@ -1053,23 +1053,23 @@
         <v>86537.12</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>19055</v>
+        <v>19315</v>
       </c>
       <c r="L12" s="9">
         <f>IF(OR(I12="",K12=""),"",K12*I12)</f>
-        <v>76220.0</v>
+        <v>77260.0</v>
       </c>
       <c r="M12" s="9">
         <f>IF(L12="","",L12-J12)</f>
-        <v>-10317.12</v>
+        <v>-9277.12</v>
       </c>
       <c r="N12" s="10">
         <f>IF(OR(H12="",K12=""),"",K12/H12-1)</f>
-        <v>-0.11922186225051612</v>
+        <v>-0.1072038976315256</v>
       </c>
       <c r="O12" s="6">
         <f>IF(G12="","",$B$3-G12)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P12" s="6" t="str">
         <f>IF(H12="","Pending buy",IF(N12&gt;=0,"In profit","In loss"))</f>
@@ -1121,23 +1121,23 @@
         <v>98177.53</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>1659</v>
+        <v>1690.8</v>
       </c>
       <c r="L13" s="9">
         <f>IF(OR(I13="",K13=""),"",K13*I13)</f>
-        <v>87927.0</v>
+        <v>89612.4</v>
       </c>
       <c r="M13" s="9">
         <f>IF(L13="","",L13-J13)</f>
-        <v>-10250.53</v>
+        <v>-8565.13</v>
       </c>
       <c r="N13" s="10">
         <f>IF(OR(H13="",K13=""),"",K13/H13-1)</f>
-        <v>-0.10440813522482284</v>
+        <v>-0.08724127488736022</v>
       </c>
       <c r="O13" s="6">
         <f>IF(G13="","",$B$3-G13)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P13" s="6" t="str">
         <f>IF(H13="","Pending buy",IF(N13&gt;=0,"In profit","In loss"))</f>
@@ -1189,23 +1189,23 @@
         <v>97667.46</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>4200</v>
+        <v>4290</v>
       </c>
       <c r="L14" s="9">
         <f>IF(OR(I14="",K14=""),"",K14*I14)</f>
-        <v>92400.0</v>
+        <v>94380.0</v>
       </c>
       <c r="M14" s="9">
         <f>IF(L14="","",L14-J14)</f>
-        <v>-5267.46</v>
+        <v>-3287.46</v>
       </c>
       <c r="N14" s="10">
         <f>IF(OR(H14="",K14=""),"",K14/H14-1)</f>
-        <v>-0.0539326399453981</v>
+        <v>-0.03365976794422798</v>
       </c>
       <c r="O14" s="6">
         <f>IF(G14="","",$B$3-G14)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P14" s="6" t="str">
         <f>IF(H14="","Pending buy",IF(N14&gt;=0,"In profit","In loss"))</f>
@@ -1257,23 +1257,23 @@
         <v>99078.19</v>
       </c>
       <c r="K15" s="9" t="n">
-        <v>1305.7</v>
+        <v>1370.7</v>
       </c>
       <c r="L15" s="9">
         <f>IF(OR(I15="",K15=""),"",K15*I15)</f>
-        <v>83564.8</v>
+        <v>87724.8</v>
       </c>
       <c r="M15" s="9">
         <f>IF(L15="","",L15-J15)</f>
-        <v>-15513.39</v>
+        <v>-11353.39</v>
       </c>
       <c r="N15" s="10">
         <f>IF(OR(H15="",K15=""),"",K15/H15-1)</f>
-        <v>-0.15657722413268316</v>
+        <v>-0.11459018236859064</v>
       </c>
       <c r="O15" s="6">
         <f>IF(G15="","",$B$3-G15)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P15" s="6" t="str">
         <f>IF(H15="","Pending buy",IF(N15&gt;=0,"In profit","In loss"))</f>
@@ -1325,23 +1325,23 @@
         <v>98557.54</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>1575</v>
+        <v>1674</v>
       </c>
       <c r="L16" s="9">
         <f>IF(OR(I16="",K16=""),"",K16*I16)</f>
-        <v>107100.0</v>
+        <v>113832.0</v>
       </c>
       <c r="M16" s="9">
         <f>IF(L16="","",L16-J16)</f>
-        <v>8542.46</v>
+        <v>15274.46</v>
       </c>
       <c r="N16" s="10">
         <f>IF(OR(H16="",K16=""),"",K16/H16-1)</f>
-        <v>0.08667488845577243</v>
+        <v>0.15498016715870655</v>
       </c>
       <c r="O16" s="6">
         <f>IF(G16="","",$B$3-G16)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P16" s="6" t="str">
         <f>IF(H16="","Pending buy",IF(N16&gt;=0,"In profit","In loss"))</f>
@@ -1393,23 +1393,23 @@
         <v>99714.35</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>796</v>
+        <v>809.15</v>
       </c>
       <c r="L17" s="9">
         <f>IF(OR(I17="",K17=""),"",K17*I17)</f>
-        <v>91540.0</v>
+        <v>93052.25</v>
       </c>
       <c r="M17" s="9">
         <f>IF(L17="","",L17-J17)</f>
-        <v>-8174.35</v>
+        <v>-6662.1</v>
       </c>
       <c r="N17" s="10">
         <f>IF(OR(H17="",K17=""),"",K17/H17-1)</f>
-        <v>-0.08197766990259359</v>
+        <v>-0.06681184874583368</v>
       </c>
       <c r="O17" s="6">
         <f>IF(G17="","",$B$3-G17)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P17" s="6" t="str">
         <f>IF(H17="","Pending buy",IF(N17&gt;=0,"In profit","In loss"))</f>
@@ -1461,23 +1461,23 @@
         <v>99596.83</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>575.8</v>
+        <v>597.5</v>
       </c>
       <c r="L18" s="9">
         <f>IF(OR(I18="",K18=""),"",K18*I18)</f>
-        <v>81187.8</v>
+        <v>84247.5</v>
       </c>
       <c r="M18" s="9">
         <f>IF(L18="","",L18-J18)</f>
-        <v>-18409.03</v>
+        <v>-15349.33</v>
       </c>
       <c r="N18" s="10">
         <f>IF(OR(H18="",K18=""),"",K18/H18-1)</f>
-        <v>-0.18483553884987824</v>
+        <v>-0.15411468298506814</v>
       </c>
       <c r="O18" s="6">
         <f>IF(G18="","",$B$3-G18)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P18" s="6" t="str">
         <f>IF(H18="","Pending buy",IF(N18&gt;=0,"In profit","In loss"))</f>
@@ -1529,23 +1529,23 @@
         <v>99993.07</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>124.69</v>
+        <v>125.81</v>
       </c>
       <c r="L19" s="9">
         <f>IF(OR(I19="",K19=""),"",K19*I19)</f>
-        <v>82669.47</v>
+        <v>83412.03</v>
       </c>
       <c r="M19" s="9">
         <f>IF(L19="","",L19-J19)</f>
-        <v>-17323.6</v>
+        <v>-16581.04</v>
       </c>
       <c r="N19" s="10">
         <f>IF(OR(H19="",K19=""),"",K19/H19-1)</f>
-        <v>-0.17324796713583435</v>
+        <v>-0.16582185215622192</v>
       </c>
       <c r="O19" s="6">
         <f>IF(G19="","",$B$3-G19)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P19" s="6" t="str">
         <f>IF(H19="","Pending buy",IF(N19&gt;=0,"In profit","In loss"))</f>
@@ -1597,23 +1597,23 @@
         <v>99896.43</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>190.71</v>
+        <v>201.12</v>
       </c>
       <c r="L20" s="9">
         <f>IF(OR(I20="",K20=""),"",K20*I20)</f>
-        <v>90968.67</v>
+        <v>95934.24</v>
       </c>
       <c r="M20" s="9">
         <f>IF(L20="","",L20-J20)</f>
-        <v>-8927.76</v>
+        <v>-3962.19</v>
       </c>
       <c r="N20" s="10">
         <f>IF(OR(H20="",K20=""),"",K20/H20-1)</f>
-        <v>-0.08937016073010595</v>
+        <v>-0.03966297900497562</v>
       </c>
       <c r="O20" s="6">
         <f>IF(G20="","",$B$3-G20)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P20" s="6" t="str">
         <f>IF(H20="","Pending buy",IF(N20&gt;=0,"In profit","In loss"))</f>
@@ -1665,23 +1665,23 @@
         <v>99449.47</v>
       </c>
       <c r="K21" s="9" t="n">
-        <v>1245.5</v>
+        <v>1311</v>
       </c>
       <c r="L21" s="9">
         <f>IF(OR(I21="",K21=""),"",K21*I21)</f>
-        <v>88430.5</v>
+        <v>93081.0</v>
       </c>
       <c r="M21" s="9">
         <f>IF(L21="","",L21-J21)</f>
-        <v>-11018.97</v>
+        <v>-6368.47</v>
       </c>
       <c r="N21" s="10">
         <f>IF(OR(H21="",K21=""),"",K21/H21-1)</f>
-        <v>-0.11079965277479642</v>
+        <v>-0.06403720978543403</v>
       </c>
       <c r="O21" s="6">
         <f>IF(G21="","",$B$3-G21)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P21" s="6" t="str">
         <f>IF(H21="","Pending buy",IF(N21&gt;=0,"In profit","In loss"))</f>
@@ -1733,23 +1733,23 @@
         <v>99837.05</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>624.8</v>
+        <v>656</v>
       </c>
       <c r="L22" s="9">
         <f>IF(OR(I22="",K22=""),"",K22*I22)</f>
-        <v>89971.2</v>
+        <v>94464.0</v>
       </c>
       <c r="M22" s="9">
         <f>IF(L22="","",L22-J22)</f>
-        <v>-9865.85</v>
+        <v>-5373.05</v>
       </c>
       <c r="N22" s="10">
         <f>IF(OR(H22="",K22=""),"",K22/H22-1)</f>
-        <v>-0.09881953652799369</v>
+        <v>-0.05381820736613918</v>
       </c>
       <c r="O22" s="6">
         <f>IF(G22="","",$B$3-G22)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P22" s="6" t="str">
         <f>IF(H22="","Pending buy",IF(N22&gt;=0,"In profit","In loss"))</f>
@@ -1801,23 +1801,23 @@
         <v>99486.88</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>560.35</v>
+        <v>564.5</v>
       </c>
       <c r="L23" s="9">
         <f>IF(OR(I23="",K23=""),"",K23*I23)</f>
-        <v>81250.75</v>
+        <v>81852.5</v>
       </c>
       <c r="M23" s="9">
         <f>IF(L23="","",L23-J23)</f>
-        <v>-18236.13</v>
+        <v>-17634.38</v>
       </c>
       <c r="N23" s="10">
         <f>IF(OR(H23="",K23=""),"",K23/H23-1)</f>
-        <v>-0.18330186826514983</v>
+        <v>-0.17725333208829674</v>
       </c>
       <c r="O23" s="6">
         <f>IF(G23="","",$B$3-G23)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P23" s="6" t="str">
         <f>IF(H23="","Pending buy",IF(N23&gt;=0,"In profit","In loss"))</f>
@@ -1869,23 +1869,23 @@
         <v>99935.4</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>210.37</v>
+        <v>215.92</v>
       </c>
       <c r="L24" s="9">
         <f>IF(OR(I24="",K24=""),"",K24*I24)</f>
-        <v>92352.43</v>
+        <v>94788.88</v>
       </c>
       <c r="M24" s="9">
         <f>IF(L24="","",L24-J24)</f>
-        <v>-7582.97</v>
+        <v>-5146.52</v>
       </c>
       <c r="N24" s="10">
         <f>IF(OR(H24="",K24=""),"",K24/H24-1)</f>
-        <v>-0.07587870473328329</v>
+        <v>-0.05149845475120285</v>
       </c>
       <c r="O24" s="6">
         <f>IF(G24="","",$B$3-G24)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P24" s="6" t="str">
         <f>IF(H24="","Pending buy",IF(N24&gt;=0,"In profit","In loss"))</f>
@@ -1937,23 +1937,23 @@
         <v>99622.64</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>713.55</v>
+        <v>720.45</v>
       </c>
       <c r="L25" s="9">
         <f>IF(OR(I25="",K25=""),"",K25*I25)</f>
-        <v>88480.2</v>
+        <v>89335.8</v>
       </c>
       <c r="M25" s="9">
         <f>IF(L25="","",L25-J25)</f>
-        <v>-11142.44</v>
+        <v>-10286.84</v>
       </c>
       <c r="N25" s="10">
         <f>IF(OR(H25="",K25=""),"",K25/H25-1)</f>
-        <v>-0.11184643164989339</v>
+        <v>-0.10325802211781321</v>
       </c>
       <c r="O25" s="6">
         <f>IF(G25="","",$B$3-G25)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P25" s="6" t="str">
         <f>IF(H25="","Pending buy",IF(N25&gt;=0,"In profit","In loss"))</f>
@@ -2005,23 +2005,23 @@
         <v>99948.17</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>170.94</v>
+        <v>188.03</v>
       </c>
       <c r="L26" s="9">
         <f>IF(OR(I26="",K26=""),"",K26*I26)</f>
-        <v>81196.5</v>
+        <v>89314.25</v>
       </c>
       <c r="M26" s="9">
         <f>IF(L26="","",L26-J26)</f>
-        <v>-18751.67</v>
+        <v>-10633.92</v>
       </c>
       <c r="N26" s="10">
         <f>IF(OR(H26="",K26=""),"",K26/H26-1)</f>
-        <v>-0.18761391327941535</v>
+        <v>-0.10639431446079595</v>
       </c>
       <c r="O26" s="6">
         <f>IF(G26="","",$B$3-G26)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P26" s="6" t="str">
         <f>IF(H26="","Pending buy",IF(N26&gt;=0,"In profit","In loss"))</f>
@@ -2073,23 +2073,23 @@
         <v>99745.27</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>208.45</v>
+        <v>215</v>
       </c>
       <c r="L27" s="9">
         <f>IF(OR(I27="",K27=""),"",K27*I27)</f>
-        <v>79627.9</v>
+        <v>82130.0</v>
       </c>
       <c r="M27" s="9">
         <f>IF(L27="","",L27-J27)</f>
-        <v>-20117.37</v>
+        <v>-17615.27</v>
       </c>
       <c r="N27" s="10">
         <f>IF(OR(H27="",K27=""),"",K27/H27-1)</f>
-        <v>-0.20168748215333965</v>
+        <v>-0.17660258413513086</v>
       </c>
       <c r="O27" s="6">
         <f>IF(G27="","",$B$3-G27)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P27" s="6" t="str">
         <f>IF(H27="","Pending buy",IF(N27&gt;=0,"In profit","In loss"))</f>
@@ -2141,23 +2141,23 @@
         <v>95334.84</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>10726</v>
+        <v>11011</v>
       </c>
       <c r="L28" s="9">
         <f>IF(OR(I28="",K28=""),"",K28*I28)</f>
-        <v>96534.0</v>
+        <v>99099.0</v>
       </c>
       <c r="M28" s="9">
         <f>IF(L28="","",L28-J28)</f>
-        <v>1199.16</v>
+        <v>3764.16</v>
       </c>
       <c r="N28" s="10">
         <f>IF(OR(H28="",K28=""),"",K28/H28-1)</f>
-        <v>0.012578377179710776</v>
+        <v>0.03948354569511414</v>
       </c>
       <c r="O28" s="6">
         <f>IF(G28="","",$B$3-G28)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P28" s="6" t="str">
         <f>IF(H28="","Pending buy",IF(N28&gt;=0,"In profit","In loss"))</f>
@@ -2209,23 +2209,23 @@
         <v>98598.59</v>
       </c>
       <c r="K29" s="9" t="n">
-        <v>1758.4</v>
+        <v>1798.8</v>
       </c>
       <c r="L29" s="9">
         <f>IF(OR(I29="",K29=""),"",K29*I29)</f>
-        <v>89678.4</v>
+        <v>91738.8</v>
       </c>
       <c r="M29" s="9">
         <f>IF(L29="","",L29-J29)</f>
-        <v>-8920.19</v>
+        <v>-6859.79</v>
       </c>
       <c r="N29" s="10">
         <f>IF(OR(H29="",K29=""),"",K29/H29-1)</f>
-        <v>-0.09046971768141243</v>
+        <v>-0.06957286633605819</v>
       </c>
       <c r="O29" s="6">
         <f>IF(G29="","",$B$3-G29)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P29" s="6" t="str">
         <f>IF(H29="","Pending buy",IF(N29&gt;=0,"In profit","In loss"))</f>
@@ -2277,23 +2277,23 @@
         <v>99998.69</v>
       </c>
       <c r="K30" s="9" t="n">
-        <v>15.69</v>
+        <v>15.38</v>
       </c>
       <c r="L30" s="9">
         <f>IF(OR(I30="",K30=""),"",K30*I30)</f>
-        <v>105797.67</v>
+        <v>103707.34</v>
       </c>
       <c r="M30" s="9">
         <f>IF(L30="","",L30-J30)</f>
-        <v>5798.98</v>
+        <v>3708.65</v>
       </c>
       <c r="N30" s="10">
         <f>IF(OR(H30="",K30=""),"",K30/H30-1)</f>
-        <v>0.05799055967633171</v>
+        <v>0.03708698583951464</v>
       </c>
       <c r="O30" s="6">
         <f>IF(G30="","",$B$3-G30)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P30" s="6" t="str">
         <f>IF(H30="","Pending buy",IF(N30&gt;=0,"In profit","In loss"))</f>
@@ -2345,23 +2345,23 @@
         <v>99977.34</v>
       </c>
       <c r="K31" s="9" t="n">
-        <v>141.07</v>
+        <v>143.9</v>
       </c>
       <c r="L31" s="9">
         <f>IF(OR(I31="",K31=""),"",K31*I31)</f>
-        <v>79563.48</v>
+        <v>81159.6</v>
       </c>
       <c r="M31" s="9">
         <f>IF(L31="","",L31-J31)</f>
-        <v>-20413.86</v>
+        <v>-18817.74</v>
       </c>
       <c r="N31" s="10">
         <f>IF(OR(H31="",K31=""),"",K31/H31-1)</f>
-        <v>-0.20418485377219653</v>
+        <v>-0.18822003585325775</v>
       </c>
       <c r="O31" s="6">
         <f>IF(G31="","",$B$3-G31)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P31" s="6" t="str">
         <f>IF(H31="","Pending buy",IF(N31&gt;=0,"In profit","In loss"))</f>
@@ -2413,27 +2413,27 @@
         <v>99923.82</v>
       </c>
       <c r="K32" s="9" t="n">
-        <v>176.23</v>
+        <v>180.65</v>
       </c>
       <c r="L32" s="9">
         <f>IF(OR(I32="",K32=""),"",K32*I32)</f>
-        <v>99569.95</v>
+        <v>102067.25</v>
       </c>
       <c r="M32" s="9">
         <f>IF(L32="","",L32-J32)</f>
-        <v>-353.87</v>
+        <v>2143.43</v>
       </c>
       <c r="N32" s="10">
         <f>IF(OR(H32="",K32=""),"",K32/H32-1)</f>
-        <v>-0.003541394546051735</v>
+        <v>0.021450644471745717</v>
       </c>
       <c r="O32" s="6">
         <f>IF(G32="","",$B$3-G32)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P32" s="6" t="str">
         <f>IF(H32="","Pending buy",IF(N32&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q32" s="6" t="n">
         <v>1</v>
@@ -2481,23 +2481,23 @@
         <v>99608.58</v>
       </c>
       <c r="K33" s="9" t="n">
-        <v>522.8</v>
+        <v>505.2</v>
       </c>
       <c r="L33" s="9">
         <f>IF(OR(I33="",K33=""),"",K33*I33)</f>
-        <v>98809.2</v>
+        <v>95482.8</v>
       </c>
       <c r="M33" s="9">
         <f>IF(L33="","",L33-J33)</f>
-        <v>-799.38</v>
+        <v>-4125.78</v>
       </c>
       <c r="N33" s="10">
         <f>IF(OR(H33="",K33=""),"",K33/H33-1)</f>
-        <v>-0.008025163707250482</v>
+        <v>-0.04141987893057175</v>
       </c>
       <c r="O33" s="6">
         <f>IF(G33="","",$B$3-G33)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P33" s="6" t="str">
         <f>IF(H33="","Pending buy",IF(N33&gt;=0,"In profit","In loss"))</f>
@@ -2549,23 +2549,23 @@
         <v>96030.46</v>
       </c>
       <c r="K34" s="9" t="n">
-        <v>4286</v>
+        <v>4351.4</v>
       </c>
       <c r="L34" s="9">
         <f>IF(OR(I34="",K34=""),"",K34*I34)</f>
-        <v>81434.0</v>
+        <v>82676.6</v>
       </c>
       <c r="M34" s="9">
         <f>IF(L34="","",L34-J34)</f>
-        <v>-14596.46</v>
+        <v>-13353.86</v>
       </c>
       <c r="N34" s="10">
         <f>IF(OR(H34="",K34=""),"",K34/H34-1)</f>
-        <v>-0.15199823696357673</v>
+        <v>-0.1390585927025917</v>
       </c>
       <c r="O34" s="6">
         <f>IF(G34="","",$B$3-G34)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P34" s="6" t="str">
         <f>IF(H34="","Pending buy",IF(N34&gt;=0,"In profit","In loss"))</f>
@@ -2617,23 +2617,23 @@
         <v>99082.89</v>
       </c>
       <c r="K35" s="9" t="n">
-        <v>903.2</v>
+        <v>909.3</v>
       </c>
       <c r="L35" s="9">
         <f>IF(OR(I35="",K35=""),"",K35*I35)</f>
-        <v>82191.2</v>
+        <v>82746.3</v>
       </c>
       <c r="M35" s="9">
         <f>IF(L35="","",L35-J35)</f>
-        <v>-16891.69</v>
+        <v>-16336.59</v>
       </c>
       <c r="N35" s="10">
         <f>IF(OR(H35="",K35=""),"",K35/H35-1)</f>
-        <v>-0.17048041784569212</v>
+        <v>-0.16487803802821954</v>
       </c>
       <c r="O35" s="6">
         <f>IF(G35="","",$B$3-G35)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="P35" s="6" t="str">
         <f>IF(H35="","Pending buy",IF(N35&gt;=0,"In profit","In loss"))</f>
@@ -2685,23 +2685,23 @@
         <v>99910.57</v>
       </c>
       <c r="K36" s="9" t="n">
-        <v>88.64</v>
+        <v>90.95</v>
       </c>
       <c r="L36" s="9">
         <f>IF(OR(I36="",K36=""),"",K36*I36)</f>
-        <v>90856.0</v>
+        <v>93223.75</v>
       </c>
       <c r="M36" s="9">
         <f>IF(L36="","",L36-J36)</f>
-        <v>-9054.57</v>
+        <v>-6686.82</v>
       </c>
       <c r="N36" s="10">
         <f>IF(OR(H36="",K36=""),"",K36/H36-1)</f>
-        <v>-0.09062675842253609</v>
+        <v>-0.06692806496536163</v>
       </c>
       <c r="O36" s="6">
         <f>IF(G36="","",$B$3-G36)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="P36" s="6" t="str">
         <f>IF(H36="","Pending buy",IF(N36&gt;=0,"In profit","In loss"))</f>
@@ -2753,23 +2753,23 @@
         <v>99436.51</v>
       </c>
       <c r="K37" s="9" t="n">
-        <v>970.8</v>
+        <v>930.3</v>
       </c>
       <c r="L37" s="9">
         <f>IF(OR(I37="",K37=""),"",K37*I37)</f>
-        <v>97080.0</v>
+        <v>93030.0</v>
       </c>
       <c r="M37" s="9">
         <f>IF(L37="","",L37-J37)</f>
-        <v>-2356.51</v>
+        <v>-6406.51</v>
       </c>
       <c r="N37" s="10">
         <f>IF(OR(H37="",K37=""),"",K37/H37-1)</f>
-        <v>-0.023698667936695172</v>
+        <v>-0.06442817344613472</v>
       </c>
       <c r="O37" s="6">
         <f>IF(G37="","",$B$3-G37)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="P37" s="6" t="str">
         <f>IF(H37="","Pending buy",IF(N37&gt;=0,"In profit","In loss"))</f>
@@ -2821,23 +2821,23 @@
         <v>99951.48</v>
       </c>
       <c r="K38" s="9" t="n">
-        <v>112.6</v>
+        <v>116.25</v>
       </c>
       <c r="L38" s="9">
         <f>IF(OR(I38="",K38=""),"",K38*I38)</f>
-        <v>92219.4</v>
+        <v>95208.75</v>
       </c>
       <c r="M38" s="9">
         <f>IF(L38="","",L38-J38)</f>
-        <v>-7732.08</v>
+        <v>-4742.73</v>
       </c>
       <c r="N38" s="10">
         <f>IF(OR(H38="",K38=""),"",K38/H38-1)</f>
-        <v>-0.07735833334992626</v>
+        <v>-0.047450321953187546</v>
       </c>
       <c r="O38" s="6">
         <f>IF(G38="","",$B$3-G38)</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="P38" s="6" t="str">
         <f>IF(H38="","Pending buy",IF(N38&gt;=0,"In profit","In loss"))</f>
@@ -2889,23 +2889,23 @@
         <v>99666.78</v>
       </c>
       <c r="K39" s="9" t="n">
-        <v>486.75</v>
+        <v>485.05</v>
       </c>
       <c r="L39" s="9">
         <f>IF(OR(I39="",K39=""),"",K39*I39)</f>
-        <v>87128.25</v>
+        <v>86823.95</v>
       </c>
       <c r="M39" s="9">
         <f>IF(L39="","",L39-J39)</f>
-        <v>-12538.53</v>
+        <v>-12842.83</v>
       </c>
       <c r="N39" s="10">
         <f>IF(OR(H39="",K39=""),"",K39/H39-1)</f>
-        <v>-0.1258044718121215</v>
+        <v>-0.12885764571642433</v>
       </c>
       <c r="O39" s="6">
         <f>IF(G39="","",$B$3-G39)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P39" s="6" t="str">
         <f>IF(H39="","Pending buy",IF(N39&gt;=0,"In profit","In loss"))</f>
@@ -2957,23 +2957,23 @@
         <v>99998.64</v>
       </c>
       <c r="K40" s="9" t="n">
-        <v>12.23</v>
+        <v>12.63</v>
       </c>
       <c r="L40" s="9">
         <f>IF(OR(I40="",K40=""),"",K40*I40)</f>
-        <v>94391.14</v>
+        <v>97478.34</v>
       </c>
       <c r="M40" s="9">
         <f>IF(L40="","",L40-J40)</f>
-        <v>-5607.5</v>
+        <v>-2520.3</v>
       </c>
       <c r="N40" s="10">
         <f>IF(OR(H40="",K40=""),"",K40/H40-1)</f>
-        <v>-0.0560757386921269</v>
+        <v>-0.025203318044281442</v>
       </c>
       <c r="O40" s="6">
         <f>IF(G40="","",$B$3-G40)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P40" s="6" t="str">
         <f>IF(H40="","Pending buy",IF(N40&gt;=0,"In profit","In loss"))</f>
@@ -3025,23 +3025,23 @@
         <v>99889.82</v>
       </c>
       <c r="K41" s="9" t="n">
-        <v>119.81</v>
+        <v>121.27</v>
       </c>
       <c r="L41" s="9">
         <f>IF(OR(I41="",K41=""),"",K41*I41)</f>
-        <v>95248.95</v>
+        <v>96409.65</v>
       </c>
       <c r="M41" s="9">
         <f>IF(L41="","",L41-J41)</f>
-        <v>-4640.87</v>
+        <v>-3480.17</v>
       </c>
       <c r="N41" s="10">
         <f>IF(OR(H41="",K41=""),"",K41/H41-1)</f>
-        <v>-0.04645987943531349</v>
+        <v>-0.034840076613976145</v>
       </c>
       <c r="O41" s="6">
         <f>IF(G41="","",$B$3-G41)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P41" s="6" t="str">
         <f>IF(H41="","Pending buy",IF(N41&gt;=0,"In profit","In loss"))</f>
@@ -3093,23 +3093,23 @@
         <v>99925.2</v>
       </c>
       <c r="K42" s="9" t="n">
-        <v>109.87</v>
+        <v>115.58</v>
       </c>
       <c r="L42" s="9">
         <f>IF(OR(I42="",K42=""),"",K42*I42)</f>
-        <v>116791.81</v>
+        <v>122861.54</v>
       </c>
       <c r="M42" s="9">
         <f>IF(L42="","",L42-J42)</f>
-        <v>16866.61</v>
+        <v>22936.34</v>
       </c>
       <c r="N42" s="10">
         <f>IF(OR(H42="",K42=""),"",K42/H42-1)</f>
-        <v>0.168792373444131</v>
+        <v>0.22953510988142933</v>
       </c>
       <c r="O42" s="6">
         <f>IF(G42="","",$B$3-G42)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P42" s="6" t="str">
         <f>IF(H42="","Pending buy",IF(N42&gt;=0,"In profit","In loss"))</f>
@@ -3161,27 +3161,27 @@
         <v>99394.67</v>
       </c>
       <c r="K43" s="9" t="n">
-        <v>620.05</v>
+        <v>639.25</v>
       </c>
       <c r="L43" s="9">
         <f>IF(OR(I43="",K43=""),"",K43*I43)</f>
-        <v>97347.85</v>
+        <v>100362.25</v>
       </c>
       <c r="M43" s="9">
         <f>IF(L43="","",L43-J43)</f>
-        <v>-2046.82</v>
+        <v>967.58</v>
       </c>
       <c r="N43" s="10">
         <f>IF(OR(H43="",K43=""),"",K43/H43-1)</f>
-        <v>-0.020592876287458872</v>
+        <v>0.009734704996761545</v>
       </c>
       <c r="O43" s="6">
         <f>IF(G43="","",$B$3-G43)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P43" s="6" t="str">
         <f>IF(H43="","Pending buy",IF(N43&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q43" s="6" t="n">
         <v>1</v>
@@ -3229,30 +3229,30 @@
         <v>99810.88</v>
       </c>
       <c r="K44" s="9" t="n">
-        <v>337.05</v>
+        <v>368.8</v>
       </c>
       <c r="L44" s="9">
         <f>IF(OR(I44="",K44=""),"",K44*I44)</f>
-        <v>101789.1</v>
+        <v>111377.6</v>
       </c>
       <c r="M44" s="9">
         <f>IF(L44="","",L44-J44)</f>
-        <v>1978.22</v>
+        <v>11566.72</v>
       </c>
       <c r="N44" s="10">
         <f>IF(OR(H44="",K44=""),"",K44/H44-1)</f>
-        <v>0.019819678815712116</v>
+        <v>0.11588635973070649</v>
       </c>
       <c r="O44" s="6">
         <f>IF(G44="","",$B$3-G44)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P44" s="6" t="str">
         <f>IF(H44="","Pending buy",IF(N44&gt;=0,"In profit","In loss"))</f>
         <v>In profit</v>
       </c>
       <c r="Q44" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45">
@@ -3297,23 +3297,23 @@
         <v>99997.44</v>
       </c>
       <c r="K45" s="9" t="n">
-        <v>271.2</v>
+        <v>273.6</v>
       </c>
       <c r="L45" s="9">
         <f>IF(OR(I45="",K45=""),"",K45*I45)</f>
-        <v>100615.2</v>
+        <v>101505.6</v>
       </c>
       <c r="M45" s="9">
         <f>IF(L45="","",L45-J45)</f>
-        <v>617.76</v>
+        <v>1508.16</v>
       </c>
       <c r="N45" s="10">
         <f>IF(OR(H45="",K45=""),"",K45/H45-1)</f>
-        <v>0.006177783184952768</v>
+        <v>0.015082011354731195</v>
       </c>
       <c r="O45" s="6">
         <f>IF(G45="","",$B$3-G45)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P45" s="6" t="str">
         <f>IF(H45="","Pending buy",IF(N45&gt;=0,"In profit","In loss"))</f>
@@ -3365,27 +3365,27 @@
         <v>99870.37</v>
       </c>
       <c r="K46" s="9" t="n">
-        <v>366.75</v>
+        <v>358.1</v>
       </c>
       <c r="L46" s="9">
         <f>IF(OR(I46="",K46=""),"",K46*I46)</f>
-        <v>101956.5</v>
+        <v>99551.8</v>
       </c>
       <c r="M46" s="9">
         <f>IF(L46="","",L46-J46)</f>
-        <v>2086.13</v>
+        <v>-318.57</v>
       </c>
       <c r="N46" s="10">
         <f>IF(OR(H46="",K46=""),"",K46/H46-1)</f>
-        <v>0.02088842662924839</v>
+        <v>-0.0031897871140180722</v>
       </c>
       <c r="O46" s="6">
         <f>IF(G46="","",$B$3-G46)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P46" s="6" t="str">
         <f>IF(H46="","Pending buy",IF(N46&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q46" s="6" t="n">
         <v>1</v>
@@ -3433,27 +3433,27 @@
         <v>99957.4</v>
       </c>
       <c r="K47" s="9" t="n">
-        <v>560.85</v>
+        <v>578.55</v>
       </c>
       <c r="L47" s="9">
         <f>IF(OR(I47="",K47=""),"",K47*I47)</f>
-        <v>97027.05</v>
+        <v>100089.15</v>
       </c>
       <c r="M47" s="9">
         <f>IF(L47="","",L47-J47)</f>
-        <v>-2930.35</v>
+        <v>131.75</v>
       </c>
       <c r="N47" s="10">
         <f>IF(OR(H47="",K47=""),"",K47/H47-1)</f>
-        <v>-0.029315978016472344</v>
+        <v>0.0013180724232322305</v>
       </c>
       <c r="O47" s="6">
         <f>IF(G47="","",$B$3-G47)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P47" s="6" t="str">
         <f>IF(H47="","Pending buy",IF(N47&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q47" s="6" t="n">
         <v>1</v>
@@ -3501,30 +3501,30 @@
         <v>99965.44</v>
       </c>
       <c r="K48" s="9" t="n">
-        <v>181.2</v>
+        <v>184.6</v>
       </c>
       <c r="L48" s="9">
         <f>IF(OR(I48="",K48=""),"",K48*I48)</f>
-        <v>100928.4</v>
+        <v>102822.2</v>
       </c>
       <c r="M48" s="9">
         <f>IF(L48="","",L48-J48)</f>
-        <v>962.96</v>
+        <v>2856.76</v>
       </c>
       <c r="N48" s="10">
         <f>IF(OR(H48="",K48=""),"",K48/H48-1)</f>
-        <v>0.009632906446016332</v>
+        <v>0.028577453255709706</v>
       </c>
       <c r="O48" s="6">
         <f>IF(G48="","",$B$3-G48)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P48" s="6" t="str">
         <f>IF(H48="","Pending buy",IF(N48&gt;=0,"In profit","In loss"))</f>
         <v>In profit</v>
       </c>
       <c r="Q48" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49">
@@ -3569,23 +3569,23 @@
         <v>99985.7</v>
       </c>
       <c r="K49" s="9" t="n">
-        <v>867.55</v>
+        <v>910.9</v>
       </c>
       <c r="L49" s="9">
         <f>IF(OR(I49="",K49=""),"",K49*I49)</f>
-        <v>104106.0</v>
+        <v>109308.0</v>
       </c>
       <c r="M49" s="9">
         <f>IF(L49="","",L49-J49)</f>
-        <v>4120.3</v>
+        <v>9322.3</v>
       </c>
       <c r="N49" s="10">
         <f>IF(OR(H49="",K49=""),"",K49/H49-1)</f>
-        <v>0.0412089274447609</v>
+        <v>0.09323636909622812</v>
       </c>
       <c r="O49" s="6">
         <f>IF(G49="","",$B$3-G49)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P49" s="6" t="str">
         <f>IF(H49="","Pending buy",IF(N49&gt;=0,"In profit","In loss"))</f>
@@ -3622,38 +3622,42 @@
       <c r="F50" s="8" t="n">
         <v>46321</v>
       </c>
-      <c r="G50" s="6" t="inlineStr"/>
-      <c r="H50" s="9" t="inlineStr"/>
-      <c r="I50" s="6" t="str">
+      <c r="G50" s="8" t="n">
+        <v>46322</v>
+      </c>
+      <c r="H50" s="9" t="n">
+        <v>96.12</v>
+      </c>
+      <c r="I50" s="6">
         <f>IF(H50="","",ROUNDDOWN($B$1/H50,0))</f>
-        <v/>
-      </c>
-      <c r="J50" s="9" t="str">
+        <v>1040</v>
+      </c>
+      <c r="J50" s="9">
         <f>IF(H50="","",H50*I50)</f>
-        <v/>
+        <v>99961.35</v>
       </c>
       <c r="K50" s="9" t="n">
-        <v>94.62</v>
-      </c>
-      <c r="L50" s="9" t="str">
+        <v>95.95</v>
+      </c>
+      <c r="L50" s="9">
         <f>IF(OR(I50="",K50=""),"",K50*I50)</f>
-        <v/>
-      </c>
-      <c r="M50" s="9" t="str">
+        <v>99788.0</v>
+      </c>
+      <c r="M50" s="9">
         <f>IF(L50="","",L50-J50)</f>
-        <v/>
-      </c>
-      <c r="N50" s="10" t="str">
+        <v>-173.35</v>
+      </c>
+      <c r="N50" s="10">
         <f>IF(OR(H50="",K50=""),"",K50/H50-1)</f>
-        <v/>
-      </c>
-      <c r="O50" s="6" t="str">
+        <v>-0.0017341526805321195</v>
+      </c>
+      <c r="O50" s="6">
         <f>IF(G50="","",$B$3-G50)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P50" s="6" t="str">
         <f>IF(H50="","Pending buy",IF(N50&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q50" s="6" t="n">
         <v>1</v>
@@ -3686,38 +3690,42 @@
       <c r="F51" s="8" t="n">
         <v>46321</v>
       </c>
-      <c r="G51" s="6" t="inlineStr"/>
-      <c r="H51" s="9" t="inlineStr"/>
-      <c r="I51" s="6" t="str">
+      <c r="G51" s="8" t="n">
+        <v>46322</v>
+      </c>
+      <c r="H51" s="9" t="n">
+        <v>2965.99</v>
+      </c>
+      <c r="I51" s="6">
         <f>IF(H51="","",ROUNDDOWN($B$1/H51,0))</f>
-        <v/>
-      </c>
-      <c r="J51" s="9" t="str">
+        <v>33</v>
+      </c>
+      <c r="J51" s="9">
         <f>IF(H51="","",H51*I51)</f>
-        <v/>
+        <v>97877.65</v>
       </c>
       <c r="K51" s="9" t="n">
-        <v>2843.9</v>
-      </c>
-      <c r="L51" s="9" t="str">
+        <v>2960.3</v>
+      </c>
+      <c r="L51" s="9">
         <f>IF(OR(I51="",K51=""),"",K51*I51)</f>
-        <v/>
-      </c>
-      <c r="M51" s="9" t="str">
+        <v>97689.9</v>
+      </c>
+      <c r="M51" s="9">
         <f>IF(L51="","",L51-J51)</f>
-        <v/>
-      </c>
-      <c r="N51" s="10" t="str">
+        <v>-187.75</v>
+      </c>
+      <c r="N51" s="10">
         <f>IF(OR(H51="",K51=""),"",K51/H51-1)</f>
-        <v/>
-      </c>
-      <c r="O51" s="6" t="str">
+        <v>-0.001918179542994336</v>
+      </c>
+      <c r="O51" s="6">
         <f>IF(G51="","",$B$3-G51)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P51" s="6" t="str">
         <f>IF(H51="","Pending buy",IF(N51&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q51" s="6" t="n">
         <v>1</v>
@@ -3750,38 +3758,42 @@
       <c r="F52" s="8" t="n">
         <v>46321</v>
       </c>
-      <c r="G52" s="6" t="inlineStr"/>
-      <c r="H52" s="9" t="inlineStr"/>
-      <c r="I52" s="6" t="str">
+      <c r="G52" s="8" t="n">
+        <v>46322</v>
+      </c>
+      <c r="H52" s="9" t="n">
+        <v>911.54</v>
+      </c>
+      <c r="I52" s="6">
         <f>IF(H52="","",ROUNDDOWN($B$1/H52,0))</f>
-        <v/>
-      </c>
-      <c r="J52" s="9" t="str">
+        <v>109</v>
+      </c>
+      <c r="J52" s="9">
         <f>IF(H52="","",H52*I52)</f>
-        <v/>
+        <v>99357.46</v>
       </c>
       <c r="K52" s="9" t="n">
-        <v>900.8</v>
-      </c>
-      <c r="L52" s="9" t="str">
+        <v>904.7</v>
+      </c>
+      <c r="L52" s="9">
         <f>IF(OR(I52="",K52=""),"",K52*I52)</f>
-        <v/>
-      </c>
-      <c r="M52" s="9" t="str">
+        <v>98612.3</v>
+      </c>
+      <c r="M52" s="9">
         <f>IF(L52="","",L52-J52)</f>
-        <v/>
-      </c>
-      <c r="N52" s="10" t="str">
+        <v>-745.16</v>
+      </c>
+      <c r="N52" s="10">
         <f>IF(OR(H52="",K52=""),"",K52/H52-1)</f>
-        <v/>
-      </c>
-      <c r="O52" s="6" t="str">
+        <v>-0.007499764891427563</v>
+      </c>
+      <c r="O52" s="6">
         <f>IF(G52="","",$B$3-G52)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P52" s="6" t="str">
         <f>IF(H52="","Pending buy",IF(N52&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q52" s="6" t="n">
         <v>1</v>
@@ -3814,45 +3826,369 @@
       <c r="F53" s="8" t="n">
         <v>46321</v>
       </c>
-      <c r="G53" s="6" t="inlineStr"/>
-      <c r="H53" s="9" t="inlineStr"/>
-      <c r="I53" s="6" t="str">
+      <c r="G53" s="8" t="n">
+        <v>46322</v>
+      </c>
+      <c r="H53" s="9" t="n">
+        <v>845.3099999999999</v>
+      </c>
+      <c r="I53" s="6">
         <f>IF(H53="","",ROUNDDOWN($B$1/H53,0))</f>
-        <v/>
-      </c>
-      <c r="J53" s="9" t="str">
+        <v>118</v>
+      </c>
+      <c r="J53" s="9">
         <f>IF(H53="","",H53*I53)</f>
-        <v/>
+        <v>99747.01</v>
       </c>
       <c r="K53" s="9" t="n">
-        <v>781.9</v>
-      </c>
-      <c r="L53" s="9" t="str">
+        <v>851.85</v>
+      </c>
+      <c r="L53" s="9">
         <f>IF(OR(I53="",K53=""),"",K53*I53)</f>
-        <v/>
-      </c>
-      <c r="M53" s="9" t="str">
+        <v>100518.3</v>
+      </c>
+      <c r="M53" s="9">
         <f>IF(L53="","",L53-J53)</f>
-        <v/>
-      </c>
-      <c r="N53" s="10" t="str">
+        <v>771.29</v>
+      </c>
+      <c r="N53" s="10">
         <f>IF(OR(H53="",K53=""),"",K53/H53-1)</f>
-        <v/>
-      </c>
-      <c r="O53" s="6" t="str">
+        <v>0.007732464821619489</v>
+      </c>
+      <c r="O53" s="6">
         <f>IF(G53="","",$B$3-G53)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P53" s="6" t="str">
         <f>IF(H53="","Pending buy",IF(N53&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In profit</v>
       </c>
       <c r="Q53" s="6" t="n">
         <v>1</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Alivus Life Sciences Limited</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>ALIVUS</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>271026</t>
+        </is>
+      </c>
+      <c r="F54" s="8" t="n">
+        <v>46322</v>
+      </c>
+      <c r="G54" s="6" t="inlineStr"/>
+      <c r="H54" s="9" t="inlineStr"/>
+      <c r="I54" s="6" t="str">
+        <f>IF(H54="","",ROUNDDOWN($B$1/H54,0))</f>
+        <v/>
+      </c>
+      <c r="J54" s="9" t="str">
+        <f>IF(H54="","",H54*I54)</f>
+        <v/>
+      </c>
+      <c r="K54" s="9" t="n">
+        <v>1343.6</v>
+      </c>
+      <c r="L54" s="9" t="str">
+        <f>IF(OR(I54="",K54=""),"",K54*I54)</f>
+        <v/>
+      </c>
+      <c r="M54" s="9" t="str">
+        <f>IF(L54="","",L54-J54)</f>
+        <v/>
+      </c>
+      <c r="N54" s="10" t="str">
+        <f>IF(OR(H54="",K54=""),"",K54/H54-1)</f>
+        <v/>
+      </c>
+      <c r="O54" s="6" t="str">
+        <f>IF(G54="","",$B$3-G54)</f>
+        <v/>
+      </c>
+      <c r="P54" s="6" t="str">
+        <f>IF(H54="","Pending buy",IF(N54&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q54" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>KDDL Limited</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>KDDL</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>271026</t>
+        </is>
+      </c>
+      <c r="F55" s="8" t="n">
+        <v>46322</v>
+      </c>
+      <c r="G55" s="6" t="inlineStr"/>
+      <c r="H55" s="9" t="inlineStr"/>
+      <c r="I55" s="6" t="str">
+        <f>IF(H55="","",ROUNDDOWN($B$1/H55,0))</f>
+        <v/>
+      </c>
+      <c r="J55" s="9" t="str">
+        <f>IF(H55="","",H55*I55)</f>
+        <v/>
+      </c>
+      <c r="K55" s="9" t="n">
+        <v>3794.5</v>
+      </c>
+      <c r="L55" s="9" t="str">
+        <f>IF(OR(I55="",K55=""),"",K55*I55)</f>
+        <v/>
+      </c>
+      <c r="M55" s="9" t="str">
+        <f>IF(L55="","",L55-J55)</f>
+        <v/>
+      </c>
+      <c r="N55" s="10" t="str">
+        <f>IF(OR(H55="",K55=""),"",K55/H55-1)</f>
+        <v/>
+      </c>
+      <c r="O55" s="6" t="str">
+        <f>IF(G55="","",$B$3-G55)</f>
+        <v/>
+      </c>
+      <c r="P55" s="6" t="str">
+        <f>IF(H55="","Pending buy",IF(N55&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q55" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Kovai Medical Center &amp; Hospital Limited</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>KOVAI</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>271026</t>
+        </is>
+      </c>
+      <c r="F56" s="8" t="n">
+        <v>46322</v>
+      </c>
+      <c r="G56" s="6" t="inlineStr"/>
+      <c r="H56" s="9" t="inlineStr"/>
+      <c r="I56" s="6" t="str">
+        <f>IF(H56="","",ROUNDDOWN($B$1/H56,0))</f>
+        <v/>
+      </c>
+      <c r="J56" s="9" t="str">
+        <f>IF(H56="","",H56*I56)</f>
+        <v/>
+      </c>
+      <c r="K56" s="9" t="n">
+        <v>5862</v>
+      </c>
+      <c r="L56" s="9" t="str">
+        <f>IF(OR(I56="",K56=""),"",K56*I56)</f>
+        <v/>
+      </c>
+      <c r="M56" s="9" t="str">
+        <f>IF(L56="","",L56-J56)</f>
+        <v/>
+      </c>
+      <c r="N56" s="10" t="str">
+        <f>IF(OR(H56="",K56=""),"",K56/H56-1)</f>
+        <v/>
+      </c>
+      <c r="O56" s="6" t="str">
+        <f>IF(G56="","",$B$3-G56)</f>
+        <v/>
+      </c>
+      <c r="P56" s="6" t="str">
+        <f>IF(H56="","Pending buy",IF(N56&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q56" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Marine Electricals (India) Limited</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>MARINE</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>271026</t>
+        </is>
+      </c>
+      <c r="F57" s="8" t="n">
+        <v>46322</v>
+      </c>
+      <c r="G57" s="6" t="inlineStr"/>
+      <c r="H57" s="9" t="inlineStr"/>
+      <c r="I57" s="6" t="str">
+        <f>IF(H57="","",ROUNDDOWN($B$1/H57,0))</f>
+        <v/>
+      </c>
+      <c r="J57" s="9" t="str">
+        <f>IF(H57="","",H57*I57)</f>
+        <v/>
+      </c>
+      <c r="K57" s="9" t="n">
+        <v>425.25</v>
+      </c>
+      <c r="L57" s="9" t="str">
+        <f>IF(OR(I57="",K57=""),"",K57*I57)</f>
+        <v/>
+      </c>
+      <c r="M57" s="9" t="str">
+        <f>IF(L57="","",L57-J57)</f>
+        <v/>
+      </c>
+      <c r="N57" s="10" t="str">
+        <f>IF(OR(H57="",K57=""),"",K57/H57-1)</f>
+        <v/>
+      </c>
+      <c r="O57" s="6" t="str">
+        <f>IF(G57="","",$B$3-G57)</f>
+        <v/>
+      </c>
+      <c r="P57" s="6" t="str">
+        <f>IF(H57="","Pending buy",IF(N57&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q57" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Paisalo Digital Limited</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>PAISALO</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>271026</t>
+        </is>
+      </c>
+      <c r="F58" s="8" t="n">
+        <v>46322</v>
+      </c>
+      <c r="G58" s="6" t="inlineStr"/>
+      <c r="H58" s="9" t="inlineStr"/>
+      <c r="I58" s="6" t="str">
+        <f>IF(H58="","",ROUNDDOWN($B$1/H58,0))</f>
+        <v/>
+      </c>
+      <c r="J58" s="9" t="str">
+        <f>IF(H58="","",H58*I58)</f>
+        <v/>
+      </c>
+      <c r="K58" s="9" t="n">
+        <v>78.14</v>
+      </c>
+      <c r="L58" s="9" t="str">
+        <f>IF(OR(I58="",K58=""),"",K58*I58)</f>
+        <v/>
+      </c>
+      <c r="M58" s="9" t="str">
+        <f>IF(L58="","",L58-J58)</f>
+        <v/>
+      </c>
+      <c r="N58" s="10" t="str">
+        <f>IF(OR(H58="",K58=""),"",K58/H58-1)</f>
+        <v/>
+      </c>
+      <c r="O58" s="6" t="str">
+        <f>IF(G58="","",$B$3-G58)</f>
+        <v/>
+      </c>
+      <c r="P58" s="6" t="str">
+        <f>IF(H58="","Pending buy",IF(N58&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q58" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A8:Q53">
+  <conditionalFormatting sqref="A8:Q58">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$N8&gt;0</formula>
     </cfRule>
@@ -3870,7 +4206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D57"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5018,6 +5354,146 @@
       <c r="D57" s="11" t="inlineStr">
         <is>
           <t>Sona BLW Precision Forgings Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>UNIONBANK</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>Union Bank of India</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>ALIVUS</t>
+        </is>
+      </c>
+      <c r="D59" s="11" t="inlineStr">
+        <is>
+          <t>Alivus Life Sciences Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>INDSWFTLAB</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>Ind-Swift Laboratories Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>KDDL</t>
+        </is>
+      </c>
+      <c r="D61" s="11" t="inlineStr">
+        <is>
+          <t>KDDL Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>KOVAI</t>
+        </is>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>Kovai Medical Center &amp; Hospital Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>MARINE</t>
+        </is>
+      </c>
+      <c r="D63" s="11" t="inlineStr">
+        <is>
+          <t>Marine Electricals (India) Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>PAISALO</t>
+        </is>
+      </c>
+      <c r="D64" s="11" t="inlineStr">
+        <is>
+          <t>Paisalo Digital Limited</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum Portfolio: weekday silent update 2026-10-28
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="E1" s="2">
         <f>SUM(J8:J58)</f>
-        <v>4559576.06</v>
+        <v>5052225.67</v>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
@@ -541,7 +541,7 @@
       </c>
       <c r="G1" s="2">
         <f>SUM(L8:L58)</f>
-        <v>4353060.57</v>
+        <v>4877626.59</v>
       </c>
     </row>
     <row r="2">
@@ -552,7 +552,7 @@
       </c>
       <c r="E2" s="2">
         <f>SUM(M8:M58)</f>
-        <v>-206515.49</v>
+        <v>-174599.08</v>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" s="3">
         <f>IF(E1=0,"",G1/E1-1)</f>
-        <v>-0.04529269547923698</v>
+        <v>-0.034558844241017406</v>
       </c>
     </row>
     <row r="3">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -580,7 +580,7 @@
       </c>
       <c r="E3">
         <f>COUNTIF(M8:M58,"&gt;0")</f>
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
@@ -589,7 +589,7 @@
       </c>
       <c r="G3">
         <f>COUNTIF(M8:M58,"&lt;0")</f>
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4">
@@ -600,7 +600,7 @@
       </c>
       <c r="E4" s="3">
         <f>IF((E3+G3)=0,"",E3/(E3+G3))</f>
-        <v>0.2826086956521739</v>
+        <v>0.3137254901960784</v>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
@@ -609,7 +609,7 @@
       </c>
       <c r="G4" s="3">
         <f>AVERAGE(N8:N58)</f>
-        <v>-0.045462774731276995</v>
+        <v>-0.03463787225409552</v>
       </c>
     </row>
     <row r="5">
@@ -640,7 +640,7 @@
       </c>
       <c r="E6" s="3">
         <f>AVERAGEIF(D8:D58,"4★*",N8:N58)</f>
-        <v>-0.08442613176186621</v>
+        <v>-0.06951575929167718</v>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
@@ -649,7 +649,7 @@
       </c>
       <c r="G6" s="3">
         <f>AVERAGEIF(D8:D58,"5★*",N8:N58)</f>
-        <v>-0.01804411608012162</v>
+        <v>-0.01392912682553141</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
@@ -781,23 +781,23 @@
         <v>99851.29</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>278.7</v>
+        <v>284.85</v>
       </c>
       <c r="L8" s="9">
         <f>IF(OR(I8="",K8=""),"",K8*I8)</f>
-        <v>92528.4</v>
+        <v>94570.2</v>
       </c>
       <c r="M8" s="9">
         <f>IF(L8="","",L8-J8)</f>
-        <v>-7322.89</v>
+        <v>-5281.09</v>
       </c>
       <c r="N8" s="10">
         <f>IF(OR(H8="",K8=""),"",K8/H8-1)</f>
-        <v>-0.07333799295476207</v>
+        <v>-0.052889584833742176</v>
       </c>
       <c r="O8" s="6">
         <f>IF(G8="","",$B$3-G8)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P8" s="6" t="str">
         <f>IF(H8="","Pending buy",IF(N8&gt;=0,"In profit","In loss"))</f>
@@ -849,23 +849,23 @@
         <v>99687.42</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="L9" s="9">
         <f>IF(OR(I9="",K9=""),"",K9*I9)</f>
-        <v>101286.0</v>
+        <v>99756.0</v>
       </c>
       <c r="M9" s="9">
         <f>IF(L9="","",L9-J9)</f>
-        <v>1598.58</v>
+        <v>68.58</v>
       </c>
       <c r="N9" s="10">
         <f>IF(OR(H9="",K9=""),"",K9/H9-1)</f>
-        <v>0.01603592307660162</v>
+        <v>0.0006879484077708664</v>
       </c>
       <c r="O9" s="6">
         <f>IF(G9="","",$B$3-G9)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P9" s="6" t="str">
         <f>IF(H9="","Pending buy",IF(N9&gt;=0,"In profit","In loss"))</f>
@@ -917,23 +917,23 @@
         <v>99607.14</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>1474</v>
+        <v>1450.6</v>
       </c>
       <c r="L10" s="9">
         <f>IF(OR(I10="",K10=""),"",K10*I10)</f>
-        <v>92862.0</v>
+        <v>91387.8</v>
       </c>
       <c r="M10" s="9">
         <f>IF(L10="","",L10-J10)</f>
-        <v>-6745.14</v>
+        <v>-8219.34</v>
       </c>
       <c r="N10" s="10">
         <f>IF(OR(H10="",K10=""),"",K10/H10-1)</f>
-        <v>-0.06771744339036267</v>
+        <v>-0.08251758709773416</v>
       </c>
       <c r="O10" s="6">
         <f>IF(G10="","",$B$3-G10)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P10" s="6" t="str">
         <f>IF(H10="","Pending buy",IF(N10&gt;=0,"In profit","In loss"))</f>
@@ -985,23 +985,23 @@
         <v>99927.23</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>61.25</v>
+        <v>61.71</v>
       </c>
       <c r="L11" s="9">
         <f>IF(OR(I11="",K11=""),"",K11*I11)</f>
-        <v>76623.75</v>
+        <v>77199.21</v>
       </c>
       <c r="M11" s="9">
         <f>IF(L11="","",L11-J11)</f>
-        <v>-23303.48</v>
+        <v>-22728.02</v>
       </c>
       <c r="N11" s="10">
         <f>IF(OR(H11="",K11=""),"",K11/H11-1)</f>
-        <v>-0.2332045058480644</v>
+        <v>-0.22744571519810697</v>
       </c>
       <c r="O11" s="6">
         <f>IF(G11="","",$B$3-G11)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P11" s="6" t="str">
         <f>IF(H11="","Pending buy",IF(N11&gt;=0,"In profit","In loss"))</f>
@@ -1053,23 +1053,23 @@
         <v>86537.12</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>19315</v>
+        <v>19970</v>
       </c>
       <c r="L12" s="9">
         <f>IF(OR(I12="",K12=""),"",K12*I12)</f>
-        <v>77260.0</v>
+        <v>79880.0</v>
       </c>
       <c r="M12" s="9">
         <f>IF(L12="","",L12-J12)</f>
-        <v>-9277.12</v>
+        <v>-6657.12</v>
       </c>
       <c r="N12" s="10">
         <f>IF(OR(H12="",K12=""),"",K12/H12-1)</f>
-        <v>-0.1072038976315256</v>
+        <v>-0.0769278713798377</v>
       </c>
       <c r="O12" s="6">
         <f>IF(G12="","",$B$3-G12)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P12" s="6" t="str">
         <f>IF(H12="","Pending buy",IF(N12&gt;=0,"In profit","In loss"))</f>
@@ -1121,23 +1121,23 @@
         <v>98177.53</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>1690.8</v>
+        <v>1744.7</v>
       </c>
       <c r="L13" s="9">
         <f>IF(OR(I13="",K13=""),"",K13*I13)</f>
-        <v>89612.4</v>
+        <v>92469.1</v>
       </c>
       <c r="M13" s="9">
         <f>IF(L13="","",L13-J13)</f>
-        <v>-8565.13</v>
+        <v>-5708.43</v>
       </c>
       <c r="N13" s="10">
         <f>IF(OR(H13="",K13=""),"",K13/H13-1)</f>
-        <v>-0.08724127488736022</v>
+        <v>-0.058143986453736196</v>
       </c>
       <c r="O13" s="6">
         <f>IF(G13="","",$B$3-G13)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P13" s="6" t="str">
         <f>IF(H13="","Pending buy",IF(N13&gt;=0,"In profit","In loss"))</f>
@@ -1189,23 +1189,23 @@
         <v>97667.46</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>4290</v>
+        <v>4135.1</v>
       </c>
       <c r="L14" s="9">
         <f>IF(OR(I14="",K14=""),"",K14*I14)</f>
-        <v>94380.0</v>
+        <v>90972.2</v>
       </c>
       <c r="M14" s="9">
         <f>IF(L14="","",L14-J14)</f>
-        <v>-3287.46</v>
+        <v>-6695.26</v>
       </c>
       <c r="N14" s="10">
         <f>IF(OR(H14="",K14=""),"",K14/H14-1)</f>
-        <v>-0.03365976794422798</v>
+        <v>-0.06855163319957502</v>
       </c>
       <c r="O14" s="6">
         <f>IF(G14="","",$B$3-G14)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P14" s="6" t="str">
         <f>IF(H14="","Pending buy",IF(N14&gt;=0,"In profit","In loss"))</f>
@@ -1257,23 +1257,23 @@
         <v>99078.19</v>
       </c>
       <c r="K15" s="9" t="n">
-        <v>1370.7</v>
+        <v>1365.4</v>
       </c>
       <c r="L15" s="9">
         <f>IF(OR(I15="",K15=""),"",K15*I15)</f>
-        <v>87724.8</v>
+        <v>87385.6</v>
       </c>
       <c r="M15" s="9">
         <f>IF(L15="","",L15-J15)</f>
-        <v>-11353.39</v>
+        <v>-11692.59</v>
       </c>
       <c r="N15" s="10">
         <f>IF(OR(H15="",K15=""),"",K15/H15-1)</f>
-        <v>-0.11459018236859064</v>
+        <v>-0.11801374115858587</v>
       </c>
       <c r="O15" s="6">
         <f>IF(G15="","",$B$3-G15)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P15" s="6" t="str">
         <f>IF(H15="","Pending buy",IF(N15&gt;=0,"In profit","In loss"))</f>
@@ -1325,23 +1325,23 @@
         <v>98557.54</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>1674</v>
+        <v>1650</v>
       </c>
       <c r="L16" s="9">
         <f>IF(OR(I16="",K16=""),"",K16*I16)</f>
-        <v>113832.0</v>
+        <v>112200.0</v>
       </c>
       <c r="M16" s="9">
         <f>IF(L16="","",L16-J16)</f>
-        <v>15274.46</v>
+        <v>13642.46</v>
       </c>
       <c r="N16" s="10">
         <f>IF(OR(H16="",K16=""),"",K16/H16-1)</f>
-        <v>0.15498016715870655</v>
+        <v>0.13842131171557104</v>
       </c>
       <c r="O16" s="6">
         <f>IF(G16="","",$B$3-G16)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P16" s="6" t="str">
         <f>IF(H16="","Pending buy",IF(N16&gt;=0,"In profit","In loss"))</f>
@@ -1393,23 +1393,23 @@
         <v>99714.35</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>809.15</v>
+        <v>811.65</v>
       </c>
       <c r="L17" s="9">
         <f>IF(OR(I17="",K17=""),"",K17*I17)</f>
-        <v>93052.25</v>
+        <v>93339.75</v>
       </c>
       <c r="M17" s="9">
         <f>IF(L17="","",L17-J17)</f>
-        <v>-6662.1</v>
+        <v>-6374.6</v>
       </c>
       <c r="N17" s="10">
         <f>IF(OR(H17="",K17=""),"",K17/H17-1)</f>
-        <v>-0.06681184874583368</v>
+        <v>-0.06392861278447248</v>
       </c>
       <c r="O17" s="6">
         <f>IF(G17="","",$B$3-G17)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P17" s="6" t="str">
         <f>IF(H17="","Pending buy",IF(N17&gt;=0,"In profit","In loss"))</f>
@@ -1461,23 +1461,23 @@
         <v>99596.83</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>597.5</v>
+        <v>591.3</v>
       </c>
       <c r="L18" s="9">
         <f>IF(OR(I18="",K18=""),"",K18*I18)</f>
-        <v>84247.5</v>
+        <v>83373.3</v>
       </c>
       <c r="M18" s="9">
         <f>IF(L18="","",L18-J18)</f>
-        <v>-15349.33</v>
+        <v>-16223.53</v>
       </c>
       <c r="N18" s="10">
         <f>IF(OR(H18="",K18=""),"",K18/H18-1)</f>
-        <v>-0.15411468298506814</v>
+        <v>-0.16289207037501396</v>
       </c>
       <c r="O18" s="6">
         <f>IF(G18="","",$B$3-G18)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P18" s="6" t="str">
         <f>IF(H18="","Pending buy",IF(N18&gt;=0,"In profit","In loss"))</f>
@@ -1529,23 +1529,23 @@
         <v>99993.07</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>125.81</v>
+        <v>126.44</v>
       </c>
       <c r="L19" s="9">
         <f>IF(OR(I19="",K19=""),"",K19*I19)</f>
-        <v>83412.03</v>
+        <v>83829.72</v>
       </c>
       <c r="M19" s="9">
         <f>IF(L19="","",L19-J19)</f>
-        <v>-16581.04</v>
+        <v>-16163.35</v>
       </c>
       <c r="N19" s="10">
         <f>IF(OR(H19="",K19=""),"",K19/H19-1)</f>
-        <v>-0.16582185215622192</v>
+        <v>-0.16164466248019005</v>
       </c>
       <c r="O19" s="6">
         <f>IF(G19="","",$B$3-G19)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P19" s="6" t="str">
         <f>IF(H19="","Pending buy",IF(N19&gt;=0,"In profit","In loss"))</f>
@@ -1597,23 +1597,23 @@
         <v>99896.43</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>201.12</v>
+        <v>207.01</v>
       </c>
       <c r="L20" s="9">
         <f>IF(OR(I20="",K20=""),"",K20*I20)</f>
-        <v>95934.24</v>
+        <v>98743.77</v>
       </c>
       <c r="M20" s="9">
         <f>IF(L20="","",L20-J20)</f>
-        <v>-3962.19</v>
+        <v>-1152.66</v>
       </c>
       <c r="N20" s="10">
         <f>IF(OR(H20="",K20=""),"",K20/H20-1)</f>
-        <v>-0.03966297900497562</v>
+        <v>-0.01153855053609798</v>
       </c>
       <c r="O20" s="6">
         <f>IF(G20="","",$B$3-G20)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P20" s="6" t="str">
         <f>IF(H20="","Pending buy",IF(N20&gt;=0,"In profit","In loss"))</f>
@@ -1665,23 +1665,23 @@
         <v>99449.47</v>
       </c>
       <c r="K21" s="9" t="n">
-        <v>1311</v>
+        <v>1324.3</v>
       </c>
       <c r="L21" s="9">
         <f>IF(OR(I21="",K21=""),"",K21*I21)</f>
-        <v>93081.0</v>
+        <v>94025.3</v>
       </c>
       <c r="M21" s="9">
         <f>IF(L21="","",L21-J21)</f>
-        <v>-6368.47</v>
+        <v>-5424.17</v>
       </c>
       <c r="N21" s="10">
         <f>IF(OR(H21="",K21=""),"",K21/H21-1)</f>
-        <v>-0.06403720978543403</v>
+        <v>-0.05454193510209793</v>
       </c>
       <c r="O21" s="6">
         <f>IF(G21="","",$B$3-G21)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P21" s="6" t="str">
         <f>IF(H21="","Pending buy",IF(N21&gt;=0,"In profit","In loss"))</f>
@@ -1733,23 +1733,23 @@
         <v>99837.05</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>656</v>
+        <v>674.8</v>
       </c>
       <c r="L22" s="9">
         <f>IF(OR(I22="",K22=""),"",K22*I22)</f>
-        <v>94464.0</v>
+        <v>97171.2</v>
       </c>
       <c r="M22" s="9">
         <f>IF(L22="","",L22-J22)</f>
-        <v>-5373.05</v>
+        <v>-2665.85</v>
       </c>
       <c r="N22" s="10">
         <f>IF(OR(H22="",K22=""),"",K22/H22-1)</f>
-        <v>-0.05381820736613918</v>
+        <v>-0.026702021845534718</v>
       </c>
       <c r="O22" s="6">
         <f>IF(G22="","",$B$3-G22)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P22" s="6" t="str">
         <f>IF(H22="","Pending buy",IF(N22&gt;=0,"In profit","In loss"))</f>
@@ -1801,23 +1801,23 @@
         <v>99486.88</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>564.5</v>
+        <v>568.45</v>
       </c>
       <c r="L23" s="9">
         <f>IF(OR(I23="",K23=""),"",K23*I23)</f>
-        <v>81852.5</v>
+        <v>82425.25</v>
       </c>
       <c r="M23" s="9">
         <f>IF(L23="","",L23-J23)</f>
-        <v>-17634.38</v>
+        <v>-17061.63</v>
       </c>
       <c r="N23" s="10">
         <f>IF(OR(H23="",K23=""),"",K23/H23-1)</f>
-        <v>-0.17725333208829674</v>
+        <v>-0.17149629163081004</v>
       </c>
       <c r="O23" s="6">
         <f>IF(G23="","",$B$3-G23)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P23" s="6" t="str">
         <f>IF(H23="","Pending buy",IF(N23&gt;=0,"In profit","In loss"))</f>
@@ -1869,27 +1869,27 @@
         <v>99935.4</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>215.92</v>
+        <v>230.04</v>
       </c>
       <c r="L24" s="9">
         <f>IF(OR(I24="",K24=""),"",K24*I24)</f>
-        <v>94788.88</v>
+        <v>100987.56</v>
       </c>
       <c r="M24" s="9">
         <f>IF(L24="","",L24-J24)</f>
-        <v>-5146.52</v>
+        <v>1052.16</v>
       </c>
       <c r="N24" s="10">
         <f>IF(OR(H24="",K24=""),"",K24/H24-1)</f>
-        <v>-0.05149845475120285</v>
+        <v>0.010528415473477715</v>
       </c>
       <c r="O24" s="6">
         <f>IF(G24="","",$B$3-G24)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="P24" s="6" t="str">
         <f>IF(H24="","Pending buy",IF(N24&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q24" s="6" t="n">
         <v>1</v>
@@ -1937,23 +1937,23 @@
         <v>99622.64</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>720.45</v>
+        <v>731.25</v>
       </c>
       <c r="L25" s="9">
         <f>IF(OR(I25="",K25=""),"",K25*I25)</f>
-        <v>89335.8</v>
+        <v>90675.0</v>
       </c>
       <c r="M25" s="9">
         <f>IF(L25="","",L25-J25)</f>
-        <v>-10286.84</v>
+        <v>-8947.64</v>
       </c>
       <c r="N25" s="10">
         <f>IF(OR(H25="",K25=""),"",K25/H25-1)</f>
-        <v>-0.10325802211781321</v>
+        <v>-0.08981529415455747</v>
       </c>
       <c r="O25" s="6">
         <f>IF(G25="","",$B$3-G25)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P25" s="6" t="str">
         <f>IF(H25="","Pending buy",IF(N25&gt;=0,"In profit","In loss"))</f>
@@ -2005,23 +2005,23 @@
         <v>99948.17</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>188.03</v>
+        <v>193.68</v>
       </c>
       <c r="L26" s="9">
         <f>IF(OR(I26="",K26=""),"",K26*I26)</f>
-        <v>89314.25</v>
+        <v>91998.0</v>
       </c>
       <c r="M26" s="9">
         <f>IF(L26="","",L26-J26)</f>
-        <v>-10633.92</v>
+        <v>-7950.17</v>
       </c>
       <c r="N26" s="10">
         <f>IF(OR(H26="",K26=""),"",K26/H26-1)</f>
-        <v>-0.10639431446079595</v>
+        <v>-0.0795428964780458</v>
       </c>
       <c r="O26" s="6">
         <f>IF(G26="","",$B$3-G26)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P26" s="6" t="str">
         <f>IF(H26="","Pending buy",IF(N26&gt;=0,"In profit","In loss"))</f>
@@ -2073,23 +2073,23 @@
         <v>99745.27</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>215</v>
+        <v>210.4</v>
       </c>
       <c r="L27" s="9">
         <f>IF(OR(I27="",K27=""),"",K27*I27)</f>
-        <v>82130.0</v>
+        <v>80372.8</v>
       </c>
       <c r="M27" s="9">
         <f>IF(L27="","",L27-J27)</f>
-        <v>-17615.27</v>
+        <v>-19372.47</v>
       </c>
       <c r="N27" s="10">
         <f>IF(OR(H27="",K27=""),"",K27/H27-1)</f>
-        <v>-0.17660258413513086</v>
+        <v>-0.19421945907921645</v>
       </c>
       <c r="O27" s="6">
         <f>IF(G27="","",$B$3-G27)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P27" s="6" t="str">
         <f>IF(H27="","Pending buy",IF(N27&gt;=0,"In profit","In loss"))</f>
@@ -2141,23 +2141,23 @@
         <v>95334.84</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>11011</v>
+        <v>11014</v>
       </c>
       <c r="L28" s="9">
         <f>IF(OR(I28="",K28=""),"",K28*I28)</f>
-        <v>99099.0</v>
+        <v>99126.0</v>
       </c>
       <c r="M28" s="9">
         <f>IF(L28="","",L28-J28)</f>
-        <v>3764.16</v>
+        <v>3791.16</v>
       </c>
       <c r="N28" s="10">
         <f>IF(OR(H28="",K28=""),"",K28/H28-1)</f>
-        <v>0.03948354569511414</v>
+        <v>0.03976675799527629</v>
       </c>
       <c r="O28" s="6">
         <f>IF(G28="","",$B$3-G28)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P28" s="6" t="str">
         <f>IF(H28="","Pending buy",IF(N28&gt;=0,"In profit","In loss"))</f>
@@ -2209,23 +2209,23 @@
         <v>98598.59</v>
       </c>
       <c r="K29" s="9" t="n">
-        <v>1798.8</v>
+        <v>1784.6</v>
       </c>
       <c r="L29" s="9">
         <f>IF(OR(I29="",K29=""),"",K29*I29)</f>
-        <v>91738.8</v>
+        <v>91014.6</v>
       </c>
       <c r="M29" s="9">
         <f>IF(L29="","",L29-J29)</f>
-        <v>-6859.79</v>
+        <v>-7583.99</v>
       </c>
       <c r="N29" s="10">
         <f>IF(OR(H29="",K29=""),"",K29/H29-1)</f>
-        <v>-0.06957286633605819</v>
+        <v>-0.07691779923467279</v>
       </c>
       <c r="O29" s="6">
         <f>IF(G29="","",$B$3-G29)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P29" s="6" t="str">
         <f>IF(H29="","Pending buy",IF(N29&gt;=0,"In profit","In loss"))</f>
@@ -2277,23 +2277,23 @@
         <v>99998.69</v>
       </c>
       <c r="K30" s="9" t="n">
-        <v>15.38</v>
+        <v>15.08</v>
       </c>
       <c r="L30" s="9">
         <f>IF(OR(I30="",K30=""),"",K30*I30)</f>
-        <v>103707.34</v>
+        <v>101684.44</v>
       </c>
       <c r="M30" s="9">
         <f>IF(L30="","",L30-J30)</f>
-        <v>3708.65</v>
+        <v>1685.75</v>
       </c>
       <c r="N30" s="10">
         <f>IF(OR(H30="",K30=""),"",K30/H30-1)</f>
-        <v>0.03708698583951464</v>
+        <v>0.016857720836142898</v>
       </c>
       <c r="O30" s="6">
         <f>IF(G30="","",$B$3-G30)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P30" s="6" t="str">
         <f>IF(H30="","Pending buy",IF(N30&gt;=0,"In profit","In loss"))</f>
@@ -2345,23 +2345,23 @@
         <v>99977.34</v>
       </c>
       <c r="K31" s="9" t="n">
-        <v>143.9</v>
+        <v>145.83</v>
       </c>
       <c r="L31" s="9">
         <f>IF(OR(I31="",K31=""),"",K31*I31)</f>
-        <v>81159.6</v>
+        <v>82248.12</v>
       </c>
       <c r="M31" s="9">
         <f>IF(L31="","",L31-J31)</f>
-        <v>-18817.74</v>
+        <v>-17729.22</v>
       </c>
       <c r="N31" s="10">
         <f>IF(OR(H31="",K31=""),"",K31/H31-1)</f>
-        <v>-0.18822003585325775</v>
+        <v>-0.1773323685092465</v>
       </c>
       <c r="O31" s="6">
         <f>IF(G31="","",$B$3-G31)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P31" s="6" t="str">
         <f>IF(H31="","Pending buy",IF(N31&gt;=0,"In profit","In loss"))</f>
@@ -2413,23 +2413,23 @@
         <v>99923.82</v>
       </c>
       <c r="K32" s="9" t="n">
-        <v>180.65</v>
+        <v>178.52</v>
       </c>
       <c r="L32" s="9">
         <f>IF(OR(I32="",K32=""),"",K32*I32)</f>
-        <v>102067.25</v>
+        <v>100863.8</v>
       </c>
       <c r="M32" s="9">
         <f>IF(L32="","",L32-J32)</f>
-        <v>2143.43</v>
+        <v>939.98</v>
       </c>
       <c r="N32" s="10">
         <f>IF(OR(H32="",K32=""),"",K32/H32-1)</f>
-        <v>0.021450644471745717</v>
+        <v>0.009406969560454392</v>
       </c>
       <c r="O32" s="6">
         <f>IF(G32="","",$B$3-G32)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P32" s="6" t="str">
         <f>IF(H32="","Pending buy",IF(N32&gt;=0,"In profit","In loss"))</f>
@@ -2481,23 +2481,23 @@
         <v>99608.58</v>
       </c>
       <c r="K33" s="9" t="n">
-        <v>505.2</v>
+        <v>508.1</v>
       </c>
       <c r="L33" s="9">
         <f>IF(OR(I33="",K33=""),"",K33*I33)</f>
-        <v>95482.8</v>
+        <v>96030.9</v>
       </c>
       <c r="M33" s="9">
         <f>IF(L33="","",L33-J33)</f>
-        <v>-4125.78</v>
+        <v>-3577.68</v>
       </c>
       <c r="N33" s="10">
         <f>IF(OR(H33="",K33=""),"",K33/H33-1)</f>
-        <v>-0.04141987893057175</v>
+        <v>-0.03591734062672891</v>
       </c>
       <c r="O33" s="6">
         <f>IF(G33="","",$B$3-G33)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P33" s="6" t="str">
         <f>IF(H33="","Pending buy",IF(N33&gt;=0,"In profit","In loss"))</f>
@@ -2549,23 +2549,23 @@
         <v>96030.46</v>
       </c>
       <c r="K34" s="9" t="n">
-        <v>4351.4</v>
+        <v>4403.9</v>
       </c>
       <c r="L34" s="9">
         <f>IF(OR(I34="",K34=""),"",K34*I34)</f>
-        <v>82676.6</v>
+        <v>83674.1</v>
       </c>
       <c r="M34" s="9">
         <f>IF(L34="","",L34-J34)</f>
-        <v>-13353.86</v>
+        <v>-12356.36</v>
       </c>
       <c r="N34" s="10">
         <f>IF(OR(H34="",K34=""),"",K34/H34-1)</f>
-        <v>-0.1390585927025917</v>
+        <v>-0.12867126359400272</v>
       </c>
       <c r="O34" s="6">
         <f>IF(G34="","",$B$3-G34)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P34" s="6" t="str">
         <f>IF(H34="","Pending buy",IF(N34&gt;=0,"In profit","In loss"))</f>
@@ -2617,23 +2617,23 @@
         <v>99082.89</v>
       </c>
       <c r="K35" s="9" t="n">
-        <v>909.3</v>
+        <v>938.5</v>
       </c>
       <c r="L35" s="9">
         <f>IF(OR(I35="",K35=""),"",K35*I35)</f>
-        <v>82746.3</v>
+        <v>85403.5</v>
       </c>
       <c r="M35" s="9">
         <f>IF(L35="","",L35-J35)</f>
-        <v>-16336.59</v>
+        <v>-13679.39</v>
       </c>
       <c r="N35" s="10">
         <f>IF(OR(H35="",K35=""),"",K35/H35-1)</f>
-        <v>-0.16487803802821954</v>
+        <v>-0.13806008873802267</v>
       </c>
       <c r="O35" s="6">
         <f>IF(G35="","",$B$3-G35)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P35" s="6" t="str">
         <f>IF(H35="","Pending buy",IF(N35&gt;=0,"In profit","In loss"))</f>
@@ -2685,23 +2685,23 @@
         <v>99910.57</v>
       </c>
       <c r="K36" s="9" t="n">
-        <v>90.95</v>
+        <v>89.41</v>
       </c>
       <c r="L36" s="9">
         <f>IF(OR(I36="",K36=""),"",K36*I36)</f>
-        <v>93223.75</v>
+        <v>91645.25</v>
       </c>
       <c r="M36" s="9">
         <f>IF(L36="","",L36-J36)</f>
-        <v>-6686.82</v>
+        <v>-8265.32</v>
       </c>
       <c r="N36" s="10">
         <f>IF(OR(H36="",K36=""),"",K36/H36-1)</f>
-        <v>-0.06692806496536163</v>
+        <v>-0.08272719393681138</v>
       </c>
       <c r="O36" s="6">
         <f>IF(G36="","",$B$3-G36)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P36" s="6" t="str">
         <f>IF(H36="","Pending buy",IF(N36&gt;=0,"In profit","In loss"))</f>
@@ -2753,23 +2753,23 @@
         <v>99436.51</v>
       </c>
       <c r="K37" s="9" t="n">
-        <v>930.3</v>
+        <v>989</v>
       </c>
       <c r="L37" s="9">
         <f>IF(OR(I37="",K37=""),"",K37*I37)</f>
-        <v>93030.0</v>
+        <v>98900.0</v>
       </c>
       <c r="M37" s="9">
         <f>IF(L37="","",L37-J37)</f>
-        <v>-6406.51</v>
+        <v>-536.51</v>
       </c>
       <c r="N37" s="10">
         <f>IF(OR(H37="",K37=""),"",K37/H37-1)</f>
-        <v>-0.06442817344613472</v>
+        <v>-0.005395532127514979</v>
       </c>
       <c r="O37" s="6">
         <f>IF(G37="","",$B$3-G37)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P37" s="6" t="str">
         <f>IF(H37="","Pending buy",IF(N37&gt;=0,"In profit","In loss"))</f>
@@ -2821,23 +2821,23 @@
         <v>99951.48</v>
       </c>
       <c r="K38" s="9" t="n">
-        <v>116.25</v>
+        <v>112.4</v>
       </c>
       <c r="L38" s="9">
         <f>IF(OR(I38="",K38=""),"",K38*I38)</f>
-        <v>95208.75</v>
+        <v>92055.6</v>
       </c>
       <c r="M38" s="9">
         <f>IF(L38="","",L38-J38)</f>
-        <v>-4742.73</v>
+        <v>-7895.88</v>
       </c>
       <c r="N38" s="10">
         <f>IF(OR(H38="",K38=""),"",K38/H38-1)</f>
-        <v>-0.047450321953187546</v>
+        <v>-0.07899712849495288</v>
       </c>
       <c r="O38" s="6">
         <f>IF(G38="","",$B$3-G38)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P38" s="6" t="str">
         <f>IF(H38="","Pending buy",IF(N38&gt;=0,"In profit","In loss"))</f>
@@ -2889,23 +2889,23 @@
         <v>99666.78</v>
       </c>
       <c r="K39" s="9" t="n">
-        <v>485.05</v>
+        <v>494.05</v>
       </c>
       <c r="L39" s="9">
         <f>IF(OR(I39="",K39=""),"",K39*I39)</f>
-        <v>86823.95</v>
+        <v>88434.95</v>
       </c>
       <c r="M39" s="9">
         <f>IF(L39="","",L39-J39)</f>
-        <v>-12842.83</v>
+        <v>-11231.83</v>
       </c>
       <c r="N39" s="10">
         <f>IF(OR(H39="",K39=""),"",K39/H39-1)</f>
-        <v>-0.12885764571642433</v>
+        <v>-0.1126937838701153</v>
       </c>
       <c r="O39" s="6">
         <f>IF(G39="","",$B$3-G39)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P39" s="6" t="str">
         <f>IF(H39="","Pending buy",IF(N39&gt;=0,"In profit","In loss"))</f>
@@ -2957,23 +2957,23 @@
         <v>99998.64</v>
       </c>
       <c r="K40" s="9" t="n">
-        <v>12.63</v>
+        <v>12.77</v>
       </c>
       <c r="L40" s="9">
         <f>IF(OR(I40="",K40=""),"",K40*I40)</f>
-        <v>97478.34</v>
+        <v>98558.86</v>
       </c>
       <c r="M40" s="9">
         <f>IF(L40="","",L40-J40)</f>
-        <v>-2520.3</v>
+        <v>-1439.78</v>
       </c>
       <c r="N40" s="10">
         <f>IF(OR(H40="",K40=""),"",K40/H40-1)</f>
-        <v>-0.025203318044281442</v>
+        <v>-0.014397970817535688</v>
       </c>
       <c r="O40" s="6">
         <f>IF(G40="","",$B$3-G40)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P40" s="6" t="str">
         <f>IF(H40="","Pending buy",IF(N40&gt;=0,"In profit","In loss"))</f>
@@ -3025,23 +3025,23 @@
         <v>99889.82</v>
       </c>
       <c r="K41" s="9" t="n">
-        <v>121.27</v>
+        <v>125.63</v>
       </c>
       <c r="L41" s="9">
         <f>IF(OR(I41="",K41=""),"",K41*I41)</f>
-        <v>96409.65</v>
+        <v>99875.85</v>
       </c>
       <c r="M41" s="9">
         <f>IF(L41="","",L41-J41)</f>
-        <v>-3480.17</v>
+        <v>-13.97</v>
       </c>
       <c r="N41" s="10">
         <f>IF(OR(H41="",K41=""),"",K41/H41-1)</f>
-        <v>-0.034840076613976145</v>
+        <v>-0.00013984353107787673</v>
       </c>
       <c r="O41" s="6">
         <f>IF(G41="","",$B$3-G41)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P41" s="6" t="str">
         <f>IF(H41="","Pending buy",IF(N41&gt;=0,"In profit","In loss"))</f>
@@ -3093,23 +3093,23 @@
         <v>99925.2</v>
       </c>
       <c r="K42" s="9" t="n">
-        <v>115.58</v>
+        <v>121.58</v>
       </c>
       <c r="L42" s="9">
         <f>IF(OR(I42="",K42=""),"",K42*I42)</f>
-        <v>122861.54</v>
+        <v>129239.54</v>
       </c>
       <c r="M42" s="9">
         <f>IF(L42="","",L42-J42)</f>
-        <v>22936.34</v>
+        <v>29314.34</v>
       </c>
       <c r="N42" s="10">
         <f>IF(OR(H42="",K42=""),"",K42/H42-1)</f>
-        <v>0.22953510988142933</v>
+        <v>0.29336285394864325</v>
       </c>
       <c r="O42" s="6">
         <f>IF(G42="","",$B$3-G42)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P42" s="6" t="str">
         <f>IF(H42="","Pending buy",IF(N42&gt;=0,"In profit","In loss"))</f>
@@ -3161,23 +3161,23 @@
         <v>99394.67</v>
       </c>
       <c r="K43" s="9" t="n">
-        <v>639.25</v>
+        <v>648.5</v>
       </c>
       <c r="L43" s="9">
         <f>IF(OR(I43="",K43=""),"",K43*I43)</f>
-        <v>100362.25</v>
+        <v>101814.5</v>
       </c>
       <c r="M43" s="9">
         <f>IF(L43="","",L43-J43)</f>
-        <v>967.58</v>
+        <v>2419.83</v>
       </c>
       <c r="N43" s="10">
         <f>IF(OR(H43="",K43=""),"",K43/H43-1)</f>
-        <v>0.009734704996761545</v>
+        <v>0.024345649105044664</v>
       </c>
       <c r="O43" s="6">
         <f>IF(G43="","",$B$3-G43)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P43" s="6" t="str">
         <f>IF(H43="","Pending buy",IF(N43&gt;=0,"In profit","In loss"))</f>
@@ -3229,23 +3229,23 @@
         <v>99810.88</v>
       </c>
       <c r="K44" s="9" t="n">
-        <v>368.8</v>
+        <v>378.95</v>
       </c>
       <c r="L44" s="9">
         <f>IF(OR(I44="",K44=""),"",K44*I44)</f>
-        <v>111377.6</v>
+        <v>114442.9</v>
       </c>
       <c r="M44" s="9">
         <f>IF(L44="","",L44-J44)</f>
-        <v>11566.72</v>
+        <v>14632.02</v>
       </c>
       <c r="N44" s="10">
         <f>IF(OR(H44="",K44=""),"",K44/H44-1)</f>
-        <v>0.11588635973070649</v>
+        <v>0.14659744040116918</v>
       </c>
       <c r="O44" s="6">
         <f>IF(G44="","",$B$3-G44)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P44" s="6" t="str">
         <f>IF(H44="","Pending buy",IF(N44&gt;=0,"In profit","In loss"))</f>
@@ -3297,27 +3297,27 @@
         <v>99997.44</v>
       </c>
       <c r="K45" s="9" t="n">
-        <v>273.6</v>
+        <v>268.8</v>
       </c>
       <c r="L45" s="9">
         <f>IF(OR(I45="",K45=""),"",K45*I45)</f>
-        <v>101505.6</v>
+        <v>99724.8</v>
       </c>
       <c r="M45" s="9">
         <f>IF(L45="","",L45-J45)</f>
-        <v>1508.16</v>
+        <v>-272.64</v>
       </c>
       <c r="N45" s="10">
         <f>IF(OR(H45="",K45=""),"",K45/H45-1)</f>
-        <v>0.015082011354731195</v>
+        <v>-0.002726444984825549</v>
       </c>
       <c r="O45" s="6">
         <f>IF(G45="","",$B$3-G45)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P45" s="6" t="str">
         <f>IF(H45="","Pending buy",IF(N45&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q45" s="6" t="n">
         <v>1</v>
@@ -3365,23 +3365,23 @@
         <v>99870.37</v>
       </c>
       <c r="K46" s="9" t="n">
-        <v>358.1</v>
+        <v>351.4</v>
       </c>
       <c r="L46" s="9">
         <f>IF(OR(I46="",K46=""),"",K46*I46)</f>
-        <v>99551.8</v>
+        <v>97689.2</v>
       </c>
       <c r="M46" s="9">
         <f>IF(L46="","",L46-J46)</f>
-        <v>-318.57</v>
+        <v>-2181.17</v>
       </c>
       <c r="N46" s="10">
         <f>IF(OR(H46="",K46=""),"",K46/H46-1)</f>
-        <v>-0.0031897871140180722</v>
+        <v>-0.0218399642330801</v>
       </c>
       <c r="O46" s="6">
         <f>IF(G46="","",$B$3-G46)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P46" s="6" t="str">
         <f>IF(H46="","Pending buy",IF(N46&gt;=0,"In profit","In loss"))</f>
@@ -3433,27 +3433,27 @@
         <v>99957.4</v>
       </c>
       <c r="K47" s="9" t="n">
-        <v>578.55</v>
+        <v>567.65</v>
       </c>
       <c r="L47" s="9">
         <f>IF(OR(I47="",K47=""),"",K47*I47)</f>
-        <v>100089.15</v>
+        <v>98203.45</v>
       </c>
       <c r="M47" s="9">
         <f>IF(L47="","",L47-J47)</f>
-        <v>131.75</v>
+        <v>-1753.95</v>
       </c>
       <c r="N47" s="10">
         <f>IF(OR(H47="",K47=""),"",K47/H47-1)</f>
-        <v>0.0013180724232322305</v>
+        <v>-0.01754696428822433</v>
       </c>
       <c r="O47" s="6">
         <f>IF(G47="","",$B$3-G47)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P47" s="6" t="str">
         <f>IF(H47="","Pending buy",IF(N47&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q47" s="6" t="n">
         <v>1</v>
@@ -3501,23 +3501,23 @@
         <v>99965.44</v>
       </c>
       <c r="K48" s="9" t="n">
-        <v>184.6</v>
+        <v>182.98</v>
       </c>
       <c r="L48" s="9">
         <f>IF(OR(I48="",K48=""),"",K48*I48)</f>
-        <v>102822.2</v>
+        <v>101919.86</v>
       </c>
       <c r="M48" s="9">
         <f>IF(L48="","",L48-J48)</f>
-        <v>2856.76</v>
+        <v>1954.42</v>
       </c>
       <c r="N48" s="10">
         <f>IF(OR(H48="",K48=""),"",K48/H48-1)</f>
-        <v>0.028577453255709706</v>
+        <v>0.01955093389344409</v>
       </c>
       <c r="O48" s="6">
         <f>IF(G48="","",$B$3-G48)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P48" s="6" t="str">
         <f>IF(H48="","Pending buy",IF(N48&gt;=0,"In profit","In loss"))</f>
@@ -3569,23 +3569,23 @@
         <v>99985.7</v>
       </c>
       <c r="K49" s="9" t="n">
-        <v>910.9</v>
+        <v>879.4</v>
       </c>
       <c r="L49" s="9">
         <f>IF(OR(I49="",K49=""),"",K49*I49)</f>
-        <v>109308.0</v>
+        <v>105528.0</v>
       </c>
       <c r="M49" s="9">
         <f>IF(L49="","",L49-J49)</f>
-        <v>9322.3</v>
+        <v>5542.3</v>
       </c>
       <c r="N49" s="10">
         <f>IF(OR(H49="",K49=""),"",K49/H49-1)</f>
-        <v>0.09323636909622812</v>
+        <v>0.05543096166782635</v>
       </c>
       <c r="O49" s="6">
         <f>IF(G49="","",$B$3-G49)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P49" s="6" t="str">
         <f>IF(H49="","Pending buy",IF(N49&gt;=0,"In profit","In loss"))</f>
@@ -3637,23 +3637,23 @@
         <v>99961.35</v>
       </c>
       <c r="K50" s="9" t="n">
-        <v>95.95</v>
+        <v>94.84999999999999</v>
       </c>
       <c r="L50" s="9">
         <f>IF(OR(I50="",K50=""),"",K50*I50)</f>
-        <v>99788.0</v>
+        <v>98644.0</v>
       </c>
       <c r="M50" s="9">
         <f>IF(L50="","",L50-J50)</f>
-        <v>-173.35</v>
+        <v>-1317.35</v>
       </c>
       <c r="N50" s="10">
         <f>IF(OR(H50="",K50=""),"",K50/H50-1)</f>
-        <v>-0.0017341526805321195</v>
+        <v>-0.013178576151625654</v>
       </c>
       <c r="O50" s="6">
         <f>IF(G50="","",$B$3-G50)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P50" s="6" t="str">
         <f>IF(H50="","Pending buy",IF(N50&gt;=0,"In profit","In loss"))</f>
@@ -3705,27 +3705,27 @@
         <v>97877.65</v>
       </c>
       <c r="K51" s="9" t="n">
-        <v>2960.3</v>
+        <v>3049</v>
       </c>
       <c r="L51" s="9">
         <f>IF(OR(I51="",K51=""),"",K51*I51)</f>
-        <v>97689.9</v>
+        <v>100617.0</v>
       </c>
       <c r="M51" s="9">
         <f>IF(L51="","",L51-J51)</f>
-        <v>-187.75</v>
+        <v>2739.35</v>
       </c>
       <c r="N51" s="10">
         <f>IF(OR(H51="",K51=""),"",K51/H51-1)</f>
-        <v>-0.001918179542994336</v>
+        <v>0.02798752510671565</v>
       </c>
       <c r="O51" s="6">
         <f>IF(G51="","",$B$3-G51)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P51" s="6" t="str">
         <f>IF(H51="","Pending buy",IF(N51&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q51" s="6" t="n">
         <v>1</v>
@@ -3773,27 +3773,27 @@
         <v>99357.46</v>
       </c>
       <c r="K52" s="9" t="n">
-        <v>904.7</v>
+        <v>932</v>
       </c>
       <c r="L52" s="9">
         <f>IF(OR(I52="",K52=""),"",K52*I52)</f>
-        <v>98612.3</v>
+        <v>101588.0</v>
       </c>
       <c r="M52" s="9">
         <f>IF(L52="","",L52-J52)</f>
-        <v>-745.16</v>
+        <v>2230.54</v>
       </c>
       <c r="N52" s="10">
         <f>IF(OR(H52="",K52=""),"",K52/H52-1)</f>
-        <v>-0.007499764891427563</v>
+        <v>0.022449672953674726</v>
       </c>
       <c r="O52" s="6">
         <f>IF(G52="","",$B$3-G52)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P52" s="6" t="str">
         <f>IF(H52="","Pending buy",IF(N52&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q52" s="6" t="n">
         <v>1</v>
@@ -3841,23 +3841,23 @@
         <v>99747.01</v>
       </c>
       <c r="K53" s="9" t="n">
-        <v>851.85</v>
+        <v>879.45</v>
       </c>
       <c r="L53" s="9">
         <f>IF(OR(I53="",K53=""),"",K53*I53)</f>
-        <v>100518.3</v>
+        <v>103775.1</v>
       </c>
       <c r="M53" s="9">
         <f>IF(L53="","",L53-J53)</f>
-        <v>771.29</v>
+        <v>4028.09</v>
       </c>
       <c r="N53" s="10">
         <f>IF(OR(H53="",K53=""),"",K53/H53-1)</f>
-        <v>0.007732464821619489</v>
+        <v>0.04038306766141142</v>
       </c>
       <c r="O53" s="6">
         <f>IF(G53="","",$B$3-G53)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P53" s="6" t="str">
         <f>IF(H53="","Pending buy",IF(N53&gt;=0,"In profit","In loss"))</f>
@@ -3894,38 +3894,42 @@
       <c r="F54" s="8" t="n">
         <v>46322</v>
       </c>
-      <c r="G54" s="6" t="inlineStr"/>
-      <c r="H54" s="9" t="inlineStr"/>
-      <c r="I54" s="6" t="str">
+      <c r="G54" s="8" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H54" s="9" t="n">
+        <v>1384.88</v>
+      </c>
+      <c r="I54" s="6">
         <f>IF(H54="","",ROUNDDOWN($B$1/H54,0))</f>
-        <v/>
-      </c>
-      <c r="J54" s="9" t="str">
+        <v>72</v>
+      </c>
+      <c r="J54" s="9">
         <f>IF(H54="","",H54*I54)</f>
-        <v/>
+        <v>99711.32</v>
       </c>
       <c r="K54" s="9" t="n">
-        <v>1343.6</v>
-      </c>
-      <c r="L54" s="9" t="str">
+        <v>1399.4</v>
+      </c>
+      <c r="L54" s="9">
         <f>IF(OR(I54="",K54=""),"",K54*I54)</f>
-        <v/>
-      </c>
-      <c r="M54" s="9" t="str">
+        <v>100756.8</v>
+      </c>
+      <c r="M54" s="9">
         <f>IF(L54="","",L54-J54)</f>
-        <v/>
-      </c>
-      <c r="N54" s="10" t="str">
+        <v>1045.48</v>
+      </c>
+      <c r="N54" s="10">
         <f>IF(OR(H54="",K54=""),"",K54/H54-1)</f>
-        <v/>
-      </c>
-      <c r="O54" s="6" t="str">
+        <v>0.010485093427737624</v>
+      </c>
+      <c r="O54" s="6">
         <f>IF(G54="","",$B$3-G54)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P54" s="6" t="str">
         <f>IF(H54="","Pending buy",IF(N54&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In profit</v>
       </c>
       <c r="Q54" s="6" t="n">
         <v>1</v>
@@ -3958,38 +3962,42 @@
       <c r="F55" s="8" t="n">
         <v>46322</v>
       </c>
-      <c r="G55" s="6" t="inlineStr"/>
-      <c r="H55" s="9" t="inlineStr"/>
-      <c r="I55" s="6" t="str">
+      <c r="G55" s="8" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H55" s="9" t="n">
+        <v>3780.05</v>
+      </c>
+      <c r="I55" s="6">
         <f>IF(H55="","",ROUNDDOWN($B$1/H55,0))</f>
-        <v/>
-      </c>
-      <c r="J55" s="9" t="str">
+        <v>26</v>
+      </c>
+      <c r="J55" s="9">
         <f>IF(H55="","",H55*I55)</f>
-        <v/>
+        <v>98281.27</v>
       </c>
       <c r="K55" s="9" t="n">
-        <v>3794.5</v>
-      </c>
-      <c r="L55" s="9" t="str">
+        <v>3766.9</v>
+      </c>
+      <c r="L55" s="9">
         <f>IF(OR(I55="",K55=""),"",K55*I55)</f>
-        <v/>
-      </c>
-      <c r="M55" s="9" t="str">
+        <v>97939.4</v>
+      </c>
+      <c r="M55" s="9">
         <f>IF(L55="","",L55-J55)</f>
-        <v/>
-      </c>
-      <c r="N55" s="10" t="str">
+        <v>-341.87</v>
+      </c>
+      <c r="N55" s="10">
         <f>IF(OR(H55="",K55=""),"",K55/H55-1)</f>
-        <v/>
-      </c>
-      <c r="O55" s="6" t="str">
+        <v>-0.003478522382164284</v>
+      </c>
+      <c r="O55" s="6">
         <f>IF(G55="","",$B$3-G55)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P55" s="6" t="str">
         <f>IF(H55="","Pending buy",IF(N55&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q55" s="6" t="n">
         <v>1</v>
@@ -4022,38 +4030,42 @@
       <c r="F56" s="8" t="n">
         <v>46322</v>
       </c>
-      <c r="G56" s="6" t="inlineStr"/>
-      <c r="H56" s="9" t="inlineStr"/>
-      <c r="I56" s="6" t="str">
+      <c r="G56" s="8" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H56" s="9" t="n">
+        <v>5931.66</v>
+      </c>
+      <c r="I56" s="6">
         <f>IF(H56="","",ROUNDDOWN($B$1/H56,0))</f>
-        <v/>
-      </c>
-      <c r="J56" s="9" t="str">
+        <v>16</v>
+      </c>
+      <c r="J56" s="9">
         <f>IF(H56="","",H56*I56)</f>
-        <v/>
+        <v>94906.63</v>
       </c>
       <c r="K56" s="9" t="n">
-        <v>5862</v>
-      </c>
-      <c r="L56" s="9" t="str">
+        <v>5929.5</v>
+      </c>
+      <c r="L56" s="9">
         <f>IF(OR(I56="",K56=""),"",K56*I56)</f>
-        <v/>
-      </c>
-      <c r="M56" s="9" t="str">
+        <v>94872.0</v>
+      </c>
+      <c r="M56" s="9">
         <f>IF(L56="","",L56-J56)</f>
-        <v/>
-      </c>
-      <c r="N56" s="10" t="str">
+        <v>-34.63</v>
+      </c>
+      <c r="N56" s="10">
         <f>IF(OR(H56="",K56=""),"",K56/H56-1)</f>
-        <v/>
-      </c>
-      <c r="O56" s="6" t="str">
+        <v>-0.0003648942089597984</v>
+      </c>
+      <c r="O56" s="6">
         <f>IF(G56="","",$B$3-G56)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P56" s="6" t="str">
         <f>IF(H56="","Pending buy",IF(N56&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q56" s="6" t="n">
         <v>1</v>
@@ -4086,38 +4098,42 @@
       <c r="F57" s="8" t="n">
         <v>46322</v>
       </c>
-      <c r="G57" s="6" t="inlineStr"/>
-      <c r="H57" s="9" t="inlineStr"/>
-      <c r="I57" s="6" t="str">
+      <c r="G57" s="8" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H57" s="9" t="n">
+        <v>424.61</v>
+      </c>
+      <c r="I57" s="6">
         <f>IF(H57="","",ROUNDDOWN($B$1/H57,0))</f>
-        <v/>
-      </c>
-      <c r="J57" s="9" t="str">
+        <v>235</v>
+      </c>
+      <c r="J57" s="9">
         <f>IF(H57="","",H57*I57)</f>
-        <v/>
+        <v>99783.3</v>
       </c>
       <c r="K57" s="9" t="n">
-        <v>425.25</v>
-      </c>
-      <c r="L57" s="9" t="str">
+        <v>417.3</v>
+      </c>
+      <c r="L57" s="9">
         <f>IF(OR(I57="",K57=""),"",K57*I57)</f>
-        <v/>
-      </c>
-      <c r="M57" s="9" t="str">
+        <v>98065.5</v>
+      </c>
+      <c r="M57" s="9">
         <f>IF(L57="","",L57-J57)</f>
-        <v/>
-      </c>
-      <c r="N57" s="10" t="str">
+        <v>-1717.8</v>
+      </c>
+      <c r="N57" s="10">
         <f>IF(OR(H57="",K57=""),"",K57/H57-1)</f>
-        <v/>
-      </c>
-      <c r="O57" s="6" t="str">
+        <v>-0.017215277250741567</v>
+      </c>
+      <c r="O57" s="6">
         <f>IF(G57="","",$B$3-G57)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P57" s="6" t="str">
         <f>IF(H57="","Pending buy",IF(N57&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q57" s="6" t="n">
         <v>1</v>
@@ -4150,38 +4166,42 @@
       <c r="F58" s="8" t="n">
         <v>46322</v>
       </c>
-      <c r="G58" s="6" t="inlineStr"/>
-      <c r="H58" s="9" t="inlineStr"/>
-      <c r="I58" s="6" t="str">
+      <c r="G58" s="8" t="n">
+        <v>46323</v>
+      </c>
+      <c r="H58" s="9" t="n">
+        <v>78.53</v>
+      </c>
+      <c r="I58" s="6">
         <f>IF(H58="","",ROUNDDOWN($B$1/H58,0))</f>
-        <v/>
-      </c>
-      <c r="J58" s="9" t="str">
+        <v>1273</v>
+      </c>
+      <c r="J58" s="9">
         <f>IF(H58="","",H58*I58)</f>
-        <v/>
+        <v>99967.09</v>
       </c>
       <c r="K58" s="9" t="n">
-        <v>78.14</v>
-      </c>
-      <c r="L58" s="9" t="str">
+        <v>78.97</v>
+      </c>
+      <c r="L58" s="9">
         <f>IF(OR(I58="",K58=""),"",K58*I58)</f>
-        <v/>
-      </c>
-      <c r="M58" s="9" t="str">
+        <v>100528.81</v>
+      </c>
+      <c r="M58" s="9">
         <f>IF(L58="","",L58-J58)</f>
-        <v/>
-      </c>
-      <c r="N58" s="10" t="str">
+        <v>561.72</v>
+      </c>
+      <c r="N58" s="10">
         <f>IF(OR(H58="",K58=""),"",K58/H58-1)</f>
-        <v/>
-      </c>
-      <c r="O58" s="6" t="str">
+        <v>0.005619063654426215</v>
+      </c>
+      <c r="O58" s="6">
         <f>IF(G58="","",$B$3-G58)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P58" s="6" t="str">
         <f>IF(H58="","Pending buy",IF(N58&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In profit</v>
       </c>
       <c r="Q58" s="6" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Momentum Portfolio: weekday silent update 2026-10-29
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q58"/>
+  <dimension ref="A1:Q60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="E1" s="2">
-        <f>SUM(J8:J58)</f>
+        <f>SUM(J8:J60)</f>
         <v>5052225.67</v>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -540,8 +540,8 @@
         </is>
       </c>
       <c r="G1" s="2">
-        <f>SUM(L8:L58)</f>
-        <v>4877626.59</v>
+        <f>SUM(L8:L60)</f>
+        <v>4891693.01</v>
       </c>
     </row>
     <row r="2">
@@ -551,8 +551,8 @@
         </is>
       </c>
       <c r="E2" s="2">
-        <f>SUM(M8:M58)</f>
-        <v>-174599.08</v>
+        <f>SUM(M8:M60)</f>
+        <v>-160532.66</v>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" s="3">
         <f>IF(E1=0,"",G1/E1-1)</f>
-        <v>-0.034558844241017406</v>
+        <v>-0.03177464161057564</v>
       </c>
     </row>
     <row r="3">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -579,8 +579,8 @@
         </is>
       </c>
       <c r="E3">
-        <f>COUNTIF(M8:M58,"&gt;0")</f>
-        <v>16</v>
+        <f>COUNTIF(M8:M60,"&gt;0")</f>
+        <v>17</v>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
@@ -588,8 +588,8 @@
         </is>
       </c>
       <c r="G3">
-        <f>COUNTIF(M8:M58,"&lt;0")</f>
-        <v>35</v>
+        <f>COUNTIF(M8:M60,"&lt;0")</f>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
@@ -600,7 +600,7 @@
       </c>
       <c r="E4" s="3">
         <f>IF((E3+G3)=0,"",E3/(E3+G3))</f>
-        <v>0.3137254901960784</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
@@ -608,8 +608,8 @@
         </is>
       </c>
       <c r="G4" s="3">
-        <f>AVERAGE(N8:N58)</f>
-        <v>-0.03463787225409552</v>
+        <f>AVERAGE(N8:N60)</f>
+        <v>-0.03195244959288102</v>
       </c>
     </row>
     <row r="5">
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="E5" t="str">
-        <f>INDEX(B8:B58,MATCH(MAX(N8:N58),N8:N58,0))</f>
+        <f>INDEX(B8:B60,MATCH(MAX(N8:N60),N8:N60,0))</f>
         <v>Pashupati Cotspin Limited</v>
       </c>
       <c r="F5" s="1" t="inlineStr">
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="G5" t="str">
-        <f>INDEX(B8:B58,MATCH(MIN(N8:N58),N8:N58,0))</f>
+        <f>INDEX(B8:B60,MATCH(MIN(N8:N60),N8:N60,0))</f>
         <v>Lloyds Enterprises Limited</v>
       </c>
     </row>
@@ -639,8 +639,8 @@
         </is>
       </c>
       <c r="E6" s="3">
-        <f>AVERAGEIF(D8:D58,"4★*",N8:N58)</f>
-        <v>-0.06951575929167718</v>
+        <f>AVERAGEIF(D8:D60,"4★*",N8:N60)</f>
+        <v>-0.05965058830936478</v>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
@@ -648,8 +648,8 @@
         </is>
       </c>
       <c r="G6" s="3">
-        <f>AVERAGEIF(D8:D58,"5★*",N8:N58)</f>
-        <v>-0.01392912682553141</v>
+        <f>AVERAGEIF(D8:D60,"5★*",N8:N60)</f>
+        <v>-0.01550667972996879</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
@@ -781,23 +781,23 @@
         <v>99851.29</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>284.85</v>
+        <v>293.25</v>
       </c>
       <c r="L8" s="9">
         <f>IF(OR(I8="",K8=""),"",K8*I8)</f>
-        <v>94570.2</v>
+        <v>97359.0</v>
       </c>
       <c r="M8" s="9">
         <f>IF(L8="","",L8-J8)</f>
-        <v>-5281.09</v>
+        <v>-2492.29</v>
       </c>
       <c r="N8" s="10">
         <f>IF(OR(H8="",K8=""),"",K8/H8-1)</f>
-        <v>-0.052889584833742176</v>
+        <v>-0.024960051790398174</v>
       </c>
       <c r="O8" s="6">
         <f>IF(G8="","",$B$3-G8)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P8" s="6" t="str">
         <f>IF(H8="","Pending buy",IF(N8&gt;=0,"In profit","In loss"))</f>
@@ -849,23 +849,23 @@
         <v>99687.42</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>326</v>
+        <v>337.85</v>
       </c>
       <c r="L9" s="9">
         <f>IF(OR(I9="",K9=""),"",K9*I9)</f>
-        <v>99756.0</v>
+        <v>103382.1</v>
       </c>
       <c r="M9" s="9">
         <f>IF(L9="","",L9-J9)</f>
-        <v>68.58</v>
+        <v>3694.68</v>
       </c>
       <c r="N9" s="10">
         <f>IF(OR(H9="",K9=""),"",K9/H9-1)</f>
-        <v>0.0006879484077708664</v>
+        <v>0.037062648372899964</v>
       </c>
       <c r="O9" s="6">
         <f>IF(G9="","",$B$3-G9)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P9" s="6" t="str">
         <f>IF(H9="","Pending buy",IF(N9&gt;=0,"In profit","In loss"))</f>
@@ -917,23 +917,23 @@
         <v>99607.14</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>1450.6</v>
+        <v>1429.2</v>
       </c>
       <c r="L10" s="9">
         <f>IF(OR(I10="",K10=""),"",K10*I10)</f>
-        <v>91387.8</v>
+        <v>90039.6</v>
       </c>
       <c r="M10" s="9">
         <f>IF(L10="","",L10-J10)</f>
-        <v>-8219.34</v>
+        <v>-9567.54</v>
       </c>
       <c r="N10" s="10">
         <f>IF(OR(H10="",K10=""),"",K10/H10-1)</f>
-        <v>-0.08251758709773416</v>
+        <v>-0.09605276125746687</v>
       </c>
       <c r="O10" s="6">
         <f>IF(G10="","",$B$3-G10)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P10" s="6" t="str">
         <f>IF(H10="","Pending buy",IF(N10&gt;=0,"In profit","In loss"))</f>
@@ -985,23 +985,23 @@
         <v>99927.23</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>61.71</v>
+        <v>62.76</v>
       </c>
       <c r="L11" s="9">
         <f>IF(OR(I11="",K11=""),"",K11*I11)</f>
-        <v>77199.21</v>
+        <v>78512.76</v>
       </c>
       <c r="M11" s="9">
         <f>IF(L11="","",L11-J11)</f>
-        <v>-22728.02</v>
+        <v>-21414.47</v>
       </c>
       <c r="N11" s="10">
         <f>IF(OR(H11="",K11=""),"",K11/H11-1)</f>
-        <v>-0.22744571519810697</v>
+        <v>-0.2143006495840739</v>
       </c>
       <c r="O11" s="6">
         <f>IF(G11="","",$B$3-G11)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P11" s="6" t="str">
         <f>IF(H11="","Pending buy",IF(N11&gt;=0,"In profit","In loss"))</f>
@@ -1053,23 +1053,23 @@
         <v>86537.12</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>19970</v>
+        <v>19280</v>
       </c>
       <c r="L12" s="9">
         <f>IF(OR(I12="",K12=""),"",K12*I12)</f>
-        <v>79880.0</v>
+        <v>77120.0</v>
       </c>
       <c r="M12" s="9">
         <f>IF(L12="","",L12-J12)</f>
-        <v>-6657.12</v>
+        <v>-9417.12</v>
       </c>
       <c r="N12" s="10">
         <f>IF(OR(H12="",K12=""),"",K12/H12-1)</f>
-        <v>-0.0769278713798377</v>
+        <v>-0.10882170056100504</v>
       </c>
       <c r="O12" s="6">
         <f>IF(G12="","",$B$3-G12)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P12" s="6" t="str">
         <f>IF(H12="","Pending buy",IF(N12&gt;=0,"In profit","In loss"))</f>
@@ -1121,23 +1121,23 @@
         <v>98177.53</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>1744.7</v>
+        <v>1783.9</v>
       </c>
       <c r="L13" s="9">
         <f>IF(OR(I13="",K13=""),"",K13*I13)</f>
-        <v>92469.1</v>
+        <v>94546.7</v>
       </c>
       <c r="M13" s="9">
         <f>IF(L13="","",L13-J13)</f>
-        <v>-5708.43</v>
+        <v>-3630.83</v>
       </c>
       <c r="N13" s="10">
         <f>IF(OR(H13="",K13=""),"",K13/H13-1)</f>
-        <v>-0.058143986453736196</v>
+        <v>-0.03698232213837338</v>
       </c>
       <c r="O13" s="6">
         <f>IF(G13="","",$B$3-G13)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P13" s="6" t="str">
         <f>IF(H13="","Pending buy",IF(N13&gt;=0,"In profit","In loss"))</f>
@@ -1189,23 +1189,23 @@
         <v>97667.46</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>4135.1</v>
+        <v>4235</v>
       </c>
       <c r="L14" s="9">
         <f>IF(OR(I14="",K14=""),"",K14*I14)</f>
-        <v>90972.2</v>
+        <v>93170.0</v>
       </c>
       <c r="M14" s="9">
         <f>IF(L14="","",L14-J14)</f>
-        <v>-6695.26</v>
+        <v>-4497.46</v>
       </c>
       <c r="N14" s="10">
         <f>IF(OR(H14="",K14=""),"",K14/H14-1)</f>
-        <v>-0.06855163319957502</v>
+        <v>-0.046048745278276404</v>
       </c>
       <c r="O14" s="6">
         <f>IF(G14="","",$B$3-G14)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P14" s="6" t="str">
         <f>IF(H14="","Pending buy",IF(N14&gt;=0,"In profit","In loss"))</f>
@@ -1257,23 +1257,23 @@
         <v>99078.19</v>
       </c>
       <c r="K15" s="9" t="n">
-        <v>1365.4</v>
+        <v>1359.2</v>
       </c>
       <c r="L15" s="9">
         <f>IF(OR(I15="",K15=""),"",K15*I15)</f>
-        <v>87385.6</v>
+        <v>86988.8</v>
       </c>
       <c r="M15" s="9">
         <f>IF(L15="","",L15-J15)</f>
-        <v>-11692.59</v>
+        <v>-12089.39</v>
       </c>
       <c r="N15" s="10">
         <f>IF(OR(H15="",K15=""),"",K15/H15-1)</f>
-        <v>-0.11801374115858587</v>
+        <v>-0.1220186589883917</v>
       </c>
       <c r="O15" s="6">
         <f>IF(G15="","",$B$3-G15)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P15" s="6" t="str">
         <f>IF(H15="","Pending buy",IF(N15&gt;=0,"In profit","In loss"))</f>
@@ -1325,23 +1325,23 @@
         <v>98557.54</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>1650</v>
+        <v>1663</v>
       </c>
       <c r="L16" s="9">
         <f>IF(OR(I16="",K16=""),"",K16*I16)</f>
-        <v>112200.0</v>
+        <v>113084.0</v>
       </c>
       <c r="M16" s="9">
         <f>IF(L16="","",L16-J16)</f>
-        <v>13642.46</v>
+        <v>14526.46</v>
       </c>
       <c r="N16" s="10">
         <f>IF(OR(H16="",K16=""),"",K16/H16-1)</f>
-        <v>0.13842131171557104</v>
+        <v>0.14739069174726938</v>
       </c>
       <c r="O16" s="6">
         <f>IF(G16="","",$B$3-G16)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P16" s="6" t="str">
         <f>IF(H16="","Pending buy",IF(N16&gt;=0,"In profit","In loss"))</f>
@@ -1393,23 +1393,23 @@
         <v>99714.35</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>811.65</v>
+        <v>821.15</v>
       </c>
       <c r="L17" s="9">
         <f>IF(OR(I17="",K17=""),"",K17*I17)</f>
-        <v>93339.75</v>
+        <v>94432.25</v>
       </c>
       <c r="M17" s="9">
         <f>IF(L17="","",L17-J17)</f>
-        <v>-6374.6</v>
+        <v>-5282.1</v>
       </c>
       <c r="N17" s="10">
         <f>IF(OR(H17="",K17=""),"",K17/H17-1)</f>
-        <v>-0.06392861278447248</v>
+        <v>-0.052972316131299935</v>
       </c>
       <c r="O17" s="6">
         <f>IF(G17="","",$B$3-G17)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P17" s="6" t="str">
         <f>IF(H17="","Pending buy",IF(N17&gt;=0,"In profit","In loss"))</f>
@@ -1461,23 +1461,23 @@
         <v>99596.83</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>591.3</v>
+        <v>590.95</v>
       </c>
       <c r="L18" s="9">
         <f>IF(OR(I18="",K18=""),"",K18*I18)</f>
-        <v>83373.3</v>
+        <v>83323.95</v>
       </c>
       <c r="M18" s="9">
         <f>IF(L18="","",L18-J18)</f>
-        <v>-16223.53</v>
+        <v>-16272.88</v>
       </c>
       <c r="N18" s="10">
         <f>IF(OR(H18="",K18=""),"",K18/H18-1)</f>
-        <v>-0.16289207037501396</v>
+        <v>-0.16338756805025267</v>
       </c>
       <c r="O18" s="6">
         <f>IF(G18="","",$B$3-G18)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P18" s="6" t="str">
         <f>IF(H18="","Pending buy",IF(N18&gt;=0,"In profit","In loss"))</f>
@@ -1529,23 +1529,23 @@
         <v>99993.07</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>126.44</v>
+        <v>126.35</v>
       </c>
       <c r="L19" s="9">
         <f>IF(OR(I19="",K19=""),"",K19*I19)</f>
-        <v>83829.72</v>
+        <v>83770.05</v>
       </c>
       <c r="M19" s="9">
         <f>IF(L19="","",L19-J19)</f>
-        <v>-16163.35</v>
+        <v>-16223.02</v>
       </c>
       <c r="N19" s="10">
         <f>IF(OR(H19="",K19=""),"",K19/H19-1)</f>
-        <v>-0.16164466248019005</v>
+        <v>-0.16224140386248032</v>
       </c>
       <c r="O19" s="6">
         <f>IF(G19="","",$B$3-G19)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P19" s="6" t="str">
         <f>IF(H19="","Pending buy",IF(N19&gt;=0,"In profit","In loss"))</f>
@@ -1597,27 +1597,27 @@
         <v>99896.43</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>207.01</v>
+        <v>213.7</v>
       </c>
       <c r="L20" s="9">
         <f>IF(OR(I20="",K20=""),"",K20*I20)</f>
-        <v>98743.77</v>
+        <v>101934.9</v>
       </c>
       <c r="M20" s="9">
         <f>IF(L20="","",L20-J20)</f>
-        <v>-1152.66</v>
+        <v>2038.47</v>
       </c>
       <c r="N20" s="10">
         <f>IF(OR(H20="",K20=""),"",K20/H20-1)</f>
-        <v>-0.01153855053609798</v>
+        <v>0.020405834261320033</v>
       </c>
       <c r="O20" s="6">
         <f>IF(G20="","",$B$3-G20)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P20" s="6" t="str">
         <f>IF(H20="","Pending buy",IF(N20&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q20" s="6" t="n">
         <v>1</v>
@@ -1665,23 +1665,23 @@
         <v>99449.47</v>
       </c>
       <c r="K21" s="9" t="n">
-        <v>1324.3</v>
+        <v>1219.2</v>
       </c>
       <c r="L21" s="9">
         <f>IF(OR(I21="",K21=""),"",K21*I21)</f>
-        <v>94025.3</v>
+        <v>86563.2</v>
       </c>
       <c r="M21" s="9">
         <f>IF(L21="","",L21-J21)</f>
-        <v>-5424.17</v>
+        <v>-12886.27</v>
       </c>
       <c r="N21" s="10">
         <f>IF(OR(H21="",K21=""),"",K21/H21-1)</f>
-        <v>-0.05454193510209793</v>
+        <v>-0.1295760230132732</v>
       </c>
       <c r="O21" s="6">
         <f>IF(G21="","",$B$3-G21)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P21" s="6" t="str">
         <f>IF(H21="","Pending buy",IF(N21&gt;=0,"In profit","In loss"))</f>
@@ -1733,23 +1733,23 @@
         <v>99837.05</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>674.8</v>
+        <v>642.85</v>
       </c>
       <c r="L22" s="9">
         <f>IF(OR(I22="",K22=""),"",K22*I22)</f>
-        <v>97171.2</v>
+        <v>92570.4</v>
       </c>
       <c r="M22" s="9">
         <f>IF(L22="","",L22-J22)</f>
-        <v>-2665.85</v>
+        <v>-7266.65</v>
       </c>
       <c r="N22" s="10">
         <f>IF(OR(H22="",K22=""),"",K22/H22-1)</f>
-        <v>-0.026702021845534718</v>
+        <v>-0.07278511372762586</v>
       </c>
       <c r="O22" s="6">
         <f>IF(G22="","",$B$3-G22)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P22" s="6" t="str">
         <f>IF(H22="","Pending buy",IF(N22&gt;=0,"In profit","In loss"))</f>
@@ -1801,23 +1801,23 @@
         <v>99486.88</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>568.45</v>
+        <v>577.85</v>
       </c>
       <c r="L23" s="9">
         <f>IF(OR(I23="",K23=""),"",K23*I23)</f>
-        <v>82425.25</v>
+        <v>83788.25</v>
       </c>
       <c r="M23" s="9">
         <f>IF(L23="","",L23-J23)</f>
-        <v>-17061.63</v>
+        <v>-15698.63</v>
       </c>
       <c r="N23" s="10">
         <f>IF(OR(H23="",K23=""),"",K23/H23-1)</f>
-        <v>-0.17149629163081004</v>
+        <v>-0.15779599282058854</v>
       </c>
       <c r="O23" s="6">
         <f>IF(G23="","",$B$3-G23)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P23" s="6" t="str">
         <f>IF(H23="","Pending buy",IF(N23&gt;=0,"In profit","In loss"))</f>
@@ -1869,30 +1869,30 @@
         <v>99935.4</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>230.04</v>
+        <v>239.94</v>
       </c>
       <c r="L24" s="9">
         <f>IF(OR(I24="",K24=""),"",K24*I24)</f>
-        <v>100987.56</v>
+        <v>105333.66</v>
       </c>
       <c r="M24" s="9">
         <f>IF(L24="","",L24-J24)</f>
-        <v>1052.16</v>
+        <v>5398.26</v>
       </c>
       <c r="N24" s="10">
         <f>IF(OR(H24="",K24=""),"",K24/H24-1)</f>
-        <v>0.010528415473477715</v>
+        <v>0.054017510036107774</v>
       </c>
       <c r="O24" s="6">
         <f>IF(G24="","",$B$3-G24)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="P24" s="6" t="str">
         <f>IF(H24="","Pending buy",IF(N24&gt;=0,"In profit","In loss"))</f>
         <v>In profit</v>
       </c>
       <c r="Q24" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -1937,23 +1937,23 @@
         <v>99622.64</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>731.25</v>
+        <v>722.85</v>
       </c>
       <c r="L25" s="9">
         <f>IF(OR(I25="",K25=""),"",K25*I25)</f>
-        <v>90675.0</v>
+        <v>89633.4</v>
       </c>
       <c r="M25" s="9">
         <f>IF(L25="","",L25-J25)</f>
-        <v>-8947.64</v>
+        <v>-9989.24</v>
       </c>
       <c r="N25" s="10">
         <f>IF(OR(H25="",K25=""),"",K25/H25-1)</f>
-        <v>-0.08981529415455747</v>
+        <v>-0.10027074923708967</v>
       </c>
       <c r="O25" s="6">
         <f>IF(G25="","",$B$3-G25)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P25" s="6" t="str">
         <f>IF(H25="","Pending buy",IF(N25&gt;=0,"In profit","In loss"))</f>
@@ -2005,23 +2005,23 @@
         <v>99948.17</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>193.68</v>
+        <v>190.02</v>
       </c>
       <c r="L26" s="9">
         <f>IF(OR(I26="",K26=""),"",K26*I26)</f>
-        <v>91998.0</v>
+        <v>90259.5</v>
       </c>
       <c r="M26" s="9">
         <f>IF(L26="","",L26-J26)</f>
-        <v>-7950.17</v>
+        <v>-9688.67</v>
       </c>
       <c r="N26" s="10">
         <f>IF(OR(H26="",K26=""),"",K26/H26-1)</f>
-        <v>-0.0795428964780458</v>
+        <v>-0.09693691237483615</v>
       </c>
       <c r="O26" s="6">
         <f>IF(G26="","",$B$3-G26)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P26" s="6" t="str">
         <f>IF(H26="","Pending buy",IF(N26&gt;=0,"In profit","In loss"))</f>
@@ -2073,23 +2073,23 @@
         <v>99745.27</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>210.4</v>
+        <v>210.9</v>
       </c>
       <c r="L27" s="9">
         <f>IF(OR(I27="",K27=""),"",K27*I27)</f>
-        <v>80372.8</v>
+        <v>80563.8</v>
       </c>
       <c r="M27" s="9">
         <f>IF(L27="","",L27-J27)</f>
-        <v>-19372.47</v>
+        <v>-19181.47</v>
       </c>
       <c r="N27" s="10">
         <f>IF(OR(H27="",K27=""),"",K27/H27-1)</f>
-        <v>-0.19421945907921645</v>
+        <v>-0.19230458136790274</v>
       </c>
       <c r="O27" s="6">
         <f>IF(G27="","",$B$3-G27)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P27" s="6" t="str">
         <f>IF(H27="","Pending buy",IF(N27&gt;=0,"In profit","In loss"))</f>
@@ -2141,23 +2141,23 @@
         <v>95334.84</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>11014</v>
+        <v>10833</v>
       </c>
       <c r="L28" s="9">
         <f>IF(OR(I28="",K28=""),"",K28*I28)</f>
-        <v>99126.0</v>
+        <v>97497.0</v>
       </c>
       <c r="M28" s="9">
         <f>IF(L28="","",L28-J28)</f>
-        <v>3791.16</v>
+        <v>2162.16</v>
       </c>
       <c r="N28" s="10">
         <f>IF(OR(H28="",K28=""),"",K28/H28-1)</f>
-        <v>0.03976675799527629</v>
+        <v>0.02267961588549383</v>
       </c>
       <c r="O28" s="6">
         <f>IF(G28="","",$B$3-G28)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P28" s="6" t="str">
         <f>IF(H28="","Pending buy",IF(N28&gt;=0,"In profit","In loss"))</f>
@@ -2209,23 +2209,23 @@
         <v>98598.59</v>
       </c>
       <c r="K29" s="9" t="n">
-        <v>1784.6</v>
+        <v>1800.1</v>
       </c>
       <c r="L29" s="9">
         <f>IF(OR(I29="",K29=""),"",K29*I29)</f>
-        <v>91014.6</v>
+        <v>91805.1</v>
       </c>
       <c r="M29" s="9">
         <f>IF(L29="","",L29-J29)</f>
-        <v>-7583.99</v>
+        <v>-6793.49</v>
       </c>
       <c r="N29" s="10">
         <f>IF(OR(H29="",K29=""),"",K29/H29-1)</f>
-        <v>-0.07691779923467279</v>
+        <v>-0.06890044290167796</v>
       </c>
       <c r="O29" s="6">
         <f>IF(G29="","",$B$3-G29)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P29" s="6" t="str">
         <f>IF(H29="","Pending buy",IF(N29&gt;=0,"In profit","In loss"))</f>
@@ -2277,23 +2277,23 @@
         <v>99998.69</v>
       </c>
       <c r="K30" s="9" t="n">
-        <v>15.08</v>
+        <v>15.28</v>
       </c>
       <c r="L30" s="9">
         <f>IF(OR(I30="",K30=""),"",K30*I30)</f>
-        <v>101684.44</v>
+        <v>103033.04</v>
       </c>
       <c r="M30" s="9">
         <f>IF(L30="","",L30-J30)</f>
-        <v>1685.75</v>
+        <v>3034.35</v>
       </c>
       <c r="N30" s="10">
         <f>IF(OR(H30="",K30=""),"",K30/H30-1)</f>
-        <v>0.016857720836142898</v>
+        <v>0.03034389750505717</v>
       </c>
       <c r="O30" s="6">
         <f>IF(G30="","",$B$3-G30)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P30" s="6" t="str">
         <f>IF(H30="","Pending buy",IF(N30&gt;=0,"In profit","In loss"))</f>
@@ -2345,23 +2345,23 @@
         <v>99977.34</v>
       </c>
       <c r="K31" s="9" t="n">
-        <v>145.83</v>
+        <v>144.85</v>
       </c>
       <c r="L31" s="9">
         <f>IF(OR(I31="",K31=""),"",K31*I31)</f>
-        <v>82248.12</v>
+        <v>81695.4</v>
       </c>
       <c r="M31" s="9">
         <f>IF(L31="","",L31-J31)</f>
-        <v>-17729.22</v>
+        <v>-18281.94</v>
       </c>
       <c r="N31" s="10">
         <f>IF(OR(H31="",K31=""),"",K31/H31-1)</f>
-        <v>-0.1773323685092465</v>
+        <v>-0.18286082135750104</v>
       </c>
       <c r="O31" s="6">
         <f>IF(G31="","",$B$3-G31)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P31" s="6" t="str">
         <f>IF(H31="","Pending buy",IF(N31&gt;=0,"In profit","In loss"))</f>
@@ -2413,27 +2413,27 @@
         <v>99923.82</v>
       </c>
       <c r="K32" s="9" t="n">
-        <v>178.52</v>
+        <v>175.16</v>
       </c>
       <c r="L32" s="9">
         <f>IF(OR(I32="",K32=""),"",K32*I32)</f>
-        <v>100863.8</v>
+        <v>98965.4</v>
       </c>
       <c r="M32" s="9">
         <f>IF(L32="","",L32-J32)</f>
-        <v>939.98</v>
+        <v>-958.42</v>
       </c>
       <c r="N32" s="10">
         <f>IF(OR(H32="",K32=""),"",K32/H32-1)</f>
-        <v>0.009406969560454392</v>
+        <v>-0.009591503539047919</v>
       </c>
       <c r="O32" s="6">
         <f>IF(G32="","",$B$3-G32)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P32" s="6" t="str">
         <f>IF(H32="","Pending buy",IF(N32&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q32" s="6" t="n">
         <v>1</v>
@@ -2481,23 +2481,23 @@
         <v>99608.58</v>
       </c>
       <c r="K33" s="9" t="n">
-        <v>508.1</v>
+        <v>498.7</v>
       </c>
       <c r="L33" s="9">
         <f>IF(OR(I33="",K33=""),"",K33*I33)</f>
-        <v>96030.9</v>
+        <v>94254.3</v>
       </c>
       <c r="M33" s="9">
         <f>IF(L33="","",L33-J33)</f>
-        <v>-3577.68</v>
+        <v>-5354.28</v>
       </c>
       <c r="N33" s="10">
         <f>IF(OR(H33="",K33=""),"",K33/H33-1)</f>
-        <v>-0.03591734062672891</v>
+        <v>-0.053753154439184714</v>
       </c>
       <c r="O33" s="6">
         <f>IF(G33="","",$B$3-G33)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P33" s="6" t="str">
         <f>IF(H33="","Pending buy",IF(N33&gt;=0,"In profit","In loss"))</f>
@@ -2549,23 +2549,23 @@
         <v>96030.46</v>
       </c>
       <c r="K34" s="9" t="n">
-        <v>4403.9</v>
+        <v>4387</v>
       </c>
       <c r="L34" s="9">
         <f>IF(OR(I34="",K34=""),"",K34*I34)</f>
-        <v>83674.1</v>
+        <v>83353.0</v>
       </c>
       <c r="M34" s="9">
         <f>IF(L34="","",L34-J34)</f>
-        <v>-12356.36</v>
+        <v>-12677.46</v>
       </c>
       <c r="N34" s="10">
         <f>IF(OR(H34="",K34=""),"",K34/H34-1)</f>
-        <v>-0.12867126359400272</v>
+        <v>-0.1320149942975294</v>
       </c>
       <c r="O34" s="6">
         <f>IF(G34="","",$B$3-G34)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P34" s="6" t="str">
         <f>IF(H34="","Pending buy",IF(N34&gt;=0,"In profit","In loss"))</f>
@@ -2617,23 +2617,23 @@
         <v>99082.89</v>
       </c>
       <c r="K35" s="9" t="n">
-        <v>938.5</v>
+        <v>946.3</v>
       </c>
       <c r="L35" s="9">
         <f>IF(OR(I35="",K35=""),"",K35*I35)</f>
-        <v>85403.5</v>
+        <v>86113.3</v>
       </c>
       <c r="M35" s="9">
         <f>IF(L35="","",L35-J35)</f>
-        <v>-13679.39</v>
+        <v>-12969.59</v>
       </c>
       <c r="N35" s="10">
         <f>IF(OR(H35="",K35=""),"",K35/H35-1)</f>
-        <v>-0.13806008873802267</v>
+        <v>-0.13089638995502495</v>
       </c>
       <c r="O35" s="6">
         <f>IF(G35="","",$B$3-G35)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P35" s="6" t="str">
         <f>IF(H35="","Pending buy",IF(N35&gt;=0,"In profit","In loss"))</f>
@@ -2685,23 +2685,23 @@
         <v>99910.57</v>
       </c>
       <c r="K36" s="9" t="n">
-        <v>89.41</v>
+        <v>89.77</v>
       </c>
       <c r="L36" s="9">
         <f>IF(OR(I36="",K36=""),"",K36*I36)</f>
-        <v>91645.25</v>
+        <v>92014.25</v>
       </c>
       <c r="M36" s="9">
         <f>IF(L36="","",L36-J36)</f>
-        <v>-8265.32</v>
+        <v>-7896.32</v>
       </c>
       <c r="N36" s="10">
         <f>IF(OR(H36="",K36=""),"",K36/H36-1)</f>
-        <v>-0.08272719393681138</v>
+        <v>-0.07903389106036862</v>
       </c>
       <c r="O36" s="6">
         <f>IF(G36="","",$B$3-G36)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P36" s="6" t="str">
         <f>IF(H36="","Pending buy",IF(N36&gt;=0,"In profit","In loss"))</f>
@@ -2753,23 +2753,23 @@
         <v>99436.51</v>
       </c>
       <c r="K37" s="9" t="n">
-        <v>989</v>
+        <v>946.5</v>
       </c>
       <c r="L37" s="9">
         <f>IF(OR(I37="",K37=""),"",K37*I37)</f>
-        <v>98900.0</v>
+        <v>94650.0</v>
       </c>
       <c r="M37" s="9">
         <f>IF(L37="","",L37-J37)</f>
-        <v>-536.51</v>
+        <v>-4786.51</v>
       </c>
       <c r="N37" s="10">
         <f>IF(OR(H37="",K37=""),"",K37/H37-1)</f>
-        <v>-0.005395532127514979</v>
+        <v>-0.04813637124235881</v>
       </c>
       <c r="O37" s="6">
         <f>IF(G37="","",$B$3-G37)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P37" s="6" t="str">
         <f>IF(H37="","Pending buy",IF(N37&gt;=0,"In profit","In loss"))</f>
@@ -2821,23 +2821,23 @@
         <v>99951.48</v>
       </c>
       <c r="K38" s="9" t="n">
-        <v>112.4</v>
+        <v>112.91</v>
       </c>
       <c r="L38" s="9">
         <f>IF(OR(I38="",K38=""),"",K38*I38)</f>
-        <v>92055.6</v>
+        <v>92473.29</v>
       </c>
       <c r="M38" s="9">
         <f>IF(L38="","",L38-J38)</f>
-        <v>-7895.88</v>
+        <v>-7478.19</v>
       </c>
       <c r="N38" s="10">
         <f>IF(OR(H38="",K38=""),"",K38/H38-1)</f>
-        <v>-0.07899712849495288</v>
+        <v>-0.07481820087513469</v>
       </c>
       <c r="O38" s="6">
         <f>IF(G38="","",$B$3-G38)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P38" s="6" t="str">
         <f>IF(H38="","Pending buy",IF(N38&gt;=0,"In profit","In loss"))</f>
@@ -2889,23 +2889,23 @@
         <v>99666.78</v>
       </c>
       <c r="K39" s="9" t="n">
-        <v>494.05</v>
+        <v>500.15</v>
       </c>
       <c r="L39" s="9">
         <f>IF(OR(I39="",K39=""),"",K39*I39)</f>
-        <v>88434.95</v>
+        <v>89526.85</v>
       </c>
       <c r="M39" s="9">
         <f>IF(L39="","",L39-J39)</f>
-        <v>-11231.83</v>
+        <v>-10139.93</v>
       </c>
       <c r="N39" s="10">
         <f>IF(OR(H39="",K39=""),"",K39/H39-1)</f>
-        <v>-0.1126937838701153</v>
+        <v>-0.1017382775076171</v>
       </c>
       <c r="O39" s="6">
         <f>IF(G39="","",$B$3-G39)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P39" s="6" t="str">
         <f>IF(H39="","Pending buy",IF(N39&gt;=0,"In profit","In loss"))</f>
@@ -2957,23 +2957,23 @@
         <v>99998.64</v>
       </c>
       <c r="K40" s="9" t="n">
-        <v>12.77</v>
+        <v>12.54</v>
       </c>
       <c r="L40" s="9">
         <f>IF(OR(I40="",K40=""),"",K40*I40)</f>
-        <v>98558.86</v>
+        <v>96783.72</v>
       </c>
       <c r="M40" s="9">
         <f>IF(L40="","",L40-J40)</f>
-        <v>-1439.78</v>
+        <v>-3214.92</v>
       </c>
       <c r="N40" s="10">
         <f>IF(OR(H40="",K40=""),"",K40/H40-1)</f>
-        <v>-0.014397970817535688</v>
+        <v>-0.03214961269004679</v>
       </c>
       <c r="O40" s="6">
         <f>IF(G40="","",$B$3-G40)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P40" s="6" t="str">
         <f>IF(H40="","Pending buy",IF(N40&gt;=0,"In profit","In loss"))</f>
@@ -3025,23 +3025,23 @@
         <v>99889.82</v>
       </c>
       <c r="K41" s="9" t="n">
-        <v>125.63</v>
+        <v>123.45</v>
       </c>
       <c r="L41" s="9">
         <f>IF(OR(I41="",K41=""),"",K41*I41)</f>
-        <v>99875.85</v>
+        <v>98142.75</v>
       </c>
       <c r="M41" s="9">
         <f>IF(L41="","",L41-J41)</f>
-        <v>-13.97</v>
+        <v>-1747.07</v>
       </c>
       <c r="N41" s="10">
         <f>IF(OR(H41="",K41=""),"",K41/H41-1)</f>
-        <v>-0.00013984353107787673</v>
+        <v>-0.01748996007252701</v>
       </c>
       <c r="O41" s="6">
         <f>IF(G41="","",$B$3-G41)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P41" s="6" t="str">
         <f>IF(H41="","Pending buy",IF(N41&gt;=0,"In profit","In loss"))</f>
@@ -3093,23 +3093,23 @@
         <v>99925.2</v>
       </c>
       <c r="K42" s="9" t="n">
-        <v>121.58</v>
+        <v>127.83</v>
       </c>
       <c r="L42" s="9">
         <f>IF(OR(I42="",K42=""),"",K42*I42)</f>
-        <v>129239.54</v>
+        <v>135883.29</v>
       </c>
       <c r="M42" s="9">
         <f>IF(L42="","",L42-J42)</f>
-        <v>29314.34</v>
+        <v>35958.09</v>
       </c>
       <c r="N42" s="10">
         <f>IF(OR(H42="",K42=""),"",K42/H42-1)</f>
-        <v>0.29336285394864325</v>
+        <v>0.359850087351991</v>
       </c>
       <c r="O42" s="6">
         <f>IF(G42="","",$B$3-G42)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="P42" s="6" t="str">
         <f>IF(H42="","Pending buy",IF(N42&gt;=0,"In profit","In loss"))</f>
@@ -3161,23 +3161,23 @@
         <v>99394.67</v>
       </c>
       <c r="K43" s="9" t="n">
-        <v>648.5</v>
+        <v>680.9</v>
       </c>
       <c r="L43" s="9">
         <f>IF(OR(I43="",K43=""),"",K43*I43)</f>
-        <v>101814.5</v>
+        <v>106901.3</v>
       </c>
       <c r="M43" s="9">
         <f>IF(L43="","",L43-J43)</f>
-        <v>2419.83</v>
+        <v>7506.63</v>
       </c>
       <c r="N43" s="10">
         <f>IF(OR(H43="",K43=""),"",K43/H43-1)</f>
-        <v>0.024345649105044664</v>
+        <v>0.07552344252216647</v>
       </c>
       <c r="O43" s="6">
         <f>IF(G43="","",$B$3-G43)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P43" s="6" t="str">
         <f>IF(H43="","Pending buy",IF(N43&gt;=0,"In profit","In loss"))</f>
@@ -3229,23 +3229,23 @@
         <v>99810.88</v>
       </c>
       <c r="K44" s="9" t="n">
-        <v>378.95</v>
+        <v>409.8</v>
       </c>
       <c r="L44" s="9">
         <f>IF(OR(I44="",K44=""),"",K44*I44)</f>
-        <v>114442.9</v>
+        <v>123759.6</v>
       </c>
       <c r="M44" s="9">
         <f>IF(L44="","",L44-J44)</f>
-        <v>14632.02</v>
+        <v>23948.72</v>
       </c>
       <c r="N44" s="10">
         <f>IF(OR(H44="",K44=""),"",K44/H44-1)</f>
-        <v>0.14659744040116918</v>
+        <v>0.2399409713059748</v>
       </c>
       <c r="O44" s="6">
         <f>IF(G44="","",$B$3-G44)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P44" s="6" t="str">
         <f>IF(H44="","Pending buy",IF(N44&gt;=0,"In profit","In loss"))</f>
@@ -3297,23 +3297,23 @@
         <v>99997.44</v>
       </c>
       <c r="K45" s="9" t="n">
-        <v>268.8</v>
+        <v>252.35</v>
       </c>
       <c r="L45" s="9">
         <f>IF(OR(I45="",K45=""),"",K45*I45)</f>
-        <v>99724.8</v>
+        <v>93621.85</v>
       </c>
       <c r="M45" s="9">
         <f>IF(L45="","",L45-J45)</f>
-        <v>-272.64</v>
+        <v>-6375.59</v>
       </c>
       <c r="N45" s="10">
         <f>IF(OR(H45="",K45=""),"",K45/H45-1)</f>
-        <v>-0.002726444984825549</v>
+        <v>-0.06375750889851461</v>
       </c>
       <c r="O45" s="6">
         <f>IF(G45="","",$B$3-G45)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P45" s="6" t="str">
         <f>IF(H45="","Pending buy",IF(N45&gt;=0,"In profit","In loss"))</f>
@@ -3365,23 +3365,23 @@
         <v>99870.37</v>
       </c>
       <c r="K46" s="9" t="n">
-        <v>351.4</v>
+        <v>357.15</v>
       </c>
       <c r="L46" s="9">
         <f>IF(OR(I46="",K46=""),"",K46*I46)</f>
-        <v>97689.2</v>
+        <v>99287.7</v>
       </c>
       <c r="M46" s="9">
         <f>IF(L46="","",L46-J46)</f>
-        <v>-2181.17</v>
+        <v>-582.67</v>
       </c>
       <c r="N46" s="10">
         <f>IF(OR(H46="",K46=""),"",K46/H46-1)</f>
-        <v>-0.0218399642330801</v>
+        <v>-0.005834215212989657</v>
       </c>
       <c r="O46" s="6">
         <f>IF(G46="","",$B$3-G46)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P46" s="6" t="str">
         <f>IF(H46="","Pending buy",IF(N46&gt;=0,"In profit","In loss"))</f>
@@ -3433,23 +3433,23 @@
         <v>99957.4</v>
       </c>
       <c r="K47" s="9" t="n">
-        <v>567.65</v>
+        <v>567.75</v>
       </c>
       <c r="L47" s="9">
         <f>IF(OR(I47="",K47=""),"",K47*I47)</f>
-        <v>98203.45</v>
+        <v>98220.75</v>
       </c>
       <c r="M47" s="9">
         <f>IF(L47="","",L47-J47)</f>
-        <v>-1753.95</v>
+        <v>-1736.65</v>
       </c>
       <c r="N47" s="10">
         <f>IF(OR(H47="",K47=""),"",K47/H47-1)</f>
-        <v>-0.01754696428822433</v>
+        <v>-0.017373890556926508</v>
       </c>
       <c r="O47" s="6">
         <f>IF(G47="","",$B$3-G47)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P47" s="6" t="str">
         <f>IF(H47="","Pending buy",IF(N47&gt;=0,"In profit","In loss"))</f>
@@ -3501,30 +3501,30 @@
         <v>99965.44</v>
       </c>
       <c r="K48" s="9" t="n">
-        <v>182.98</v>
+        <v>186.5</v>
       </c>
       <c r="L48" s="9">
         <f>IF(OR(I48="",K48=""),"",K48*I48)</f>
-        <v>101919.86</v>
+        <v>103880.5</v>
       </c>
       <c r="M48" s="9">
         <f>IF(L48="","",L48-J48)</f>
-        <v>1954.42</v>
+        <v>3915.06</v>
       </c>
       <c r="N48" s="10">
         <f>IF(OR(H48="",K48=""),"",K48/H48-1)</f>
-        <v>0.01955093389344409</v>
+        <v>0.03916411176700918</v>
       </c>
       <c r="O48" s="6">
         <f>IF(G48="","",$B$3-G48)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P48" s="6" t="str">
         <f>IF(H48="","Pending buy",IF(N48&gt;=0,"In profit","In loss"))</f>
         <v>In profit</v>
       </c>
       <c r="Q48" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49">
@@ -3569,23 +3569,23 @@
         <v>99985.7</v>
       </c>
       <c r="K49" s="9" t="n">
-        <v>879.4</v>
+        <v>867.85</v>
       </c>
       <c r="L49" s="9">
         <f>IF(OR(I49="",K49=""),"",K49*I49)</f>
-        <v>105528.0</v>
+        <v>104142.0</v>
       </c>
       <c r="M49" s="9">
         <f>IF(L49="","",L49-J49)</f>
-        <v>5542.3</v>
+        <v>4156.3</v>
       </c>
       <c r="N49" s="10">
         <f>IF(OR(H49="",K49=""),"",K49/H49-1)</f>
-        <v>0.05543096166782635</v>
+        <v>0.04156897894407918</v>
       </c>
       <c r="O49" s="6">
         <f>IF(G49="","",$B$3-G49)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P49" s="6" t="str">
         <f>IF(H49="","Pending buy",IF(N49&gt;=0,"In profit","In loss"))</f>
@@ -3637,23 +3637,23 @@
         <v>99961.35</v>
       </c>
       <c r="K50" s="9" t="n">
-        <v>94.84999999999999</v>
+        <v>93.76000000000001</v>
       </c>
       <c r="L50" s="9">
         <f>IF(OR(I50="",K50=""),"",K50*I50)</f>
-        <v>98644.0</v>
+        <v>97510.4</v>
       </c>
       <c r="M50" s="9">
         <f>IF(L50="","",L50-J50)</f>
-        <v>-1317.35</v>
+        <v>-2450.95</v>
       </c>
       <c r="N50" s="10">
         <f>IF(OR(H50="",K50=""),"",K50/H50-1)</f>
-        <v>-0.013178576151625654</v>
+        <v>-0.024518959409345342</v>
       </c>
       <c r="O50" s="6">
         <f>IF(G50="","",$B$3-G50)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P50" s="6" t="str">
         <f>IF(H50="","Pending buy",IF(N50&gt;=0,"In profit","In loss"))</f>
@@ -3705,23 +3705,23 @@
         <v>97877.65</v>
       </c>
       <c r="K51" s="9" t="n">
-        <v>3049</v>
+        <v>3074.5</v>
       </c>
       <c r="L51" s="9">
         <f>IF(OR(I51="",K51=""),"",K51*I51)</f>
-        <v>100617.0</v>
+        <v>101458.5</v>
       </c>
       <c r="M51" s="9">
         <f>IF(L51="","",L51-J51)</f>
-        <v>2739.35</v>
+        <v>3580.85</v>
       </c>
       <c r="N51" s="10">
         <f>IF(OR(H51="",K51=""),"",K51/H51-1)</f>
-        <v>0.02798752510671565</v>
+        <v>0.036584993748965955</v>
       </c>
       <c r="O51" s="6">
         <f>IF(G51="","",$B$3-G51)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P51" s="6" t="str">
         <f>IF(H51="","Pending buy",IF(N51&gt;=0,"In profit","In loss"))</f>
@@ -3773,23 +3773,23 @@
         <v>99357.46</v>
       </c>
       <c r="K52" s="9" t="n">
-        <v>932</v>
+        <v>935.6</v>
       </c>
       <c r="L52" s="9">
         <f>IF(OR(I52="",K52=""),"",K52*I52)</f>
-        <v>101588.0</v>
+        <v>101980.4</v>
       </c>
       <c r="M52" s="9">
         <f>IF(L52="","",L52-J52)</f>
-        <v>2230.54</v>
+        <v>2622.94</v>
       </c>
       <c r="N52" s="10">
         <f>IF(OR(H52="",K52=""),"",K52/H52-1)</f>
-        <v>0.022449672953674726</v>
+        <v>0.026399049372809014</v>
       </c>
       <c r="O52" s="6">
         <f>IF(G52="","",$B$3-G52)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P52" s="6" t="str">
         <f>IF(H52="","Pending buy",IF(N52&gt;=0,"In profit","In loss"))</f>
@@ -3841,23 +3841,23 @@
         <v>99747.01</v>
       </c>
       <c r="K53" s="9" t="n">
-        <v>879.45</v>
+        <v>873.6</v>
       </c>
       <c r="L53" s="9">
         <f>IF(OR(I53="",K53=""),"",K53*I53)</f>
-        <v>103775.1</v>
+        <v>103084.8</v>
       </c>
       <c r="M53" s="9">
         <f>IF(L53="","",L53-J53)</f>
-        <v>4028.09</v>
+        <v>3337.79</v>
       </c>
       <c r="N53" s="10">
         <f>IF(OR(H53="",K53=""),"",K53/H53-1)</f>
-        <v>0.04038306766141142</v>
+        <v>0.03346255945080334</v>
       </c>
       <c r="O53" s="6">
         <f>IF(G53="","",$B$3-G53)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P53" s="6" t="str">
         <f>IF(H53="","Pending buy",IF(N53&gt;=0,"In profit","In loss"))</f>
@@ -3909,23 +3909,23 @@
         <v>99711.32</v>
       </c>
       <c r="K54" s="9" t="n">
-        <v>1399.4</v>
+        <v>1397.4</v>
       </c>
       <c r="L54" s="9">
         <f>IF(OR(I54="",K54=""),"",K54*I54)</f>
-        <v>100756.8</v>
+        <v>100612.8</v>
       </c>
       <c r="M54" s="9">
         <f>IF(L54="","",L54-J54)</f>
-        <v>1045.48</v>
+        <v>901.48</v>
       </c>
       <c r="N54" s="10">
         <f>IF(OR(H54="",K54=""),"",K54/H54-1)</f>
-        <v>0.010485093427737624</v>
+        <v>0.009040924364670966</v>
       </c>
       <c r="O54" s="6">
         <f>IF(G54="","",$B$3-G54)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P54" s="6" t="str">
         <f>IF(H54="","Pending buy",IF(N54&gt;=0,"In profit","In loss"))</f>
@@ -3977,27 +3977,27 @@
         <v>98281.27</v>
       </c>
       <c r="K55" s="9" t="n">
-        <v>3766.9</v>
+        <v>3860.2</v>
       </c>
       <c r="L55" s="9">
         <f>IF(OR(I55="",K55=""),"",K55*I55)</f>
-        <v>97939.4</v>
+        <v>100365.2</v>
       </c>
       <c r="M55" s="9">
         <f>IF(L55="","",L55-J55)</f>
-        <v>-341.87</v>
+        <v>2083.93</v>
       </c>
       <c r="N55" s="10">
         <f>IF(OR(H55="",K55=""),"",K55/H55-1)</f>
-        <v>-0.003478522382164284</v>
+        <v>0.021203697443619163</v>
       </c>
       <c r="O55" s="6">
         <f>IF(G55="","",$B$3-G55)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P55" s="6" t="str">
         <f>IF(H55="","Pending buy",IF(N55&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q55" s="6" t="n">
         <v>1</v>
@@ -4045,23 +4045,23 @@
         <v>94906.63</v>
       </c>
       <c r="K56" s="9" t="n">
-        <v>5929.5</v>
+        <v>5896</v>
       </c>
       <c r="L56" s="9">
         <f>IF(OR(I56="",K56=""),"",K56*I56)</f>
-        <v>94872.0</v>
+        <v>94336.0</v>
       </c>
       <c r="M56" s="9">
         <f>IF(L56="","",L56-J56)</f>
-        <v>-34.63</v>
+        <v>-570.63</v>
       </c>
       <c r="N56" s="10">
         <f>IF(OR(H56="",K56=""),"",K56/H56-1)</f>
-        <v>-0.0003648942089597984</v>
+        <v>-0.006012550173880915</v>
       </c>
       <c r="O56" s="6">
         <f>IF(G56="","",$B$3-G56)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P56" s="6" t="str">
         <f>IF(H56="","Pending buy",IF(N56&gt;=0,"In profit","In loss"))</f>
@@ -4113,23 +4113,23 @@
         <v>99783.3</v>
       </c>
       <c r="K57" s="9" t="n">
-        <v>417.3</v>
+        <v>420.8</v>
       </c>
       <c r="L57" s="9">
         <f>IF(OR(I57="",K57=""),"",K57*I57)</f>
-        <v>98065.5</v>
+        <v>98888.0</v>
       </c>
       <c r="M57" s="9">
         <f>IF(L57="","",L57-J57)</f>
-        <v>-1717.8</v>
+        <v>-895.3</v>
       </c>
       <c r="N57" s="10">
         <f>IF(OR(H57="",K57=""),"",K57/H57-1)</f>
-        <v>-0.017215277250741567</v>
+        <v>-0.008972414730678335</v>
       </c>
       <c r="O57" s="6">
         <f>IF(G57="","",$B$3-G57)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P57" s="6" t="str">
         <f>IF(H57="","Pending buy",IF(N57&gt;=0,"In profit","In loss"))</f>
@@ -4181,23 +4181,23 @@
         <v>99967.09</v>
       </c>
       <c r="K58" s="9" t="n">
-        <v>78.97</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="L58" s="9">
         <f>IF(OR(I58="",K58=""),"",K58*I58)</f>
-        <v>100528.81</v>
+        <v>101076.2</v>
       </c>
       <c r="M58" s="9">
         <f>IF(L58="","",L58-J58)</f>
-        <v>561.72</v>
+        <v>1109.11</v>
       </c>
       <c r="N58" s="10">
         <f>IF(OR(H58="",K58=""),"",K58/H58-1)</f>
-        <v>0.005619063654426215</v>
+        <v>0.011094765786519467</v>
       </c>
       <c r="O58" s="6">
         <f>IF(G58="","",$B$3-G58)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P58" s="6" t="str">
         <f>IF(H58="","Pending buy",IF(N58&gt;=0,"In profit","In loss"))</f>
@@ -4207,8 +4207,136 @@
         <v>1</v>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Cemindia Projects Limited</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>CEMPRO</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>291026</t>
+        </is>
+      </c>
+      <c r="F59" s="8" t="n">
+        <v>46324</v>
+      </c>
+      <c r="G59" s="6" t="inlineStr"/>
+      <c r="H59" s="9" t="inlineStr"/>
+      <c r="I59" s="6" t="str">
+        <f>IF(H59="","",ROUNDDOWN($B$1/H59,0))</f>
+        <v/>
+      </c>
+      <c r="J59" s="9" t="str">
+        <f>IF(H59="","",H59*I59)</f>
+        <v/>
+      </c>
+      <c r="K59" s="9" t="n">
+        <v>1287.4</v>
+      </c>
+      <c r="L59" s="9" t="str">
+        <f>IF(OR(I59="",K59=""),"",K59*I59)</f>
+        <v/>
+      </c>
+      <c r="M59" s="9" t="str">
+        <f>IF(L59="","",L59-J59)</f>
+        <v/>
+      </c>
+      <c r="N59" s="10" t="str">
+        <f>IF(OR(H59="",K59=""),"",K59/H59-1)</f>
+        <v/>
+      </c>
+      <c r="O59" s="6" t="str">
+        <f>IF(G59="","",$B$3-G59)</f>
+        <v/>
+      </c>
+      <c r="P59" s="6" t="str">
+        <f>IF(H59="","Pending buy",IF(N59&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q59" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>Diamond Power Infrastructure Limited</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>DIACABS</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>291026</t>
+        </is>
+      </c>
+      <c r="F60" s="8" t="n">
+        <v>46324</v>
+      </c>
+      <c r="G60" s="6" t="inlineStr"/>
+      <c r="H60" s="9" t="inlineStr"/>
+      <c r="I60" s="6" t="str">
+        <f>IF(H60="","",ROUNDDOWN($B$1/H60,0))</f>
+        <v/>
+      </c>
+      <c r="J60" s="9" t="str">
+        <f>IF(H60="","",H60*I60)</f>
+        <v/>
+      </c>
+      <c r="K60" s="9" t="n">
+        <v>341.65</v>
+      </c>
+      <c r="L60" s="9" t="str">
+        <f>IF(OR(I60="",K60=""),"",K60*I60)</f>
+        <v/>
+      </c>
+      <c r="M60" s="9" t="str">
+        <f>IF(L60="","",L60-J60)</f>
+        <v/>
+      </c>
+      <c r="N60" s="10" t="str">
+        <f>IF(OR(H60="",K60=""),"",K60/H60-1)</f>
+        <v/>
+      </c>
+      <c r="O60" s="6" t="str">
+        <f>IF(G60="","",$B$3-G60)</f>
+        <v/>
+      </c>
+      <c r="P60" s="6" t="str">
+        <f>IF(H60="","Pending buy",IF(N60&gt;=0,"In profit","In loss"))</f>
+        <v>Pending buy</v>
+      </c>
+      <c r="Q60" s="6" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A8:Q58">
+  <conditionalFormatting sqref="A8:Q60">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$N8&gt;0</formula>
     </cfRule>
@@ -4226,7 +4354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5514,6 +5642,106 @@
       <c r="D64" s="11" t="inlineStr">
         <is>
           <t>Paisalo Digital Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>CEMPRO</t>
+        </is>
+      </c>
+      <c r="D65" s="11" t="inlineStr">
+        <is>
+          <t>Cemindia Projects Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>MANCREDIT</t>
+        </is>
+      </c>
+      <c r="D66" s="11" t="inlineStr">
+        <is>
+          <t>Mangal Credit and Fincorp Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>4★</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>UNIONBANK</t>
+        </is>
+      </c>
+      <c r="D67" s="11" t="inlineStr">
+        <is>
+          <t>Union Bank of India</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>DIACABS</t>
+        </is>
+      </c>
+      <c r="D68" s="11" t="inlineStr">
+        <is>
+          <t>Diamond Power Infrastructure Limited</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>5★</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>DIACABS</t>
+        </is>
+      </c>
+      <c r="D69" s="11" t="inlineStr">
+        <is>
+          <t>Diamond Power Infrastructure Limited</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum Portfolio: Friday report 2026-10-30
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -532,7 +532,7 @@
       </c>
       <c r="E1" s="2">
         <f>SUM(J8:J60)</f>
-        <v>5052225.67</v>
+        <v>5251124.56</v>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
@@ -541,7 +541,7 @@
       </c>
       <c r="G1" s="2">
         <f>SUM(L8:L60)</f>
-        <v>4891693.01</v>
+        <v>4995088.27</v>
       </c>
     </row>
     <row r="2">
@@ -552,7 +552,7 @@
       </c>
       <c r="E2" s="2">
         <f>SUM(M8:M60)</f>
-        <v>-160532.66</v>
+        <v>-256036.29</v>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" s="3">
         <f>IF(E1=0,"",G1/E1-1)</f>
-        <v>-0.03177464161057564</v>
+        <v>-0.04875837300648611</v>
       </c>
     </row>
     <row r="3">
@@ -571,7 +571,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
@@ -580,7 +580,7 @@
       </c>
       <c r="E3">
         <f>COUNTIF(M8:M60,"&gt;0")</f>
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
@@ -589,7 +589,7 @@
       </c>
       <c r="G3">
         <f>COUNTIF(M8:M60,"&lt;0")</f>
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4">
@@ -600,7 +600,7 @@
       </c>
       <c r="E4" s="3">
         <f>IF((E3+G3)=0,"",E3/(E3+G3))</f>
-        <v>0.3333333333333333</v>
+        <v>0.2830188679245283</v>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
@@ -609,7 +609,7 @@
       </c>
       <c r="G4" s="3">
         <f>AVERAGE(N8:N60)</f>
-        <v>-0.03195244959288102</v>
+        <v>-0.048869122008295456</v>
       </c>
     </row>
     <row r="5">
@@ -640,7 +640,7 @@
       </c>
       <c r="E6" s="3">
         <f>AVERAGEIF(D8:D60,"4★*",N8:N60)</f>
-        <v>-0.05965058830936478</v>
+        <v>-0.07623968635321751</v>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
@@ -649,7 +649,7 @@
       </c>
       <c r="G6" s="3">
         <f>AVERAGEIF(D8:D60,"5★*",N8:N60)</f>
-        <v>-0.01550667972996879</v>
+        <v>-0.03228090119319117</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
@@ -781,23 +781,23 @@
         <v>99851.29</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>293.25</v>
+        <v>288.75</v>
       </c>
       <c r="L8" s="9">
         <f>IF(OR(I8="",K8=""),"",K8*I8)</f>
-        <v>97359.0</v>
+        <v>95865.0</v>
       </c>
       <c r="M8" s="9">
         <f>IF(L8="","",L8-J8)</f>
-        <v>-2492.29</v>
+        <v>-3986.29</v>
       </c>
       <c r="N8" s="10">
         <f>IF(OR(H8="",K8=""),"",K8/H8-1)</f>
-        <v>-0.024960051790398174</v>
+        <v>-0.03992230163504673</v>
       </c>
       <c r="O8" s="6">
         <f>IF(G8="","",$B$3-G8)</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="P8" s="6" t="str">
         <f>IF(H8="","Pending buy",IF(N8&gt;=0,"In profit","In loss"))</f>
@@ -849,23 +849,23 @@
         <v>99687.42</v>
       </c>
       <c r="K9" s="9" t="n">
-        <v>337.85</v>
+        <v>343.65</v>
       </c>
       <c r="L9" s="9">
         <f>IF(OR(I9="",K9=""),"",K9*I9)</f>
-        <v>103382.1</v>
+        <v>105156.9</v>
       </c>
       <c r="M9" s="9">
         <f>IF(L9="","",L9-J9)</f>
-        <v>3694.68</v>
+        <v>5469.48</v>
       </c>
       <c r="N9" s="10">
         <f>IF(OR(H9="",K9=""),"",K9/H9-1)</f>
-        <v>0.037062648372899964</v>
+        <v>0.05486629898874362</v>
       </c>
       <c r="O9" s="6">
         <f>IF(G9="","",$B$3-G9)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P9" s="6" t="str">
         <f>IF(H9="","Pending buy",IF(N9&gt;=0,"In profit","In loss"))</f>
@@ -917,23 +917,23 @@
         <v>99607.14</v>
       </c>
       <c r="K10" s="9" t="n">
-        <v>1429.2</v>
+        <v>1394.4</v>
       </c>
       <c r="L10" s="9">
         <f>IF(OR(I10="",K10=""),"",K10*I10)</f>
-        <v>90039.6</v>
+        <v>87847.2</v>
       </c>
       <c r="M10" s="9">
         <f>IF(L10="","",L10-J10)</f>
-        <v>-9567.54</v>
+        <v>-11759.94</v>
       </c>
       <c r="N10" s="10">
         <f>IF(OR(H10="",K10=""),"",K10/H10-1)</f>
-        <v>-0.09605276125746687</v>
+        <v>-0.11806323138637831</v>
       </c>
       <c r="O10" s="6">
         <f>IF(G10="","",$B$3-G10)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P10" s="6" t="str">
         <f>IF(H10="","Pending buy",IF(N10&gt;=0,"In profit","In loss"))</f>
@@ -985,23 +985,23 @@
         <v>99927.23</v>
       </c>
       <c r="K11" s="9" t="n">
-        <v>62.76</v>
+        <v>60.98</v>
       </c>
       <c r="L11" s="9">
         <f>IF(OR(I11="",K11=""),"",K11*I11)</f>
-        <v>78512.76</v>
+        <v>76285.98</v>
       </c>
       <c r="M11" s="9">
         <f>IF(L11="","",L11-J11)</f>
-        <v>-21414.47</v>
+        <v>-23641.25</v>
       </c>
       <c r="N11" s="10">
         <f>IF(OR(H11="",K11=""),"",K11/H11-1)</f>
-        <v>-0.2143006495840739</v>
+        <v>-0.23658466557738733</v>
       </c>
       <c r="O11" s="6">
         <f>IF(G11="","",$B$3-G11)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P11" s="6" t="str">
         <f>IF(H11="","Pending buy",IF(N11&gt;=0,"In profit","In loss"))</f>
@@ -1053,23 +1053,23 @@
         <v>86537.12</v>
       </c>
       <c r="K12" s="9" t="n">
-        <v>19280</v>
+        <v>19700</v>
       </c>
       <c r="L12" s="9">
         <f>IF(OR(I12="",K12=""),"",K12*I12)</f>
-        <v>77120.0</v>
+        <v>78800.0</v>
       </c>
       <c r="M12" s="9">
         <f>IF(L12="","",L12-J12)</f>
-        <v>-9417.12</v>
+        <v>-7737.12</v>
       </c>
       <c r="N12" s="10">
         <f>IF(OR(H12="",K12=""),"",K12/H12-1)</f>
-        <v>-0.10882170056100504</v>
+        <v>-0.08940806540725099</v>
       </c>
       <c r="O12" s="6">
         <f>IF(G12="","",$B$3-G12)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P12" s="6" t="str">
         <f>IF(H12="","Pending buy",IF(N12&gt;=0,"In profit","In loss"))</f>
@@ -1121,23 +1121,23 @@
         <v>98177.53</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>1783.9</v>
+        <v>1736</v>
       </c>
       <c r="L13" s="9">
         <f>IF(OR(I13="",K13=""),"",K13*I13)</f>
-        <v>94546.7</v>
+        <v>92008.0</v>
       </c>
       <c r="M13" s="9">
         <f>IF(L13="","",L13-J13)</f>
-        <v>-3630.83</v>
+        <v>-6169.53</v>
       </c>
       <c r="N13" s="10">
         <f>IF(OR(H13="",K13=""),"",K13/H13-1)</f>
-        <v>-0.03698232213837338</v>
+        <v>-0.0628405803196459</v>
       </c>
       <c r="O13" s="6">
         <f>IF(G13="","",$B$3-G13)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P13" s="6" t="str">
         <f>IF(H13="","Pending buy",IF(N13&gt;=0,"In profit","In loss"))</f>
@@ -1189,23 +1189,23 @@
         <v>97667.46</v>
       </c>
       <c r="K14" s="9" t="n">
-        <v>4235</v>
+        <v>4086.7</v>
       </c>
       <c r="L14" s="9">
         <f>IF(OR(I14="",K14=""),"",K14*I14)</f>
-        <v>93170.0</v>
+        <v>89907.4</v>
       </c>
       <c r="M14" s="9">
         <f>IF(L14="","",L14-J14)</f>
-        <v>-4497.46</v>
+        <v>-7760.06</v>
       </c>
       <c r="N14" s="10">
         <f>IF(OR(H14="",K14=""),"",K14/H14-1)</f>
-        <v>-0.046048745278276404</v>
+        <v>-0.07945393325353767</v>
       </c>
       <c r="O14" s="6">
         <f>IF(G14="","",$B$3-G14)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="P14" s="6" t="str">
         <f>IF(H14="","Pending buy",IF(N14&gt;=0,"In profit","In loss"))</f>
@@ -1257,23 +1257,23 @@
         <v>99078.19</v>
       </c>
       <c r="K15" s="9" t="n">
-        <v>1359.2</v>
+        <v>1330.9</v>
       </c>
       <c r="L15" s="9">
         <f>IF(OR(I15="",K15=""),"",K15*I15)</f>
-        <v>86988.8</v>
+        <v>85177.6</v>
       </c>
       <c r="M15" s="9">
         <f>IF(L15="","",L15-J15)</f>
-        <v>-12089.39</v>
+        <v>-13900.59</v>
       </c>
       <c r="N15" s="10">
         <f>IF(OR(H15="",K15=""),"",K15/H15-1)</f>
-        <v>-0.1220186589883917</v>
+        <v>-0.14029917101798883</v>
       </c>
       <c r="O15" s="6">
         <f>IF(G15="","",$B$3-G15)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P15" s="6" t="str">
         <f>IF(H15="","Pending buy",IF(N15&gt;=0,"In profit","In loss"))</f>
@@ -1325,23 +1325,23 @@
         <v>98557.54</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>1663</v>
+        <v>1756</v>
       </c>
       <c r="L16" s="9">
         <f>IF(OR(I16="",K16=""),"",K16*I16)</f>
-        <v>113084.0</v>
+        <v>119408.0</v>
       </c>
       <c r="M16" s="9">
         <f>IF(L16="","",L16-J16)</f>
-        <v>14526.46</v>
+        <v>20850.46</v>
       </c>
       <c r="N16" s="10">
         <f>IF(OR(H16="",K16=""),"",K16/H16-1)</f>
-        <v>0.14739069174726938</v>
+        <v>0.2115562565894198</v>
       </c>
       <c r="O16" s="6">
         <f>IF(G16="","",$B$3-G16)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P16" s="6" t="str">
         <f>IF(H16="","Pending buy",IF(N16&gt;=0,"In profit","In loss"))</f>
@@ -1393,23 +1393,23 @@
         <v>99714.35</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>821.15</v>
+        <v>796.75</v>
       </c>
       <c r="L17" s="9">
         <f>IF(OR(I17="",K17=""),"",K17*I17)</f>
-        <v>94432.25</v>
+        <v>91626.25</v>
       </c>
       <c r="M17" s="9">
         <f>IF(L17="","",L17-J17)</f>
-        <v>-5282.1</v>
+        <v>-8088.1</v>
       </c>
       <c r="N17" s="10">
         <f>IF(OR(H17="",K17=""),"",K17/H17-1)</f>
-        <v>-0.052972316131299935</v>
+        <v>-0.08111269911418517</v>
       </c>
       <c r="O17" s="6">
         <f>IF(G17="","",$B$3-G17)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P17" s="6" t="str">
         <f>IF(H17="","Pending buy",IF(N17&gt;=0,"In profit","In loss"))</f>
@@ -1461,23 +1461,23 @@
         <v>99596.83</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>590.95</v>
+        <v>566.4</v>
       </c>
       <c r="L18" s="9">
         <f>IF(OR(I18="",K18=""),"",K18*I18)</f>
-        <v>83323.95</v>
+        <v>79862.4</v>
       </c>
       <c r="M18" s="9">
         <f>IF(L18="","",L18-J18)</f>
-        <v>-16272.88</v>
+        <v>-19734.43</v>
       </c>
       <c r="N18" s="10">
         <f>IF(OR(H18="",K18=""),"",K18/H18-1)</f>
-        <v>-0.16338756805025267</v>
+        <v>-0.19814319069915087</v>
       </c>
       <c r="O18" s="6">
         <f>IF(G18="","",$B$3-G18)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P18" s="6" t="str">
         <f>IF(H18="","Pending buy",IF(N18&gt;=0,"In profit","In loss"))</f>
@@ -1529,23 +1529,23 @@
         <v>99993.07</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>126.35</v>
+        <v>120.86</v>
       </c>
       <c r="L19" s="9">
         <f>IF(OR(I19="",K19=""),"",K19*I19)</f>
-        <v>83770.05</v>
+        <v>80130.18</v>
       </c>
       <c r="M19" s="9">
         <f>IF(L19="","",L19-J19)</f>
-        <v>-16223.02</v>
+        <v>-19862.89</v>
       </c>
       <c r="N19" s="10">
         <f>IF(OR(H19="",K19=""),"",K19/H19-1)</f>
-        <v>-0.16224140386248032</v>
+        <v>-0.19864262818218736</v>
       </c>
       <c r="O19" s="6">
         <f>IF(G19="","",$B$3-G19)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P19" s="6" t="str">
         <f>IF(H19="","Pending buy",IF(N19&gt;=0,"In profit","In loss"))</f>
@@ -1597,27 +1597,27 @@
         <v>99896.43</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>213.7</v>
+        <v>200.01</v>
       </c>
       <c r="L20" s="9">
         <f>IF(OR(I20="",K20=""),"",K20*I20)</f>
-        <v>101934.9</v>
+        <v>95404.77</v>
       </c>
       <c r="M20" s="9">
         <f>IF(L20="","",L20-J20)</f>
-        <v>2038.47</v>
+        <v>-4491.66</v>
       </c>
       <c r="N20" s="10">
         <f>IF(OR(H20="",K20=""),"",K20/H20-1)</f>
-        <v>0.020405834261320033</v>
+        <v>-0.04496316841082537</v>
       </c>
       <c r="O20" s="6">
         <f>IF(G20="","",$B$3-G20)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P20" s="6" t="str">
         <f>IF(H20="","Pending buy",IF(N20&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q20" s="6" t="n">
         <v>1</v>
@@ -1665,23 +1665,23 @@
         <v>99449.47</v>
       </c>
       <c r="K21" s="9" t="n">
-        <v>1219.2</v>
+        <v>1133.9</v>
       </c>
       <c r="L21" s="9">
         <f>IF(OR(I21="",K21=""),"",K21*I21)</f>
-        <v>86563.2</v>
+        <v>80506.9</v>
       </c>
       <c r="M21" s="9">
         <f>IF(L21="","",L21-J21)</f>
-        <v>-12886.27</v>
+        <v>-18942.57</v>
       </c>
       <c r="N21" s="10">
         <f>IF(OR(H21="",K21=""),"",K21/H21-1)</f>
-        <v>-0.1295760230132732</v>
+        <v>-0.19047428846354197</v>
       </c>
       <c r="O21" s="6">
         <f>IF(G21="","",$B$3-G21)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P21" s="6" t="str">
         <f>IF(H21="","Pending buy",IF(N21&gt;=0,"In profit","In loss"))</f>
@@ -1733,23 +1733,23 @@
         <v>99837.05</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>642.85</v>
+        <v>635.05</v>
       </c>
       <c r="L22" s="9">
         <f>IF(OR(I22="",K22=""),"",K22*I22)</f>
-        <v>92570.4</v>
+        <v>91447.2</v>
       </c>
       <c r="M22" s="9">
         <f>IF(L22="","",L22-J22)</f>
-        <v>-7266.65</v>
+        <v>-8389.85</v>
       </c>
       <c r="N22" s="10">
         <f>IF(OR(H22="",K22=""),"",K22/H22-1)</f>
-        <v>-0.07278511372762586</v>
+        <v>-0.08403544601808954</v>
       </c>
       <c r="O22" s="6">
         <f>IF(G22="","",$B$3-G22)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P22" s="6" t="str">
         <f>IF(H22="","Pending buy",IF(N22&gt;=0,"In profit","In loss"))</f>
@@ -1801,23 +1801,23 @@
         <v>99486.88</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>577.85</v>
+        <v>542.15</v>
       </c>
       <c r="L23" s="9">
         <f>IF(OR(I23="",K23=""),"",K23*I23)</f>
-        <v>83788.25</v>
+        <v>78611.75</v>
       </c>
       <c r="M23" s="9">
         <f>IF(L23="","",L23-J23)</f>
-        <v>-15698.63</v>
+        <v>-20875.13</v>
       </c>
       <c r="N23" s="10">
         <f>IF(OR(H23="",K23=""),"",K23/H23-1)</f>
-        <v>-0.15779599282058854</v>
+        <v>-0.20982797872749348</v>
       </c>
       <c r="O23" s="6">
         <f>IF(G23="","",$B$3-G23)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P23" s="6" t="str">
         <f>IF(H23="","Pending buy",IF(N23&gt;=0,"In profit","In loss"))</f>
@@ -1869,23 +1869,23 @@
         <v>99935.4</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>239.94</v>
+        <v>237.2</v>
       </c>
       <c r="L24" s="9">
         <f>IF(OR(I24="",K24=""),"",K24*I24)</f>
-        <v>105333.66</v>
+        <v>104130.8</v>
       </c>
       <c r="M24" s="9">
         <f>IF(L24="","",L24-J24)</f>
-        <v>5398.26</v>
+        <v>4195.4</v>
       </c>
       <c r="N24" s="10">
         <f>IF(OR(H24="",K24=""),"",K24/H24-1)</f>
-        <v>0.054017510036107774</v>
+        <v>0.04198113436927886</v>
       </c>
       <c r="O24" s="6">
         <f>IF(G24="","",$B$3-G24)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="P24" s="6" t="str">
         <f>IF(H24="","Pending buy",IF(N24&gt;=0,"In profit","In loss"))</f>
@@ -1937,23 +1937,23 @@
         <v>99622.64</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>722.85</v>
+        <v>715.45</v>
       </c>
       <c r="L25" s="9">
         <f>IF(OR(I25="",K25=""),"",K25*I25)</f>
-        <v>89633.4</v>
+        <v>88715.8</v>
       </c>
       <c r="M25" s="9">
         <f>IF(L25="","",L25-J25)</f>
-        <v>-9989.24</v>
+        <v>-10906.84</v>
       </c>
       <c r="N25" s="10">
         <f>IF(OR(H25="",K25=""),"",K25/H25-1)</f>
-        <v>-0.10027074923708967</v>
+        <v>-0.10948150728598716</v>
       </c>
       <c r="O25" s="6">
         <f>IF(G25="","",$B$3-G25)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="P25" s="6" t="str">
         <f>IF(H25="","Pending buy",IF(N25&gt;=0,"In profit","In loss"))</f>
@@ -2005,23 +2005,23 @@
         <v>99948.17</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>190.02</v>
+        <v>186.29</v>
       </c>
       <c r="L26" s="9">
         <f>IF(OR(I26="",K26=""),"",K26*I26)</f>
-        <v>90259.5</v>
+        <v>88487.75</v>
       </c>
       <c r="M26" s="9">
         <f>IF(L26="","",L26-J26)</f>
-        <v>-9688.67</v>
+        <v>-11460.42</v>
       </c>
       <c r="N26" s="10">
         <f>IF(OR(H26="",K26=""),"",K26/H26-1)</f>
-        <v>-0.09693691237483615</v>
+        <v>-0.11466360070681114</v>
       </c>
       <c r="O26" s="6">
         <f>IF(G26="","",$B$3-G26)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="P26" s="6" t="str">
         <f>IF(H26="","Pending buy",IF(N26&gt;=0,"In profit","In loss"))</f>
@@ -2073,23 +2073,23 @@
         <v>99745.27</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>210.9</v>
+        <v>203.1</v>
       </c>
       <c r="L27" s="9">
         <f>IF(OR(I27="",K27=""),"",K27*I27)</f>
-        <v>80563.8</v>
+        <v>77584.2</v>
       </c>
       <c r="M27" s="9">
         <f>IF(L27="","",L27-J27)</f>
-        <v>-19181.47</v>
+        <v>-22161.07</v>
       </c>
       <c r="N27" s="10">
         <f>IF(OR(H27="",K27=""),"",K27/H27-1)</f>
-        <v>-0.19230458136790274</v>
+        <v>-0.22217667366439575</v>
       </c>
       <c r="O27" s="6">
         <f>IF(G27="","",$B$3-G27)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P27" s="6" t="str">
         <f>IF(H27="","Pending buy",IF(N27&gt;=0,"In profit","In loss"))</f>
@@ -2141,27 +2141,27 @@
         <v>95334.84</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>10833</v>
+        <v>10271</v>
       </c>
       <c r="L28" s="9">
         <f>IF(OR(I28="",K28=""),"",K28*I28)</f>
-        <v>97497.0</v>
+        <v>92439.0</v>
       </c>
       <c r="M28" s="9">
         <f>IF(L28="","",L28-J28)</f>
-        <v>2162.16</v>
+        <v>-2895.84</v>
       </c>
       <c r="N28" s="10">
         <f>IF(OR(H28="",K28=""),"",K28/H28-1)</f>
-        <v>0.02267961588549383</v>
+        <v>-0.030375488344880797</v>
       </c>
       <c r="O28" s="6">
         <f>IF(G28="","",$B$3-G28)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P28" s="6" t="str">
         <f>IF(H28="","Pending buy",IF(N28&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q28" s="6" t="n">
         <v>1</v>
@@ -2209,23 +2209,23 @@
         <v>98598.59</v>
       </c>
       <c r="K29" s="9" t="n">
-        <v>1800.1</v>
+        <v>1748.2</v>
       </c>
       <c r="L29" s="9">
         <f>IF(OR(I29="",K29=""),"",K29*I29)</f>
-        <v>91805.1</v>
+        <v>89158.2</v>
       </c>
       <c r="M29" s="9">
         <f>IF(L29="","",L29-J29)</f>
-        <v>-6793.49</v>
+        <v>-9440.39</v>
       </c>
       <c r="N29" s="10">
         <f>IF(OR(H29="",K29=""),"",K29/H29-1)</f>
-        <v>-0.06890044290167796</v>
+        <v>-0.09574565539731872</v>
       </c>
       <c r="O29" s="6">
         <f>IF(G29="","",$B$3-G29)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P29" s="6" t="str">
         <f>IF(H29="","Pending buy",IF(N29&gt;=0,"In profit","In loss"))</f>
@@ -2277,23 +2277,23 @@
         <v>99998.69</v>
       </c>
       <c r="K30" s="9" t="n">
-        <v>15.28</v>
+        <v>14.98</v>
       </c>
       <c r="L30" s="9">
         <f>IF(OR(I30="",K30=""),"",K30*I30)</f>
-        <v>103033.04</v>
+        <v>101010.14</v>
       </c>
       <c r="M30" s="9">
         <f>IF(L30="","",L30-J30)</f>
-        <v>3034.35</v>
+        <v>1011.45</v>
       </c>
       <c r="N30" s="10">
         <f>IF(OR(H30="",K30=""),"",K30/H30-1)</f>
-        <v>0.03034389750505717</v>
+        <v>0.010114632501685872</v>
       </c>
       <c r="O30" s="6">
         <f>IF(G30="","",$B$3-G30)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="P30" s="6" t="str">
         <f>IF(H30="","Pending buy",IF(N30&gt;=0,"In profit","In loss"))</f>
@@ -2345,23 +2345,23 @@
         <v>99977.34</v>
       </c>
       <c r="K31" s="9" t="n">
-        <v>144.85</v>
+        <v>139.28</v>
       </c>
       <c r="L31" s="9">
         <f>IF(OR(I31="",K31=""),"",K31*I31)</f>
-        <v>81695.4</v>
+        <v>78553.92</v>
       </c>
       <c r="M31" s="9">
         <f>IF(L31="","",L31-J31)</f>
-        <v>-18281.94</v>
+        <v>-21423.42</v>
       </c>
       <c r="N31" s="10">
         <f>IF(OR(H31="",K31=""),"",K31/H31-1)</f>
-        <v>-0.18286082135750104</v>
+        <v>-0.21428274213788567</v>
       </c>
       <c r="O31" s="6">
         <f>IF(G31="","",$B$3-G31)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P31" s="6" t="str">
         <f>IF(H31="","Pending buy",IF(N31&gt;=0,"In profit","In loss"))</f>
@@ -2413,23 +2413,23 @@
         <v>99923.82</v>
       </c>
       <c r="K32" s="9" t="n">
-        <v>175.16</v>
+        <v>167.34</v>
       </c>
       <c r="L32" s="9">
         <f>IF(OR(I32="",K32=""),"",K32*I32)</f>
-        <v>98965.4</v>
+        <v>94547.1</v>
       </c>
       <c r="M32" s="9">
         <f>IF(L32="","",L32-J32)</f>
-        <v>-958.42</v>
+        <v>-5376.72</v>
       </c>
       <c r="N32" s="10">
         <f>IF(OR(H32="",K32=""),"",K32/H32-1)</f>
-        <v>-0.009591503539047919</v>
+        <v>-0.05380818795515119</v>
       </c>
       <c r="O32" s="6">
         <f>IF(G32="","",$B$3-G32)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P32" s="6" t="str">
         <f>IF(H32="","Pending buy",IF(N32&gt;=0,"In profit","In loss"))</f>
@@ -2481,23 +2481,23 @@
         <v>99608.58</v>
       </c>
       <c r="K33" s="9" t="n">
-        <v>498.7</v>
+        <v>489.7</v>
       </c>
       <c r="L33" s="9">
         <f>IF(OR(I33="",K33=""),"",K33*I33)</f>
-        <v>94254.3</v>
+        <v>92553.3</v>
       </c>
       <c r="M33" s="9">
         <f>IF(L33="","",L33-J33)</f>
-        <v>-5354.28</v>
+        <v>-7055.28</v>
       </c>
       <c r="N33" s="10">
         <f>IF(OR(H33="",K33=""),"",K33/H33-1)</f>
-        <v>-0.053753154439184714</v>
+        <v>-0.0708299974511104</v>
       </c>
       <c r="O33" s="6">
         <f>IF(G33="","",$B$3-G33)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P33" s="6" t="str">
         <f>IF(H33="","Pending buy",IF(N33&gt;=0,"In profit","In loss"))</f>
@@ -2549,23 +2549,23 @@
         <v>96030.46</v>
       </c>
       <c r="K34" s="9" t="n">
-        <v>4387</v>
+        <v>4172.6</v>
       </c>
       <c r="L34" s="9">
         <f>IF(OR(I34="",K34=""),"",K34*I34)</f>
-        <v>83353.0</v>
+        <v>79279.4</v>
       </c>
       <c r="M34" s="9">
         <f>IF(L34="","",L34-J34)</f>
-        <v>-12677.46</v>
+        <v>-16751.06</v>
       </c>
       <c r="N34" s="10">
         <f>IF(OR(H34="",K34=""),"",K34/H34-1)</f>
-        <v>-0.1320149942975294</v>
+        <v>-0.17443486783812878</v>
       </c>
       <c r="O34" s="6">
         <f>IF(G34="","",$B$3-G34)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P34" s="6" t="str">
         <f>IF(H34="","Pending buy",IF(N34&gt;=0,"In profit","In loss"))</f>
@@ -2617,23 +2617,23 @@
         <v>99082.89</v>
       </c>
       <c r="K35" s="9" t="n">
-        <v>946.3</v>
+        <v>932</v>
       </c>
       <c r="L35" s="9">
         <f>IF(OR(I35="",K35=""),"",K35*I35)</f>
-        <v>86113.3</v>
+        <v>84812.0</v>
       </c>
       <c r="M35" s="9">
         <f>IF(L35="","",L35-J35)</f>
-        <v>-12969.59</v>
+        <v>-14270.89</v>
       </c>
       <c r="N35" s="10">
         <f>IF(OR(H35="",K35=""),"",K35/H35-1)</f>
-        <v>-0.13089638995502495</v>
+        <v>-0.14402983772385414</v>
       </c>
       <c r="O35" s="6">
         <f>IF(G35="","",$B$3-G35)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P35" s="6" t="str">
         <f>IF(H35="","Pending buy",IF(N35&gt;=0,"In profit","In loss"))</f>
@@ -2685,23 +2685,23 @@
         <v>99910.57</v>
       </c>
       <c r="K36" s="9" t="n">
-        <v>89.77</v>
+        <v>87.06999999999999</v>
       </c>
       <c r="L36" s="9">
         <f>IF(OR(I36="",K36=""),"",K36*I36)</f>
-        <v>92014.25</v>
+        <v>89246.75</v>
       </c>
       <c r="M36" s="9">
         <f>IF(L36="","",L36-J36)</f>
-        <v>-7896.32</v>
+        <v>-10663.82</v>
       </c>
       <c r="N36" s="10">
         <f>IF(OR(H36="",K36=""),"",K36/H36-1)</f>
-        <v>-0.07903389106036862</v>
+        <v>-0.10673366263368933</v>
       </c>
       <c r="O36" s="6">
         <f>IF(G36="","",$B$3-G36)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P36" s="6" t="str">
         <f>IF(H36="","Pending buy",IF(N36&gt;=0,"In profit","In loss"))</f>
@@ -2753,23 +2753,23 @@
         <v>99436.51</v>
       </c>
       <c r="K37" s="9" t="n">
-        <v>946.5</v>
+        <v>944.8</v>
       </c>
       <c r="L37" s="9">
         <f>IF(OR(I37="",K37=""),"",K37*I37)</f>
-        <v>94650.0</v>
+        <v>94480.0</v>
       </c>
       <c r="M37" s="9">
         <f>IF(L37="","",L37-J37)</f>
-        <v>-4786.51</v>
+        <v>-4956.51</v>
       </c>
       <c r="N37" s="10">
         <f>IF(OR(H37="",K37=""),"",K37/H37-1)</f>
-        <v>-0.04813637124235881</v>
+        <v>-0.04984600480695267</v>
       </c>
       <c r="O37" s="6">
         <f>IF(G37="","",$B$3-G37)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P37" s="6" t="str">
         <f>IF(H37="","Pending buy",IF(N37&gt;=0,"In profit","In loss"))</f>
@@ -2821,23 +2821,23 @@
         <v>99951.48</v>
       </c>
       <c r="K38" s="9" t="n">
-        <v>112.91</v>
+        <v>114.85</v>
       </c>
       <c r="L38" s="9">
         <f>IF(OR(I38="",K38=""),"",K38*I38)</f>
-        <v>92473.29</v>
+        <v>94062.15</v>
       </c>
       <c r="M38" s="9">
         <f>IF(L38="","",L38-J38)</f>
-        <v>-7478.19</v>
+        <v>-5889.33</v>
       </c>
       <c r="N38" s="10">
         <f>IF(OR(H38="",K38=""),"",K38/H38-1)</f>
-        <v>-0.07481820087513469</v>
+        <v>-0.05892188796837505</v>
       </c>
       <c r="O38" s="6">
         <f>IF(G38="","",$B$3-G38)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P38" s="6" t="str">
         <f>IF(H38="","Pending buy",IF(N38&gt;=0,"In profit","In loss"))</f>
@@ -2889,23 +2889,23 @@
         <v>99666.78</v>
       </c>
       <c r="K39" s="9" t="n">
-        <v>500.15</v>
+        <v>492.15</v>
       </c>
       <c r="L39" s="9">
         <f>IF(OR(I39="",K39=""),"",K39*I39)</f>
-        <v>89526.85</v>
+        <v>88094.85</v>
       </c>
       <c r="M39" s="9">
         <f>IF(L39="","",L39-J39)</f>
-        <v>-10139.93</v>
+        <v>-11571.93</v>
       </c>
       <c r="N39" s="10">
         <f>IF(OR(H39="",K39=""),"",K39/H39-1)</f>
-        <v>-0.1017382775076171</v>
+        <v>-0.11610615470433616</v>
       </c>
       <c r="O39" s="6">
         <f>IF(G39="","",$B$3-G39)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P39" s="6" t="str">
         <f>IF(H39="","Pending buy",IF(N39&gt;=0,"In profit","In loss"))</f>
@@ -2957,23 +2957,23 @@
         <v>99998.64</v>
       </c>
       <c r="K40" s="9" t="n">
-        <v>12.54</v>
+        <v>12.03</v>
       </c>
       <c r="L40" s="9">
         <f>IF(OR(I40="",K40=""),"",K40*I40)</f>
-        <v>96783.72</v>
+        <v>92847.54</v>
       </c>
       <c r="M40" s="9">
         <f>IF(L40="","",L40-J40)</f>
-        <v>-3214.92</v>
+        <v>-7151.1</v>
       </c>
       <c r="N40" s="10">
         <f>IF(OR(H40="",K40=""),"",K40/H40-1)</f>
-        <v>-0.03214961269004679</v>
+        <v>-0.07151194901604963</v>
       </c>
       <c r="O40" s="6">
         <f>IF(G40="","",$B$3-G40)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="P40" s="6" t="str">
         <f>IF(H40="","Pending buy",IF(N40&gt;=0,"In profit","In loss"))</f>
@@ -3025,23 +3025,23 @@
         <v>99889.82</v>
       </c>
       <c r="K41" s="9" t="n">
-        <v>123.45</v>
+        <v>120.56</v>
       </c>
       <c r="L41" s="9">
         <f>IF(OR(I41="",K41=""),"",K41*I41)</f>
-        <v>98142.75</v>
+        <v>95845.2</v>
       </c>
       <c r="M41" s="9">
         <f>IF(L41="","",L41-J41)</f>
-        <v>-1747.07</v>
+        <v>-4044.62</v>
       </c>
       <c r="N41" s="10">
         <f>IF(OR(H41="",K41=""),"",K41/H41-1)</f>
-        <v>-0.01748996007252701</v>
+        <v>-0.040490802643530555</v>
       </c>
       <c r="O41" s="6">
         <f>IF(G41="","",$B$3-G41)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P41" s="6" t="str">
         <f>IF(H41="","Pending buy",IF(N41&gt;=0,"In profit","In loss"))</f>
@@ -3093,23 +3093,23 @@
         <v>99925.2</v>
       </c>
       <c r="K42" s="9" t="n">
-        <v>127.83</v>
+        <v>134.6</v>
       </c>
       <c r="L42" s="9">
         <f>IF(OR(I42="",K42=""),"",K42*I42)</f>
-        <v>135883.29</v>
+        <v>143079.8</v>
       </c>
       <c r="M42" s="9">
         <f>IF(L42="","",L42-J42)</f>
-        <v>35958.09</v>
+        <v>43154.6</v>
       </c>
       <c r="N42" s="10">
         <f>IF(OR(H42="",K42=""),"",K42/H42-1)</f>
-        <v>0.359850087351991</v>
+        <v>0.4318690585744971</v>
       </c>
       <c r="O42" s="6">
         <f>IF(G42="","",$B$3-G42)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P42" s="6" t="str">
         <f>IF(H42="","Pending buy",IF(N42&gt;=0,"In profit","In loss"))</f>
@@ -3161,23 +3161,23 @@
         <v>99394.67</v>
       </c>
       <c r="K43" s="9" t="n">
-        <v>680.9</v>
+        <v>647.5</v>
       </c>
       <c r="L43" s="9">
         <f>IF(OR(I43="",K43=""),"",K43*I43)</f>
-        <v>106901.3</v>
+        <v>101657.5</v>
       </c>
       <c r="M43" s="9">
         <f>IF(L43="","",L43-J43)</f>
-        <v>7506.63</v>
+        <v>2262.83</v>
       </c>
       <c r="N43" s="10">
         <f>IF(OR(H43="",K43=""),"",K43/H43-1)</f>
-        <v>0.07552344252216647</v>
+        <v>0.022766087579825012</v>
       </c>
       <c r="O43" s="6">
         <f>IF(G43="","",$B$3-G43)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P43" s="6" t="str">
         <f>IF(H43="","Pending buy",IF(N43&gt;=0,"In profit","In loss"))</f>
@@ -3229,23 +3229,23 @@
         <v>99810.88</v>
       </c>
       <c r="K44" s="9" t="n">
-        <v>409.8</v>
+        <v>368.2</v>
       </c>
       <c r="L44" s="9">
         <f>IF(OR(I44="",K44=""),"",K44*I44)</f>
-        <v>123759.6</v>
+        <v>111196.4</v>
       </c>
       <c r="M44" s="9">
         <f>IF(L44="","",L44-J44)</f>
-        <v>23948.72</v>
+        <v>11385.52</v>
       </c>
       <c r="N44" s="10">
         <f>IF(OR(H44="",K44=""),"",K44/H44-1)</f>
-        <v>0.2399409713059748</v>
+        <v>0.11407092639058058</v>
       </c>
       <c r="O44" s="6">
         <f>IF(G44="","",$B$3-G44)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P44" s="6" t="str">
         <f>IF(H44="","Pending buy",IF(N44&gt;=0,"In profit","In loss"))</f>
@@ -3297,27 +3297,27 @@
         <v>99997.44</v>
       </c>
       <c r="K45" s="9" t="n">
-        <v>252.35</v>
+        <v>276.2</v>
       </c>
       <c r="L45" s="9">
         <f>IF(OR(I45="",K45=""),"",K45*I45)</f>
-        <v>93621.85</v>
+        <v>102470.2</v>
       </c>
       <c r="M45" s="9">
         <f>IF(L45="","",L45-J45)</f>
-        <v>-6375.59</v>
+        <v>2472.76</v>
       </c>
       <c r="N45" s="10">
         <f>IF(OR(H45="",K45=""),"",K45/H45-1)</f>
-        <v>-0.06375750889851461</v>
+        <v>0.024728258538657677</v>
       </c>
       <c r="O45" s="6">
         <f>IF(G45="","",$B$3-G45)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P45" s="6" t="str">
         <f>IF(H45="","Pending buy",IF(N45&gt;=0,"In profit","In loss"))</f>
-        <v>In loss</v>
+        <v>In profit</v>
       </c>
       <c r="Q45" s="6" t="n">
         <v>1</v>
@@ -3365,23 +3365,23 @@
         <v>99870.37</v>
       </c>
       <c r="K46" s="9" t="n">
-        <v>357.15</v>
+        <v>326.95</v>
       </c>
       <c r="L46" s="9">
         <f>IF(OR(I46="",K46=""),"",K46*I46)</f>
-        <v>99287.7</v>
+        <v>90892.1</v>
       </c>
       <c r="M46" s="9">
         <f>IF(L46="","",L46-J46)</f>
-        <v>-582.67</v>
+        <v>-8978.27</v>
       </c>
       <c r="N46" s="10">
         <f>IF(OR(H46="",K46=""),"",K46/H46-1)</f>
-        <v>-0.005834215212989657</v>
+        <v>-0.08989919267502999</v>
       </c>
       <c r="O46" s="6">
         <f>IF(G46="","",$B$3-G46)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P46" s="6" t="str">
         <f>IF(H46="","Pending buy",IF(N46&gt;=0,"In profit","In loss"))</f>
@@ -3433,23 +3433,23 @@
         <v>99957.4</v>
       </c>
       <c r="K47" s="9" t="n">
-        <v>567.75</v>
+        <v>573.6</v>
       </c>
       <c r="L47" s="9">
         <f>IF(OR(I47="",K47=""),"",K47*I47)</f>
-        <v>98220.75</v>
+        <v>99232.8</v>
       </c>
       <c r="M47" s="9">
         <f>IF(L47="","",L47-J47)</f>
-        <v>-1736.65</v>
+        <v>-724.6</v>
       </c>
       <c r="N47" s="10">
         <f>IF(OR(H47="",K47=""),"",K47/H47-1)</f>
-        <v>-0.017373890556926508</v>
+        <v>-0.007249077276007099</v>
       </c>
       <c r="O47" s="6">
         <f>IF(G47="","",$B$3-G47)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P47" s="6" t="str">
         <f>IF(H47="","Pending buy",IF(N47&gt;=0,"In profit","In loss"))</f>
@@ -3501,23 +3501,23 @@
         <v>99965.44</v>
       </c>
       <c r="K48" s="9" t="n">
-        <v>186.5</v>
+        <v>186</v>
       </c>
       <c r="L48" s="9">
         <f>IF(OR(I48="",K48=""),"",K48*I48)</f>
-        <v>103880.5</v>
+        <v>103602.0</v>
       </c>
       <c r="M48" s="9">
         <f>IF(L48="","",L48-J48)</f>
-        <v>3915.06</v>
+        <v>3636.56</v>
       </c>
       <c r="N48" s="10">
         <f>IF(OR(H48="",K48=""),"",K48/H48-1)</f>
-        <v>0.03916411176700918</v>
+        <v>0.03637814900087766</v>
       </c>
       <c r="O48" s="6">
         <f>IF(G48="","",$B$3-G48)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P48" s="6" t="str">
         <f>IF(H48="","Pending buy",IF(N48&gt;=0,"In profit","In loss"))</f>
@@ -3569,27 +3569,27 @@
         <v>99985.7</v>
       </c>
       <c r="K49" s="9" t="n">
-        <v>867.85</v>
+        <v>824.5</v>
       </c>
       <c r="L49" s="9">
         <f>IF(OR(I49="",K49=""),"",K49*I49)</f>
-        <v>104142.0</v>
+        <v>98940.0</v>
       </c>
       <c r="M49" s="9">
         <f>IF(L49="","",L49-J49)</f>
-        <v>4156.3</v>
+        <v>-1045.7</v>
       </c>
       <c r="N49" s="10">
         <f>IF(OR(H49="",K49=""),"",K49/H49-1)</f>
-        <v>0.04156897894407918</v>
+        <v>-0.01045846270738815</v>
       </c>
       <c r="O49" s="6">
         <f>IF(G49="","",$B$3-G49)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P49" s="6" t="str">
         <f>IF(H49="","Pending buy",IF(N49&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q49" s="6" t="n">
         <v>1</v>
@@ -3637,23 +3637,23 @@
         <v>99961.35</v>
       </c>
       <c r="K50" s="9" t="n">
-        <v>93.76000000000001</v>
+        <v>89.26000000000001</v>
       </c>
       <c r="L50" s="9">
         <f>IF(OR(I50="",K50=""),"",K50*I50)</f>
-        <v>97510.4</v>
+        <v>92830.4</v>
       </c>
       <c r="M50" s="9">
         <f>IF(L50="","",L50-J50)</f>
-        <v>-2450.95</v>
+        <v>-7130.95</v>
       </c>
       <c r="N50" s="10">
         <f>IF(OR(H50="",K50=""),"",K50/H50-1)</f>
-        <v>-0.024518959409345342</v>
+        <v>-0.07133705542745483</v>
       </c>
       <c r="O50" s="6">
         <f>IF(G50="","",$B$3-G50)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P50" s="6" t="str">
         <f>IF(H50="","Pending buy",IF(N50&gt;=0,"In profit","In loss"))</f>
@@ -3705,23 +3705,23 @@
         <v>97877.65</v>
       </c>
       <c r="K51" s="9" t="n">
-        <v>3074.5</v>
+        <v>3095.9</v>
       </c>
       <c r="L51" s="9">
         <f>IF(OR(I51="",K51=""),"",K51*I51)</f>
-        <v>101458.5</v>
+        <v>102164.7</v>
       </c>
       <c r="M51" s="9">
         <f>IF(L51="","",L51-J51)</f>
-        <v>3580.85</v>
+        <v>4287.05</v>
       </c>
       <c r="N51" s="10">
         <f>IF(OR(H51="",K51=""),"",K51/H51-1)</f>
-        <v>0.036584993748965955</v>
+        <v>0.04380012429579572</v>
       </c>
       <c r="O51" s="6">
         <f>IF(G51="","",$B$3-G51)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P51" s="6" t="str">
         <f>IF(H51="","Pending buy",IF(N51&gt;=0,"In profit","In loss"))</f>
@@ -3773,23 +3773,23 @@
         <v>99357.46</v>
       </c>
       <c r="K52" s="9" t="n">
-        <v>935.6</v>
+        <v>955.6</v>
       </c>
       <c r="L52" s="9">
         <f>IF(OR(I52="",K52=""),"",K52*I52)</f>
-        <v>101980.4</v>
+        <v>104160.4</v>
       </c>
       <c r="M52" s="9">
         <f>IF(L52="","",L52-J52)</f>
-        <v>2622.94</v>
+        <v>4802.94</v>
       </c>
       <c r="N52" s="10">
         <f>IF(OR(H52="",K52=""),"",K52/H52-1)</f>
-        <v>0.026399049372809014</v>
+        <v>0.04834002947911098</v>
       </c>
       <c r="O52" s="6">
         <f>IF(G52="","",$B$3-G52)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P52" s="6" t="str">
         <f>IF(H52="","Pending buy",IF(N52&gt;=0,"In profit","In loss"))</f>
@@ -3841,23 +3841,23 @@
         <v>99747.01</v>
       </c>
       <c r="K53" s="9" t="n">
-        <v>873.6</v>
+        <v>890.5</v>
       </c>
       <c r="L53" s="9">
         <f>IF(OR(I53="",K53=""),"",K53*I53)</f>
-        <v>103084.8</v>
+        <v>105079.0</v>
       </c>
       <c r="M53" s="9">
         <f>IF(L53="","",L53-J53)</f>
-        <v>3337.79</v>
+        <v>5331.99</v>
       </c>
       <c r="N53" s="10">
         <f>IF(OR(H53="",K53=""),"",K53/H53-1)</f>
-        <v>0.03346255945080334</v>
+        <v>0.05345513872589325</v>
       </c>
       <c r="O53" s="6">
         <f>IF(G53="","",$B$3-G53)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P53" s="6" t="str">
         <f>IF(H53="","Pending buy",IF(N53&gt;=0,"In profit","In loss"))</f>
@@ -3909,23 +3909,23 @@
         <v>99711.32</v>
       </c>
       <c r="K54" s="9" t="n">
-        <v>1397.4</v>
+        <v>1415.3</v>
       </c>
       <c r="L54" s="9">
         <f>IF(OR(I54="",K54=""),"",K54*I54)</f>
-        <v>100612.8</v>
+        <v>101901.6</v>
       </c>
       <c r="M54" s="9">
         <f>IF(L54="","",L54-J54)</f>
-        <v>901.48</v>
+        <v>2190.28</v>
       </c>
       <c r="N54" s="10">
         <f>IF(OR(H54="",K54=""),"",K54/H54-1)</f>
-        <v>0.009040924364670966</v>
+        <v>0.021966237479117412</v>
       </c>
       <c r="O54" s="6">
         <f>IF(G54="","",$B$3-G54)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P54" s="6" t="str">
         <f>IF(H54="","Pending buy",IF(N54&gt;=0,"In profit","In loss"))</f>
@@ -3977,27 +3977,27 @@
         <v>98281.27</v>
       </c>
       <c r="K55" s="9" t="n">
-        <v>3860.2</v>
+        <v>3743.8</v>
       </c>
       <c r="L55" s="9">
         <f>IF(OR(I55="",K55=""),"",K55*I55)</f>
-        <v>100365.2</v>
+        <v>97338.8</v>
       </c>
       <c r="M55" s="9">
         <f>IF(L55="","",L55-J55)</f>
-        <v>2083.93</v>
+        <v>-942.47</v>
       </c>
       <c r="N55" s="10">
         <f>IF(OR(H55="",K55=""),"",K55/H55-1)</f>
-        <v>0.021203697443619163</v>
+        <v>-0.009589554300445058</v>
       </c>
       <c r="O55" s="6">
         <f>IF(G55="","",$B$3-G55)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P55" s="6" t="str">
         <f>IF(H55="","Pending buy",IF(N55&gt;=0,"In profit","In loss"))</f>
-        <v>In profit</v>
+        <v>In loss</v>
       </c>
       <c r="Q55" s="6" t="n">
         <v>1</v>
@@ -4045,23 +4045,23 @@
         <v>94906.63</v>
       </c>
       <c r="K56" s="9" t="n">
-        <v>5896</v>
+        <v>5816</v>
       </c>
       <c r="L56" s="9">
         <f>IF(OR(I56="",K56=""),"",K56*I56)</f>
-        <v>94336.0</v>
+        <v>93056.0</v>
       </c>
       <c r="M56" s="9">
         <f>IF(L56="","",L56-J56)</f>
-        <v>-570.63</v>
+        <v>-1850.63</v>
       </c>
       <c r="N56" s="10">
         <f>IF(OR(H56="",K56=""),"",K56/H56-1)</f>
-        <v>-0.006012550173880915</v>
+        <v>-0.019499489791602986</v>
       </c>
       <c r="O56" s="6">
         <f>IF(G56="","",$B$3-G56)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P56" s="6" t="str">
         <f>IF(H56="","Pending buy",IF(N56&gt;=0,"In profit","In loss"))</f>
@@ -4113,23 +4113,23 @@
         <v>99783.3</v>
       </c>
       <c r="K57" s="9" t="n">
-        <v>420.8</v>
+        <v>399.65</v>
       </c>
       <c r="L57" s="9">
         <f>IF(OR(I57="",K57=""),"",K57*I57)</f>
-        <v>98888.0</v>
+        <v>93917.75</v>
       </c>
       <c r="M57" s="9">
         <f>IF(L57="","",L57-J57)</f>
-        <v>-895.3</v>
+        <v>-5865.55</v>
       </c>
       <c r="N57" s="10">
         <f>IF(OR(H57="",K57=""),"",K57/H57-1)</f>
-        <v>-0.008972414730678335</v>
+        <v>-0.05878285538763217</v>
       </c>
       <c r="O57" s="6">
         <f>IF(G57="","",$B$3-G57)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P57" s="6" t="str">
         <f>IF(H57="","Pending buy",IF(N57&gt;=0,"In profit","In loss"))</f>
@@ -4181,23 +4181,23 @@
         <v>99967.09</v>
       </c>
       <c r="K58" s="9" t="n">
-        <v>79.40000000000001</v>
+        <v>78.63</v>
       </c>
       <c r="L58" s="9">
         <f>IF(OR(I58="",K58=""),"",K58*I58)</f>
-        <v>101076.2</v>
+        <v>100095.99</v>
       </c>
       <c r="M58" s="9">
         <f>IF(L58="","",L58-J58)</f>
-        <v>1109.11</v>
+        <v>128.9</v>
       </c>
       <c r="N58" s="10">
         <f>IF(OR(H58="",K58=""),"",K58/H58-1)</f>
-        <v>0.011094765786519467</v>
+        <v>0.001289438712770874</v>
       </c>
       <c r="O58" s="6">
         <f>IF(G58="","",$B$3-G58)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P58" s="6" t="str">
         <f>IF(H58="","Pending buy",IF(N58&gt;=0,"In profit","In loss"))</f>
@@ -4234,38 +4234,42 @@
       <c r="F59" s="8" t="n">
         <v>46324</v>
       </c>
-      <c r="G59" s="6" t="inlineStr"/>
-      <c r="H59" s="9" t="inlineStr"/>
-      <c r="I59" s="6" t="str">
+      <c r="G59" s="8" t="n">
+        <v>46325</v>
+      </c>
+      <c r="H59" s="9" t="n">
+        <v>1269.45</v>
+      </c>
+      <c r="I59" s="6">
         <f>IF(H59="","",ROUNDDOWN($B$1/H59,0))</f>
-        <v/>
-      </c>
-      <c r="J59" s="9" t="str">
+        <v>78</v>
+      </c>
+      <c r="J59" s="9">
         <f>IF(H59="","",H59*I59)</f>
-        <v/>
+        <v>99017.08</v>
       </c>
       <c r="K59" s="9" t="n">
-        <v>1287.4</v>
-      </c>
-      <c r="L59" s="9" t="str">
+        <v>1265</v>
+      </c>
+      <c r="L59" s="9">
         <f>IF(OR(I59="",K59=""),"",K59*I59)</f>
-        <v/>
-      </c>
-      <c r="M59" s="9" t="str">
+        <v>98670.0</v>
+      </c>
+      <c r="M59" s="9">
         <f>IF(L59="","",L59-J59)</f>
-        <v/>
-      </c>
-      <c r="N59" s="10" t="str">
+        <v>-347.08</v>
+      </c>
+      <c r="N59" s="10">
         <f>IF(OR(H59="",K59=""),"",K59/H59-1)</f>
-        <v/>
-      </c>
-      <c r="O59" s="6" t="str">
+        <v>-0.0035052816374550044</v>
+      </c>
+      <c r="O59" s="6">
         <f>IF(G59="","",$B$3-G59)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P59" s="6" t="str">
         <f>IF(H59="","Pending buy",IF(N59&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In loss</v>
       </c>
       <c r="Q59" s="6" t="n">
         <v>1</v>
@@ -4298,38 +4302,42 @@
       <c r="F60" s="8" t="n">
         <v>46324</v>
       </c>
-      <c r="G60" s="6" t="inlineStr"/>
-      <c r="H60" s="9" t="inlineStr"/>
-      <c r="I60" s="6" t="str">
+      <c r="G60" s="8" t="n">
+        <v>46325</v>
+      </c>
+      <c r="H60" s="9" t="n">
+        <v>340.89</v>
+      </c>
+      <c r="I60" s="6">
         <f>IF(H60="","",ROUNDDOWN($B$1/H60,0))</f>
-        <v/>
-      </c>
-      <c r="J60" s="9" t="str">
+        <v>293</v>
+      </c>
+      <c r="J60" s="9">
         <f>IF(H60="","",H60*I60)</f>
-        <v/>
+        <v>99881.81</v>
       </c>
       <c r="K60" s="9" t="n">
-        <v>341.65</v>
-      </c>
-      <c r="L60" s="9" t="str">
+        <v>344.4</v>
+      </c>
+      <c r="L60" s="9">
         <f>IF(OR(I60="",K60=""),"",K60*I60)</f>
-        <v/>
-      </c>
-      <c r="M60" s="9" t="str">
+        <v>100909.2</v>
+      </c>
+      <c r="M60" s="9">
         <f>IF(L60="","",L60-J60)</f>
-        <v/>
-      </c>
-      <c r="N60" s="10" t="str">
+        <v>1027.39</v>
+      </c>
+      <c r="N60" s="10">
         <f>IF(OR(H60="",K60=""),"",K60/H60-1)</f>
-        <v/>
-      </c>
-      <c r="O60" s="6" t="str">
+        <v>0.010286100028268352</v>
+      </c>
+      <c r="O60" s="6">
         <f>IF(G60="","",$B$3-G60)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P60" s="6" t="str">
         <f>IF(H60="","Pending buy",IF(N60&gt;=0,"In profit","In loss"))</f>
-        <v>Pending buy</v>
+        <v>In profit</v>
       </c>
       <c r="Q60" s="6" t="n">
         <v>2</v>

</xml_diff>